<commit_message>
finished almos all the papers´summary
</commit_message>
<xml_diff>
--- a/Papers/Resumen Papers.xlsx
+++ b/Papers/Resumen Papers.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sophiaaristizabal/Documents/GitHub/LLMS_Project/Papers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33C289D6-356E-4347-AB52-44CFC41B1C6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FF8BB10-140D-0343-9A87-B611EBE97255}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16220" activeTab="1" xr2:uid="{400AC57E-08F9-B346-9132-4F74AEBC2D15}"/>
+    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16220" activeTab="3" xr2:uid="{400AC57E-08F9-B346-9132-4F74AEBC2D15}"/>
   </bookViews>
   <sheets>
     <sheet name="MANAGERIAL LEADERSHIP" sheetId="1" r:id="rId1"/>
     <sheet name="Strategic Environment" sheetId="2" r:id="rId2"/>
+    <sheet name="Trust and Promises over Time" sheetId="3" r:id="rId3"/>
+    <sheet name="Underreporting of AI Use" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -72,8 +74,44 @@
 </comments>
 </file>
 
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={9A4E8FE0-8687-DC4A-AC8C-A8F523668577}</author>
+  </authors>
+  <commentList>
+    <comment ref="B20" authorId="0" shapeId="0" xr:uid="{9A4E8FE0-8687-DC4A-AC8C-A8F523668577}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    https://www.aeaweb.org/content/file?id=17090</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={0A408D3A-459E-F246-830F-7CF5C0FA2D8C}</author>
+  </authors>
+  <commentList>
+    <comment ref="B20" authorId="0" shapeId="0" xr:uid="{0A408D3A-459E-F246-830F-7CF5C0FA2D8C}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    https://www.aeaweb.org/content/file?id=17090</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="110">
   <si>
     <t>Autores</t>
   </si>
@@ -1282,12 +1320,618 @@
 Chat-based classification reveals that gradual moves toward cooperation are more common in complementarity settings, while jumps or abrupt decisions are observed in substitution treatments .</t>
     </r>
   </si>
+  <si>
+    <t>Trust and Promises over Time</t>
+  </si>
+  <si>
+    <t>By FLORIAN EDERER AND FRÉDÉRIC SCHNEIDER</t>
+  </si>
+  <si>
+    <t>American Economic Journal: Microeconomics</t>
+  </si>
+  <si>
+    <t>https://www.jstor.org/stable/10.2307/27154558</t>
+  </si>
+  <si>
+    <t>This paper provides the first experimental investigation of the strength of trust, trustworthiness, and promises over time. We document that communication (pri-marily through the use of promises) has a large effect on trust, trustworthiness, and cooperation that remains remarkably persistent over time. Specifically, to investigate how the passage of time affects trust, trustworthiness, and the power of communication (and promises in particular). We find that preplay communication raises cooperation by about 50 percent.
+More importantly, we document that the increase in cooperation, trust, and trustworthiness resulting from communication is not diminished even when three weeks pass before the trustee's actual decision. Thus, we provide evidence for the lasting power of communication and of promises in particular.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>El experimento se basa en el trust game de Charness &amp; Dufwenberg (2006), jugado una sola vez y entre dos personas:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Trustor (él)
+Trustee (ella)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2. Estructura del juego</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+El trustor decide entre:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">OUT: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">ambos reciben $15.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>IN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: pasa el turno a la trustee.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Si el trustor elige IN, la trustee decide entre:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DON’T ROLL</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: ella recibe $42, el trustor $0. (La opción egoísta)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ROLL</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: ella recibe $30 y el trustor obtiene:
+$36 con prob. 5/6,
+$0 con prob. 1/6.
+Elegir IN requiere confianza de que la trustee elegirá ROLL, ya que DON’T ROLL es el comportamiento egoísta dominante.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3. Tratamientos de comunicación (siguiendo C&amp;D 2006)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Antes de que el trustor tome su decisión, se introduce un posible mensaje de la trustee:
+COMM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: la trustee puede escribir un mensaje libre.
+Puede prometer explícitamente que elegirá ROLL.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NOCOMM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: no hay comunicación.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Importante:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+El trustor nunca observa la acción real de la trustee; solo su propio pago. Si recibe $0, puede deberse a que ella eligió DON’T ROLL o a que ella eligió ROLL pero salió la mala suerte (1/6). Esto genera incertidumbre estratégica e inferencia sobre intenciones.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4. Información de la trustee al tomar decisiones</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+La trustee no sabe si el trustor eligió IN u OUT cuando elige entre ROLL y DON’T ROLL.
+Esto permite recoger decisiones de todas las trustees, independientemente de si fueron efectivamente “activadas”.</t>
+    </r>
+  </si>
+  <si>
+    <t>we analyze the behavior of over 700 subjects in a one-shot, two-person trust game with and without preplay communication. 40 experimental sessions with a total of 707 student subjects at the University of Zurich and at Yale University.</t>
+  </si>
+  <si>
+    <t>messages were classified according to whether they contained an explicit promise of choosing ROLL (e.g., “I will choose ROLL” or “I promise to choose ROLL”) or whether they did not (e.g., “a singer in a smoky room, a smell of wine and cheap perfume”)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> “Promise,”</t>
+  </si>
+  <si>
+    <t>“Other Content,”</t>
+  </si>
+  <si>
+    <t>“No Message.”</t>
+  </si>
+  <si>
+    <t>Two ­ hypothesis-blind research assistants classified the messages independently. received a monetary incentive for indicating the same categories as the other coder.
+The correlation between the two research assistants was high (for the Promise category, Pearson correlation is 0.87 and Cronbach’s α = 0.93).</t>
+  </si>
+  <si>
+    <t>3  We allowed three levels for the coding: 0 (category not present in message); 1 (category somewhat present in message); 2 (category strongly present in message).</t>
+  </si>
+  <si>
+    <t>We classified a message as a promise if both assistants coded the message as such</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sistema de clasificación humana (gold standard) APPENDIX </t>
+  </si>
+  <si>
+    <t>Underreporting of AI Use: The Role of Social Desirability Bias</t>
+  </si>
+  <si>
+    <t>Yier Ling, Alex Kale, Alex Imas</t>
+  </si>
+  <si>
+    <t>http://dx.doi.org/10.2139/ssrn.5464215</t>
+  </si>
+  <si>
+    <t>SSRN</t>
+  </si>
+  <si>
+    <t>This study looks into how people might not always admit to using AI, especially in schools, because they want to avoid judgment. It shows that when students are asked about their own AI use versus their peers’, they tend to underreport their own use by a lot.
+about 60% say they use AI, while 90% say their friends do. This gap points to a social desirability bias where folks shape their answers to look better or avoid criticism.
+Self-reports on AI use can be way off because of wanting to appear socially acceptable.
+In education, admitting to using AI might be seen as cheating or lowering one’s credibility.
+A smarter survey method that asks about others helps reveal the real usage rates.</t>
+  </si>
+  <si>
+    <t>The primary participant population in this experiment consisted of undergraduate students from a medium-sized Midwestern university. Specifically, the sample size for the main survey was 338 students after data cleaning, and among these, about 76.3% reported at least one STEM major.</t>
+  </si>
+  <si>
+    <t>In the main survey, participants answered questions regarding their own AI reliance and frequency of use, as well as their perceptions of their peers’ AI usage. The survey included direct questions about whether students used LLMs, how often, and why they might report different usage levels for themselves versus others. The responses about reliance and frequency were then analyzed statistically, with logistic regression used to examine factors influencing reported AI use, including gender, major, and the nature of the report (self vs. peer).
+Following this, a follow-up survey was conducted with a separate sample of 96 undergraduate students recruited via Prolific. This phase aimed to explore reasons behind the observed reporting gap. Participants were shown initial findings from the first survey and then asked open-ended and multiple-choice questions about their explanations for this gap, such as social desirability bias or lack of knowledge about others’ AI use. The qualitative responses were analyzed via thematic coding to categorize explanations</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Dependent Variables:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Self-reported AI use: Whether students report using large language models (LLMs), including reliance level and frequency of use (e.g., days per week). This was often binarized into “use” vs. “no use” for analysis.
+Perceived peer AI use: Participants’ reports about their peers’ reliance and frequency of AI use, including categorical levels and estimated percentages.
+Reporting gap: The difference between self-reported and peer-reported AI use, analyzed both quantitatively (via regression) and qualitatively (explanations).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Independent Variables:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Report type: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Whether the response pertains to personal use (“own”) or perceived peer use (“others”).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Gender: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Participant gender identity.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Major: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Whether the participant is in a STEM major or not.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Interactions: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Interactions between report type, gender, and major to analyze differential effects.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Other measured variables include:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Reasons for the reporting gap: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Qualitative categories such as embarrassment, lack of knowledge, social desirability bias, or inflation.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Participant demographics: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Age, year in college, race, ethnicity, international status, English first language, family income, and part-time work related or unrelated to their major. These were collected via demographic questionnaires.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">In this survey, we first described to participants the findings from the initial student survey, showing both the percentage of students’ own self-reported reliance and frequency of AI use as well as their answers about peer use.
+All participants were then asked three questions about this gap. The first question was a free-text entry directly asking for their explanation of the gap. The second question asked whether they believed this gap was due to the overreporting of others’ use or the underreporting the students’ own use. The last question asked participants to choose the most likely explanation: students being embarrassed to admit LLM use; students inflate others’ use; students are unaware of others’ use; and none of the above.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Initial Coding Process:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+The first author conducted open coding to identify initial descriptive categories based on the responses.
+All authors then discussed these initial codes to agree on a set of inductive, mutually exclusive categories that best captured the themes in the responses.
+The first author recoded responses according to these refined codes, iterating as necessary to ensure clarity and consistency.
+Among 96 respondents, 71 provide valid responses; 25 are removed for providing nonsensical responses (e.g., random integers), or for implying that they misunderstood or were confused by the question (e.g., explaining a reporting gap in the reverse direction).</t>
+    </r>
+  </si>
+  <si>
+    <t>The researchers</t>
+  </si>
+  <si>
+    <t>Social Desirability Bias</t>
+  </si>
+  <si>
+    <t>Overestimating Others’ Usage</t>
+  </si>
+  <si>
+    <t>Information Asymmetry</t>
+  </si>
+  <si>
+    <t>Underestimating Own Usage</t>
+  </si>
+  <si>
+    <t>Self-esteem</t>
+  </si>
+  <si>
+    <t>Privacy Concerns</t>
+  </si>
+  <si>
+    <t>Self-reporting Bias</t>
+  </si>
+  <si>
+    <t>Truthful Reporting</t>
+  </si>
+  <si>
+    <t>Believe the reporting gap accurately reflects a gap in AI usage between survey respondents and their peers, and the students were truthfully reporting.</t>
+  </si>
+  <si>
+    <t>Definición (that's what it was said in the paper)</t>
+  </si>
+  <si>
+    <t>The underreporting can be an outcome of students exhibiting a self-favoring bias when reporting.</t>
+  </si>
+  <si>
+    <t>privacy concerns as a reason behind the underreporting of own AI usage</t>
+  </si>
+  <si>
+    <t>students may underreport their AI usage to protect their self-esteem, a motivation similar to SDB but different in caring about students’ self-image</t>
+  </si>
+  <si>
+    <t>students may be underestimating. their true AI usage</t>
+  </si>
+  <si>
+    <t>students are unaware of other students’ actual AI adoption</t>
+  </si>
+  <si>
+    <t>A varied range of sources of social desirability associated with reporting AI usage are provided by the respondents
+as well. Academic integrity concerns, such as casting AI usage as cheating or dishonest, is most frequently mentioned</t>
+  </si>
+  <si>
+    <t>The reporting gap is overestimation of others’ usage (22/71). Among these participants, multiple respondents suggest that this overestimation could come from biased perception: students are “primed” by AI reliance in certain groups and overgeneralize it to all other students</t>
+  </si>
+  <si>
+    <t>Majority Attribution to Social Desirability Bias: Most participants (around 70%) explained the reporting gap between their own and others' AI use as due to embarrassment or shame—indicating that students are underreporting their own AI use because of social stigma or moral concerns .
+Perception of Peer Use: Participants tend to overestimate others’ AI use, attributing higher AI reliance to peers than to themselves, which is consistent with availability bias and social perceptions .
+Explanations Focused on Self-Reporting Concerns: Free-text responses and forced-choice questions primarily reflect moral panic or social norms that discourage openly admitting to AI use, pointing to moral or ethical concerns as barriers to honest self-reporting  .
+Biases in Self- and Peer-Reporting: The research uncovers that social desirability bias drives underreporting of own AI use, especially in educational settings where stigma is high, leading to significant measurement error in self-reported data</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1329,14 +1973,8 @@
       <color theme="1"/>
       <name val="Aptos Narrow (Body)"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1359,6 +1997,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF002060"/>
         <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1515,133 +2165,205 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1649,56 +2371,32 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -1706,53 +2404,35 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2262,6 +2942,34 @@
 </ThreadedComments>
 </file>
 
+<file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="B20" dT="2025-11-25T06:22:34.58" personId="{8E3B53E8-6818-164C-AE00-EDEC79BF3325}" id="{9A4E8FE0-8687-DC4A-AC8C-A8F523668577}">
+    <text>https://www.aeaweb.org/content/file?id=17090</text>
+    <extLst>
+      <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
+        <xltc2:checksum>1271413348</xltc2:checksum>
+        <xltc2:hyperlink startIndex="0" length="44" url="https://www.aeaweb.org/content/file?id=17090"/>
+      </x:ext>
+    </extLst>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment4.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="B20" dT="2025-11-25T06:22:34.58" personId="{8E3B53E8-6818-164C-AE00-EDEC79BF3325}" id="{0A408D3A-459E-F246-830F-7CF5C0FA2D8C}">
+    <text>https://www.aeaweb.org/content/file?id=17090</text>
+    <extLst>
+      <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
+        <xltc2:checksum>1271413348</xltc2:checksum>
+        <xltc2:hyperlink startIndex="0" length="44" url="https://www.aeaweb.org/content/file?id=17090"/>
+      </x:ext>
+    </extLst>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F9C7557-9F52-EA41-8CAF-23F9F254837D}">
   <dimension ref="B2:I40"/>
@@ -2275,537 +2983,523 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="57" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="58" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="58"/>
+      <c r="H4" s="58"/>
+      <c r="I4" s="58"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="50">
         <v>2025</v>
       </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
+      <c r="D5" s="50"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="50"/>
+      <c r="G5" s="50"/>
+      <c r="H5" s="50"/>
+      <c r="I5" s="50"/>
     </row>
     <row r="6" spans="2:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
+      <c r="D6" s="50"/>
+      <c r="E6" s="50"/>
+      <c r="F6" s="50"/>
+      <c r="G6" s="50"/>
+      <c r="H6" s="50"/>
+      <c r="I6" s="50"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="59" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
+      <c r="D7" s="50"/>
+      <c r="E7" s="50"/>
+      <c r="F7" s="50"/>
+      <c r="G7" s="50"/>
+      <c r="H7" s="50"/>
+      <c r="I7" s="50"/>
     </row>
     <row r="8" spans="2:9" ht="9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
     </row>
     <row r="9" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
+      <c r="C9" s="46"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="46"/>
+      <c r="F9" s="46"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="46"/>
+      <c r="I9" s="46"/>
     </row>
     <row r="10" spans="2:9" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
-      <c r="I10" s="21"/>
+      <c r="C10" s="47"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="47"/>
+      <c r="G10" s="47"/>
+      <c r="H10" s="47"/>
+      <c r="I10" s="47"/>
     </row>
     <row r="11" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="21"/>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="21"/>
-      <c r="G11" s="21"/>
-      <c r="H11" s="21"/>
-      <c r="I11" s="21"/>
+      <c r="B11" s="47"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47"/>
+      <c r="F11" s="47"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="47"/>
+      <c r="I11" s="47"/>
     </row>
     <row r="12" spans="2:9" ht="11" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="21"/>
-      <c r="C12" s="21"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21"/>
-      <c r="G12" s="21"/>
-      <c r="H12" s="21"/>
-      <c r="I12" s="21"/>
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="47"/>
+      <c r="F12" s="47"/>
+      <c r="G12" s="47"/>
+      <c r="H12" s="47"/>
+      <c r="I12" s="47"/>
     </row>
     <row r="13" spans="2:9" ht="9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
+      <c r="C14" s="46"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="46"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="46"/>
+      <c r="I14" s="46"/>
     </row>
     <row r="15" spans="2:9" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="23" t="s">
+      <c r="B15" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="49" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
+      <c r="D15" s="50"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="50"/>
+      <c r="G15" s="50"/>
+      <c r="H15" s="50"/>
+      <c r="I15" s="50"/>
     </row>
     <row r="16" spans="2:9" ht="125" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="19" t="s">
+      <c r="C16" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="15"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="38"/>
+      <c r="G16" s="38"/>
+      <c r="H16" s="38"/>
+      <c r="I16" s="39"/>
     </row>
     <row r="17" spans="2:9" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="26"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="17"/>
-      <c r="I17" s="18"/>
+      <c r="B17" s="36"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="41"/>
+      <c r="F17" s="41"/>
+      <c r="G17" s="41"/>
+      <c r="H17" s="41"/>
+      <c r="I17" s="42"/>
     </row>
     <row r="18" spans="2:9" ht="67" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
+      <c r="D18" s="50"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="50"/>
+      <c r="G18" s="50"/>
+      <c r="H18" s="50"/>
+      <c r="I18" s="50"/>
     </row>
     <row r="19" spans="2:9" ht="7" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="26"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
+      <c r="C20" s="46"/>
+      <c r="D20" s="46"/>
+      <c r="E20" s="46"/>
+      <c r="F20" s="46"/>
+      <c r="G20" s="46"/>
+      <c r="H20" s="46"/>
+      <c r="I20" s="46"/>
     </row>
     <row r="21" spans="2:9" ht="43" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="22" t="s">
+      <c r="B21" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="35" t="s">
+      <c r="C21" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="33"/>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="33"/>
-      <c r="H21" s="33"/>
-      <c r="I21" s="34"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="30"/>
+      <c r="F21" s="30"/>
+      <c r="G21" s="30"/>
+      <c r="H21" s="30"/>
+      <c r="I21" s="31"/>
     </row>
     <row r="22" spans="2:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="30">
+      <c r="C22" s="32">
         <v>9</v>
       </c>
-      <c r="D22" s="31"/>
-      <c r="E22" s="31"/>
-      <c r="F22" s="31"/>
-      <c r="G22" s="31"/>
-      <c r="H22" s="31"/>
-      <c r="I22" s="32"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="34"/>
     </row>
     <row r="23" spans="2:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="12" t="s">
+      <c r="C23" s="55" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="12"/>
-      <c r="E23" s="6" t="s">
+      <c r="D23" s="55"/>
+      <c r="E23" s="56" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
+      <c r="F23" s="56"/>
+      <c r="G23" s="56"/>
+      <c r="H23" s="56"/>
+      <c r="I23" s="56"/>
     </row>
     <row r="24" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="41">
+      <c r="B24" s="6">
         <v>1</v>
       </c>
-      <c r="C24" s="45" t="s">
+      <c r="C24" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="D24" s="48"/>
-      <c r="E24" s="35" t="s">
+      <c r="D24" s="23"/>
+      <c r="E24" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="F24" s="46"/>
-      <c r="G24" s="46"/>
-      <c r="H24" s="46"/>
-      <c r="I24" s="47"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="20"/>
+      <c r="H24" s="20"/>
+      <c r="I24" s="21"/>
     </row>
     <row r="25" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="41">
+      <c r="B25" s="6">
         <v>2</v>
       </c>
-      <c r="C25" s="45" t="s">
+      <c r="C25" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="D25" s="48"/>
-      <c r="E25" s="45"/>
-      <c r="F25" s="49"/>
-      <c r="G25" s="49"/>
-      <c r="H25" s="49"/>
-      <c r="I25" s="48"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="24"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="24"/>
+      <c r="I25" s="23"/>
     </row>
     <row r="26" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="57">
+      <c r="B26" s="7">
         <v>3</v>
       </c>
-      <c r="C26" s="50" t="s">
+      <c r="C26" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D26" s="51"/>
-      <c r="E26" s="38" t="s">
+      <c r="D26" s="10"/>
+      <c r="E26" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="F26" s="38"/>
-      <c r="G26" s="49" t="s">
+      <c r="F26" s="25"/>
+      <c r="G26" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="H26" s="49"/>
-      <c r="I26" s="48"/>
+      <c r="H26" s="24"/>
+      <c r="I26" s="23"/>
     </row>
     <row r="27" spans="2:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="58"/>
-      <c r="C27" s="52"/>
-      <c r="D27" s="53"/>
-      <c r="E27" s="39" t="s">
+      <c r="B27" s="8"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="F27" s="40"/>
-      <c r="G27" s="54" t="s">
+      <c r="F27" s="14"/>
+      <c r="G27" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="H27" s="55"/>
-      <c r="I27" s="56"/>
+      <c r="H27" s="16"/>
+      <c r="I27" s="17"/>
     </row>
     <row r="28" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="41">
+      <c r="B28" s="6">
         <v>4</v>
       </c>
-      <c r="C28" s="39" t="s">
+      <c r="C28" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="D28" s="40"/>
-      <c r="E28" s="27" t="s">
+      <c r="D28" s="14"/>
+      <c r="E28" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="F28" s="33"/>
-      <c r="G28" s="33"/>
-      <c r="H28" s="33"/>
-      <c r="I28" s="34"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="H28" s="30"/>
+      <c r="I28" s="31"/>
     </row>
     <row r="29" spans="2:9" ht="43" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="41">
+      <c r="B29" s="6">
         <v>5</v>
       </c>
-      <c r="C29" s="38" t="s">
+      <c r="C29" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="D29" s="38"/>
-      <c r="E29" s="36" t="s">
+      <c r="D29" s="25"/>
+      <c r="E29" s="51" t="s">
         <v>33</v>
       </c>
-      <c r="F29" s="36"/>
-      <c r="G29" s="36"/>
-      <c r="H29" s="36"/>
-      <c r="I29" s="36"/>
+      <c r="F29" s="51"/>
+      <c r="G29" s="51"/>
+      <c r="H29" s="51"/>
+      <c r="I29" s="51"/>
     </row>
     <row r="30" spans="2:9" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="41">
+      <c r="B30" s="6">
         <v>6</v>
       </c>
-      <c r="C30" s="39" t="s">
+      <c r="C30" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="D30" s="40"/>
-      <c r="E30" s="27" t="s">
+      <c r="D30" s="14"/>
+      <c r="E30" s="43" t="s">
         <v>34</v>
       </c>
-      <c r="F30" s="28"/>
-      <c r="G30" s="28"/>
-      <c r="H30" s="28"/>
-      <c r="I30" s="29"/>
+      <c r="F30" s="44"/>
+      <c r="G30" s="44"/>
+      <c r="H30" s="44"/>
+      <c r="I30" s="45"/>
     </row>
     <row r="31" spans="2:9" ht="53" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="41">
+      <c r="B31" s="6">
         <v>7</v>
       </c>
-      <c r="C31" s="38" t="s">
+      <c r="C31" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="D31" s="38"/>
-      <c r="E31" s="36" t="s">
+      <c r="D31" s="25"/>
+      <c r="E31" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="F31" s="37"/>
-      <c r="G31" s="37"/>
-      <c r="H31" s="37"/>
-      <c r="I31" s="37"/>
+      <c r="F31" s="52"/>
+      <c r="G31" s="52"/>
+      <c r="H31" s="52"/>
+      <c r="I31" s="52"/>
     </row>
     <row r="32" spans="2:9" ht="53" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="41">
+      <c r="B32" s="6">
         <v>8</v>
       </c>
-      <c r="C32" s="39" t="s">
+      <c r="C32" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="D32" s="40"/>
-      <c r="E32" s="39"/>
-      <c r="F32" s="59"/>
-      <c r="G32" s="59"/>
-      <c r="H32" s="59"/>
-      <c r="I32" s="40"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="13"/>
+      <c r="F32" s="18"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="18"/>
+      <c r="I32" s="14"/>
     </row>
     <row r="33" spans="2:9" ht="102" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="41">
+      <c r="B33" s="6">
         <v>9</v>
       </c>
-      <c r="C33" s="39" t="s">
+      <c r="C33" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="D33" s="40"/>
-      <c r="E33" s="30" t="s">
+      <c r="D33" s="14"/>
+      <c r="E33" s="32" t="s">
         <v>46</v>
       </c>
-      <c r="F33" s="60"/>
-      <c r="G33" s="60"/>
-      <c r="H33" s="60"/>
-      <c r="I33" s="61"/>
+      <c r="F33" s="53"/>
+      <c r="G33" s="53"/>
+      <c r="H33" s="53"/>
+      <c r="I33" s="54"/>
     </row>
     <row r="34" spans="2:9" ht="190" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="24" t="s">
+      <c r="B34" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C34" s="36" t="s">
+      <c r="C34" s="51" t="s">
         <v>31</v>
       </c>
-      <c r="D34" s="36"/>
-      <c r="E34" s="36"/>
-      <c r="F34" s="36"/>
-      <c r="G34" s="36"/>
-      <c r="H34" s="36"/>
-      <c r="I34" s="36"/>
+      <c r="D34" s="51"/>
+      <c r="E34" s="51"/>
+      <c r="F34" s="51"/>
+      <c r="G34" s="51"/>
+      <c r="H34" s="51"/>
+      <c r="I34" s="51"/>
     </row>
     <row r="35" spans="2:9" ht="10" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="9"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10"/>
-      <c r="H35" s="10"/>
-      <c r="I35" s="11"/>
+      <c r="B35" s="27"/>
+      <c r="C35" s="28"/>
+      <c r="D35" s="28"/>
+      <c r="E35" s="28"/>
+      <c r="F35" s="28"/>
+      <c r="G35" s="28"/>
+      <c r="H35" s="28"/>
+      <c r="I35" s="29"/>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
+      <c r="C36" s="46"/>
+      <c r="D36" s="46"/>
+      <c r="E36" s="46"/>
+      <c r="F36" s="46"/>
+      <c r="G36" s="46"/>
+      <c r="H36" s="46"/>
+      <c r="I36" s="46"/>
     </row>
     <row r="37" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="20" t="s">
+      <c r="B37" s="48" t="s">
         <v>48</v>
       </c>
-      <c r="C37" s="20"/>
-      <c r="D37" s="20"/>
-      <c r="E37" s="20"/>
-      <c r="F37" s="20"/>
-      <c r="G37" s="20"/>
-      <c r="H37" s="20"/>
-      <c r="I37" s="20"/>
+      <c r="C37" s="48"/>
+      <c r="D37" s="48"/>
+      <c r="E37" s="48"/>
+      <c r="F37" s="48"/>
+      <c r="G37" s="48"/>
+      <c r="H37" s="48"/>
+      <c r="I37" s="48"/>
     </row>
     <row r="38" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="20"/>
-      <c r="C38" s="20"/>
-      <c r="D38" s="20"/>
-      <c r="E38" s="20"/>
-      <c r="F38" s="20"/>
-      <c r="G38" s="20"/>
-      <c r="H38" s="20"/>
-      <c r="I38" s="20"/>
+      <c r="B38" s="48"/>
+      <c r="C38" s="48"/>
+      <c r="D38" s="48"/>
+      <c r="E38" s="48"/>
+      <c r="F38" s="48"/>
+      <c r="G38" s="48"/>
+      <c r="H38" s="48"/>
+      <c r="I38" s="48"/>
     </row>
     <row r="39" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="20"/>
-      <c r="C39" s="20"/>
-      <c r="D39" s="20"/>
-      <c r="E39" s="20"/>
-      <c r="F39" s="20"/>
-      <c r="G39" s="20"/>
-      <c r="H39" s="20"/>
-      <c r="I39" s="20"/>
+      <c r="B39" s="48"/>
+      <c r="C39" s="48"/>
+      <c r="D39" s="48"/>
+      <c r="E39" s="48"/>
+      <c r="F39" s="48"/>
+      <c r="G39" s="48"/>
+      <c r="H39" s="48"/>
+      <c r="I39" s="48"/>
     </row>
     <row r="40" spans="2:9" ht="76" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B40" s="20"/>
-      <c r="C40" s="20"/>
-      <c r="D40" s="20"/>
-      <c r="E40" s="20"/>
-      <c r="F40" s="20"/>
-      <c r="G40" s="20"/>
-      <c r="H40" s="20"/>
-      <c r="I40" s="20"/>
+      <c r="B40" s="48"/>
+      <c r="C40" s="48"/>
+      <c r="D40" s="48"/>
+      <c r="E40" s="48"/>
+      <c r="F40" s="48"/>
+      <c r="G40" s="48"/>
+      <c r="H40" s="48"/>
+      <c r="I40" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="C26:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="E32:I32"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="B35:I35"/>
-    <mergeCell ref="B13:I13"/>
-    <mergeCell ref="C21:I21"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="C6:I6"/>
     <mergeCell ref="B36:I36"/>
     <mergeCell ref="B10:I12"/>
     <mergeCell ref="B9:I9"/>
@@ -2822,17 +3516,31 @@
     <mergeCell ref="C28:D28"/>
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="C31:D31"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:I30"/>
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="B14:I14"/>
     <mergeCell ref="B20:I20"/>
     <mergeCell ref="C23:D23"/>
     <mergeCell ref="E23:I23"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="C3:I3"/>
-    <mergeCell ref="C4:I4"/>
-    <mergeCell ref="C5:I5"/>
-    <mergeCell ref="C6:I6"/>
-    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="C26:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="E32:I32"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{C9E9977D-5134-FE4B-852F-8DEBDCB543E0}"/>
@@ -2856,433 +3564,433 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="62" t="s">
+      <c r="C3" s="78" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
-      <c r="I3" s="63"/>
+      <c r="D3" s="79"/>
+      <c r="E3" s="79"/>
+      <c r="F3" s="79"/>
+      <c r="G3" s="79"/>
+      <c r="H3" s="79"/>
+      <c r="I3" s="79"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="50" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
+      <c r="D4" s="50"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="50"/>
+      <c r="G4" s="50"/>
+      <c r="H4" s="50"/>
+      <c r="I4" s="50"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="50">
         <v>2020</v>
       </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
+      <c r="D5" s="50"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="50"/>
+      <c r="G5" s="50"/>
+      <c r="H5" s="50"/>
+      <c r="I5" s="50"/>
     </row>
     <row r="6" spans="2:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="37" t="s">
+      <c r="C6" s="52" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="37"/>
-      <c r="I6" s="37"/>
+      <c r="D6" s="52"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="52"/>
+      <c r="I6" s="52"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="59" t="s">
         <v>51</v>
       </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
+      <c r="D7" s="50"/>
+      <c r="E7" s="50"/>
+      <c r="F7" s="50"/>
+      <c r="G7" s="50"/>
+      <c r="H7" s="50"/>
+      <c r="I7" s="50"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
+      <c r="C9" s="46"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="46"/>
+      <c r="F9" s="46"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="46"/>
+      <c r="I9" s="46"/>
     </row>
     <row r="10" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="47" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
-      <c r="I10" s="21"/>
+      <c r="C10" s="47"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="47"/>
+      <c r="G10" s="47"/>
+      <c r="H10" s="47"/>
+      <c r="I10" s="47"/>
     </row>
     <row r="11" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="21"/>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="21"/>
-      <c r="G11" s="21"/>
-      <c r="H11" s="21"/>
-      <c r="I11" s="21"/>
+      <c r="B11" s="47"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47"/>
+      <c r="F11" s="47"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="47"/>
+      <c r="I11" s="47"/>
     </row>
     <row r="12" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="21"/>
-      <c r="C12" s="21"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21"/>
-      <c r="G12" s="21"/>
-      <c r="H12" s="21"/>
-      <c r="I12" s="21"/>
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="47"/>
+      <c r="F12" s="47"/>
+      <c r="G12" s="47"/>
+      <c r="H12" s="47"/>
+      <c r="I12" s="47"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
+      <c r="C14" s="46"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="46"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="46"/>
+      <c r="I14" s="46"/>
     </row>
     <row r="15" spans="2:9" ht="64" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="23" t="s">
+      <c r="B15" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="49" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
+      <c r="D15" s="50"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="50"/>
+      <c r="G15" s="50"/>
+      <c r="H15" s="50"/>
+      <c r="I15" s="50"/>
     </row>
     <row r="16" spans="2:9" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="64" t="s">
+      <c r="C16" s="69" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="65"/>
-      <c r="E16" s="65"/>
-      <c r="F16" s="65"/>
-      <c r="G16" s="65"/>
-      <c r="H16" s="65"/>
-      <c r="I16" s="66"/>
+      <c r="D16" s="70"/>
+      <c r="E16" s="70"/>
+      <c r="F16" s="70"/>
+      <c r="G16" s="70"/>
+      <c r="H16" s="70"/>
+      <c r="I16" s="71"/>
     </row>
     <row r="17" spans="2:9" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="26"/>
-      <c r="C17" s="67"/>
-      <c r="D17" s="68"/>
-      <c r="E17" s="68"/>
-      <c r="F17" s="68"/>
-      <c r="G17" s="68"/>
-      <c r="H17" s="68"/>
-      <c r="I17" s="69"/>
+      <c r="B17" s="36"/>
+      <c r="C17" s="72"/>
+      <c r="D17" s="73"/>
+      <c r="E17" s="73"/>
+      <c r="F17" s="73"/>
+      <c r="G17" s="73"/>
+      <c r="H17" s="73"/>
+      <c r="I17" s="74"/>
     </row>
     <row r="18" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="49" t="s">
         <v>56</v>
       </c>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
+      <c r="D18" s="50"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="50"/>
+      <c r="G18" s="50"/>
+      <c r="H18" s="50"/>
+      <c r="I18" s="50"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="26"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
+      <c r="C20" s="46"/>
+      <c r="D20" s="46"/>
+      <c r="E20" s="46"/>
+      <c r="F20" s="46"/>
+      <c r="G20" s="46"/>
+      <c r="H20" s="46"/>
+      <c r="I20" s="46"/>
     </row>
     <row r="21" spans="2:9" ht="160" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="24" t="s">
+      <c r="B21" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="70" t="s">
+      <c r="C21" s="75" t="s">
         <v>57</v>
       </c>
-      <c r="D21" s="71"/>
-      <c r="E21" s="71"/>
-      <c r="F21" s="71"/>
-      <c r="G21" s="71"/>
-      <c r="H21" s="71"/>
-      <c r="I21" s="72"/>
+      <c r="D21" s="76"/>
+      <c r="E21" s="76"/>
+      <c r="F21" s="76"/>
+      <c r="G21" s="76"/>
+      <c r="H21" s="76"/>
+      <c r="I21" s="77"/>
     </row>
     <row r="22" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B22" s="41" t="s">
+      <c r="B22" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="30">
+      <c r="C22" s="32">
         <v>3</v>
       </c>
-      <c r="D22" s="31"/>
-      <c r="E22" s="31"/>
-      <c r="F22" s="31"/>
-      <c r="G22" s="31"/>
-      <c r="H22" s="31"/>
-      <c r="I22" s="32"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="34"/>
     </row>
     <row r="23" spans="2:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="12" t="s">
+      <c r="C23" s="55" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="12"/>
-      <c r="E23" s="6" t="s">
+      <c r="D23" s="55"/>
+      <c r="E23" s="56" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
+      <c r="F23" s="56"/>
+      <c r="G23" s="56"/>
+      <c r="H23" s="56"/>
+      <c r="I23" s="56"/>
     </row>
     <row r="24" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="57">
+      <c r="B24" s="7">
         <v>1</v>
       </c>
-      <c r="C24" s="73" t="s">
+      <c r="C24" s="60" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="74"/>
-      <c r="E24" s="42" t="s">
+      <c r="D24" s="61"/>
+      <c r="E24" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F24" s="77" t="s">
+      <c r="F24" s="64" t="s">
         <v>63</v>
       </c>
-      <c r="G24" s="77"/>
-      <c r="H24" s="77"/>
-      <c r="I24" s="78"/>
+      <c r="G24" s="64"/>
+      <c r="H24" s="64"/>
+      <c r="I24" s="65"/>
     </row>
     <row r="25" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="58"/>
-      <c r="C25" s="75"/>
-      <c r="D25" s="76"/>
-      <c r="E25" s="42" t="s">
+      <c r="B25" s="8"/>
+      <c r="C25" s="62"/>
+      <c r="D25" s="63"/>
+      <c r="E25" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="F25" s="49" t="s">
+      <c r="F25" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="G25" s="49"/>
-      <c r="H25" s="49"/>
-      <c r="I25" s="48"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="24"/>
+      <c r="I25" s="23"/>
     </row>
     <row r="26" spans="2:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="41">
+      <c r="B26" s="6">
         <v>2</v>
       </c>
-      <c r="C26" s="43" t="s">
+      <c r="C26" s="67" t="s">
         <v>59</v>
       </c>
-      <c r="D26" s="44"/>
-      <c r="E26" s="39"/>
-      <c r="F26" s="59"/>
-      <c r="G26" s="59"/>
-      <c r="H26" s="59"/>
-      <c r="I26" s="40"/>
+      <c r="D26" s="68"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="18"/>
+      <c r="I26" s="14"/>
     </row>
     <row r="27" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="41">
+      <c r="B27" s="6">
         <v>3</v>
       </c>
-      <c r="C27" s="75" t="s">
+      <c r="C27" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="D27" s="76"/>
-      <c r="E27" s="39"/>
-      <c r="F27" s="59"/>
-      <c r="G27" s="59"/>
-      <c r="H27" s="59"/>
-      <c r="I27" s="40"/>
+      <c r="D27" s="63"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="18"/>
+      <c r="H27" s="18"/>
+      <c r="I27" s="14"/>
     </row>
     <row r="28" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B28" s="24" t="s">
+      <c r="B28" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C28" s="36" t="s">
+      <c r="C28" s="51" t="s">
         <v>65</v>
       </c>
-      <c r="D28" s="36"/>
-      <c r="E28" s="36"/>
-      <c r="F28" s="36"/>
-      <c r="G28" s="36"/>
-      <c r="H28" s="36"/>
-      <c r="I28" s="36"/>
+      <c r="D28" s="51"/>
+      <c r="E28" s="51"/>
+      <c r="F28" s="51"/>
+      <c r="G28" s="51"/>
+      <c r="H28" s="51"/>
+      <c r="I28" s="51"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B29" s="9"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10"/>
-      <c r="G29" s="10"/>
-      <c r="H29" s="10"/>
-      <c r="I29" s="11"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="28"/>
+      <c r="F29" s="28"/>
+      <c r="G29" s="28"/>
+      <c r="H29" s="28"/>
+      <c r="I29" s="29"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
+      <c r="C30" s="46"/>
+      <c r="D30" s="46"/>
+      <c r="E30" s="46"/>
+      <c r="F30" s="46"/>
+      <c r="G30" s="46"/>
+      <c r="H30" s="46"/>
+      <c r="I30" s="46"/>
     </row>
     <row r="31" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="79" t="s">
+      <c r="B31" s="66" t="s">
         <v>66</v>
       </c>
-      <c r="C31" s="20"/>
-      <c r="D31" s="20"/>
-      <c r="E31" s="20"/>
-      <c r="F31" s="20"/>
-      <c r="G31" s="20"/>
-      <c r="H31" s="20"/>
-      <c r="I31" s="20"/>
+      <c r="C31" s="48"/>
+      <c r="D31" s="48"/>
+      <c r="E31" s="48"/>
+      <c r="F31" s="48"/>
+      <c r="G31" s="48"/>
+      <c r="H31" s="48"/>
+      <c r="I31" s="48"/>
     </row>
     <row r="32" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
-      <c r="D32" s="20"/>
-      <c r="E32" s="20"/>
-      <c r="F32" s="20"/>
-      <c r="G32" s="20"/>
-      <c r="H32" s="20"/>
-      <c r="I32" s="20"/>
+      <c r="B32" s="48"/>
+      <c r="C32" s="48"/>
+      <c r="D32" s="48"/>
+      <c r="E32" s="48"/>
+      <c r="F32" s="48"/>
+      <c r="G32" s="48"/>
+      <c r="H32" s="48"/>
+      <c r="I32" s="48"/>
     </row>
     <row r="33" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
-      <c r="D33" s="20"/>
-      <c r="E33" s="20"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="20"/>
-      <c r="H33" s="20"/>
-      <c r="I33" s="20"/>
+      <c r="B33" s="48"/>
+      <c r="C33" s="48"/>
+      <c r="D33" s="48"/>
+      <c r="E33" s="48"/>
+      <c r="F33" s="48"/>
+      <c r="G33" s="48"/>
+      <c r="H33" s="48"/>
+      <c r="I33" s="48"/>
     </row>
     <row r="34" spans="2:9" ht="254" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="20"/>
-      <c r="C34" s="20"/>
-      <c r="D34" s="20"/>
-      <c r="E34" s="20"/>
-      <c r="F34" s="20"/>
-      <c r="G34" s="20"/>
-      <c r="H34" s="20"/>
-      <c r="I34" s="20"/>
+      <c r="B34" s="48"/>
+      <c r="C34" s="48"/>
+      <c r="D34" s="48"/>
+      <c r="E34" s="48"/>
+      <c r="F34" s="48"/>
+      <c r="G34" s="48"/>
+      <c r="H34" s="48"/>
+      <c r="I34" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:D25"/>
-    <mergeCell ref="F24:I24"/>
-    <mergeCell ref="F25:I25"/>
-    <mergeCell ref="C28:I28"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="B31:I34"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:I27"/>
-    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="C15:I15"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B9:I9"/>
+    <mergeCell ref="B10:I12"/>
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="B14:I14"/>
     <mergeCell ref="C22:I22"/>
     <mergeCell ref="C23:D23"/>
     <mergeCell ref="E23:I23"/>
@@ -3292,18 +4000,18 @@
     <mergeCell ref="B19:I19"/>
     <mergeCell ref="B20:I20"/>
     <mergeCell ref="C21:I21"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="B9:I9"/>
-    <mergeCell ref="B10:I12"/>
-    <mergeCell ref="B13:I13"/>
-    <mergeCell ref="B14:I14"/>
-    <mergeCell ref="C15:I15"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="C3:I3"/>
-    <mergeCell ref="C4:I4"/>
-    <mergeCell ref="C5:I5"/>
-    <mergeCell ref="C6:I6"/>
-    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="B31:I34"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:D25"/>
+    <mergeCell ref="F24:I24"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="C28:I28"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{4DBC988E-4FF2-2C49-AA18-DD92CA6A87E8}"/>
@@ -3312,4 +4020,998 @@
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6FFA9D1-69E4-904A-A96B-F62928B9B513}">
+  <dimension ref="B2:I33"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="23.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18.33203125" customWidth="1"/>
+    <col min="9" max="9" width="49.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B2" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+    </row>
+    <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="78" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" s="79"/>
+      <c r="E3" s="79"/>
+      <c r="F3" s="79"/>
+      <c r="G3" s="79"/>
+      <c r="H3" s="79"/>
+      <c r="I3" s="79"/>
+    </row>
+    <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D4" s="50"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="50"/>
+      <c r="G4" s="50"/>
+      <c r="H4" s="50"/>
+      <c r="I4" s="50"/>
+    </row>
+    <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="50">
+        <v>2022</v>
+      </c>
+      <c r="D5" s="50"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="50"/>
+      <c r="G5" s="50"/>
+      <c r="H5" s="50"/>
+      <c r="I5" s="50"/>
+    </row>
+    <row r="6" spans="2:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="D6" s="52"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="52"/>
+      <c r="I6" s="52"/>
+    </row>
+    <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="59" t="s">
+        <v>70</v>
+      </c>
+      <c r="D7" s="50"/>
+      <c r="E7" s="50"/>
+      <c r="F7" s="50"/>
+      <c r="G7" s="50"/>
+      <c r="H7" s="50"/>
+      <c r="I7" s="50"/>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B9" s="46" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="46"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="46"/>
+      <c r="F9" s="46"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="46"/>
+      <c r="I9" s="46"/>
+    </row>
+    <row r="10" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="47" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" s="47"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="47"/>
+      <c r="G10" s="47"/>
+      <c r="H10" s="47"/>
+      <c r="I10" s="47"/>
+    </row>
+    <row r="11" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="47"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47"/>
+      <c r="F11" s="47"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="47"/>
+      <c r="I11" s="47"/>
+    </row>
+    <row r="12" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="47"/>
+      <c r="F12" s="47"/>
+      <c r="G12" s="47"/>
+      <c r="H12" s="47"/>
+      <c r="I12" s="47"/>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B14" s="46" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="46"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="46"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="46"/>
+      <c r="I14" s="46"/>
+    </row>
+    <row r="15" spans="2:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="49" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="50"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="50"/>
+      <c r="G15" s="50"/>
+      <c r="H15" s="50"/>
+      <c r="I15" s="50"/>
+    </row>
+    <row r="16" spans="2:9" ht="247" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="69" t="s">
+        <v>72</v>
+      </c>
+      <c r="D16" s="70"/>
+      <c r="E16" s="70"/>
+      <c r="F16" s="70"/>
+      <c r="G16" s="70"/>
+      <c r="H16" s="70"/>
+      <c r="I16" s="71"/>
+    </row>
+    <row r="17" spans="2:9" ht="247" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="36"/>
+      <c r="C17" s="72"/>
+      <c r="D17" s="73"/>
+      <c r="E17" s="73"/>
+      <c r="F17" s="73"/>
+      <c r="G17" s="73"/>
+      <c r="H17" s="73"/>
+      <c r="I17" s="74"/>
+    </row>
+    <row r="18" spans="2:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B18" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="83"/>
+      <c r="D18" s="84"/>
+      <c r="E18" s="84"/>
+      <c r="F18" s="84"/>
+      <c r="G18" s="84"/>
+      <c r="H18" s="84"/>
+      <c r="I18" s="84"/>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="26"/>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B20" s="46" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" s="46"/>
+      <c r="D20" s="46"/>
+      <c r="E20" s="46"/>
+      <c r="F20" s="46"/>
+      <c r="G20" s="46"/>
+      <c r="H20" s="46"/>
+      <c r="I20" s="46"/>
+    </row>
+    <row r="21" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" s="75" t="s">
+        <v>74</v>
+      </c>
+      <c r="D21" s="76"/>
+      <c r="E21" s="76"/>
+      <c r="F21" s="76"/>
+      <c r="G21" s="76"/>
+      <c r="H21" s="76"/>
+      <c r="I21" s="77"/>
+    </row>
+    <row r="22" spans="2:9" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="34"/>
+    </row>
+    <row r="23" spans="2:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="B23" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="55" t="s">
+        <v>16</v>
+      </c>
+      <c r="D23" s="55"/>
+      <c r="E23" s="56" t="s">
+        <v>17</v>
+      </c>
+      <c r="F23" s="56"/>
+      <c r="G23" s="56"/>
+      <c r="H23" s="56"/>
+      <c r="I23" s="56"/>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B24" s="6">
+        <v>1</v>
+      </c>
+      <c r="C24" s="82" t="s">
+        <v>75</v>
+      </c>
+      <c r="D24" s="82"/>
+      <c r="E24" s="55" t="s">
+        <v>80</v>
+      </c>
+      <c r="F24" s="55"/>
+      <c r="G24" s="55"/>
+      <c r="H24" s="55"/>
+      <c r="I24" s="55"/>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B25" s="6">
+        <v>2</v>
+      </c>
+      <c r="C25" s="82" t="s">
+        <v>76</v>
+      </c>
+      <c r="D25" s="82"/>
+      <c r="E25" s="55"/>
+      <c r="F25" s="55"/>
+      <c r="G25" s="55"/>
+      <c r="H25" s="55"/>
+      <c r="I25" s="55"/>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B26" s="6">
+        <v>3</v>
+      </c>
+      <c r="C26" s="67" t="s">
+        <v>77</v>
+      </c>
+      <c r="D26" s="68"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="18"/>
+      <c r="I26" s="14"/>
+    </row>
+    <row r="27" spans="2:9" ht="68" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B27" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27" s="51" t="s">
+        <v>78</v>
+      </c>
+      <c r="D27" s="51"/>
+      <c r="E27" s="51"/>
+      <c r="F27" s="51"/>
+      <c r="G27" s="51"/>
+      <c r="H27" s="51"/>
+      <c r="I27" s="51"/>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B28" s="27"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="28"/>
+      <c r="E28" s="28"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="28"/>
+      <c r="H28" s="28"/>
+      <c r="I28" s="29"/>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B29" s="46" t="s">
+        <v>18</v>
+      </c>
+      <c r="C29" s="46"/>
+      <c r="D29" s="46"/>
+      <c r="E29" s="46"/>
+      <c r="F29" s="46"/>
+      <c r="G29" s="46"/>
+      <c r="H29" s="46"/>
+      <c r="I29" s="46"/>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B30" s="80"/>
+      <c r="C30" s="81"/>
+      <c r="D30" s="81"/>
+      <c r="E30" s="81"/>
+      <c r="F30" s="81"/>
+      <c r="G30" s="81"/>
+      <c r="H30" s="81"/>
+      <c r="I30" s="81"/>
+    </row>
+    <row r="31" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B31" s="81"/>
+      <c r="C31" s="81"/>
+      <c r="D31" s="81"/>
+      <c r="E31" s="81"/>
+      <c r="F31" s="81"/>
+      <c r="G31" s="81"/>
+      <c r="H31" s="81"/>
+      <c r="I31" s="81"/>
+    </row>
+    <row r="32" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B32" s="81"/>
+      <c r="C32" s="81"/>
+      <c r="D32" s="81"/>
+      <c r="E32" s="81"/>
+      <c r="F32" s="81"/>
+      <c r="G32" s="81"/>
+      <c r="H32" s="81"/>
+      <c r="I32" s="81"/>
+    </row>
+    <row r="33" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B33" s="81"/>
+      <c r="C33" s="81"/>
+      <c r="D33" s="81"/>
+      <c r="E33" s="81"/>
+      <c r="F33" s="81"/>
+      <c r="G33" s="81"/>
+      <c r="H33" s="81"/>
+      <c r="I33" s="81"/>
+    </row>
+  </sheetData>
+  <mergeCells count="31">
+    <mergeCell ref="C15:I15"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B9:I9"/>
+    <mergeCell ref="B10:I12"/>
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:I33"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="C27:I27"/>
+    <mergeCell ref="B28:I28"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C7" r:id="rId1" xr:uid="{60ABBC95-3763-1140-8147-BC4DA0DFC780}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{625A714D-2F1D-8548-AF4D-43E8CCED86F0}">
+  <dimension ref="B2:I38"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="28.83203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18.33203125" customWidth="1"/>
+    <col min="9" max="9" width="49.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B2" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+    </row>
+    <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="78" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3" s="79"/>
+      <c r="E3" s="79"/>
+      <c r="F3" s="79"/>
+      <c r="G3" s="79"/>
+      <c r="H3" s="79"/>
+      <c r="I3" s="79"/>
+    </row>
+    <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="50" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" s="50"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="50"/>
+      <c r="G4" s="50"/>
+      <c r="H4" s="50"/>
+      <c r="I4" s="50"/>
+    </row>
+    <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="50">
+        <v>2025</v>
+      </c>
+      <c r="D5" s="50"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="50"/>
+      <c r="G5" s="50"/>
+      <c r="H5" s="50"/>
+      <c r="I5" s="50"/>
+    </row>
+    <row r="6" spans="2:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="52" t="s">
+        <v>85</v>
+      </c>
+      <c r="D6" s="52"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="52"/>
+      <c r="I6" s="52"/>
+    </row>
+    <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="59" t="s">
+        <v>84</v>
+      </c>
+      <c r="D7" s="50"/>
+      <c r="E7" s="50"/>
+      <c r="F7" s="50"/>
+      <c r="G7" s="50"/>
+      <c r="H7" s="50"/>
+      <c r="I7" s="50"/>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B9" s="46" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="46"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="46"/>
+      <c r="F9" s="46"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="46"/>
+      <c r="I9" s="46"/>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B10" s="47" t="s">
+        <v>86</v>
+      </c>
+      <c r="C10" s="47"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="47"/>
+      <c r="G10" s="47"/>
+      <c r="H10" s="47"/>
+      <c r="I10" s="47"/>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B11" s="47"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47"/>
+      <c r="F11" s="47"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="47"/>
+      <c r="I11" s="47"/>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="47"/>
+      <c r="F12" s="47"/>
+      <c r="G12" s="47"/>
+      <c r="H12" s="47"/>
+      <c r="I12" s="47"/>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B14" s="46" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="46"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="46"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="46"/>
+      <c r="I14" s="46"/>
+    </row>
+    <row r="15" spans="2:9" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="51" t="s">
+        <v>87</v>
+      </c>
+      <c r="D15" s="52"/>
+      <c r="E15" s="52"/>
+      <c r="F15" s="52"/>
+      <c r="G15" s="52"/>
+      <c r="H15" s="52"/>
+      <c r="I15" s="52"/>
+    </row>
+    <row r="16" spans="2:9" ht="59" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="69" t="s">
+        <v>88</v>
+      </c>
+      <c r="D16" s="70"/>
+      <c r="E16" s="70"/>
+      <c r="F16" s="70"/>
+      <c r="G16" s="70"/>
+      <c r="H16" s="70"/>
+      <c r="I16" s="71"/>
+    </row>
+    <row r="17" spans="2:9" ht="92" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="36"/>
+      <c r="C17" s="72"/>
+      <c r="D17" s="73"/>
+      <c r="E17" s="73"/>
+      <c r="F17" s="73"/>
+      <c r="G17" s="73"/>
+      <c r="H17" s="73"/>
+      <c r="I17" s="74"/>
+    </row>
+    <row r="18" spans="2:9" ht="256" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="78" t="s">
+        <v>89</v>
+      </c>
+      <c r="D18" s="50"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="50"/>
+      <c r="G18" s="50"/>
+      <c r="H18" s="50"/>
+      <c r="I18" s="50"/>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="26"/>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B20" s="46" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" s="46"/>
+      <c r="D20" s="46"/>
+      <c r="E20" s="46"/>
+      <c r="F20" s="46"/>
+      <c r="G20" s="46"/>
+      <c r="H20" s="46"/>
+      <c r="I20" s="46"/>
+    </row>
+    <row r="21" spans="2:9" ht="246" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" s="75" t="s">
+        <v>90</v>
+      </c>
+      <c r="D21" s="76"/>
+      <c r="E21" s="76"/>
+      <c r="F21" s="76"/>
+      <c r="G21" s="76"/>
+      <c r="H21" s="76"/>
+      <c r="I21" s="77"/>
+    </row>
+    <row r="22" spans="2:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B22" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" s="32">
+        <v>8</v>
+      </c>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="34"/>
+    </row>
+    <row r="23" spans="2:9" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="55" t="s">
+        <v>16</v>
+      </c>
+      <c r="D23" s="55"/>
+      <c r="E23" s="56" t="s">
+        <v>101</v>
+      </c>
+      <c r="F23" s="56"/>
+      <c r="G23" s="56"/>
+      <c r="H23" s="56"/>
+      <c r="I23" s="56"/>
+    </row>
+    <row r="24" spans="2:9" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B24" s="6">
+        <v>1</v>
+      </c>
+      <c r="C24" s="88" t="s">
+        <v>92</v>
+      </c>
+      <c r="D24" s="89"/>
+      <c r="E24" s="78" t="s">
+        <v>107</v>
+      </c>
+      <c r="F24" s="78"/>
+      <c r="G24" s="78"/>
+      <c r="H24" s="78"/>
+      <c r="I24" s="78"/>
+    </row>
+    <row r="25" spans="2:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="6">
+        <v>2</v>
+      </c>
+      <c r="C25" s="86" t="s">
+        <v>93</v>
+      </c>
+      <c r="D25" s="87"/>
+      <c r="E25" s="78" t="s">
+        <v>108</v>
+      </c>
+      <c r="F25" s="78"/>
+      <c r="G25" s="78"/>
+      <c r="H25" s="78"/>
+      <c r="I25" s="78"/>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B26" s="6">
+        <v>3</v>
+      </c>
+      <c r="C26" s="86" t="s">
+        <v>94</v>
+      </c>
+      <c r="D26" s="87"/>
+      <c r="E26" s="78" t="s">
+        <v>106</v>
+      </c>
+      <c r="F26" s="78"/>
+      <c r="G26" s="78"/>
+      <c r="H26" s="78"/>
+      <c r="I26" s="78"/>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B27" s="6">
+        <v>4</v>
+      </c>
+      <c r="C27" s="86" t="s">
+        <v>95</v>
+      </c>
+      <c r="D27" s="87"/>
+      <c r="E27" s="78" t="s">
+        <v>105</v>
+      </c>
+      <c r="F27" s="78"/>
+      <c r="G27" s="78"/>
+      <c r="H27" s="78"/>
+      <c r="I27" s="78"/>
+    </row>
+    <row r="28" spans="2:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B28" s="6">
+        <v>5</v>
+      </c>
+      <c r="C28" s="86" t="s">
+        <v>96</v>
+      </c>
+      <c r="D28" s="87"/>
+      <c r="E28" s="78" t="s">
+        <v>104</v>
+      </c>
+      <c r="F28" s="78"/>
+      <c r="G28" s="78"/>
+      <c r="H28" s="78"/>
+      <c r="I28" s="78"/>
+    </row>
+    <row r="29" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B29" s="6">
+        <v>6</v>
+      </c>
+      <c r="C29" s="82" t="s">
+        <v>97</v>
+      </c>
+      <c r="D29" s="82"/>
+      <c r="E29" s="78" t="s">
+        <v>103</v>
+      </c>
+      <c r="F29" s="78"/>
+      <c r="G29" s="78"/>
+      <c r="H29" s="78"/>
+      <c r="I29" s="78"/>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B30" s="6">
+        <v>7</v>
+      </c>
+      <c r="C30" s="82" t="s">
+        <v>98</v>
+      </c>
+      <c r="D30" s="82"/>
+      <c r="E30" s="78" t="s">
+        <v>102</v>
+      </c>
+      <c r="F30" s="85"/>
+      <c r="G30" s="85"/>
+      <c r="H30" s="85"/>
+      <c r="I30" s="85"/>
+    </row>
+    <row r="31" spans="2:9" ht="37" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B31" s="6">
+        <v>8</v>
+      </c>
+      <c r="C31" s="86" t="s">
+        <v>99</v>
+      </c>
+      <c r="D31" s="87"/>
+      <c r="E31" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="F31" s="53"/>
+      <c r="G31" s="53"/>
+      <c r="H31" s="53"/>
+      <c r="I31" s="54"/>
+    </row>
+    <row r="32" spans="2:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B32" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C32" s="51" t="s">
+        <v>91</v>
+      </c>
+      <c r="D32" s="51"/>
+      <c r="E32" s="51"/>
+      <c r="F32" s="51"/>
+      <c r="G32" s="51"/>
+      <c r="H32" s="51"/>
+      <c r="I32" s="51"/>
+    </row>
+    <row r="33" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B33" s="27"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="28"/>
+      <c r="H33" s="28"/>
+      <c r="I33" s="29"/>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B34" s="46" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" s="46"/>
+      <c r="D34" s="46"/>
+      <c r="E34" s="46"/>
+      <c r="F34" s="46"/>
+      <c r="G34" s="46"/>
+      <c r="H34" s="46"/>
+      <c r="I34" s="46"/>
+    </row>
+    <row r="35" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B35" s="66" t="s">
+        <v>109</v>
+      </c>
+      <c r="C35" s="48"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="48"/>
+      <c r="F35" s="48"/>
+      <c r="G35" s="48"/>
+      <c r="H35" s="48"/>
+      <c r="I35" s="48"/>
+    </row>
+    <row r="36" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B36" s="48"/>
+      <c r="C36" s="48"/>
+      <c r="D36" s="48"/>
+      <c r="E36" s="48"/>
+      <c r="F36" s="48"/>
+      <c r="G36" s="48"/>
+      <c r="H36" s="48"/>
+      <c r="I36" s="48"/>
+    </row>
+    <row r="37" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B37" s="48"/>
+      <c r="C37" s="48"/>
+      <c r="D37" s="48"/>
+      <c r="E37" s="48"/>
+      <c r="F37" s="48"/>
+      <c r="G37" s="48"/>
+      <c r="H37" s="48"/>
+      <c r="I37" s="48"/>
+    </row>
+    <row r="38" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B38" s="48"/>
+      <c r="C38" s="48"/>
+      <c r="D38" s="48"/>
+      <c r="E38" s="48"/>
+      <c r="F38" s="48"/>
+      <c r="G38" s="48"/>
+      <c r="H38" s="48"/>
+      <c r="I38" s="48"/>
+    </row>
+  </sheetData>
+  <mergeCells count="41">
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B9:I9"/>
+    <mergeCell ref="B10:I12"/>
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="C15:I15"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="B35:I38"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="E29:I29"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:I28"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:I31"/>
+    <mergeCell ref="C32:I32"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="B34:I34"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C7" r:id="rId1" xr:uid="{69FD07AD-7FCA-E141-8126-AFB63E0A1511}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
did all what it was in my hands to leave the dataset prepared for the prompts
</commit_message>
<xml_diff>
--- a/Papers/Resumen Papers.xlsx
+++ b/Papers/Resumen Papers.xlsx
@@ -8,15 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sophiaaristizabal/Documents/GitHub/LLMS_Project/Papers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FF8BB10-140D-0343-9A87-B611EBE97255}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{183EE981-4C46-A645-8BD3-D7D0C4D79BC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16220" activeTab="3" xr2:uid="{400AC57E-08F9-B346-9132-4F74AEBC2D15}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16220" activeTab="1" xr2:uid="{400AC57E-08F9-B346-9132-4F74AEBC2D15}"/>
   </bookViews>
   <sheets>
     <sheet name="MANAGERIAL LEADERSHIP" sheetId="1" r:id="rId1"/>
-    <sheet name="Strategic Environment" sheetId="2" r:id="rId2"/>
-    <sheet name="Trust and Promises over Time" sheetId="3" r:id="rId3"/>
-    <sheet name="Underreporting of AI Use" sheetId="4" r:id="rId4"/>
+    <sheet name="MANAGERIAL LEADERSHIP data" sheetId="5" r:id="rId2"/>
+    <sheet name="Strategic Environment" sheetId="2" r:id="rId3"/>
+    <sheet name="Strategic Environment data" sheetId="6" r:id="rId4"/>
+    <sheet name="Trust and Promises over Time" sheetId="3" r:id="rId5"/>
+    <sheet name="Trust and Promises data" sheetId="7" r:id="rId6"/>
+    <sheet name="Underreporting of AI Use" sheetId="4" r:id="rId7"/>
+    <sheet name="Underreporting of AI Use data" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -111,7 +115,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="176">
   <si>
     <t>Autores</t>
   </si>
@@ -1925,6 +1929,204 @@
 Perception of Peer Use: Participants tend to overestimate others’ AI use, attributing higher AI reliance to peers than to themselves, which is consistent with availability bias and social perceptions .
 Explanations Focused on Self-Reporting Concerns: Free-text responses and forced-choice questions primarily reflect moral panic or social norms that discourage openly admitting to AI use, pointing to moral or ethical concerns as barriers to honest self-reporting  .
 Biases in Self- and Peer-Reporting: The research uncovers that social desirability bias drives underreporting of own AI use, especially in educational settings where stigma is high, leading to significant measurement error in self-reported data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">variable </t>
+  </si>
+  <si>
+    <t>file</t>
+  </si>
+  <si>
+    <t>und</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>any_suggestion</t>
+  </si>
+  <si>
+    <t>suggest_safe</t>
+  </si>
+  <si>
+    <t>suggest_efficient</t>
+  </si>
+  <si>
+    <t xml:space="preserve">agree_proposal </t>
+  </si>
+  <si>
+    <t>discuss_coordinate</t>
+  </si>
+  <si>
+    <t>discuss_fairness</t>
+  </si>
+  <si>
+    <t>discuss_efficient</t>
+  </si>
+  <si>
+    <t>discuss_rules</t>
+  </si>
+  <si>
+    <t>discuss_howtoplay</t>
+  </si>
+  <si>
+    <t>explanation</t>
+  </si>
+  <si>
+    <t>ask_game</t>
+  </si>
+  <si>
+    <t>truthful</t>
+  </si>
+  <si>
+    <t>falsehood</t>
+  </si>
+  <si>
+    <t>contradict</t>
+  </si>
+  <si>
+    <t>BC Coding Data, Main Experiment.dta</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Any Suggestion</t>
+  </si>
+  <si>
+    <t>Suggest Safe Outcome</t>
+  </si>
+  <si>
+    <t>Suggest Efficient Outcome</t>
+  </si>
+  <si>
+    <t>Agreement to Suggestion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tabla 6 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Discuss Need to Coordinate</t>
+  </si>
+  <si>
+    <t>Discuss Fairness</t>
+  </si>
+  <si>
+    <t>Discuss Efficiency</t>
+  </si>
+  <si>
+    <t>Questions About Rules of the Experiment</t>
+  </si>
+  <si>
+    <t>Questions About How to Play</t>
+  </si>
+  <si>
+    <t>Explanation</t>
+  </si>
+  <si>
+    <t>Ask What Game Is Being Played (M)</t>
+  </si>
+  <si>
+    <t>truthfully reveal game</t>
+  </si>
+  <si>
+    <t>lie about game</t>
+  </si>
+  <si>
+    <t>Contradict (One tells truth, other lies)</t>
+  </si>
+  <si>
+    <t>message</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> messagecode</t>
+  </si>
+  <si>
+    <t>BC Master Data, Follow Up Experiment.dta</t>
+  </si>
+  <si>
+    <t>is_promise</t>
+  </si>
+  <si>
+    <t>Classified as promise</t>
+  </si>
+  <si>
+    <t>recalled_as_promise</t>
+  </si>
+  <si>
+    <t>Trustee recalled message as promise</t>
+  </si>
+  <si>
+    <t>is_efficiency</t>
+  </si>
+  <si>
+    <t>Classified as appeal to efficiency</t>
+  </si>
+  <si>
+    <t>is_ethics</t>
+  </si>
+  <si>
+    <t>Classified as appeal to fairness</t>
+  </si>
+  <si>
+    <t>Message</t>
+  </si>
+  <si>
+    <t>Recalled_Message</t>
+  </si>
+  <si>
+    <t>Trustee's message to trustor</t>
+  </si>
+  <si>
+    <t>Trustee's message (recalled)</t>
+  </si>
+  <si>
+    <t>datapaper_anonymized.csv</t>
+  </si>
+  <si>
+    <t>Underreporting of AI Use.csv</t>
+  </si>
+  <si>
+    <t>uninformative</t>
+  </si>
+  <si>
+    <t>SDB</t>
+  </si>
+  <si>
+    <t>overest. Others</t>
+  </si>
+  <si>
+    <t>underest. Own</t>
+  </si>
+  <si>
+    <t>academic integrity</t>
+  </si>
+  <si>
+    <t>T, F or F?</t>
+  </si>
+  <si>
+    <t>info asymmetry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI discussion priming </t>
+  </si>
+  <si>
+    <t>privacy concerns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">self - esteem </t>
+  </si>
+  <si>
+    <t>self-report bias</t>
+  </si>
+  <si>
+    <t>network effect</t>
+  </si>
+  <si>
+    <t>TRUE or FALSE</t>
+  </si>
+  <si>
+    <t>session period group game</t>
+  </si>
+  <si>
+    <t>0          . . .             *</t>
   </si>
 </sst>
 </file>
@@ -2165,11 +2367,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -2185,6 +2393,142 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -2204,12 +2548,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2221,128 +2559,53 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2350,58 +2613,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2413,26 +2634,39 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2983,523 +3217,542 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="57" t="s">
+      <c r="C3" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="58" t="s">
+      <c r="C4" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="58"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="58"/>
-      <c r="I4" s="58"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="16"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="50">
+      <c r="C5" s="13">
         <v>2025</v>
       </c>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="50"/>
-      <c r="G5" s="50"/>
-      <c r="H5" s="50"/>
-      <c r="I5" s="50"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
+      <c r="I5" s="13"/>
     </row>
     <row r="6" spans="2:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="50" t="s">
+      <c r="C6" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="50"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="50"/>
-      <c r="G6" s="50"/>
-      <c r="H6" s="50"/>
-      <c r="I6" s="50"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
+      <c r="I6" s="13"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="59" t="s">
+      <c r="C7" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="50"/>
-      <c r="E7" s="50"/>
-      <c r="F7" s="50"/>
-      <c r="G7" s="50"/>
-      <c r="H7" s="50"/>
-      <c r="I7" s="50"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
     </row>
     <row r="8" spans="2:9" ht="9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
     </row>
     <row r="9" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="46" t="s">
+      <c r="B9" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="46"/>
-      <c r="D9" s="46"/>
-      <c r="E9" s="46"/>
-      <c r="F9" s="46"/>
-      <c r="G9" s="46"/>
-      <c r="H9" s="46"/>
-      <c r="I9" s="46"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
     </row>
     <row r="10" spans="2:9" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="47" t="s">
+      <c r="B10" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="47"/>
-      <c r="F10" s="47"/>
-      <c r="G10" s="47"/>
-      <c r="H10" s="47"/>
-      <c r="I10" s="47"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
     </row>
     <row r="11" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="47"/>
-      <c r="C11" s="47"/>
-      <c r="D11" s="47"/>
-      <c r="E11" s="47"/>
-      <c r="F11" s="47"/>
-      <c r="G11" s="47"/>
-      <c r="H11" s="47"/>
-      <c r="I11" s="47"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
     </row>
     <row r="12" spans="2:9" ht="11" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="47"/>
-      <c r="C12" s="47"/>
-      <c r="D12" s="47"/>
-      <c r="E12" s="47"/>
-      <c r="F12" s="47"/>
-      <c r="G12" s="47"/>
-      <c r="H12" s="47"/>
-      <c r="I12" s="47"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
     </row>
     <row r="13" spans="2:9" ht="9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="26"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="46" t="s">
+      <c r="B14" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
-      <c r="E14" s="46"/>
-      <c r="F14" s="46"/>
-      <c r="G14" s="46"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="46"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
+      <c r="I14" s="14"/>
     </row>
     <row r="15" spans="2:9" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="49" t="s">
+      <c r="C15" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="50"/>
-      <c r="E15" s="50"/>
-      <c r="F15" s="50"/>
-      <c r="G15" s="50"/>
-      <c r="H15" s="50"/>
-      <c r="I15" s="50"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13"/>
     </row>
     <row r="16" spans="2:9" ht="125" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="35" t="s">
+      <c r="B16" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="37" t="s">
+      <c r="C16" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="D16" s="38"/>
-      <c r="E16" s="38"/>
-      <c r="F16" s="38"/>
-      <c r="G16" s="38"/>
-      <c r="H16" s="38"/>
-      <c r="I16" s="39"/>
+      <c r="D16" s="41"/>
+      <c r="E16" s="41"/>
+      <c r="F16" s="41"/>
+      <c r="G16" s="41"/>
+      <c r="H16" s="41"/>
+      <c r="I16" s="42"/>
     </row>
     <row r="17" spans="2:9" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="36"/>
-      <c r="C17" s="40"/>
-      <c r="D17" s="41"/>
-      <c r="E17" s="41"/>
-      <c r="F17" s="41"/>
-      <c r="G17" s="41"/>
-      <c r="H17" s="41"/>
-      <c r="I17" s="42"/>
+      <c r="B17" s="39"/>
+      <c r="C17" s="43"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="44"/>
+      <c r="F17" s="44"/>
+      <c r="G17" s="44"/>
+      <c r="H17" s="44"/>
+      <c r="I17" s="45"/>
     </row>
     <row r="18" spans="2:9" ht="67" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="49" t="s">
+      <c r="C18" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="50"/>
-      <c r="E18" s="50"/>
-      <c r="F18" s="50"/>
-      <c r="G18" s="50"/>
-      <c r="H18" s="50"/>
-      <c r="I18" s="50"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="13"/>
     </row>
     <row r="19" spans="2:9" ht="7" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="20"/>
+      <c r="I19" s="20"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="46" t="s">
+      <c r="B20" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="46"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="46"/>
-      <c r="F20" s="46"/>
-      <c r="G20" s="46"/>
-      <c r="H20" s="46"/>
-      <c r="I20" s="46"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="14"/>
     </row>
     <row r="21" spans="2:9" ht="43" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="19" t="s">
+      <c r="C21" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="30"/>
-      <c r="E21" s="30"/>
-      <c r="F21" s="30"/>
-      <c r="G21" s="30"/>
-      <c r="H21" s="30"/>
-      <c r="I21" s="31"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="22"/>
+      <c r="H21" s="22"/>
+      <c r="I21" s="23"/>
     </row>
     <row r="22" spans="2:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="32">
+      <c r="C22" s="28">
         <v>9</v>
       </c>
-      <c r="D22" s="33"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="33"/>
-      <c r="H22" s="33"/>
-      <c r="I22" s="34"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="36"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="36"/>
+      <c r="I22" s="37"/>
     </row>
     <row r="23" spans="2:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="55" t="s">
+      <c r="C23" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="55"/>
-      <c r="E23" s="56" t="s">
+      <c r="D23" s="50"/>
+      <c r="E23" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="56"/>
-      <c r="G23" s="56"/>
-      <c r="H23" s="56"/>
-      <c r="I23" s="56"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="51"/>
+      <c r="H23" s="51"/>
+      <c r="I23" s="51"/>
     </row>
     <row r="24" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="6">
+      <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="22" t="s">
+      <c r="C24" s="48" t="s">
         <v>38</v>
       </c>
-      <c r="D24" s="23"/>
-      <c r="E24" s="19" t="s">
+      <c r="D24" s="49"/>
+      <c r="E24" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="F24" s="20"/>
-      <c r="G24" s="20"/>
-      <c r="H24" s="20"/>
-      <c r="I24" s="21"/>
+      <c r="F24" s="52"/>
+      <c r="G24" s="52"/>
+      <c r="H24" s="52"/>
+      <c r="I24" s="53"/>
     </row>
     <row r="25" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="6">
+      <c r="B25" s="8">
         <v>2</v>
       </c>
-      <c r="C25" s="22" t="s">
+      <c r="C25" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="D25" s="23"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="24"/>
-      <c r="G25" s="24"/>
-      <c r="H25" s="24"/>
-      <c r="I25" s="23"/>
+      <c r="D25" s="49"/>
+      <c r="E25" s="48"/>
+      <c r="F25" s="54"/>
+      <c r="G25" s="54"/>
+      <c r="H25" s="54"/>
+      <c r="I25" s="49"/>
     </row>
     <row r="26" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="7">
+      <c r="B26" s="55">
         <v>3</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="57" t="s">
         <v>40</v>
       </c>
-      <c r="D26" s="10"/>
-      <c r="E26" s="25" t="s">
+      <c r="D26" s="58"/>
+      <c r="E26" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="F26" s="25"/>
-      <c r="G26" s="24" t="s">
+      <c r="F26" s="31"/>
+      <c r="G26" s="54" t="s">
         <v>41</v>
       </c>
-      <c r="H26" s="24"/>
-      <c r="I26" s="23"/>
+      <c r="H26" s="54"/>
+      <c r="I26" s="49"/>
     </row>
     <row r="27" spans="2:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="8"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="13" t="s">
+      <c r="B27" s="56"/>
+      <c r="C27" s="59"/>
+      <c r="D27" s="60"/>
+      <c r="E27" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="F27" s="14"/>
-      <c r="G27" s="15" t="s">
+      <c r="F27" s="27"/>
+      <c r="G27" s="61" t="s">
         <v>43</v>
       </c>
-      <c r="H27" s="16"/>
-      <c r="I27" s="17"/>
+      <c r="H27" s="62"/>
+      <c r="I27" s="63"/>
     </row>
     <row r="28" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="6">
+      <c r="B28" s="8">
         <v>4</v>
       </c>
-      <c r="C28" s="13" t="s">
+      <c r="C28" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="D28" s="14"/>
-      <c r="E28" s="43" t="s">
+      <c r="D28" s="27"/>
+      <c r="E28" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="F28" s="30"/>
-      <c r="G28" s="30"/>
-      <c r="H28" s="30"/>
-      <c r="I28" s="31"/>
+      <c r="F28" s="22"/>
+      <c r="G28" s="22"/>
+      <c r="H28" s="22"/>
+      <c r="I28" s="23"/>
     </row>
     <row r="29" spans="2:9" ht="43" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="6">
+      <c r="B29" s="8">
         <v>5</v>
       </c>
-      <c r="C29" s="25" t="s">
+      <c r="C29" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="D29" s="25"/>
-      <c r="E29" s="51" t="s">
+      <c r="D29" s="31"/>
+      <c r="E29" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="F29" s="51"/>
-      <c r="G29" s="51"/>
-      <c r="H29" s="51"/>
-      <c r="I29" s="51"/>
+      <c r="F29" s="24"/>
+      <c r="G29" s="24"/>
+      <c r="H29" s="24"/>
+      <c r="I29" s="24"/>
     </row>
     <row r="30" spans="2:9" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="6">
+      <c r="B30" s="8">
         <v>6</v>
       </c>
-      <c r="C30" s="13" t="s">
+      <c r="C30" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="D30" s="14"/>
-      <c r="E30" s="43" t="s">
+      <c r="D30" s="27"/>
+      <c r="E30" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="F30" s="44"/>
-      <c r="G30" s="44"/>
-      <c r="H30" s="44"/>
-      <c r="I30" s="45"/>
+      <c r="F30" s="46"/>
+      <c r="G30" s="46"/>
+      <c r="H30" s="46"/>
+      <c r="I30" s="47"/>
     </row>
     <row r="31" spans="2:9" ht="53" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="6">
+      <c r="B31" s="8">
         <v>7</v>
       </c>
-      <c r="C31" s="25" t="s">
+      <c r="C31" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="D31" s="25"/>
-      <c r="E31" s="51" t="s">
+      <c r="D31" s="31"/>
+      <c r="E31" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="F31" s="52"/>
-      <c r="G31" s="52"/>
-      <c r="H31" s="52"/>
-      <c r="I31" s="52"/>
+      <c r="F31" s="25"/>
+      <c r="G31" s="25"/>
+      <c r="H31" s="25"/>
+      <c r="I31" s="25"/>
     </row>
     <row r="32" spans="2:9" ht="53" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="6">
+      <c r="B32" s="8">
         <v>8</v>
       </c>
-      <c r="C32" s="13" t="s">
+      <c r="C32" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="D32" s="14"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="18"/>
-      <c r="G32" s="18"/>
-      <c r="H32" s="18"/>
-      <c r="I32" s="14"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="64"/>
+      <c r="G32" s="64"/>
+      <c r="H32" s="64"/>
+      <c r="I32" s="27"/>
     </row>
     <row r="33" spans="2:9" ht="102" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="6">
+      <c r="B33" s="8">
         <v>9</v>
       </c>
-      <c r="C33" s="13" t="s">
+      <c r="C33" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="D33" s="14"/>
-      <c r="E33" s="32" t="s">
+      <c r="D33" s="27"/>
+      <c r="E33" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="F33" s="53"/>
-      <c r="G33" s="53"/>
-      <c r="H33" s="53"/>
-      <c r="I33" s="54"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="29"/>
+      <c r="H33" s="29"/>
+      <c r="I33" s="30"/>
     </row>
     <row r="34" spans="2:9" ht="190" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C34" s="51" t="s">
+      <c r="C34" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="D34" s="51"/>
-      <c r="E34" s="51"/>
-      <c r="F34" s="51"/>
-      <c r="G34" s="51"/>
-      <c r="H34" s="51"/>
-      <c r="I34" s="51"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="24"/>
+      <c r="I34" s="24"/>
     </row>
     <row r="35" spans="2:9" ht="10" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="27"/>
-      <c r="C35" s="28"/>
-      <c r="D35" s="28"/>
-      <c r="E35" s="28"/>
-      <c r="F35" s="28"/>
-      <c r="G35" s="28"/>
-      <c r="H35" s="28"/>
-      <c r="I35" s="29"/>
+      <c r="B35" s="32"/>
+      <c r="C35" s="33"/>
+      <c r="D35" s="33"/>
+      <c r="E35" s="33"/>
+      <c r="F35" s="33"/>
+      <c r="G35" s="33"/>
+      <c r="H35" s="33"/>
+      <c r="I35" s="34"/>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B36" s="46" t="s">
+      <c r="B36" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C36" s="46"/>
-      <c r="D36" s="46"/>
-      <c r="E36" s="46"/>
-      <c r="F36" s="46"/>
-      <c r="G36" s="46"/>
-      <c r="H36" s="46"/>
-      <c r="I36" s="46"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="14"/>
+      <c r="H36" s="14"/>
+      <c r="I36" s="14"/>
     </row>
     <row r="37" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="48" t="s">
+      <c r="B37" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="C37" s="48"/>
-      <c r="D37" s="48"/>
-      <c r="E37" s="48"/>
-      <c r="F37" s="48"/>
-      <c r="G37" s="48"/>
-      <c r="H37" s="48"/>
-      <c r="I37" s="48"/>
+      <c r="C37" s="18"/>
+      <c r="D37" s="18"/>
+      <c r="E37" s="18"/>
+      <c r="F37" s="18"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="18"/>
+      <c r="I37" s="18"/>
     </row>
     <row r="38" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="48"/>
-      <c r="C38" s="48"/>
-      <c r="D38" s="48"/>
-      <c r="E38" s="48"/>
-      <c r="F38" s="48"/>
-      <c r="G38" s="48"/>
-      <c r="H38" s="48"/>
-      <c r="I38" s="48"/>
+      <c r="B38" s="18"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="18"/>
+      <c r="E38" s="18"/>
+      <c r="F38" s="18"/>
+      <c r="G38" s="18"/>
+      <c r="H38" s="18"/>
+      <c r="I38" s="18"/>
     </row>
     <row r="39" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="48"/>
-      <c r="C39" s="48"/>
-      <c r="D39" s="48"/>
-      <c r="E39" s="48"/>
-      <c r="F39" s="48"/>
-      <c r="G39" s="48"/>
-      <c r="H39" s="48"/>
-      <c r="I39" s="48"/>
+      <c r="B39" s="18"/>
+      <c r="C39" s="18"/>
+      <c r="D39" s="18"/>
+      <c r="E39" s="18"/>
+      <c r="F39" s="18"/>
+      <c r="G39" s="18"/>
+      <c r="H39" s="18"/>
+      <c r="I39" s="18"/>
     </row>
     <row r="40" spans="2:9" ht="76" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B40" s="48"/>
-      <c r="C40" s="48"/>
-      <c r="D40" s="48"/>
-      <c r="E40" s="48"/>
-      <c r="F40" s="48"/>
-      <c r="G40" s="48"/>
-      <c r="H40" s="48"/>
-      <c r="I40" s="48"/>
+      <c r="B40" s="18"/>
+      <c r="C40" s="18"/>
+      <c r="D40" s="18"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="18"/>
+      <c r="G40" s="18"/>
+      <c r="H40" s="18"/>
+      <c r="I40" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="C7:I7"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="C3:I3"/>
-    <mergeCell ref="C4:I4"/>
-    <mergeCell ref="C5:I5"/>
-    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="E32:I32"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="C26:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="C25:D25"/>
     <mergeCell ref="B36:I36"/>
     <mergeCell ref="B10:I12"/>
     <mergeCell ref="B9:I9"/>
@@ -3516,31 +3769,12 @@
     <mergeCell ref="C28:D28"/>
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="C31:D31"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="B35:I35"/>
-    <mergeCell ref="B13:I13"/>
-    <mergeCell ref="C21:I21"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:I30"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="B14:I14"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="C26:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="E32:I32"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="C6:I6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{C9E9977D-5134-FE4B-852F-8DEBDCB543E0}"/>
@@ -3552,6 +3786,287 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33691873-C7AA-8F42-A0C0-0DDE1CD59CDD}">
+  <dimension ref="B4:I27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.6640625" customWidth="1"/>
+    <col min="2" max="2" width="26" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
+    <col min="4" max="4" width="38.5" customWidth="1"/>
+    <col min="5" max="5" width="24.5" customWidth="1"/>
+    <col min="6" max="6" width="26.6640625" customWidth="1"/>
+    <col min="7" max="7" width="33.33203125" customWidth="1"/>
+    <col min="8" max="8" width="16.1640625" customWidth="1"/>
+    <col min="9" max="9" width="37" customWidth="1"/>
+    <col min="10" max="10" width="25.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B4" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+    </row>
+    <row r="5" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B7" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="C20" s="10"/>
+      <c r="D20" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B21" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="C21" s="10"/>
+      <c r="D21" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="C27">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B4:E4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24F74443-37D3-BE4C-BB6A-E284A6B9B524}">
   <dimension ref="B2:I34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3564,421 +4079,442 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="78" t="s">
+      <c r="C3" s="65" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="79"/>
-      <c r="E3" s="79"/>
-      <c r="F3" s="79"/>
-      <c r="G3" s="79"/>
-      <c r="H3" s="79"/>
-      <c r="I3" s="79"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="66"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="66"/>
+      <c r="H3" s="66"/>
+      <c r="I3" s="66"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="50" t="s">
+      <c r="C4" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="50"/>
-      <c r="H4" s="50"/>
-      <c r="I4" s="50"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
+      <c r="I4" s="13"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="50">
+      <c r="C5" s="13">
         <v>2020</v>
       </c>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="50"/>
-      <c r="G5" s="50"/>
-      <c r="H5" s="50"/>
-      <c r="I5" s="50"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
+      <c r="I5" s="13"/>
     </row>
     <row r="6" spans="2:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="52" t="s">
+      <c r="C6" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="52"/>
-      <c r="E6" s="52"/>
-      <c r="F6" s="52"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="52"/>
-      <c r="I6" s="52"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="25"/>
+      <c r="I6" s="25"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="59" t="s">
+      <c r="C7" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="D7" s="50"/>
-      <c r="E7" s="50"/>
-      <c r="F7" s="50"/>
-      <c r="G7" s="50"/>
-      <c r="H7" s="50"/>
-      <c r="I7" s="50"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="46" t="s">
+      <c r="B9" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="46"/>
-      <c r="D9" s="46"/>
-      <c r="E9" s="46"/>
-      <c r="F9" s="46"/>
-      <c r="G9" s="46"/>
-      <c r="H9" s="46"/>
-      <c r="I9" s="46"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
     </row>
     <row r="10" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="47" t="s">
+      <c r="B10" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="47"/>
-      <c r="F10" s="47"/>
-      <c r="G10" s="47"/>
-      <c r="H10" s="47"/>
-      <c r="I10" s="47"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
     </row>
     <row r="11" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="47"/>
-      <c r="C11" s="47"/>
-      <c r="D11" s="47"/>
-      <c r="E11" s="47"/>
-      <c r="F11" s="47"/>
-      <c r="G11" s="47"/>
-      <c r="H11" s="47"/>
-      <c r="I11" s="47"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
     </row>
     <row r="12" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="47"/>
-      <c r="C12" s="47"/>
-      <c r="D12" s="47"/>
-      <c r="E12" s="47"/>
-      <c r="F12" s="47"/>
-      <c r="G12" s="47"/>
-      <c r="H12" s="47"/>
-      <c r="I12" s="47"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="26"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="46" t="s">
+      <c r="B14" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
-      <c r="E14" s="46"/>
-      <c r="F14" s="46"/>
-      <c r="G14" s="46"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="46"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
+      <c r="I14" s="14"/>
     </row>
     <row r="15" spans="2:9" ht="64" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="49" t="s">
+      <c r="C15" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="50"/>
-      <c r="E15" s="50"/>
-      <c r="F15" s="50"/>
-      <c r="G15" s="50"/>
-      <c r="H15" s="50"/>
-      <c r="I15" s="50"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13"/>
     </row>
     <row r="16" spans="2:9" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="35" t="s">
+      <c r="B16" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="69" t="s">
+      <c r="C16" s="67" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="70"/>
-      <c r="E16" s="70"/>
-      <c r="F16" s="70"/>
-      <c r="G16" s="70"/>
-      <c r="H16" s="70"/>
-      <c r="I16" s="71"/>
+      <c r="D16" s="68"/>
+      <c r="E16" s="68"/>
+      <c r="F16" s="68"/>
+      <c r="G16" s="68"/>
+      <c r="H16" s="68"/>
+      <c r="I16" s="69"/>
     </row>
     <row r="17" spans="2:9" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="36"/>
-      <c r="C17" s="72"/>
-      <c r="D17" s="73"/>
-      <c r="E17" s="73"/>
-      <c r="F17" s="73"/>
-      <c r="G17" s="73"/>
-      <c r="H17" s="73"/>
-      <c r="I17" s="74"/>
+      <c r="B17" s="39"/>
+      <c r="C17" s="70"/>
+      <c r="D17" s="71"/>
+      <c r="E17" s="71"/>
+      <c r="F17" s="71"/>
+      <c r="G17" s="71"/>
+      <c r="H17" s="71"/>
+      <c r="I17" s="72"/>
     </row>
     <row r="18" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="49" t="s">
+      <c r="C18" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="D18" s="50"/>
-      <c r="E18" s="50"/>
-      <c r="F18" s="50"/>
-      <c r="G18" s="50"/>
-      <c r="H18" s="50"/>
-      <c r="I18" s="50"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="13"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="20"/>
+      <c r="I19" s="20"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="46" t="s">
+      <c r="B20" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="46"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="46"/>
-      <c r="F20" s="46"/>
-      <c r="G20" s="46"/>
-      <c r="H20" s="46"/>
-      <c r="I20" s="46"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="14"/>
     </row>
     <row r="21" spans="2:9" ht="160" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="75" t="s">
+      <c r="C21" s="73" t="s">
         <v>57</v>
       </c>
-      <c r="D21" s="76"/>
-      <c r="E21" s="76"/>
-      <c r="F21" s="76"/>
-      <c r="G21" s="76"/>
-      <c r="H21" s="76"/>
-      <c r="I21" s="77"/>
+      <c r="D21" s="74"/>
+      <c r="E21" s="74"/>
+      <c r="F21" s="74"/>
+      <c r="G21" s="74"/>
+      <c r="H21" s="74"/>
+      <c r="I21" s="75"/>
     </row>
     <row r="22" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="32">
+      <c r="C22" s="28">
         <v>3</v>
       </c>
-      <c r="D22" s="33"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="33"/>
-      <c r="H22" s="33"/>
-      <c r="I22" s="34"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="36"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="36"/>
+      <c r="I22" s="37"/>
     </row>
     <row r="23" spans="2:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="55" t="s">
+      <c r="C23" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="55"/>
-      <c r="E23" s="56" t="s">
+      <c r="D23" s="50"/>
+      <c r="E23" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="56"/>
-      <c r="G23" s="56"/>
-      <c r="H23" s="56"/>
-      <c r="I23" s="56"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="51"/>
+      <c r="H23" s="51"/>
+      <c r="I23" s="51"/>
     </row>
     <row r="24" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="7">
+      <c r="B24" s="55">
         <v>1</v>
       </c>
-      <c r="C24" s="60" t="s">
+      <c r="C24" s="81" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="61"/>
-      <c r="E24" s="2" t="s">
+      <c r="D24" s="82"/>
+      <c r="E24" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="F24" s="64" t="s">
+      <c r="F24" s="83" t="s">
         <v>63</v>
       </c>
-      <c r="G24" s="64"/>
-      <c r="H24" s="64"/>
-      <c r="I24" s="65"/>
+      <c r="G24" s="83"/>
+      <c r="H24" s="83"/>
+      <c r="I24" s="84"/>
     </row>
     <row r="25" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="8"/>
-      <c r="C25" s="62"/>
-      <c r="D25" s="63"/>
-      <c r="E25" s="2" t="s">
+      <c r="B25" s="56"/>
+      <c r="C25" s="79"/>
+      <c r="D25" s="80"/>
+      <c r="E25" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="F25" s="24" t="s">
+      <c r="F25" s="54" t="s">
         <v>64</v>
       </c>
-      <c r="G25" s="24"/>
-      <c r="H25" s="24"/>
-      <c r="I25" s="23"/>
+      <c r="G25" s="54"/>
+      <c r="H25" s="54"/>
+      <c r="I25" s="49"/>
     </row>
     <row r="26" spans="2:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="6">
+      <c r="B26" s="8">
         <v>2</v>
       </c>
-      <c r="C26" s="67" t="s">
+      <c r="C26" s="77" t="s">
         <v>59</v>
       </c>
-      <c r="D26" s="68"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="18"/>
-      <c r="G26" s="18"/>
-      <c r="H26" s="18"/>
-      <c r="I26" s="14"/>
+      <c r="D26" s="78"/>
+      <c r="E26" s="26"/>
+      <c r="F26" s="64"/>
+      <c r="G26" s="64"/>
+      <c r="H26" s="64"/>
+      <c r="I26" s="27"/>
     </row>
     <row r="27" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="6">
+      <c r="B27" s="8">
         <v>3</v>
       </c>
-      <c r="C27" s="62" t="s">
+      <c r="C27" s="79" t="s">
         <v>60</v>
       </c>
-      <c r="D27" s="63"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="18"/>
-      <c r="G27" s="18"/>
-      <c r="H27" s="18"/>
-      <c r="I27" s="14"/>
+      <c r="D27" s="80"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="64"/>
+      <c r="G27" s="64"/>
+      <c r="H27" s="64"/>
+      <c r="I27" s="27"/>
     </row>
     <row r="28" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C28" s="51" t="s">
+      <c r="C28" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="D28" s="51"/>
-      <c r="E28" s="51"/>
-      <c r="F28" s="51"/>
-      <c r="G28" s="51"/>
-      <c r="H28" s="51"/>
-      <c r="I28" s="51"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="24"/>
+      <c r="I28" s="24"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B29" s="27"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="28"/>
-      <c r="I29" s="29"/>
+      <c r="B29" s="32"/>
+      <c r="C29" s="33"/>
+      <c r="D29" s="33"/>
+      <c r="E29" s="33"/>
+      <c r="F29" s="33"/>
+      <c r="G29" s="33"/>
+      <c r="H29" s="33"/>
+      <c r="I29" s="34"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B30" s="46" t="s">
+      <c r="B30" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C30" s="46"/>
-      <c r="D30" s="46"/>
-      <c r="E30" s="46"/>
-      <c r="F30" s="46"/>
-      <c r="G30" s="46"/>
-      <c r="H30" s="46"/>
-      <c r="I30" s="46"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="14"/>
+      <c r="H30" s="14"/>
+      <c r="I30" s="14"/>
     </row>
     <row r="31" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="66" t="s">
+      <c r="B31" s="76" t="s">
         <v>66</v>
       </c>
-      <c r="C31" s="48"/>
-      <c r="D31" s="48"/>
-      <c r="E31" s="48"/>
-      <c r="F31" s="48"/>
-      <c r="G31" s="48"/>
-      <c r="H31" s="48"/>
-      <c r="I31" s="48"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="18"/>
+      <c r="E31" s="18"/>
+      <c r="F31" s="18"/>
+      <c r="G31" s="18"/>
+      <c r="H31" s="18"/>
+      <c r="I31" s="18"/>
     </row>
     <row r="32" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="48"/>
-      <c r="C32" s="48"/>
-      <c r="D32" s="48"/>
-      <c r="E32" s="48"/>
-      <c r="F32" s="48"/>
-      <c r="G32" s="48"/>
-      <c r="H32" s="48"/>
-      <c r="I32" s="48"/>
+      <c r="B32" s="18"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="18"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="18"/>
+      <c r="I32" s="18"/>
     </row>
     <row r="33" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="48"/>
-      <c r="C33" s="48"/>
-      <c r="D33" s="48"/>
-      <c r="E33" s="48"/>
-      <c r="F33" s="48"/>
-      <c r="G33" s="48"/>
-      <c r="H33" s="48"/>
-      <c r="I33" s="48"/>
+      <c r="B33" s="18"/>
+      <c r="C33" s="18"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="18"/>
+      <c r="G33" s="18"/>
+      <c r="H33" s="18"/>
+      <c r="I33" s="18"/>
     </row>
     <row r="34" spans="2:9" ht="254" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="48"/>
-      <c r="C34" s="48"/>
-      <c r="D34" s="48"/>
-      <c r="E34" s="48"/>
-      <c r="F34" s="48"/>
-      <c r="G34" s="48"/>
-      <c r="H34" s="48"/>
-      <c r="I34" s="48"/>
+      <c r="B34" s="18"/>
+      <c r="C34" s="18"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="18"/>
+      <c r="F34" s="18"/>
+      <c r="G34" s="18"/>
+      <c r="H34" s="18"/>
+      <c r="I34" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:D25"/>
+    <mergeCell ref="F24:I24"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="C28:I28"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="B31:I34"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="C21:I21"/>
     <mergeCell ref="C15:I15"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -3991,27 +4527,6 @@
     <mergeCell ref="B10:I12"/>
     <mergeCell ref="B13:I13"/>
     <mergeCell ref="B14:I14"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="C21:I21"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="B31:I34"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:I27"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:D25"/>
-    <mergeCell ref="F24:I24"/>
-    <mergeCell ref="F25:I25"/>
-    <mergeCell ref="C28:I28"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{4DBC988E-4FF2-2C49-AA18-DD92CA6A87E8}"/>
@@ -4022,7 +4537,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57DE7B14-DB2E-8641-B8BE-3D9A44A8DF71}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6FFA9D1-69E4-904A-A96B-F62928B9B513}">
   <dimension ref="B2:I33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4035,401 +4559,420 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="78" t="s">
+      <c r="C3" s="65" t="s">
         <v>67</v>
       </c>
-      <c r="D3" s="79"/>
-      <c r="E3" s="79"/>
-      <c r="F3" s="79"/>
-      <c r="G3" s="79"/>
-      <c r="H3" s="79"/>
-      <c r="I3" s="79"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="66"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="66"/>
+      <c r="H3" s="66"/>
+      <c r="I3" s="66"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="50" t="s">
+      <c r="C4" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="50"/>
-      <c r="H4" s="50"/>
-      <c r="I4" s="50"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
+      <c r="I4" s="13"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="50">
+      <c r="C5" s="13">
         <v>2022</v>
       </c>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="50"/>
-      <c r="G5" s="50"/>
-      <c r="H5" s="50"/>
-      <c r="I5" s="50"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
+      <c r="I5" s="13"/>
     </row>
     <row r="6" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="52" t="s">
+      <c r="C6" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="D6" s="52"/>
-      <c r="E6" s="52"/>
-      <c r="F6" s="52"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="52"/>
-      <c r="I6" s="52"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="25"/>
+      <c r="I6" s="25"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="59" t="s">
+      <c r="C7" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="D7" s="50"/>
-      <c r="E7" s="50"/>
-      <c r="F7" s="50"/>
-      <c r="G7" s="50"/>
-      <c r="H7" s="50"/>
-      <c r="I7" s="50"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="46" t="s">
+      <c r="B9" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="46"/>
-      <c r="D9" s="46"/>
-      <c r="E9" s="46"/>
-      <c r="F9" s="46"/>
-      <c r="G9" s="46"/>
-      <c r="H9" s="46"/>
-      <c r="I9" s="46"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
     </row>
     <row r="10" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="47" t="s">
+      <c r="B10" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="47"/>
-      <c r="F10" s="47"/>
-      <c r="G10" s="47"/>
-      <c r="H10" s="47"/>
-      <c r="I10" s="47"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
     </row>
     <row r="11" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="47"/>
-      <c r="C11" s="47"/>
-      <c r="D11" s="47"/>
-      <c r="E11" s="47"/>
-      <c r="F11" s="47"/>
-      <c r="G11" s="47"/>
-      <c r="H11" s="47"/>
-      <c r="I11" s="47"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
     </row>
     <row r="12" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="47"/>
-      <c r="C12" s="47"/>
-      <c r="D12" s="47"/>
-      <c r="E12" s="47"/>
-      <c r="F12" s="47"/>
-      <c r="G12" s="47"/>
-      <c r="H12" s="47"/>
-      <c r="I12" s="47"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="26"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="46" t="s">
+      <c r="B14" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
-      <c r="E14" s="46"/>
-      <c r="F14" s="46"/>
-      <c r="G14" s="46"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="46"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
+      <c r="I14" s="14"/>
     </row>
     <row r="15" spans="2:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="49" t="s">
+      <c r="C15" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="D15" s="50"/>
-      <c r="E15" s="50"/>
-      <c r="F15" s="50"/>
-      <c r="G15" s="50"/>
-      <c r="H15" s="50"/>
-      <c r="I15" s="50"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13"/>
     </row>
     <row r="16" spans="2:9" ht="247" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="35" t="s">
+      <c r="B16" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="69" t="s">
+      <c r="C16" s="67" t="s">
         <v>72</v>
       </c>
-      <c r="D16" s="70"/>
-      <c r="E16" s="70"/>
-      <c r="F16" s="70"/>
-      <c r="G16" s="70"/>
-      <c r="H16" s="70"/>
-      <c r="I16" s="71"/>
+      <c r="D16" s="68"/>
+      <c r="E16" s="68"/>
+      <c r="F16" s="68"/>
+      <c r="G16" s="68"/>
+      <c r="H16" s="68"/>
+      <c r="I16" s="69"/>
     </row>
     <row r="17" spans="2:9" ht="247" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="36"/>
-      <c r="C17" s="72"/>
-      <c r="D17" s="73"/>
-      <c r="E17" s="73"/>
-      <c r="F17" s="73"/>
-      <c r="G17" s="73"/>
-      <c r="H17" s="73"/>
-      <c r="I17" s="74"/>
+      <c r="B17" s="39"/>
+      <c r="C17" s="70"/>
+      <c r="D17" s="71"/>
+      <c r="E17" s="71"/>
+      <c r="F17" s="71"/>
+      <c r="G17" s="71"/>
+      <c r="H17" s="71"/>
+      <c r="I17" s="72"/>
     </row>
     <row r="18" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="83"/>
-      <c r="D18" s="84"/>
-      <c r="E18" s="84"/>
-      <c r="F18" s="84"/>
-      <c r="G18" s="84"/>
-      <c r="H18" s="84"/>
-      <c r="I18" s="84"/>
+      <c r="C18" s="85"/>
+      <c r="D18" s="86"/>
+      <c r="E18" s="86"/>
+      <c r="F18" s="86"/>
+      <c r="G18" s="86"/>
+      <c r="H18" s="86"/>
+      <c r="I18" s="86"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="20"/>
+      <c r="I19" s="20"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="46" t="s">
+      <c r="B20" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="C20" s="46"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="46"/>
-      <c r="F20" s="46"/>
-      <c r="G20" s="46"/>
-      <c r="H20" s="46"/>
-      <c r="I20" s="46"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="14"/>
     </row>
     <row r="21" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="75" t="s">
+      <c r="C21" s="73" t="s">
         <v>74</v>
       </c>
-      <c r="D21" s="76"/>
-      <c r="E21" s="76"/>
-      <c r="F21" s="76"/>
-      <c r="G21" s="76"/>
-      <c r="H21" s="76"/>
-      <c r="I21" s="77"/>
+      <c r="D21" s="74"/>
+      <c r="E21" s="74"/>
+      <c r="F21" s="74"/>
+      <c r="G21" s="74"/>
+      <c r="H21" s="74"/>
+      <c r="I21" s="75"/>
     </row>
     <row r="22" spans="2:9" ht="39" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="32" t="s">
+      <c r="C22" s="28" t="s">
         <v>79</v>
       </c>
-      <c r="D22" s="33"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="33"/>
-      <c r="H22" s="33"/>
-      <c r="I22" s="34"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="36"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="36"/>
+      <c r="I22" s="37"/>
     </row>
     <row r="23" spans="2:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="55" t="s">
+      <c r="C23" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="55"/>
-      <c r="E23" s="56" t="s">
+      <c r="D23" s="50"/>
+      <c r="E23" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="56"/>
-      <c r="G23" s="56"/>
-      <c r="H23" s="56"/>
-      <c r="I23" s="56"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="51"/>
+      <c r="H23" s="51"/>
+      <c r="I23" s="51"/>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B24" s="6">
+      <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="82" t="s">
+      <c r="C24" s="89" t="s">
         <v>75</v>
       </c>
-      <c r="D24" s="82"/>
-      <c r="E24" s="55" t="s">
+      <c r="D24" s="89"/>
+      <c r="E24" s="50" t="s">
         <v>80</v>
       </c>
-      <c r="F24" s="55"/>
-      <c r="G24" s="55"/>
-      <c r="H24" s="55"/>
-      <c r="I24" s="55"/>
+      <c r="F24" s="50"/>
+      <c r="G24" s="50"/>
+      <c r="H24" s="50"/>
+      <c r="I24" s="50"/>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B25" s="6">
+      <c r="B25" s="8">
         <v>2</v>
       </c>
-      <c r="C25" s="82" t="s">
+      <c r="C25" s="89" t="s">
         <v>76</v>
       </c>
-      <c r="D25" s="82"/>
-      <c r="E25" s="55"/>
-      <c r="F25" s="55"/>
-      <c r="G25" s="55"/>
-      <c r="H25" s="55"/>
-      <c r="I25" s="55"/>
+      <c r="D25" s="89"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="50"/>
+      <c r="G25" s="50"/>
+      <c r="H25" s="50"/>
+      <c r="I25" s="50"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B26" s="6">
+      <c r="B26" s="8">
         <v>3</v>
       </c>
-      <c r="C26" s="67" t="s">
+      <c r="C26" s="77" t="s">
         <v>77</v>
       </c>
-      <c r="D26" s="68"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="18"/>
-      <c r="G26" s="18"/>
-      <c r="H26" s="18"/>
-      <c r="I26" s="14"/>
+      <c r="D26" s="78"/>
+      <c r="E26" s="26"/>
+      <c r="F26" s="64"/>
+      <c r="G26" s="64"/>
+      <c r="H26" s="64"/>
+      <c r="I26" s="27"/>
     </row>
     <row r="27" spans="2:9" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="51" t="s">
+      <c r="C27" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="D27" s="51"/>
-      <c r="E27" s="51"/>
-      <c r="F27" s="51"/>
-      <c r="G27" s="51"/>
-      <c r="H27" s="51"/>
-      <c r="I27" s="51"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="24"/>
+      <c r="I27" s="24"/>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B28" s="27"/>
-      <c r="C28" s="28"/>
-      <c r="D28" s="28"/>
-      <c r="E28" s="28"/>
-      <c r="F28" s="28"/>
-      <c r="G28" s="28"/>
-      <c r="H28" s="28"/>
-      <c r="I28" s="29"/>
+      <c r="B28" s="32"/>
+      <c r="C28" s="33"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
+      <c r="H28" s="33"/>
+      <c r="I28" s="34"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B29" s="46" t="s">
+      <c r="B29" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C29" s="46"/>
-      <c r="D29" s="46"/>
-      <c r="E29" s="46"/>
-      <c r="F29" s="46"/>
-      <c r="G29" s="46"/>
-      <c r="H29" s="46"/>
-      <c r="I29" s="46"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="14"/>
+      <c r="H29" s="14"/>
+      <c r="I29" s="14"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B30" s="80"/>
-      <c r="C30" s="81"/>
-      <c r="D30" s="81"/>
-      <c r="E30" s="81"/>
-      <c r="F30" s="81"/>
-      <c r="G30" s="81"/>
-      <c r="H30" s="81"/>
-      <c r="I30" s="81"/>
+      <c r="B30" s="87"/>
+      <c r="C30" s="88"/>
+      <c r="D30" s="88"/>
+      <c r="E30" s="88"/>
+      <c r="F30" s="88"/>
+      <c r="G30" s="88"/>
+      <c r="H30" s="88"/>
+      <c r="I30" s="88"/>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B31" s="81"/>
-      <c r="C31" s="81"/>
-      <c r="D31" s="81"/>
-      <c r="E31" s="81"/>
-      <c r="F31" s="81"/>
-      <c r="G31" s="81"/>
-      <c r="H31" s="81"/>
-      <c r="I31" s="81"/>
+      <c r="B31" s="88"/>
+      <c r="C31" s="88"/>
+      <c r="D31" s="88"/>
+      <c r="E31" s="88"/>
+      <c r="F31" s="88"/>
+      <c r="G31" s="88"/>
+      <c r="H31" s="88"/>
+      <c r="I31" s="88"/>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B32" s="81"/>
-      <c r="C32" s="81"/>
-      <c r="D32" s="81"/>
-      <c r="E32" s="81"/>
-      <c r="F32" s="81"/>
-      <c r="G32" s="81"/>
-      <c r="H32" s="81"/>
-      <c r="I32" s="81"/>
+      <c r="B32" s="88"/>
+      <c r="C32" s="88"/>
+      <c r="D32" s="88"/>
+      <c r="E32" s="88"/>
+      <c r="F32" s="88"/>
+      <c r="G32" s="88"/>
+      <c r="H32" s="88"/>
+      <c r="I32" s="88"/>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B33" s="81"/>
-      <c r="C33" s="81"/>
-      <c r="D33" s="81"/>
-      <c r="E33" s="81"/>
-      <c r="F33" s="81"/>
-      <c r="G33" s="81"/>
-      <c r="H33" s="81"/>
-      <c r="I33" s="81"/>
+      <c r="B33" s="88"/>
+      <c r="C33" s="88"/>
+      <c r="D33" s="88"/>
+      <c r="E33" s="88"/>
+      <c r="F33" s="88"/>
+      <c r="G33" s="88"/>
+      <c r="H33" s="88"/>
+      <c r="I33" s="88"/>
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:I33"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="C27:I27"/>
+    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="C21:I21"/>
     <mergeCell ref="C15:I15"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -4442,25 +4985,6 @@
     <mergeCell ref="B10:I12"/>
     <mergeCell ref="B13:I13"/>
     <mergeCell ref="B14:I14"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="C21:I21"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:I33"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="C27:I27"/>
-    <mergeCell ref="B28:I28"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{60ABBC95-3763-1140-8147-BC4DA0DFC780}"/>
@@ -4470,7 +4994,154 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24EB2CC3-0FD4-CD4B-B868-F439D6ACDB2E}">
+  <dimension ref="C4:E21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="30.5" customWidth="1"/>
+    <col min="4" max="4" width="41" customWidth="1"/>
+    <col min="5" max="5" width="37.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C4" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="5" spans="3:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="C5" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="6" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C6" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="7" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C7" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="8" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C8" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="9" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C9" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="10" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C10" s="95" t="s">
+        <v>156</v>
+      </c>
+      <c r="D10" s="96" t="s">
+        <v>158</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="11" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C11" s="100"/>
+      <c r="D11" s="101"/>
+      <c r="E11" s="101"/>
+    </row>
+    <row r="12" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C12" s="97"/>
+      <c r="D12" s="98"/>
+      <c r="E12" s="98"/>
+    </row>
+    <row r="13" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C13" s="97"/>
+      <c r="D13" s="98"/>
+      <c r="E13" s="98"/>
+    </row>
+    <row r="14" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C14" s="97"/>
+      <c r="D14" s="98"/>
+      <c r="E14" s="98"/>
+    </row>
+    <row r="15" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C15" s="97"/>
+      <c r="D15" s="98"/>
+      <c r="E15" s="98"/>
+    </row>
+    <row r="16" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C16" s="97"/>
+      <c r="D16" s="98"/>
+      <c r="E16" s="98"/>
+    </row>
+    <row r="17" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C17" s="97"/>
+      <c r="D17" s="98"/>
+      <c r="E17" s="98"/>
+    </row>
+    <row r="18" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C18" s="97"/>
+      <c r="D18" s="98"/>
+      <c r="E18" s="98"/>
+    </row>
+    <row r="19" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C19" s="97"/>
+      <c r="D19" s="99"/>
+      <c r="E19" s="98"/>
+    </row>
+    <row r="20" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C20" s="97"/>
+      <c r="D20" s="99"/>
+      <c r="E20" s="98"/>
+    </row>
+    <row r="21" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C21" s="99"/>
+      <c r="D21" s="99"/>
+      <c r="E21" s="99"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{625A714D-2F1D-8548-AF4D-43E8CCED86F0}">
   <dimension ref="B2:I38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4483,515 +5154,489 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="78" t="s">
+      <c r="C3" s="65" t="s">
         <v>82</v>
       </c>
-      <c r="D3" s="79"/>
-      <c r="E3" s="79"/>
-      <c r="F3" s="79"/>
-      <c r="G3" s="79"/>
-      <c r="H3" s="79"/>
-      <c r="I3" s="79"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="66"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="66"/>
+      <c r="H3" s="66"/>
+      <c r="I3" s="66"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="50" t="s">
+      <c r="C4" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="50"/>
-      <c r="H4" s="50"/>
-      <c r="I4" s="50"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
+      <c r="I4" s="13"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="50">
+      <c r="C5" s="13">
         <v>2025</v>
       </c>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="50"/>
-      <c r="G5" s="50"/>
-      <c r="H5" s="50"/>
-      <c r="I5" s="50"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
+      <c r="I5" s="13"/>
     </row>
     <row r="6" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="52" t="s">
+      <c r="C6" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="52"/>
-      <c r="E6" s="52"/>
-      <c r="F6" s="52"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="52"/>
-      <c r="I6" s="52"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="25"/>
+      <c r="I6" s="25"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="59" t="s">
+      <c r="C7" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="D7" s="50"/>
-      <c r="E7" s="50"/>
-      <c r="F7" s="50"/>
-      <c r="G7" s="50"/>
-      <c r="H7" s="50"/>
-      <c r="I7" s="50"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="46" t="s">
+      <c r="B9" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="46"/>
-      <c r="D9" s="46"/>
-      <c r="E9" s="46"/>
-      <c r="F9" s="46"/>
-      <c r="G9" s="46"/>
-      <c r="H9" s="46"/>
-      <c r="I9" s="46"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B10" s="47" t="s">
+      <c r="B10" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="47"/>
-      <c r="F10" s="47"/>
-      <c r="G10" s="47"/>
-      <c r="H10" s="47"/>
-      <c r="I10" s="47"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B11" s="47"/>
-      <c r="C11" s="47"/>
-      <c r="D11" s="47"/>
-      <c r="E11" s="47"/>
-      <c r="F11" s="47"/>
-      <c r="G11" s="47"/>
-      <c r="H11" s="47"/>
-      <c r="I11" s="47"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B12" s="47"/>
-      <c r="C12" s="47"/>
-      <c r="D12" s="47"/>
-      <c r="E12" s="47"/>
-      <c r="F12" s="47"/>
-      <c r="G12" s="47"/>
-      <c r="H12" s="47"/>
-      <c r="I12" s="47"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="26"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="46" t="s">
+      <c r="B14" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
-      <c r="E14" s="46"/>
-      <c r="F14" s="46"/>
-      <c r="G14" s="46"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="46"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
+      <c r="I14" s="14"/>
     </row>
     <row r="15" spans="2:9" ht="46" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="51" t="s">
+      <c r="C15" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="D15" s="52"/>
-      <c r="E15" s="52"/>
-      <c r="F15" s="52"/>
-      <c r="G15" s="52"/>
-      <c r="H15" s="52"/>
-      <c r="I15" s="52"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="25"/>
+      <c r="H15" s="25"/>
+      <c r="I15" s="25"/>
     </row>
     <row r="16" spans="2:9" ht="59" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="35" t="s">
+      <c r="B16" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="69" t="s">
+      <c r="C16" s="67" t="s">
         <v>88</v>
       </c>
-      <c r="D16" s="70"/>
-      <c r="E16" s="70"/>
-      <c r="F16" s="70"/>
-      <c r="G16" s="70"/>
-      <c r="H16" s="70"/>
-      <c r="I16" s="71"/>
+      <c r="D16" s="68"/>
+      <c r="E16" s="68"/>
+      <c r="F16" s="68"/>
+      <c r="G16" s="68"/>
+      <c r="H16" s="68"/>
+      <c r="I16" s="69"/>
     </row>
     <row r="17" spans="2:9" ht="92" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="36"/>
-      <c r="C17" s="72"/>
-      <c r="D17" s="73"/>
-      <c r="E17" s="73"/>
-      <c r="F17" s="73"/>
-      <c r="G17" s="73"/>
-      <c r="H17" s="73"/>
-      <c r="I17" s="74"/>
+      <c r="B17" s="39"/>
+      <c r="C17" s="70"/>
+      <c r="D17" s="71"/>
+      <c r="E17" s="71"/>
+      <c r="F17" s="71"/>
+      <c r="G17" s="71"/>
+      <c r="H17" s="71"/>
+      <c r="I17" s="72"/>
     </row>
     <row r="18" spans="2:9" ht="256" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="78" t="s">
+      <c r="C18" s="65" t="s">
         <v>89</v>
       </c>
-      <c r="D18" s="50"/>
-      <c r="E18" s="50"/>
-      <c r="F18" s="50"/>
-      <c r="G18" s="50"/>
-      <c r="H18" s="50"/>
-      <c r="I18" s="50"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="13"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="20"/>
+      <c r="I19" s="20"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="46" t="s">
+      <c r="B20" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="C20" s="46"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="46"/>
-      <c r="F20" s="46"/>
-      <c r="G20" s="46"/>
-      <c r="H20" s="46"/>
-      <c r="I20" s="46"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="14"/>
     </row>
     <row r="21" spans="2:9" ht="246" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="75" t="s">
+      <c r="C21" s="73" t="s">
         <v>90</v>
       </c>
-      <c r="D21" s="76"/>
-      <c r="E21" s="76"/>
-      <c r="F21" s="76"/>
-      <c r="G21" s="76"/>
-      <c r="H21" s="76"/>
-      <c r="I21" s="77"/>
+      <c r="D21" s="74"/>
+      <c r="E21" s="74"/>
+      <c r="F21" s="74"/>
+      <c r="G21" s="74"/>
+      <c r="H21" s="74"/>
+      <c r="I21" s="75"/>
     </row>
     <row r="22" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="32">
+      <c r="C22" s="28">
         <v>8</v>
       </c>
-      <c r="D22" s="33"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="33"/>
-      <c r="H22" s="33"/>
-      <c r="I22" s="34"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="36"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="36"/>
+      <c r="I22" s="37"/>
     </row>
     <row r="23" spans="2:9" ht="19" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="55" t="s">
+      <c r="C23" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="55"/>
-      <c r="E23" s="56" t="s">
+      <c r="D23" s="50"/>
+      <c r="E23" s="51" t="s">
         <v>101</v>
       </c>
-      <c r="F23" s="56"/>
-      <c r="G23" s="56"/>
-      <c r="H23" s="56"/>
-      <c r="I23" s="56"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="51"/>
+      <c r="H23" s="51"/>
+      <c r="I23" s="51"/>
     </row>
     <row r="24" spans="2:9" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="6">
+      <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="88" t="s">
+      <c r="C24" s="90" t="s">
         <v>92</v>
       </c>
-      <c r="D24" s="89"/>
-      <c r="E24" s="78" t="s">
+      <c r="D24" s="91"/>
+      <c r="E24" s="65" t="s">
         <v>107</v>
       </c>
-      <c r="F24" s="78"/>
-      <c r="G24" s="78"/>
-      <c r="H24" s="78"/>
-      <c r="I24" s="78"/>
+      <c r="F24" s="65"/>
+      <c r="G24" s="65"/>
+      <c r="H24" s="65"/>
+      <c r="I24" s="65"/>
     </row>
     <row r="25" spans="2:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="6">
+      <c r="B25" s="8">
         <v>2</v>
       </c>
-      <c r="C25" s="86" t="s">
+      <c r="C25" s="92" t="s">
         <v>93</v>
       </c>
-      <c r="D25" s="87"/>
-      <c r="E25" s="78" t="s">
+      <c r="D25" s="93"/>
+      <c r="E25" s="65" t="s">
         <v>108</v>
       </c>
-      <c r="F25" s="78"/>
-      <c r="G25" s="78"/>
-      <c r="H25" s="78"/>
-      <c r="I25" s="78"/>
+      <c r="F25" s="65"/>
+      <c r="G25" s="65"/>
+      <c r="H25" s="65"/>
+      <c r="I25" s="65"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B26" s="6">
+      <c r="B26" s="8">
         <v>3</v>
       </c>
-      <c r="C26" s="86" t="s">
+      <c r="C26" s="92" t="s">
         <v>94</v>
       </c>
-      <c r="D26" s="87"/>
-      <c r="E26" s="78" t="s">
+      <c r="D26" s="93"/>
+      <c r="E26" s="65" t="s">
         <v>106</v>
       </c>
-      <c r="F26" s="78"/>
-      <c r="G26" s="78"/>
-      <c r="H26" s="78"/>
-      <c r="I26" s="78"/>
+      <c r="F26" s="65"/>
+      <c r="G26" s="65"/>
+      <c r="H26" s="65"/>
+      <c r="I26" s="65"/>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B27" s="6">
+      <c r="B27" s="8">
         <v>4</v>
       </c>
-      <c r="C27" s="86" t="s">
+      <c r="C27" s="92" t="s">
         <v>95</v>
       </c>
-      <c r="D27" s="87"/>
-      <c r="E27" s="78" t="s">
+      <c r="D27" s="93"/>
+      <c r="E27" s="65" t="s">
         <v>105</v>
       </c>
-      <c r="F27" s="78"/>
-      <c r="G27" s="78"/>
-      <c r="H27" s="78"/>
-      <c r="I27" s="78"/>
+      <c r="F27" s="65"/>
+      <c r="G27" s="65"/>
+      <c r="H27" s="65"/>
+      <c r="I27" s="65"/>
     </row>
     <row r="28" spans="2:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="6">
+      <c r="B28" s="8">
         <v>5</v>
       </c>
-      <c r="C28" s="86" t="s">
+      <c r="C28" s="92" t="s">
         <v>96</v>
       </c>
-      <c r="D28" s="87"/>
-      <c r="E28" s="78" t="s">
+      <c r="D28" s="93"/>
+      <c r="E28" s="65" t="s">
         <v>104</v>
       </c>
-      <c r="F28" s="78"/>
-      <c r="G28" s="78"/>
-      <c r="H28" s="78"/>
-      <c r="I28" s="78"/>
+      <c r="F28" s="65"/>
+      <c r="G28" s="65"/>
+      <c r="H28" s="65"/>
+      <c r="I28" s="65"/>
     </row>
     <row r="29" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="6">
+      <c r="B29" s="8">
         <v>6</v>
       </c>
-      <c r="C29" s="82" t="s">
+      <c r="C29" s="89" t="s">
         <v>97</v>
       </c>
-      <c r="D29" s="82"/>
-      <c r="E29" s="78" t="s">
+      <c r="D29" s="89"/>
+      <c r="E29" s="65" t="s">
         <v>103</v>
       </c>
-      <c r="F29" s="78"/>
-      <c r="G29" s="78"/>
-      <c r="H29" s="78"/>
-      <c r="I29" s="78"/>
+      <c r="F29" s="65"/>
+      <c r="G29" s="65"/>
+      <c r="H29" s="65"/>
+      <c r="I29" s="65"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B30" s="6">
+      <c r="B30" s="8">
         <v>7</v>
       </c>
-      <c r="C30" s="82" t="s">
+      <c r="C30" s="89" t="s">
         <v>98</v>
       </c>
-      <c r="D30" s="82"/>
-      <c r="E30" s="78" t="s">
+      <c r="D30" s="89"/>
+      <c r="E30" s="65" t="s">
         <v>102</v>
       </c>
-      <c r="F30" s="85"/>
-      <c r="G30" s="85"/>
-      <c r="H30" s="85"/>
-      <c r="I30" s="85"/>
+      <c r="F30" s="94"/>
+      <c r="G30" s="94"/>
+      <c r="H30" s="94"/>
+      <c r="I30" s="94"/>
     </row>
     <row r="31" spans="2:9" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="6">
+      <c r="B31" s="8">
         <v>8</v>
       </c>
-      <c r="C31" s="86" t="s">
+      <c r="C31" s="92" t="s">
         <v>99</v>
       </c>
-      <c r="D31" s="87"/>
-      <c r="E31" s="32" t="s">
+      <c r="D31" s="93"/>
+      <c r="E31" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="F31" s="53"/>
-      <c r="G31" s="53"/>
-      <c r="H31" s="53"/>
-      <c r="I31" s="54"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="29"/>
+      <c r="H31" s="29"/>
+      <c r="I31" s="30"/>
     </row>
     <row r="32" spans="2:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C32" s="51" t="s">
+      <c r="C32" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="D32" s="51"/>
-      <c r="E32" s="51"/>
-      <c r="F32" s="51"/>
-      <c r="G32" s="51"/>
-      <c r="H32" s="51"/>
-      <c r="I32" s="51"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="24"/>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B33" s="27"/>
-      <c r="C33" s="28"/>
-      <c r="D33" s="28"/>
-      <c r="E33" s="28"/>
-      <c r="F33" s="28"/>
-      <c r="G33" s="28"/>
-      <c r="H33" s="28"/>
-      <c r="I33" s="29"/>
+      <c r="B33" s="32"/>
+      <c r="C33" s="33"/>
+      <c r="D33" s="33"/>
+      <c r="E33" s="33"/>
+      <c r="F33" s="33"/>
+      <c r="G33" s="33"/>
+      <c r="H33" s="33"/>
+      <c r="I33" s="34"/>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B34" s="46" t="s">
+      <c r="B34" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C34" s="46"/>
-      <c r="D34" s="46"/>
-      <c r="E34" s="46"/>
-      <c r="F34" s="46"/>
-      <c r="G34" s="46"/>
-      <c r="H34" s="46"/>
-      <c r="I34" s="46"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14"/>
+      <c r="I34" s="14"/>
     </row>
     <row r="35" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="66" t="s">
+      <c r="B35" s="76" t="s">
         <v>109</v>
       </c>
-      <c r="C35" s="48"/>
-      <c r="D35" s="48"/>
-      <c r="E35" s="48"/>
-      <c r="F35" s="48"/>
-      <c r="G35" s="48"/>
-      <c r="H35" s="48"/>
-      <c r="I35" s="48"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="18"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="18"/>
+      <c r="G35" s="18"/>
+      <c r="H35" s="18"/>
+      <c r="I35" s="18"/>
     </row>
     <row r="36" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="48"/>
-      <c r="C36" s="48"/>
-      <c r="D36" s="48"/>
-      <c r="E36" s="48"/>
-      <c r="F36" s="48"/>
-      <c r="G36" s="48"/>
-      <c r="H36" s="48"/>
-      <c r="I36" s="48"/>
+      <c r="B36" s="18"/>
+      <c r="C36" s="18"/>
+      <c r="D36" s="18"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="18"/>
+      <c r="G36" s="18"/>
+      <c r="H36" s="18"/>
+      <c r="I36" s="18"/>
     </row>
     <row r="37" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="48"/>
-      <c r="C37" s="48"/>
-      <c r="D37" s="48"/>
-      <c r="E37" s="48"/>
-      <c r="F37" s="48"/>
-      <c r="G37" s="48"/>
-      <c r="H37" s="48"/>
-      <c r="I37" s="48"/>
+      <c r="B37" s="18"/>
+      <c r="C37" s="18"/>
+      <c r="D37" s="18"/>
+      <c r="E37" s="18"/>
+      <c r="F37" s="18"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="18"/>
+      <c r="I37" s="18"/>
     </row>
     <row r="38" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="48"/>
-      <c r="C38" s="48"/>
-      <c r="D38" s="48"/>
-      <c r="E38" s="48"/>
-      <c r="F38" s="48"/>
-      <c r="G38" s="48"/>
-      <c r="H38" s="48"/>
-      <c r="I38" s="48"/>
+      <c r="B38" s="18"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="18"/>
+      <c r="E38" s="18"/>
+      <c r="F38" s="18"/>
+      <c r="G38" s="18"/>
+      <c r="H38" s="18"/>
+      <c r="I38" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="C7:I7"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="E27:I27"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="C3:I3"/>
-    <mergeCell ref="C4:I4"/>
-    <mergeCell ref="C5:I5"/>
-    <mergeCell ref="C6:I6"/>
-    <mergeCell ref="C21:I21"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="B9:I9"/>
-    <mergeCell ref="B10:I12"/>
-    <mergeCell ref="B13:I13"/>
-    <mergeCell ref="B14:I14"/>
-    <mergeCell ref="C15:I15"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
     <mergeCell ref="B35:I38"/>
     <mergeCell ref="C22:I22"/>
     <mergeCell ref="C23:D23"/>
@@ -5007,6 +5652,32 @@
     <mergeCell ref="C32:I32"/>
     <mergeCell ref="B33:I33"/>
     <mergeCell ref="B34:I34"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B9:I9"/>
+    <mergeCell ref="B10:I12"/>
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="C15:I15"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{69FD07AD-7FCA-E141-8126-AFB63E0A1511}"/>
@@ -5014,4 +5685,184 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{134BA8C2-F108-0848-8F24-448939A23463}">
+  <dimension ref="C3:E17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="4" width="32.83203125" customWidth="1"/>
+    <col min="5" max="5" width="29.1640625" customWidth="1"/>
+    <col min="6" max="6" width="32.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C3" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="4" spans="3:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="C4" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="5" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C5" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="6" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C6" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="7" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C7" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="8" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C8" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="9" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C9" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="10" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C10" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="11" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C11" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="12" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C12" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="13" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C13" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="14" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C14" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="15" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C15" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="16" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C16" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="17" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C17" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
created a word doc for the process that gonna be made for the prompts´construction
</commit_message>
<xml_diff>
--- a/Papers/Resumen Papers.xlsx
+++ b/Papers/Resumen Papers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sophiaaristizabal/Documents/GitHub/LLMS_Project/Papers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{183EE981-4C46-A645-8BD3-D7D0C4D79BC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82B2D0B8-B0C4-0740-9951-86CE8CCB62E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16220" activeTab="1" xr2:uid="{400AC57E-08F9-B346-9132-4F74AEBC2D15}"/>
+    <workbookView xWindow="13020" yWindow="500" windowWidth="15780" windowHeight="16180" activeTab="1" xr2:uid="{400AC57E-08F9-B346-9132-4F74AEBC2D15}"/>
   </bookViews>
   <sheets>
     <sheet name="MANAGERIAL LEADERSHIP" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
obtained the new dataset from Jordi's paper and merged it with one of the previous dta. Decided to merge the chat and the  respective tags with R in stead of Stata 🌞
</commit_message>
<xml_diff>
--- a/Papers/Resumen Papers.xlsx
+++ b/Papers/Resumen Papers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sophiaaristizabal/Documents/GitHub/LLMS_Project/Papers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82B2D0B8-B0C4-0740-9951-86CE8CCB62E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C530E70-6F68-C345-BA07-AC8460941B51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13020" yWindow="500" windowWidth="15780" windowHeight="16180" activeTab="1" xr2:uid="{400AC57E-08F9-B346-9132-4F74AEBC2D15}"/>
+    <workbookView xWindow="5880" yWindow="500" windowWidth="18460" windowHeight="16180" activeTab="2" xr2:uid="{400AC57E-08F9-B346-9132-4F74AEBC2D15}"/>
   </bookViews>
   <sheets>
     <sheet name="MANAGERIAL LEADERSHIP" sheetId="1" r:id="rId1"/>
@@ -2367,7 +2367,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2400,164 +2400,236 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -2565,59 +2637,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -2625,13 +2652,13 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2639,34 +2666,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3217,542 +3216,523 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="55" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="69" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
+      <c r="D3" s="69"/>
+      <c r="E3" s="69"/>
+      <c r="F3" s="69"/>
+      <c r="G3" s="69"/>
+      <c r="H3" s="69"/>
+      <c r="I3" s="69"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="16"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="70"/>
+      <c r="F4" s="70"/>
+      <c r="G4" s="70"/>
+      <c r="H4" s="70"/>
+      <c r="I4" s="70"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="63">
         <v>2025</v>
       </c>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
+      <c r="D5" s="63"/>
+      <c r="E5" s="63"/>
+      <c r="F5" s="63"/>
+      <c r="G5" s="63"/>
+      <c r="H5" s="63"/>
+      <c r="I5" s="63"/>
     </row>
     <row r="6" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="63" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
+      <c r="D6" s="63"/>
+      <c r="E6" s="63"/>
+      <c r="F6" s="63"/>
+      <c r="G6" s="63"/>
+      <c r="H6" s="63"/>
+      <c r="I6" s="63"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="68" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
+      <c r="D7" s="63"/>
+      <c r="E7" s="63"/>
+      <c r="F7" s="63"/>
+      <c r="G7" s="63"/>
+      <c r="H7" s="63"/>
+      <c r="I7" s="63"/>
     </row>
     <row r="8" spans="2:9" ht="9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="20"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="34"/>
     </row>
     <row r="9" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
+      <c r="C9" s="55"/>
+      <c r="D9" s="55"/>
+      <c r="E9" s="55"/>
+      <c r="F9" s="55"/>
+      <c r="G9" s="55"/>
+      <c r="H9" s="55"/>
+      <c r="I9" s="55"/>
     </row>
     <row r="10" spans="2:9" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
+      <c r="C10" s="60"/>
+      <c r="D10" s="60"/>
+      <c r="E10" s="60"/>
+      <c r="F10" s="60"/>
+      <c r="G10" s="60"/>
+      <c r="H10" s="60"/>
+      <c r="I10" s="60"/>
     </row>
     <row r="11" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
+      <c r="B11" s="60"/>
+      <c r="C11" s="60"/>
+      <c r="D11" s="60"/>
+      <c r="E11" s="60"/>
+      <c r="F11" s="60"/>
+      <c r="G11" s="60"/>
+      <c r="H11" s="60"/>
+      <c r="I11" s="60"/>
     </row>
     <row r="12" spans="2:9" ht="11" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
+      <c r="B12" s="60"/>
+      <c r="C12" s="60"/>
+      <c r="D12" s="60"/>
+      <c r="E12" s="60"/>
+      <c r="F12" s="60"/>
+      <c r="G12" s="60"/>
+      <c r="H12" s="60"/>
+      <c r="I12" s="60"/>
     </row>
     <row r="13" spans="2:9" ht="9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="20"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="34"/>
+      <c r="I13" s="34"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="14"/>
+      <c r="C14" s="55"/>
+      <c r="D14" s="55"/>
+      <c r="E14" s="55"/>
+      <c r="F14" s="55"/>
+      <c r="G14" s="55"/>
+      <c r="H14" s="55"/>
+      <c r="I14" s="55"/>
     </row>
     <row r="15" spans="2:9" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="62" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="13"/>
+      <c r="D15" s="63"/>
+      <c r="E15" s="63"/>
+      <c r="F15" s="63"/>
+      <c r="G15" s="63"/>
+      <c r="H15" s="63"/>
+      <c r="I15" s="63"/>
     </row>
     <row r="16" spans="2:9" ht="125" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="38" t="s">
+      <c r="B16" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="40" t="s">
+      <c r="C16" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="D16" s="41"/>
-      <c r="E16" s="41"/>
-      <c r="F16" s="41"/>
-      <c r="G16" s="41"/>
-      <c r="H16" s="41"/>
-      <c r="I16" s="42"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="47"/>
+      <c r="G16" s="47"/>
+      <c r="H16" s="47"/>
+      <c r="I16" s="48"/>
     </row>
     <row r="17" spans="2:9" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="39"/>
-      <c r="C17" s="43"/>
-      <c r="D17" s="44"/>
-      <c r="E17" s="44"/>
-      <c r="F17" s="44"/>
-      <c r="G17" s="44"/>
-      <c r="H17" s="44"/>
-      <c r="I17" s="45"/>
+      <c r="B17" s="45"/>
+      <c r="C17" s="49"/>
+      <c r="D17" s="50"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="50"/>
+      <c r="G17" s="50"/>
+      <c r="H17" s="50"/>
+      <c r="I17" s="51"/>
     </row>
     <row r="18" spans="2:9" ht="67" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="19" t="s">
+      <c r="C18" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13"/>
+      <c r="D18" s="63"/>
+      <c r="E18" s="63"/>
+      <c r="F18" s="63"/>
+      <c r="G18" s="63"/>
+      <c r="H18" s="63"/>
+      <c r="I18" s="63"/>
     </row>
     <row r="19" spans="2:9" ht="7" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
+      <c r="B19" s="34"/>
+      <c r="C19" s="34"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="34"/>
+      <c r="I19" s="34"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="55" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="14"/>
+      <c r="C20" s="55"/>
+      <c r="D20" s="55"/>
+      <c r="E20" s="55"/>
+      <c r="F20" s="55"/>
+      <c r="G20" s="55"/>
+      <c r="H20" s="55"/>
+      <c r="I20" s="55"/>
     </row>
     <row r="21" spans="2:9" ht="43" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="35" t="s">
+      <c r="C21" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="22"/>
-      <c r="I21" s="23"/>
+      <c r="D21" s="39"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="39"/>
+      <c r="H21" s="39"/>
+      <c r="I21" s="40"/>
     </row>
     <row r="22" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B22" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="28">
+      <c r="C22" s="41">
         <v>9</v>
       </c>
-      <c r="D22" s="36"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="36"/>
-      <c r="G22" s="36"/>
-      <c r="H22" s="36"/>
-      <c r="I22" s="37"/>
+      <c r="D22" s="42"/>
+      <c r="E22" s="42"/>
+      <c r="F22" s="42"/>
+      <c r="G22" s="42"/>
+      <c r="H22" s="42"/>
+      <c r="I22" s="43"/>
     </row>
     <row r="23" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="50" t="s">
+      <c r="C23" s="56" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="50"/>
-      <c r="E23" s="51" t="s">
+      <c r="D23" s="56"/>
+      <c r="E23" s="57" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="51"/>
-      <c r="G23" s="51"/>
-      <c r="H23" s="51"/>
-      <c r="I23" s="51"/>
+      <c r="F23" s="57"/>
+      <c r="G23" s="57"/>
+      <c r="H23" s="57"/>
+      <c r="I23" s="57"/>
     </row>
     <row r="24" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="48" t="s">
+      <c r="C24" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="D24" s="49"/>
-      <c r="E24" s="35" t="s">
+      <c r="D24" s="23"/>
+      <c r="E24" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="F24" s="52"/>
-      <c r="G24" s="52"/>
-      <c r="H24" s="52"/>
-      <c r="I24" s="53"/>
+      <c r="F24" s="58"/>
+      <c r="G24" s="58"/>
+      <c r="H24" s="58"/>
+      <c r="I24" s="59"/>
     </row>
     <row r="25" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="8">
         <v>2</v>
       </c>
-      <c r="C25" s="48" t="s">
+      <c r="C25" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="D25" s="49"/>
-      <c r="E25" s="48"/>
-      <c r="F25" s="54"/>
-      <c r="G25" s="54"/>
-      <c r="H25" s="54"/>
-      <c r="I25" s="49"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="23"/>
     </row>
     <row r="26" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="55">
+      <c r="B26" s="25">
         <v>3</v>
       </c>
-      <c r="C26" s="57" t="s">
+      <c r="C26" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="D26" s="58"/>
-      <c r="E26" s="31" t="s">
+      <c r="D26" s="28"/>
+      <c r="E26" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="F26" s="31"/>
-      <c r="G26" s="54" t="s">
+      <c r="F26" s="24"/>
+      <c r="G26" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="H26" s="54"/>
-      <c r="I26" s="49"/>
+      <c r="H26" s="22"/>
+      <c r="I26" s="23"/>
     </row>
     <row r="27" spans="2:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="56"/>
-      <c r="C27" s="59"/>
-      <c r="D27" s="60"/>
-      <c r="E27" s="26" t="s">
+      <c r="B27" s="26"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="30"/>
+      <c r="E27" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="F27" s="27"/>
-      <c r="G27" s="61" t="s">
+      <c r="F27" s="19"/>
+      <c r="G27" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="H27" s="62"/>
-      <c r="I27" s="63"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="33"/>
     </row>
     <row r="28" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="8">
         <v>4</v>
       </c>
-      <c r="C28" s="26" t="s">
+      <c r="C28" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="D28" s="27"/>
-      <c r="E28" s="21" t="s">
+      <c r="D28" s="19"/>
+      <c r="E28" s="52" t="s">
         <v>32</v>
       </c>
-      <c r="F28" s="22"/>
-      <c r="G28" s="22"/>
-      <c r="H28" s="22"/>
-      <c r="I28" s="23"/>
+      <c r="F28" s="39"/>
+      <c r="G28" s="39"/>
+      <c r="H28" s="39"/>
+      <c r="I28" s="40"/>
     </row>
     <row r="29" spans="2:9" ht="43" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="8">
         <v>5</v>
       </c>
-      <c r="C29" s="31" t="s">
+      <c r="C29" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="D29" s="31"/>
-      <c r="E29" s="24" t="s">
+      <c r="D29" s="24"/>
+      <c r="E29" s="64" t="s">
         <v>33</v>
       </c>
-      <c r="F29" s="24"/>
-      <c r="G29" s="24"/>
-      <c r="H29" s="24"/>
-      <c r="I29" s="24"/>
+      <c r="F29" s="64"/>
+      <c r="G29" s="64"/>
+      <c r="H29" s="64"/>
+      <c r="I29" s="64"/>
     </row>
     <row r="30" spans="2:9" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="8">
         <v>6</v>
       </c>
-      <c r="C30" s="26" t="s">
+      <c r="C30" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="D30" s="27"/>
-      <c r="E30" s="21" t="s">
+      <c r="D30" s="19"/>
+      <c r="E30" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="F30" s="46"/>
-      <c r="G30" s="46"/>
-      <c r="H30" s="46"/>
-      <c r="I30" s="47"/>
+      <c r="F30" s="53"/>
+      <c r="G30" s="53"/>
+      <c r="H30" s="53"/>
+      <c r="I30" s="54"/>
     </row>
     <row r="31" spans="2:9" ht="53" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="8">
         <v>7</v>
       </c>
-      <c r="C31" s="31" t="s">
+      <c r="C31" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="D31" s="31"/>
-      <c r="E31" s="24" t="s">
+      <c r="D31" s="24"/>
+      <c r="E31" s="64" t="s">
         <v>35</v>
       </c>
-      <c r="F31" s="25"/>
-      <c r="G31" s="25"/>
-      <c r="H31" s="25"/>
-      <c r="I31" s="25"/>
+      <c r="F31" s="65"/>
+      <c r="G31" s="65"/>
+      <c r="H31" s="65"/>
+      <c r="I31" s="65"/>
     </row>
     <row r="32" spans="2:9" ht="53" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="8">
         <v>8</v>
       </c>
-      <c r="C32" s="26" t="s">
+      <c r="C32" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="D32" s="27"/>
-      <c r="E32" s="26"/>
-      <c r="F32" s="64"/>
-      <c r="G32" s="64"/>
-      <c r="H32" s="64"/>
-      <c r="I32" s="27"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="20"/>
+      <c r="G32" s="20"/>
+      <c r="H32" s="20"/>
+      <c r="I32" s="19"/>
     </row>
     <row r="33" spans="2:9" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="8">
         <v>9</v>
       </c>
-      <c r="C33" s="26" t="s">
+      <c r="C33" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="D33" s="27"/>
-      <c r="E33" s="28" t="s">
+      <c r="D33" s="19"/>
+      <c r="E33" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="F33" s="29"/>
-      <c r="G33" s="29"/>
-      <c r="H33" s="29"/>
-      <c r="I33" s="30"/>
+      <c r="F33" s="66"/>
+      <c r="G33" s="66"/>
+      <c r="H33" s="66"/>
+      <c r="I33" s="67"/>
     </row>
     <row r="34" spans="2:9" ht="190" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C34" s="24" t="s">
+      <c r="C34" s="64" t="s">
         <v>31</v>
       </c>
-      <c r="D34" s="24"/>
-      <c r="E34" s="24"/>
-      <c r="F34" s="24"/>
-      <c r="G34" s="24"/>
-      <c r="H34" s="24"/>
-      <c r="I34" s="24"/>
+      <c r="D34" s="64"/>
+      <c r="E34" s="64"/>
+      <c r="F34" s="64"/>
+      <c r="G34" s="64"/>
+      <c r="H34" s="64"/>
+      <c r="I34" s="64"/>
     </row>
     <row r="35" spans="2:9" ht="10" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="32"/>
-      <c r="C35" s="33"/>
-      <c r="D35" s="33"/>
-      <c r="E35" s="33"/>
-      <c r="F35" s="33"/>
-      <c r="G35" s="33"/>
-      <c r="H35" s="33"/>
-      <c r="I35" s="34"/>
+      <c r="B35" s="35"/>
+      <c r="C35" s="36"/>
+      <c r="D35" s="36"/>
+      <c r="E35" s="36"/>
+      <c r="F35" s="36"/>
+      <c r="G35" s="36"/>
+      <c r="H35" s="36"/>
+      <c r="I35" s="37"/>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B36" s="14" t="s">
+      <c r="B36" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="14"/>
-      <c r="H36" s="14"/>
-      <c r="I36" s="14"/>
+      <c r="C36" s="55"/>
+      <c r="D36" s="55"/>
+      <c r="E36" s="55"/>
+      <c r="F36" s="55"/>
+      <c r="G36" s="55"/>
+      <c r="H36" s="55"/>
+      <c r="I36" s="55"/>
     </row>
     <row r="37" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="18" t="s">
+      <c r="B37" s="61" t="s">
         <v>48</v>
       </c>
-      <c r="C37" s="18"/>
-      <c r="D37" s="18"/>
-      <c r="E37" s="18"/>
-      <c r="F37" s="18"/>
-      <c r="G37" s="18"/>
-      <c r="H37" s="18"/>
-      <c r="I37" s="18"/>
+      <c r="C37" s="61"/>
+      <c r="D37" s="61"/>
+      <c r="E37" s="61"/>
+      <c r="F37" s="61"/>
+      <c r="G37" s="61"/>
+      <c r="H37" s="61"/>
+      <c r="I37" s="61"/>
     </row>
     <row r="38" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="18"/>
-      <c r="C38" s="18"/>
-      <c r="D38" s="18"/>
-      <c r="E38" s="18"/>
-      <c r="F38" s="18"/>
-      <c r="G38" s="18"/>
-      <c r="H38" s="18"/>
-      <c r="I38" s="18"/>
+      <c r="B38" s="61"/>
+      <c r="C38" s="61"/>
+      <c r="D38" s="61"/>
+      <c r="E38" s="61"/>
+      <c r="F38" s="61"/>
+      <c r="G38" s="61"/>
+      <c r="H38" s="61"/>
+      <c r="I38" s="61"/>
     </row>
     <row r="39" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="18"/>
-      <c r="C39" s="18"/>
-      <c r="D39" s="18"/>
-      <c r="E39" s="18"/>
-      <c r="F39" s="18"/>
-      <c r="G39" s="18"/>
-      <c r="H39" s="18"/>
-      <c r="I39" s="18"/>
+      <c r="B39" s="61"/>
+      <c r="C39" s="61"/>
+      <c r="D39" s="61"/>
+      <c r="E39" s="61"/>
+      <c r="F39" s="61"/>
+      <c r="G39" s="61"/>
+      <c r="H39" s="61"/>
+      <c r="I39" s="61"/>
     </row>
     <row r="40" spans="2:9" ht="76" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B40" s="18"/>
-      <c r="C40" s="18"/>
-      <c r="D40" s="18"/>
-      <c r="E40" s="18"/>
-      <c r="F40" s="18"/>
-      <c r="G40" s="18"/>
-      <c r="H40" s="18"/>
-      <c r="I40" s="18"/>
+      <c r="B40" s="61"/>
+      <c r="C40" s="61"/>
+      <c r="D40" s="61"/>
+      <c r="E40" s="61"/>
+      <c r="F40" s="61"/>
+      <c r="G40" s="61"/>
+      <c r="H40" s="61"/>
+      <c r="I40" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="E32:I32"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="C26:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="B35:I35"/>
-    <mergeCell ref="B13:I13"/>
-    <mergeCell ref="C21:I21"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:I30"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="B14:I14"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="C6:I6"/>
     <mergeCell ref="B36:I36"/>
     <mergeCell ref="B10:I12"/>
     <mergeCell ref="B9:I9"/>
@@ -3769,12 +3749,31 @@
     <mergeCell ref="C28:D28"/>
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C7:I7"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="C3:I3"/>
-    <mergeCell ref="C4:I4"/>
-    <mergeCell ref="C5:I5"/>
-    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="C26:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="E32:I32"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="G26:I26"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{C9E9977D-5134-FE4B-852F-8DEBDCB543E0}"/>
@@ -3803,12 +3802,12 @@
   </cols>
   <sheetData>
     <row r="4" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="70" t="s">
         <v>133</v>
       </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
+      <c r="C4" s="70"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="70"/>
     </row>
     <row r="5" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="11" t="s">
@@ -4079,442 +4078,421 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="55" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="65" t="s">
+      <c r="C3" s="89" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
-      <c r="I3" s="66"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="90"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="63" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
+      <c r="D4" s="63"/>
+      <c r="E4" s="63"/>
+      <c r="F4" s="63"/>
+      <c r="G4" s="63"/>
+      <c r="H4" s="63"/>
+      <c r="I4" s="63"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="63">
         <v>2020</v>
       </c>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
+      <c r="D5" s="63"/>
+      <c r="E5" s="63"/>
+      <c r="F5" s="63"/>
+      <c r="G5" s="63"/>
+      <c r="H5" s="63"/>
+      <c r="I5" s="63"/>
     </row>
     <row r="6" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="65" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="25"/>
+      <c r="D6" s="65"/>
+      <c r="E6" s="65"/>
+      <c r="F6" s="65"/>
+      <c r="G6" s="65"/>
+      <c r="H6" s="65"/>
+      <c r="I6" s="65"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="68" t="s">
         <v>51</v>
       </c>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
+      <c r="D7" s="63"/>
+      <c r="E7" s="63"/>
+      <c r="F7" s="63"/>
+      <c r="G7" s="63"/>
+      <c r="H7" s="63"/>
+      <c r="I7" s="63"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="20"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="34"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
+      <c r="C9" s="55"/>
+      <c r="D9" s="55"/>
+      <c r="E9" s="55"/>
+      <c r="F9" s="55"/>
+      <c r="G9" s="55"/>
+      <c r="H9" s="55"/>
+      <c r="I9" s="55"/>
     </row>
     <row r="10" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="60" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
+      <c r="C10" s="60"/>
+      <c r="D10" s="60"/>
+      <c r="E10" s="60"/>
+      <c r="F10" s="60"/>
+      <c r="G10" s="60"/>
+      <c r="H10" s="60"/>
+      <c r="I10" s="60"/>
     </row>
     <row r="11" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
+      <c r="B11" s="60"/>
+      <c r="C11" s="60"/>
+      <c r="D11" s="60"/>
+      <c r="E11" s="60"/>
+      <c r="F11" s="60"/>
+      <c r="G11" s="60"/>
+      <c r="H11" s="60"/>
+      <c r="I11" s="60"/>
     </row>
     <row r="12" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
+      <c r="B12" s="60"/>
+      <c r="C12" s="60"/>
+      <c r="D12" s="60"/>
+      <c r="E12" s="60"/>
+      <c r="F12" s="60"/>
+      <c r="G12" s="60"/>
+      <c r="H12" s="60"/>
+      <c r="I12" s="60"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="20"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="34"/>
+      <c r="I13" s="34"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="14"/>
+      <c r="C14" s="55"/>
+      <c r="D14" s="55"/>
+      <c r="E14" s="55"/>
+      <c r="F14" s="55"/>
+      <c r="G14" s="55"/>
+      <c r="H14" s="55"/>
+      <c r="I14" s="55"/>
     </row>
     <row r="15" spans="2:9" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="62" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="13"/>
+      <c r="D15" s="63"/>
+      <c r="E15" s="63"/>
+      <c r="F15" s="63"/>
+      <c r="G15" s="63"/>
+      <c r="H15" s="63"/>
+      <c r="I15" s="63"/>
     </row>
     <row r="16" spans="2:9" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="38" t="s">
+      <c r="B16" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="67" t="s">
+      <c r="C16" s="80" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="68"/>
-      <c r="E16" s="68"/>
-      <c r="F16" s="68"/>
-      <c r="G16" s="68"/>
-      <c r="H16" s="68"/>
-      <c r="I16" s="69"/>
+      <c r="D16" s="81"/>
+      <c r="E16" s="81"/>
+      <c r="F16" s="81"/>
+      <c r="G16" s="81"/>
+      <c r="H16" s="81"/>
+      <c r="I16" s="82"/>
     </row>
     <row r="17" spans="2:9" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="39"/>
-      <c r="C17" s="70"/>
-      <c r="D17" s="71"/>
-      <c r="E17" s="71"/>
-      <c r="F17" s="71"/>
-      <c r="G17" s="71"/>
-      <c r="H17" s="71"/>
-      <c r="I17" s="72"/>
+      <c r="B17" s="45"/>
+      <c r="C17" s="83"/>
+      <c r="D17" s="84"/>
+      <c r="E17" s="84"/>
+      <c r="F17" s="84"/>
+      <c r="G17" s="84"/>
+      <c r="H17" s="84"/>
+      <c r="I17" s="85"/>
     </row>
     <row r="18" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="19" t="s">
+      <c r="C18" s="62" t="s">
         <v>56</v>
       </c>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13"/>
+      <c r="D18" s="63"/>
+      <c r="E18" s="63"/>
+      <c r="F18" s="63"/>
+      <c r="G18" s="63"/>
+      <c r="H18" s="63"/>
+      <c r="I18" s="63"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
+      <c r="B19" s="34"/>
+      <c r="C19" s="34"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="34"/>
+      <c r="I19" s="34"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="55" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="14"/>
+      <c r="C20" s="55"/>
+      <c r="D20" s="55"/>
+      <c r="E20" s="55"/>
+      <c r="F20" s="55"/>
+      <c r="G20" s="55"/>
+      <c r="H20" s="55"/>
+      <c r="I20" s="55"/>
     </row>
     <row r="21" spans="2:9" ht="160" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="73" t="s">
+      <c r="C21" s="86" t="s">
         <v>57</v>
       </c>
-      <c r="D21" s="74"/>
-      <c r="E21" s="74"/>
-      <c r="F21" s="74"/>
-      <c r="G21" s="74"/>
-      <c r="H21" s="74"/>
-      <c r="I21" s="75"/>
+      <c r="D21" s="87"/>
+      <c r="E21" s="87"/>
+      <c r="F21" s="87"/>
+      <c r="G21" s="87"/>
+      <c r="H21" s="87"/>
+      <c r="I21" s="88"/>
     </row>
     <row r="22" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="28">
+      <c r="C22" s="41">
         <v>3</v>
       </c>
-      <c r="D22" s="36"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="36"/>
-      <c r="G22" s="36"/>
-      <c r="H22" s="36"/>
-      <c r="I22" s="37"/>
+      <c r="D22" s="42"/>
+      <c r="E22" s="42"/>
+      <c r="F22" s="42"/>
+      <c r="G22" s="42"/>
+      <c r="H22" s="42"/>
+      <c r="I22" s="43"/>
     </row>
     <row r="23" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="50" t="s">
+      <c r="C23" s="56" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="50"/>
-      <c r="E23" s="51" t="s">
+      <c r="D23" s="56"/>
+      <c r="E23" s="57" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="51"/>
-      <c r="G23" s="51"/>
-      <c r="H23" s="51"/>
-      <c r="I23" s="51"/>
+      <c r="F23" s="57"/>
+      <c r="G23" s="57"/>
+      <c r="H23" s="57"/>
+      <c r="I23" s="57"/>
     </row>
     <row r="24" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="55">
+      <c r="B24" s="25">
         <v>1</v>
       </c>
-      <c r="C24" s="81" t="s">
+      <c r="C24" s="71" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="82"/>
+      <c r="D24" s="72"/>
       <c r="E24" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="F24" s="83" t="s">
+      <c r="F24" s="75" t="s">
         <v>63</v>
       </c>
-      <c r="G24" s="83"/>
-      <c r="H24" s="83"/>
-      <c r="I24" s="84"/>
+      <c r="G24" s="75"/>
+      <c r="H24" s="75"/>
+      <c r="I24" s="76"/>
     </row>
     <row r="25" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="56"/>
-      <c r="C25" s="79"/>
-      <c r="D25" s="80"/>
+      <c r="B25" s="26"/>
+      <c r="C25" s="73"/>
+      <c r="D25" s="74"/>
       <c r="E25" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="F25" s="54" t="s">
+      <c r="F25" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="G25" s="54"/>
-      <c r="H25" s="54"/>
-      <c r="I25" s="49"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="23"/>
     </row>
     <row r="26" spans="2:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="8">
         <v>2</v>
       </c>
-      <c r="C26" s="77" t="s">
+      <c r="C26" s="78" t="s">
         <v>59</v>
       </c>
-      <c r="D26" s="78"/>
-      <c r="E26" s="26"/>
-      <c r="F26" s="64"/>
-      <c r="G26" s="64"/>
-      <c r="H26" s="64"/>
-      <c r="I26" s="27"/>
+      <c r="D26" s="79"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="20"/>
+      <c r="H26" s="20"/>
+      <c r="I26" s="19"/>
     </row>
     <row r="27" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="8">
         <v>3</v>
       </c>
-      <c r="C27" s="79" t="s">
+      <c r="C27" s="73" t="s">
         <v>60</v>
       </c>
-      <c r="D27" s="80"/>
-      <c r="E27" s="26"/>
-      <c r="F27" s="64"/>
-      <c r="G27" s="64"/>
-      <c r="H27" s="64"/>
-      <c r="I27" s="27"/>
+      <c r="D27" s="74"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="20"/>
+      <c r="I27" s="19"/>
     </row>
     <row r="28" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B28" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C28" s="24" t="s">
+      <c r="C28" s="64" t="s">
         <v>65</v>
       </c>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
-      <c r="G28" s="24"/>
-      <c r="H28" s="24"/>
-      <c r="I28" s="24"/>
+      <c r="D28" s="64"/>
+      <c r="E28" s="64"/>
+      <c r="F28" s="64"/>
+      <c r="G28" s="64"/>
+      <c r="H28" s="64"/>
+      <c r="I28" s="64"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B29" s="32"/>
-      <c r="C29" s="33"/>
-      <c r="D29" s="33"/>
-      <c r="E29" s="33"/>
-      <c r="F29" s="33"/>
-      <c r="G29" s="33"/>
-      <c r="H29" s="33"/>
-      <c r="I29" s="34"/>
+      <c r="B29" s="35"/>
+      <c r="C29" s="36"/>
+      <c r="D29" s="36"/>
+      <c r="E29" s="36"/>
+      <c r="F29" s="36"/>
+      <c r="G29" s="36"/>
+      <c r="H29" s="36"/>
+      <c r="I29" s="37"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B30" s="14" t="s">
+      <c r="B30" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="14"/>
+      <c r="C30" s="55"/>
+      <c r="D30" s="55"/>
+      <c r="E30" s="55"/>
+      <c r="F30" s="55"/>
+      <c r="G30" s="55"/>
+      <c r="H30" s="55"/>
+      <c r="I30" s="55"/>
     </row>
     <row r="31" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="76" t="s">
+      <c r="B31" s="77" t="s">
         <v>66</v>
       </c>
-      <c r="C31" s="18"/>
-      <c r="D31" s="18"/>
-      <c r="E31" s="18"/>
-      <c r="F31" s="18"/>
-      <c r="G31" s="18"/>
-      <c r="H31" s="18"/>
-      <c r="I31" s="18"/>
+      <c r="C31" s="61"/>
+      <c r="D31" s="61"/>
+      <c r="E31" s="61"/>
+      <c r="F31" s="61"/>
+      <c r="G31" s="61"/>
+      <c r="H31" s="61"/>
+      <c r="I31" s="61"/>
     </row>
     <row r="32" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="18"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="18"/>
-      <c r="E32" s="18"/>
-      <c r="F32" s="18"/>
-      <c r="G32" s="18"/>
-      <c r="H32" s="18"/>
-      <c r="I32" s="18"/>
+      <c r="B32" s="61"/>
+      <c r="C32" s="61"/>
+      <c r="D32" s="61"/>
+      <c r="E32" s="61"/>
+      <c r="F32" s="61"/>
+      <c r="G32" s="61"/>
+      <c r="H32" s="61"/>
+      <c r="I32" s="61"/>
     </row>
     <row r="33" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="18"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="18"/>
-      <c r="G33" s="18"/>
-      <c r="H33" s="18"/>
-      <c r="I33" s="18"/>
+      <c r="B33" s="61"/>
+      <c r="C33" s="61"/>
+      <c r="D33" s="61"/>
+      <c r="E33" s="61"/>
+      <c r="F33" s="61"/>
+      <c r="G33" s="61"/>
+      <c r="H33" s="61"/>
+      <c r="I33" s="61"/>
     </row>
     <row r="34" spans="2:9" ht="254" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="18"/>
-      <c r="C34" s="18"/>
-      <c r="D34" s="18"/>
-      <c r="E34" s="18"/>
-      <c r="F34" s="18"/>
-      <c r="G34" s="18"/>
-      <c r="H34" s="18"/>
-      <c r="I34" s="18"/>
+      <c r="B34" s="61"/>
+      <c r="C34" s="61"/>
+      <c r="D34" s="61"/>
+      <c r="E34" s="61"/>
+      <c r="F34" s="61"/>
+      <c r="G34" s="61"/>
+      <c r="H34" s="61"/>
+      <c r="I34" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:D25"/>
-    <mergeCell ref="F24:I24"/>
-    <mergeCell ref="F25:I25"/>
-    <mergeCell ref="C28:I28"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="B31:I34"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:I27"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="C21:I21"/>
     <mergeCell ref="C15:I15"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -4527,6 +4505,27 @@
     <mergeCell ref="B10:I12"/>
     <mergeCell ref="B13:I13"/>
     <mergeCell ref="B14:I14"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="B31:I34"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:D25"/>
+    <mergeCell ref="F24:I24"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="C28:I28"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{4DBC988E-4FF2-2C49-AA18-DD92CA6A87E8}"/>
@@ -4559,420 +4558,401 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="55" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="65" t="s">
+      <c r="C3" s="89" t="s">
         <v>67</v>
       </c>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
-      <c r="I3" s="66"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="90"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="63" t="s">
         <v>68</v>
       </c>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
+      <c r="D4" s="63"/>
+      <c r="E4" s="63"/>
+      <c r="F4" s="63"/>
+      <c r="G4" s="63"/>
+      <c r="H4" s="63"/>
+      <c r="I4" s="63"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="63">
         <v>2022</v>
       </c>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
+      <c r="D5" s="63"/>
+      <c r="E5" s="63"/>
+      <c r="F5" s="63"/>
+      <c r="G5" s="63"/>
+      <c r="H5" s="63"/>
+      <c r="I5" s="63"/>
     </row>
     <row r="6" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="65" t="s">
         <v>69</v>
       </c>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="25"/>
+      <c r="D6" s="65"/>
+      <c r="E6" s="65"/>
+      <c r="F6" s="65"/>
+      <c r="G6" s="65"/>
+      <c r="H6" s="65"/>
+      <c r="I6" s="65"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="68" t="s">
         <v>70</v>
       </c>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
+      <c r="D7" s="63"/>
+      <c r="E7" s="63"/>
+      <c r="F7" s="63"/>
+      <c r="G7" s="63"/>
+      <c r="H7" s="63"/>
+      <c r="I7" s="63"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="20"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="34"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
+      <c r="C9" s="55"/>
+      <c r="D9" s="55"/>
+      <c r="E9" s="55"/>
+      <c r="F9" s="55"/>
+      <c r="G9" s="55"/>
+      <c r="H9" s="55"/>
+      <c r="I9" s="55"/>
     </row>
     <row r="10" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="60" t="s">
         <v>71</v>
       </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
+      <c r="C10" s="60"/>
+      <c r="D10" s="60"/>
+      <c r="E10" s="60"/>
+      <c r="F10" s="60"/>
+      <c r="G10" s="60"/>
+      <c r="H10" s="60"/>
+      <c r="I10" s="60"/>
     </row>
     <row r="11" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
+      <c r="B11" s="60"/>
+      <c r="C11" s="60"/>
+      <c r="D11" s="60"/>
+      <c r="E11" s="60"/>
+      <c r="F11" s="60"/>
+      <c r="G11" s="60"/>
+      <c r="H11" s="60"/>
+      <c r="I11" s="60"/>
     </row>
     <row r="12" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
+      <c r="B12" s="60"/>
+      <c r="C12" s="60"/>
+      <c r="D12" s="60"/>
+      <c r="E12" s="60"/>
+      <c r="F12" s="60"/>
+      <c r="G12" s="60"/>
+      <c r="H12" s="60"/>
+      <c r="I12" s="60"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="20"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="34"/>
+      <c r="I13" s="34"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="14"/>
+      <c r="C14" s="55"/>
+      <c r="D14" s="55"/>
+      <c r="E14" s="55"/>
+      <c r="F14" s="55"/>
+      <c r="G14" s="55"/>
+      <c r="H14" s="55"/>
+      <c r="I14" s="55"/>
     </row>
     <row r="15" spans="2:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="62" t="s">
         <v>73</v>
       </c>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="13"/>
+      <c r="D15" s="63"/>
+      <c r="E15" s="63"/>
+      <c r="F15" s="63"/>
+      <c r="G15" s="63"/>
+      <c r="H15" s="63"/>
+      <c r="I15" s="63"/>
     </row>
     <row r="16" spans="2:9" ht="247" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="38" t="s">
+      <c r="B16" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="67" t="s">
+      <c r="C16" s="80" t="s">
         <v>72</v>
       </c>
-      <c r="D16" s="68"/>
-      <c r="E16" s="68"/>
-      <c r="F16" s="68"/>
-      <c r="G16" s="68"/>
-      <c r="H16" s="68"/>
-      <c r="I16" s="69"/>
+      <c r="D16" s="81"/>
+      <c r="E16" s="81"/>
+      <c r="F16" s="81"/>
+      <c r="G16" s="81"/>
+      <c r="H16" s="81"/>
+      <c r="I16" s="82"/>
     </row>
     <row r="17" spans="2:9" ht="247" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="39"/>
-      <c r="C17" s="70"/>
-      <c r="D17" s="71"/>
-      <c r="E17" s="71"/>
-      <c r="F17" s="71"/>
-      <c r="G17" s="71"/>
-      <c r="H17" s="71"/>
-      <c r="I17" s="72"/>
+      <c r="B17" s="45"/>
+      <c r="C17" s="83"/>
+      <c r="D17" s="84"/>
+      <c r="E17" s="84"/>
+      <c r="F17" s="84"/>
+      <c r="G17" s="84"/>
+      <c r="H17" s="84"/>
+      <c r="I17" s="85"/>
     </row>
     <row r="18" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="85"/>
-      <c r="D18" s="86"/>
-      <c r="E18" s="86"/>
-      <c r="F18" s="86"/>
-      <c r="G18" s="86"/>
-      <c r="H18" s="86"/>
-      <c r="I18" s="86"/>
+      <c r="C18" s="94"/>
+      <c r="D18" s="95"/>
+      <c r="E18" s="95"/>
+      <c r="F18" s="95"/>
+      <c r="G18" s="95"/>
+      <c r="H18" s="95"/>
+      <c r="I18" s="95"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
+      <c r="B19" s="34"/>
+      <c r="C19" s="34"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="34"/>
+      <c r="I19" s="34"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="14"/>
+      <c r="C20" s="55"/>
+      <c r="D20" s="55"/>
+      <c r="E20" s="55"/>
+      <c r="F20" s="55"/>
+      <c r="G20" s="55"/>
+      <c r="H20" s="55"/>
+      <c r="I20" s="55"/>
     </row>
     <row r="21" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="73" t="s">
+      <c r="C21" s="86" t="s">
         <v>74</v>
       </c>
-      <c r="D21" s="74"/>
-      <c r="E21" s="74"/>
-      <c r="F21" s="74"/>
-      <c r="G21" s="74"/>
-      <c r="H21" s="74"/>
-      <c r="I21" s="75"/>
+      <c r="D21" s="87"/>
+      <c r="E21" s="87"/>
+      <c r="F21" s="87"/>
+      <c r="G21" s="87"/>
+      <c r="H21" s="87"/>
+      <c r="I21" s="88"/>
     </row>
     <row r="22" spans="2:9" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="28" t="s">
+      <c r="C22" s="41" t="s">
         <v>79</v>
       </c>
-      <c r="D22" s="36"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="36"/>
-      <c r="G22" s="36"/>
-      <c r="H22" s="36"/>
-      <c r="I22" s="37"/>
+      <c r="D22" s="42"/>
+      <c r="E22" s="42"/>
+      <c r="F22" s="42"/>
+      <c r="G22" s="42"/>
+      <c r="H22" s="42"/>
+      <c r="I22" s="43"/>
     </row>
     <row r="23" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="50" t="s">
+      <c r="C23" s="56" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="50"/>
-      <c r="E23" s="51" t="s">
+      <c r="D23" s="56"/>
+      <c r="E23" s="57" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="51"/>
-      <c r="G23" s="51"/>
-      <c r="H23" s="51"/>
-      <c r="I23" s="51"/>
+      <c r="F23" s="57"/>
+      <c r="G23" s="57"/>
+      <c r="H23" s="57"/>
+      <c r="I23" s="57"/>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="89" t="s">
+      <c r="C24" s="93" t="s">
         <v>75</v>
       </c>
-      <c r="D24" s="89"/>
-      <c r="E24" s="50" t="s">
+      <c r="D24" s="93"/>
+      <c r="E24" s="56" t="s">
         <v>80</v>
       </c>
-      <c r="F24" s="50"/>
-      <c r="G24" s="50"/>
-      <c r="H24" s="50"/>
-      <c r="I24" s="50"/>
+      <c r="F24" s="56"/>
+      <c r="G24" s="56"/>
+      <c r="H24" s="56"/>
+      <c r="I24" s="56"/>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B25" s="8">
         <v>2</v>
       </c>
-      <c r="C25" s="89" t="s">
+      <c r="C25" s="93" t="s">
         <v>76</v>
       </c>
-      <c r="D25" s="89"/>
-      <c r="E25" s="50"/>
-      <c r="F25" s="50"/>
-      <c r="G25" s="50"/>
-      <c r="H25" s="50"/>
-      <c r="I25" s="50"/>
+      <c r="D25" s="93"/>
+      <c r="E25" s="56"/>
+      <c r="F25" s="56"/>
+      <c r="G25" s="56"/>
+      <c r="H25" s="56"/>
+      <c r="I25" s="56"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B26" s="8">
         <v>3</v>
       </c>
-      <c r="C26" s="77" t="s">
+      <c r="C26" s="78" t="s">
         <v>77</v>
       </c>
-      <c r="D26" s="78"/>
-      <c r="E26" s="26"/>
-      <c r="F26" s="64"/>
-      <c r="G26" s="64"/>
-      <c r="H26" s="64"/>
-      <c r="I26" s="27"/>
+      <c r="D26" s="79"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="20"/>
+      <c r="H26" s="20"/>
+      <c r="I26" s="19"/>
     </row>
     <row r="27" spans="2:9" ht="68" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="24" t="s">
+      <c r="C27" s="64" t="s">
         <v>78</v>
       </c>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
-      <c r="G27" s="24"/>
-      <c r="H27" s="24"/>
-      <c r="I27" s="24"/>
+      <c r="D27" s="64"/>
+      <c r="E27" s="64"/>
+      <c r="F27" s="64"/>
+      <c r="G27" s="64"/>
+      <c r="H27" s="64"/>
+      <c r="I27" s="64"/>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B28" s="32"/>
-      <c r="C28" s="33"/>
-      <c r="D28" s="33"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="33"/>
-      <c r="H28" s="33"/>
-      <c r="I28" s="34"/>
+      <c r="B28" s="35"/>
+      <c r="C28" s="36"/>
+      <c r="D28" s="36"/>
+      <c r="E28" s="36"/>
+      <c r="F28" s="36"/>
+      <c r="G28" s="36"/>
+      <c r="H28" s="36"/>
+      <c r="I28" s="37"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B29" s="14" t="s">
+      <c r="B29" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="14"/>
+      <c r="C29" s="55"/>
+      <c r="D29" s="55"/>
+      <c r="E29" s="55"/>
+      <c r="F29" s="55"/>
+      <c r="G29" s="55"/>
+      <c r="H29" s="55"/>
+      <c r="I29" s="55"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B30" s="87"/>
-      <c r="C30" s="88"/>
-      <c r="D30" s="88"/>
-      <c r="E30" s="88"/>
-      <c r="F30" s="88"/>
-      <c r="G30" s="88"/>
-      <c r="H30" s="88"/>
-      <c r="I30" s="88"/>
+      <c r="B30" s="91"/>
+      <c r="C30" s="92"/>
+      <c r="D30" s="92"/>
+      <c r="E30" s="92"/>
+      <c r="F30" s="92"/>
+      <c r="G30" s="92"/>
+      <c r="H30" s="92"/>
+      <c r="I30" s="92"/>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B31" s="88"/>
-      <c r="C31" s="88"/>
-      <c r="D31" s="88"/>
-      <c r="E31" s="88"/>
-      <c r="F31" s="88"/>
-      <c r="G31" s="88"/>
-      <c r="H31" s="88"/>
-      <c r="I31" s="88"/>
+      <c r="B31" s="92"/>
+      <c r="C31" s="92"/>
+      <c r="D31" s="92"/>
+      <c r="E31" s="92"/>
+      <c r="F31" s="92"/>
+      <c r="G31" s="92"/>
+      <c r="H31" s="92"/>
+      <c r="I31" s="92"/>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B32" s="88"/>
-      <c r="C32" s="88"/>
-      <c r="D32" s="88"/>
-      <c r="E32" s="88"/>
-      <c r="F32" s="88"/>
-      <c r="G32" s="88"/>
-      <c r="H32" s="88"/>
-      <c r="I32" s="88"/>
+      <c r="B32" s="92"/>
+      <c r="C32" s="92"/>
+      <c r="D32" s="92"/>
+      <c r="E32" s="92"/>
+      <c r="F32" s="92"/>
+      <c r="G32" s="92"/>
+      <c r="H32" s="92"/>
+      <c r="I32" s="92"/>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B33" s="88"/>
-      <c r="C33" s="88"/>
-      <c r="D33" s="88"/>
-      <c r="E33" s="88"/>
-      <c r="F33" s="88"/>
-      <c r="G33" s="88"/>
-      <c r="H33" s="88"/>
-      <c r="I33" s="88"/>
+      <c r="B33" s="92"/>
+      <c r="C33" s="92"/>
+      <c r="D33" s="92"/>
+      <c r="E33" s="92"/>
+      <c r="F33" s="92"/>
+      <c r="G33" s="92"/>
+      <c r="H33" s="92"/>
+      <c r="I33" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:I33"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="C27:I27"/>
-    <mergeCell ref="B28:I28"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="C21:I21"/>
     <mergeCell ref="C15:I15"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -4985,6 +4965,25 @@
     <mergeCell ref="B10:I12"/>
     <mergeCell ref="B13:I13"/>
     <mergeCell ref="B14:I14"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:I33"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="C27:I27"/>
+    <mergeCell ref="B28:I28"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{60ABBC95-3763-1140-8147-BC4DA0DFC780}"/>
@@ -4996,7 +4995,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24EB2CC3-0FD4-CD4B-B868-F439D6ACDB2E}">
-  <dimension ref="C4:E21"/>
+  <dimension ref="C4:E20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="30.5" customWidth="1"/>
@@ -5071,10 +5070,10 @@
       </c>
     </row>
     <row r="10" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C10" s="95" t="s">
+      <c r="C10" s="12" t="s">
         <v>156</v>
       </c>
-      <c r="D10" s="96" t="s">
+      <c r="D10" s="13" t="s">
         <v>158</v>
       </c>
       <c r="E10" s="2" t="s">
@@ -5082,59 +5081,52 @@
       </c>
     </row>
     <row r="11" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C11" s="100"/>
-      <c r="D11" s="101"/>
-      <c r="E11" s="101"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
     </row>
     <row r="12" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C12" s="97"/>
-      <c r="D12" s="98"/>
-      <c r="E12" s="98"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
     </row>
     <row r="13" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C13" s="97"/>
-      <c r="D13" s="98"/>
-      <c r="E13" s="98"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
     </row>
     <row r="14" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C14" s="97"/>
-      <c r="D14" s="98"/>
-      <c r="E14" s="98"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
     </row>
     <row r="15" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C15" s="97"/>
-      <c r="D15" s="98"/>
-      <c r="E15" s="98"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
     </row>
     <row r="16" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C16" s="97"/>
-      <c r="D16" s="98"/>
-      <c r="E16" s="98"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
     </row>
     <row r="17" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C17" s="97"/>
-      <c r="D17" s="98"/>
-      <c r="E17" s="98"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
     </row>
     <row r="18" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C18" s="97"/>
-      <c r="D18" s="98"/>
-      <c r="E18" s="98"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
     </row>
     <row r="19" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C19" s="97"/>
-      <c r="D19" s="99"/>
-      <c r="E19" s="98"/>
+      <c r="C19" s="14"/>
+      <c r="E19" s="15"/>
     </row>
     <row r="20" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C20" s="97"/>
-      <c r="D20" s="99"/>
-      <c r="E20" s="98"/>
-    </row>
-    <row r="21" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C21" s="99"/>
-      <c r="D21" s="99"/>
-      <c r="E21" s="99"/>
+      <c r="C20" s="14"/>
+      <c r="E20" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5154,514 +5146,489 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="55" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="65" t="s">
+      <c r="C3" s="89" t="s">
         <v>82</v>
       </c>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
-      <c r="I3" s="66"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="90"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="63" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
+      <c r="D4" s="63"/>
+      <c r="E4" s="63"/>
+      <c r="F4" s="63"/>
+      <c r="G4" s="63"/>
+      <c r="H4" s="63"/>
+      <c r="I4" s="63"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="63">
         <v>2025</v>
       </c>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
+      <c r="D5" s="63"/>
+      <c r="E5" s="63"/>
+      <c r="F5" s="63"/>
+      <c r="G5" s="63"/>
+      <c r="H5" s="63"/>
+      <c r="I5" s="63"/>
     </row>
     <row r="6" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="65" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="25"/>
+      <c r="D6" s="65"/>
+      <c r="E6" s="65"/>
+      <c r="F6" s="65"/>
+      <c r="G6" s="65"/>
+      <c r="H6" s="65"/>
+      <c r="I6" s="65"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="68" t="s">
         <v>84</v>
       </c>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
+      <c r="D7" s="63"/>
+      <c r="E7" s="63"/>
+      <c r="F7" s="63"/>
+      <c r="G7" s="63"/>
+      <c r="H7" s="63"/>
+      <c r="I7" s="63"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="20"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="34"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
+      <c r="C9" s="55"/>
+      <c r="D9" s="55"/>
+      <c r="E9" s="55"/>
+      <c r="F9" s="55"/>
+      <c r="G9" s="55"/>
+      <c r="H9" s="55"/>
+      <c r="I9" s="55"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="60" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
+      <c r="C10" s="60"/>
+      <c r="D10" s="60"/>
+      <c r="E10" s="60"/>
+      <c r="F10" s="60"/>
+      <c r="G10" s="60"/>
+      <c r="H10" s="60"/>
+      <c r="I10" s="60"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
+      <c r="B11" s="60"/>
+      <c r="C11" s="60"/>
+      <c r="D11" s="60"/>
+      <c r="E11" s="60"/>
+      <c r="F11" s="60"/>
+      <c r="G11" s="60"/>
+      <c r="H11" s="60"/>
+      <c r="I11" s="60"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
+      <c r="B12" s="60"/>
+      <c r="C12" s="60"/>
+      <c r="D12" s="60"/>
+      <c r="E12" s="60"/>
+      <c r="F12" s="60"/>
+      <c r="G12" s="60"/>
+      <c r="H12" s="60"/>
+      <c r="I12" s="60"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="20"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="34"/>
+      <c r="I13" s="34"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="14"/>
+      <c r="C14" s="55"/>
+      <c r="D14" s="55"/>
+      <c r="E14" s="55"/>
+      <c r="F14" s="55"/>
+      <c r="G14" s="55"/>
+      <c r="H14" s="55"/>
+      <c r="I14" s="55"/>
     </row>
     <row r="15" spans="2:9" ht="46" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="24" t="s">
+      <c r="C15" s="64" t="s">
         <v>87</v>
       </c>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
-      <c r="I15" s="25"/>
+      <c r="D15" s="65"/>
+      <c r="E15" s="65"/>
+      <c r="F15" s="65"/>
+      <c r="G15" s="65"/>
+      <c r="H15" s="65"/>
+      <c r="I15" s="65"/>
     </row>
     <row r="16" spans="2:9" ht="59" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="38" t="s">
+      <c r="B16" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="67" t="s">
+      <c r="C16" s="80" t="s">
         <v>88</v>
       </c>
-      <c r="D16" s="68"/>
-      <c r="E16" s="68"/>
-      <c r="F16" s="68"/>
-      <c r="G16" s="68"/>
-      <c r="H16" s="68"/>
-      <c r="I16" s="69"/>
+      <c r="D16" s="81"/>
+      <c r="E16" s="81"/>
+      <c r="F16" s="81"/>
+      <c r="G16" s="81"/>
+      <c r="H16" s="81"/>
+      <c r="I16" s="82"/>
     </row>
     <row r="17" spans="2:9" ht="92" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="39"/>
-      <c r="C17" s="70"/>
-      <c r="D17" s="71"/>
-      <c r="E17" s="71"/>
-      <c r="F17" s="71"/>
-      <c r="G17" s="71"/>
-      <c r="H17" s="71"/>
-      <c r="I17" s="72"/>
+      <c r="B17" s="45"/>
+      <c r="C17" s="83"/>
+      <c r="D17" s="84"/>
+      <c r="E17" s="84"/>
+      <c r="F17" s="84"/>
+      <c r="G17" s="84"/>
+      <c r="H17" s="84"/>
+      <c r="I17" s="85"/>
     </row>
     <row r="18" spans="2:9" ht="256" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="65" t="s">
+      <c r="C18" s="89" t="s">
         <v>89</v>
       </c>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13"/>
+      <c r="D18" s="63"/>
+      <c r="E18" s="63"/>
+      <c r="F18" s="63"/>
+      <c r="G18" s="63"/>
+      <c r="H18" s="63"/>
+      <c r="I18" s="63"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
+      <c r="B19" s="34"/>
+      <c r="C19" s="34"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="34"/>
+      <c r="I19" s="34"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="14"/>
+      <c r="C20" s="55"/>
+      <c r="D20" s="55"/>
+      <c r="E20" s="55"/>
+      <c r="F20" s="55"/>
+      <c r="G20" s="55"/>
+      <c r="H20" s="55"/>
+      <c r="I20" s="55"/>
     </row>
     <row r="21" spans="2:9" ht="246" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="73" t="s">
+      <c r="C21" s="86" t="s">
         <v>90</v>
       </c>
-      <c r="D21" s="74"/>
-      <c r="E21" s="74"/>
-      <c r="F21" s="74"/>
-      <c r="G21" s="74"/>
-      <c r="H21" s="74"/>
-      <c r="I21" s="75"/>
+      <c r="D21" s="87"/>
+      <c r="E21" s="87"/>
+      <c r="F21" s="87"/>
+      <c r="G21" s="87"/>
+      <c r="H21" s="87"/>
+      <c r="I21" s="88"/>
     </row>
     <row r="22" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="28">
+      <c r="C22" s="41">
         <v>8</v>
       </c>
-      <c r="D22" s="36"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="36"/>
-      <c r="G22" s="36"/>
-      <c r="H22" s="36"/>
-      <c r="I22" s="37"/>
+      <c r="D22" s="42"/>
+      <c r="E22" s="42"/>
+      <c r="F22" s="42"/>
+      <c r="G22" s="42"/>
+      <c r="H22" s="42"/>
+      <c r="I22" s="43"/>
     </row>
     <row r="23" spans="2:9" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="50" t="s">
+      <c r="C23" s="56" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="50"/>
-      <c r="E23" s="51" t="s">
+      <c r="D23" s="56"/>
+      <c r="E23" s="57" t="s">
         <v>101</v>
       </c>
-      <c r="F23" s="51"/>
-      <c r="G23" s="51"/>
-      <c r="H23" s="51"/>
-      <c r="I23" s="51"/>
+      <c r="F23" s="57"/>
+      <c r="G23" s="57"/>
+      <c r="H23" s="57"/>
+      <c r="I23" s="57"/>
     </row>
     <row r="24" spans="2:9" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="90" t="s">
+      <c r="C24" s="99" t="s">
         <v>92</v>
       </c>
-      <c r="D24" s="91"/>
-      <c r="E24" s="65" t="s">
+      <c r="D24" s="100"/>
+      <c r="E24" s="89" t="s">
         <v>107</v>
       </c>
-      <c r="F24" s="65"/>
-      <c r="G24" s="65"/>
-      <c r="H24" s="65"/>
-      <c r="I24" s="65"/>
+      <c r="F24" s="89"/>
+      <c r="G24" s="89"/>
+      <c r="H24" s="89"/>
+      <c r="I24" s="89"/>
     </row>
     <row r="25" spans="2:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="8">
         <v>2</v>
       </c>
-      <c r="C25" s="92" t="s">
+      <c r="C25" s="97" t="s">
         <v>93</v>
       </c>
-      <c r="D25" s="93"/>
-      <c r="E25" s="65" t="s">
+      <c r="D25" s="98"/>
+      <c r="E25" s="89" t="s">
         <v>108</v>
       </c>
-      <c r="F25" s="65"/>
-      <c r="G25" s="65"/>
-      <c r="H25" s="65"/>
-      <c r="I25" s="65"/>
+      <c r="F25" s="89"/>
+      <c r="G25" s="89"/>
+      <c r="H25" s="89"/>
+      <c r="I25" s="89"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B26" s="8">
         <v>3</v>
       </c>
-      <c r="C26" s="92" t="s">
+      <c r="C26" s="97" t="s">
         <v>94</v>
       </c>
-      <c r="D26" s="93"/>
-      <c r="E26" s="65" t="s">
+      <c r="D26" s="98"/>
+      <c r="E26" s="89" t="s">
         <v>106</v>
       </c>
-      <c r="F26" s="65"/>
-      <c r="G26" s="65"/>
-      <c r="H26" s="65"/>
-      <c r="I26" s="65"/>
+      <c r="F26" s="89"/>
+      <c r="G26" s="89"/>
+      <c r="H26" s="89"/>
+      <c r="I26" s="89"/>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B27" s="8">
         <v>4</v>
       </c>
-      <c r="C27" s="92" t="s">
+      <c r="C27" s="97" t="s">
         <v>95</v>
       </c>
-      <c r="D27" s="93"/>
-      <c r="E27" s="65" t="s">
+      <c r="D27" s="98"/>
+      <c r="E27" s="89" t="s">
         <v>105</v>
       </c>
-      <c r="F27" s="65"/>
-      <c r="G27" s="65"/>
-      <c r="H27" s="65"/>
-      <c r="I27" s="65"/>
+      <c r="F27" s="89"/>
+      <c r="G27" s="89"/>
+      <c r="H27" s="89"/>
+      <c r="I27" s="89"/>
     </row>
     <row r="28" spans="2:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="8">
         <v>5</v>
       </c>
-      <c r="C28" s="92" t="s">
+      <c r="C28" s="97" t="s">
         <v>96</v>
       </c>
-      <c r="D28" s="93"/>
-      <c r="E28" s="65" t="s">
+      <c r="D28" s="98"/>
+      <c r="E28" s="89" t="s">
         <v>104</v>
       </c>
-      <c r="F28" s="65"/>
-      <c r="G28" s="65"/>
-      <c r="H28" s="65"/>
-      <c r="I28" s="65"/>
+      <c r="F28" s="89"/>
+      <c r="G28" s="89"/>
+      <c r="H28" s="89"/>
+      <c r="I28" s="89"/>
     </row>
     <row r="29" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="8">
         <v>6</v>
       </c>
-      <c r="C29" s="89" t="s">
+      <c r="C29" s="93" t="s">
         <v>97</v>
       </c>
-      <c r="D29" s="89"/>
-      <c r="E29" s="65" t="s">
+      <c r="D29" s="93"/>
+      <c r="E29" s="89" t="s">
         <v>103</v>
       </c>
-      <c r="F29" s="65"/>
-      <c r="G29" s="65"/>
-      <c r="H29" s="65"/>
-      <c r="I29" s="65"/>
+      <c r="F29" s="89"/>
+      <c r="G29" s="89"/>
+      <c r="H29" s="89"/>
+      <c r="I29" s="89"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B30" s="8">
         <v>7</v>
       </c>
-      <c r="C30" s="89" t="s">
+      <c r="C30" s="93" t="s">
         <v>98</v>
       </c>
-      <c r="D30" s="89"/>
-      <c r="E30" s="65" t="s">
+      <c r="D30" s="93"/>
+      <c r="E30" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="F30" s="94"/>
-      <c r="G30" s="94"/>
-      <c r="H30" s="94"/>
-      <c r="I30" s="94"/>
+      <c r="F30" s="96"/>
+      <c r="G30" s="96"/>
+      <c r="H30" s="96"/>
+      <c r="I30" s="96"/>
     </row>
     <row r="31" spans="2:9" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="8">
         <v>8</v>
       </c>
-      <c r="C31" s="92" t="s">
+      <c r="C31" s="97" t="s">
         <v>99</v>
       </c>
-      <c r="D31" s="93"/>
-      <c r="E31" s="28" t="s">
+      <c r="D31" s="98"/>
+      <c r="E31" s="41" t="s">
         <v>100</v>
       </c>
-      <c r="F31" s="29"/>
-      <c r="G31" s="29"/>
-      <c r="H31" s="29"/>
-      <c r="I31" s="30"/>
+      <c r="F31" s="66"/>
+      <c r="G31" s="66"/>
+      <c r="H31" s="66"/>
+      <c r="I31" s="67"/>
     </row>
     <row r="32" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B32" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C32" s="24" t="s">
+      <c r="C32" s="64" t="s">
         <v>91</v>
       </c>
-      <c r="D32" s="24"/>
-      <c r="E32" s="24"/>
-      <c r="F32" s="24"/>
-      <c r="G32" s="24"/>
-      <c r="H32" s="24"/>
-      <c r="I32" s="24"/>
+      <c r="D32" s="64"/>
+      <c r="E32" s="64"/>
+      <c r="F32" s="64"/>
+      <c r="G32" s="64"/>
+      <c r="H32" s="64"/>
+      <c r="I32" s="64"/>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B33" s="32"/>
-      <c r="C33" s="33"/>
-      <c r="D33" s="33"/>
-      <c r="E33" s="33"/>
-      <c r="F33" s="33"/>
-      <c r="G33" s="33"/>
-      <c r="H33" s="33"/>
-      <c r="I33" s="34"/>
+      <c r="B33" s="35"/>
+      <c r="C33" s="36"/>
+      <c r="D33" s="36"/>
+      <c r="E33" s="36"/>
+      <c r="F33" s="36"/>
+      <c r="G33" s="36"/>
+      <c r="H33" s="36"/>
+      <c r="I33" s="37"/>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B34" s="14" t="s">
+      <c r="B34" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="14"/>
+      <c r="C34" s="55"/>
+      <c r="D34" s="55"/>
+      <c r="E34" s="55"/>
+      <c r="F34" s="55"/>
+      <c r="G34" s="55"/>
+      <c r="H34" s="55"/>
+      <c r="I34" s="55"/>
     </row>
     <row r="35" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="76" t="s">
+      <c r="B35" s="77" t="s">
         <v>109</v>
       </c>
-      <c r="C35" s="18"/>
-      <c r="D35" s="18"/>
-      <c r="E35" s="18"/>
-      <c r="F35" s="18"/>
-      <c r="G35" s="18"/>
-      <c r="H35" s="18"/>
-      <c r="I35" s="18"/>
+      <c r="C35" s="61"/>
+      <c r="D35" s="61"/>
+      <c r="E35" s="61"/>
+      <c r="F35" s="61"/>
+      <c r="G35" s="61"/>
+      <c r="H35" s="61"/>
+      <c r="I35" s="61"/>
     </row>
     <row r="36" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="18"/>
-      <c r="C36" s="18"/>
-      <c r="D36" s="18"/>
-      <c r="E36" s="18"/>
-      <c r="F36" s="18"/>
-      <c r="G36" s="18"/>
-      <c r="H36" s="18"/>
-      <c r="I36" s="18"/>
+      <c r="B36" s="61"/>
+      <c r="C36" s="61"/>
+      <c r="D36" s="61"/>
+      <c r="E36" s="61"/>
+      <c r="F36" s="61"/>
+      <c r="G36" s="61"/>
+      <c r="H36" s="61"/>
+      <c r="I36" s="61"/>
     </row>
     <row r="37" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="18"/>
-      <c r="C37" s="18"/>
-      <c r="D37" s="18"/>
-      <c r="E37" s="18"/>
-      <c r="F37" s="18"/>
-      <c r="G37" s="18"/>
-      <c r="H37" s="18"/>
-      <c r="I37" s="18"/>
+      <c r="B37" s="61"/>
+      <c r="C37" s="61"/>
+      <c r="D37" s="61"/>
+      <c r="E37" s="61"/>
+      <c r="F37" s="61"/>
+      <c r="G37" s="61"/>
+      <c r="H37" s="61"/>
+      <c r="I37" s="61"/>
     </row>
     <row r="38" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="18"/>
-      <c r="C38" s="18"/>
-      <c r="D38" s="18"/>
-      <c r="E38" s="18"/>
-      <c r="F38" s="18"/>
-      <c r="G38" s="18"/>
-      <c r="H38" s="18"/>
-      <c r="I38" s="18"/>
+      <c r="B38" s="61"/>
+      <c r="C38" s="61"/>
+      <c r="D38" s="61"/>
+      <c r="E38" s="61"/>
+      <c r="F38" s="61"/>
+      <c r="G38" s="61"/>
+      <c r="H38" s="61"/>
+      <c r="I38" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="B35:I38"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="E29:I29"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:I30"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E28:I28"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:I31"/>
-    <mergeCell ref="C32:I32"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="B34:I34"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="C3:I3"/>
-    <mergeCell ref="C4:I4"/>
-    <mergeCell ref="C5:I5"/>
-    <mergeCell ref="C6:I6"/>
     <mergeCell ref="C7:I7"/>
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="C25:D25"/>
@@ -5678,6 +5645,31 @@
     <mergeCell ref="B13:I13"/>
     <mergeCell ref="B14:I14"/>
     <mergeCell ref="C15:I15"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="B35:I38"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="E29:I29"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:I28"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:I31"/>
+    <mergeCell ref="C32:I32"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="B34:I34"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{69FD07AD-7FCA-E141-8126-AFB63E0A1511}"/>

</xml_diff>

<commit_message>
did the first prompt planning
</commit_message>
<xml_diff>
--- a/Papers/Resumen Papers.xlsx
+++ b/Papers/Resumen Papers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sophiaaristizabal/Documents/GitHub/LLMS_Project/Papers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C530E70-6F68-C345-BA07-AC8460941B51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AEFC2EB-2F32-6648-AAC1-0337E8C17ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5880" yWindow="500" windowWidth="18460" windowHeight="16180" activeTab="2" xr2:uid="{400AC57E-08F9-B346-9132-4F74AEBC2D15}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" firstSheet="2" activeTab="4" xr2:uid="{400AC57E-08F9-B346-9132-4F74AEBC2D15}"/>
   </bookViews>
   <sheets>
     <sheet name="MANAGERIAL LEADERSHIP" sheetId="1" r:id="rId1"/>
@@ -2418,164 +2418,212 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2583,58 +2631,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2646,26 +2652,20 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3216,176 +3216,176 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="69" t="s">
+      <c r="C3" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="69"/>
-      <c r="E3" s="69"/>
-      <c r="F3" s="69"/>
-      <c r="G3" s="69"/>
-      <c r="H3" s="69"/>
-      <c r="I3" s="69"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="70" t="s">
+      <c r="C4" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="70"/>
-      <c r="F4" s="70"/>
-      <c r="G4" s="70"/>
-      <c r="H4" s="70"/>
-      <c r="I4" s="70"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="63">
+      <c r="C5" s="19">
         <v>2025</v>
       </c>
-      <c r="D5" s="63"/>
-      <c r="E5" s="63"/>
-      <c r="F5" s="63"/>
-      <c r="G5" s="63"/>
-      <c r="H5" s="63"/>
-      <c r="I5" s="63"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
     </row>
     <row r="6" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="63" t="s">
+      <c r="C6" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="63"/>
-      <c r="E6" s="63"/>
-      <c r="F6" s="63"/>
-      <c r="G6" s="63"/>
-      <c r="H6" s="63"/>
-      <c r="I6" s="63"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="68" t="s">
+      <c r="C7" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="63"/>
-      <c r="E7" s="63"/>
-      <c r="F7" s="63"/>
-      <c r="G7" s="63"/>
-      <c r="H7" s="63"/>
-      <c r="I7" s="63"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
     </row>
     <row r="8" spans="2:9" ht="9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="34"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="34"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
     </row>
     <row r="9" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="55" t="s">
+      <c r="B9" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="55"/>
-      <c r="D9" s="55"/>
-      <c r="E9" s="55"/>
-      <c r="F9" s="55"/>
-      <c r="G9" s="55"/>
-      <c r="H9" s="55"/>
-      <c r="I9" s="55"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
     </row>
     <row r="10" spans="2:9" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="60" t="s">
+      <c r="B10" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="60"/>
-      <c r="D10" s="60"/>
-      <c r="E10" s="60"/>
-      <c r="F10" s="60"/>
-      <c r="G10" s="60"/>
-      <c r="H10" s="60"/>
-      <c r="I10" s="60"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
     </row>
     <row r="11" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="60"/>
-      <c r="C11" s="60"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="60"/>
-      <c r="H11" s="60"/>
-      <c r="I11" s="60"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
     </row>
     <row r="12" spans="2:9" ht="11" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="60"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="60"/>
-      <c r="H12" s="60"/>
-      <c r="I12" s="60"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
     </row>
     <row r="13" spans="2:9" ht="9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="34"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="34"/>
-      <c r="I13" s="34"/>
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="55" t="s">
+      <c r="B14" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="55"/>
-      <c r="D14" s="55"/>
-      <c r="E14" s="55"/>
-      <c r="F14" s="55"/>
-      <c r="G14" s="55"/>
-      <c r="H14" s="55"/>
-      <c r="I14" s="55"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="20"/>
+      <c r="I14" s="20"/>
     </row>
     <row r="15" spans="2:9" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="62" t="s">
+      <c r="C15" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="63"/>
-      <c r="E15" s="63"/>
-      <c r="F15" s="63"/>
-      <c r="G15" s="63"/>
-      <c r="H15" s="63"/>
-      <c r="I15" s="63"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="19"/>
+      <c r="I15" s="19"/>
     </row>
     <row r="16" spans="2:9" ht="125" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="44" t="s">
@@ -3415,57 +3415,57 @@
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="62" t="s">
+      <c r="C18" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="63"/>
-      <c r="E18" s="63"/>
-      <c r="F18" s="63"/>
-      <c r="G18" s="63"/>
-      <c r="H18" s="63"/>
-      <c r="I18" s="63"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="19"/>
+      <c r="H18" s="19"/>
+      <c r="I18" s="19"/>
     </row>
     <row r="19" spans="2:9" ht="7" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="34"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="34"/>
-      <c r="I19" s="34"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="26"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="55" t="s">
+      <c r="B20" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="55"/>
-      <c r="D20" s="55"/>
-      <c r="E20" s="55"/>
-      <c r="F20" s="55"/>
-      <c r="G20" s="55"/>
-      <c r="H20" s="55"/>
-      <c r="I20" s="55"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="20"/>
+      <c r="I20" s="20"/>
     </row>
     <row r="21" spans="2:9" ht="43" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="38" t="s">
+      <c r="C21" s="41" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="39"/>
-      <c r="E21" s="39"/>
-      <c r="F21" s="39"/>
-      <c r="G21" s="39"/>
-      <c r="H21" s="39"/>
-      <c r="I21" s="40"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="28"/>
+      <c r="F21" s="28"/>
+      <c r="G21" s="28"/>
+      <c r="H21" s="28"/>
+      <c r="I21" s="29"/>
     </row>
     <row r="22" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B22" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="41">
+      <c r="C22" s="34">
         <v>9</v>
       </c>
       <c r="D22" s="42"/>
@@ -3495,11 +3495,11 @@
       <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="21" t="s">
+      <c r="C24" s="54" t="s">
         <v>38</v>
       </c>
-      <c r="D24" s="23"/>
-      <c r="E24" s="38" t="s">
+      <c r="D24" s="55"/>
+      <c r="E24" s="41" t="s">
         <v>37</v>
       </c>
       <c r="F24" s="58"/>
@@ -3511,228 +3511,247 @@
       <c r="B25" s="8">
         <v>2</v>
       </c>
-      <c r="C25" s="21" t="s">
+      <c r="C25" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="D25" s="23"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="22"/>
-      <c r="H25" s="22"/>
-      <c r="I25" s="23"/>
+      <c r="D25" s="55"/>
+      <c r="E25" s="54"/>
+      <c r="F25" s="70"/>
+      <c r="G25" s="70"/>
+      <c r="H25" s="70"/>
+      <c r="I25" s="55"/>
     </row>
     <row r="26" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="25">
+      <c r="B26" s="60">
         <v>3</v>
       </c>
-      <c r="C26" s="27" t="s">
+      <c r="C26" s="62" t="s">
         <v>40</v>
       </c>
-      <c r="D26" s="28"/>
-      <c r="E26" s="24" t="s">
+      <c r="D26" s="63"/>
+      <c r="E26" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="F26" s="24"/>
-      <c r="G26" s="22" t="s">
+      <c r="F26" s="37"/>
+      <c r="G26" s="70" t="s">
         <v>41</v>
       </c>
-      <c r="H26" s="22"/>
-      <c r="I26" s="23"/>
+      <c r="H26" s="70"/>
+      <c r="I26" s="55"/>
     </row>
     <row r="27" spans="2:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="26"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="30"/>
-      <c r="E27" s="18" t="s">
+      <c r="B27" s="61"/>
+      <c r="C27" s="64"/>
+      <c r="D27" s="65"/>
+      <c r="E27" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="F27" s="19"/>
-      <c r="G27" s="31" t="s">
+      <c r="F27" s="33"/>
+      <c r="G27" s="66" t="s">
         <v>43</v>
       </c>
-      <c r="H27" s="32"/>
-      <c r="I27" s="33"/>
+      <c r="H27" s="67"/>
+      <c r="I27" s="68"/>
     </row>
     <row r="28" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="8">
         <v>4</v>
       </c>
-      <c r="C28" s="18" t="s">
+      <c r="C28" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="D28" s="19"/>
-      <c r="E28" s="52" t="s">
+      <c r="D28" s="33"/>
+      <c r="E28" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="F28" s="39"/>
-      <c r="G28" s="39"/>
-      <c r="H28" s="39"/>
-      <c r="I28" s="40"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="28"/>
+      <c r="H28" s="28"/>
+      <c r="I28" s="29"/>
     </row>
     <row r="29" spans="2:9" ht="43" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="8">
         <v>5</v>
       </c>
-      <c r="C29" s="24" t="s">
+      <c r="C29" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="D29" s="24"/>
-      <c r="E29" s="64" t="s">
+      <c r="D29" s="37"/>
+      <c r="E29" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="F29" s="64"/>
-      <c r="G29" s="64"/>
-      <c r="H29" s="64"/>
-      <c r="I29" s="64"/>
+      <c r="F29" s="30"/>
+      <c r="G29" s="30"/>
+      <c r="H29" s="30"/>
+      <c r="I29" s="30"/>
     </row>
     <row r="30" spans="2:9" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="8">
         <v>6</v>
       </c>
-      <c r="C30" s="18" t="s">
+      <c r="C30" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="D30" s="19"/>
-      <c r="E30" s="52" t="s">
+      <c r="D30" s="33"/>
+      <c r="E30" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="F30" s="53"/>
-      <c r="G30" s="53"/>
-      <c r="H30" s="53"/>
-      <c r="I30" s="54"/>
+      <c r="F30" s="52"/>
+      <c r="G30" s="52"/>
+      <c r="H30" s="52"/>
+      <c r="I30" s="53"/>
     </row>
     <row r="31" spans="2:9" ht="53" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="8">
         <v>7</v>
       </c>
-      <c r="C31" s="24" t="s">
+      <c r="C31" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="D31" s="24"/>
-      <c r="E31" s="64" t="s">
+      <c r="D31" s="37"/>
+      <c r="E31" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="F31" s="65"/>
-      <c r="G31" s="65"/>
-      <c r="H31" s="65"/>
-      <c r="I31" s="65"/>
+      <c r="F31" s="31"/>
+      <c r="G31" s="31"/>
+      <c r="H31" s="31"/>
+      <c r="I31" s="31"/>
     </row>
     <row r="32" spans="2:9" ht="53" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="8">
         <v>8</v>
       </c>
-      <c r="C32" s="18" t="s">
+      <c r="C32" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="D32" s="19"/>
-      <c r="E32" s="18"/>
-      <c r="F32" s="20"/>
-      <c r="G32" s="20"/>
-      <c r="H32" s="20"/>
-      <c r="I32" s="19"/>
+      <c r="D32" s="33"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="69"/>
+      <c r="G32" s="69"/>
+      <c r="H32" s="69"/>
+      <c r="I32" s="33"/>
     </row>
     <row r="33" spans="2:9" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="8">
         <v>9</v>
       </c>
-      <c r="C33" s="18" t="s">
+      <c r="C33" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="D33" s="19"/>
-      <c r="E33" s="41" t="s">
+      <c r="D33" s="33"/>
+      <c r="E33" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="F33" s="66"/>
-      <c r="G33" s="66"/>
-      <c r="H33" s="66"/>
-      <c r="I33" s="67"/>
+      <c r="F33" s="35"/>
+      <c r="G33" s="35"/>
+      <c r="H33" s="35"/>
+      <c r="I33" s="36"/>
     </row>
     <row r="34" spans="2:9" ht="190" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C34" s="64" t="s">
+      <c r="C34" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="D34" s="64"/>
-      <c r="E34" s="64"/>
-      <c r="F34" s="64"/>
-      <c r="G34" s="64"/>
-      <c r="H34" s="64"/>
-      <c r="I34" s="64"/>
+      <c r="D34" s="30"/>
+      <c r="E34" s="30"/>
+      <c r="F34" s="30"/>
+      <c r="G34" s="30"/>
+      <c r="H34" s="30"/>
+      <c r="I34" s="30"/>
     </row>
     <row r="35" spans="2:9" ht="10" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="35"/>
-      <c r="C35" s="36"/>
-      <c r="D35" s="36"/>
-      <c r="E35" s="36"/>
-      <c r="F35" s="36"/>
-      <c r="G35" s="36"/>
-      <c r="H35" s="36"/>
-      <c r="I35" s="37"/>
+      <c r="B35" s="38"/>
+      <c r="C35" s="39"/>
+      <c r="D35" s="39"/>
+      <c r="E35" s="39"/>
+      <c r="F35" s="39"/>
+      <c r="G35" s="39"/>
+      <c r="H35" s="39"/>
+      <c r="I35" s="40"/>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B36" s="55" t="s">
+      <c r="B36" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="C36" s="55"/>
-      <c r="D36" s="55"/>
-      <c r="E36" s="55"/>
-      <c r="F36" s="55"/>
-      <c r="G36" s="55"/>
-      <c r="H36" s="55"/>
-      <c r="I36" s="55"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="20"/>
+      <c r="E36" s="20"/>
+      <c r="F36" s="20"/>
+      <c r="G36" s="20"/>
+      <c r="H36" s="20"/>
+      <c r="I36" s="20"/>
     </row>
     <row r="37" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="61" t="s">
+      <c r="B37" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="C37" s="61"/>
-      <c r="D37" s="61"/>
-      <c r="E37" s="61"/>
-      <c r="F37" s="61"/>
-      <c r="G37" s="61"/>
-      <c r="H37" s="61"/>
-      <c r="I37" s="61"/>
+      <c r="C37" s="24"/>
+      <c r="D37" s="24"/>
+      <c r="E37" s="24"/>
+      <c r="F37" s="24"/>
+      <c r="G37" s="24"/>
+      <c r="H37" s="24"/>
+      <c r="I37" s="24"/>
     </row>
     <row r="38" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="61"/>
-      <c r="C38" s="61"/>
-      <c r="D38" s="61"/>
-      <c r="E38" s="61"/>
-      <c r="F38" s="61"/>
-      <c r="G38" s="61"/>
-      <c r="H38" s="61"/>
-      <c r="I38" s="61"/>
+      <c r="B38" s="24"/>
+      <c r="C38" s="24"/>
+      <c r="D38" s="24"/>
+      <c r="E38" s="24"/>
+      <c r="F38" s="24"/>
+      <c r="G38" s="24"/>
+      <c r="H38" s="24"/>
+      <c r="I38" s="24"/>
     </row>
     <row r="39" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="61"/>
-      <c r="C39" s="61"/>
-      <c r="D39" s="61"/>
-      <c r="E39" s="61"/>
-      <c r="F39" s="61"/>
-      <c r="G39" s="61"/>
-      <c r="H39" s="61"/>
-      <c r="I39" s="61"/>
+      <c r="B39" s="24"/>
+      <c r="C39" s="24"/>
+      <c r="D39" s="24"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="24"/>
+      <c r="G39" s="24"/>
+      <c r="H39" s="24"/>
+      <c r="I39" s="24"/>
     </row>
     <row r="40" spans="2:9" ht="76" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B40" s="61"/>
-      <c r="C40" s="61"/>
-      <c r="D40" s="61"/>
-      <c r="E40" s="61"/>
-      <c r="F40" s="61"/>
-      <c r="G40" s="61"/>
-      <c r="H40" s="61"/>
-      <c r="I40" s="61"/>
+      <c r="B40" s="24"/>
+      <c r="C40" s="24"/>
+      <c r="D40" s="24"/>
+      <c r="E40" s="24"/>
+      <c r="F40" s="24"/>
+      <c r="G40" s="24"/>
+      <c r="H40" s="24"/>
+      <c r="I40" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="C7:I7"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="C3:I3"/>
-    <mergeCell ref="C4:I4"/>
-    <mergeCell ref="C5:I5"/>
-    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="C26:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="E32:I32"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="B26:B27"/>
     <mergeCell ref="B36:I36"/>
     <mergeCell ref="B10:I12"/>
     <mergeCell ref="B9:I9"/>
@@ -3749,31 +3768,12 @@
     <mergeCell ref="C28:D28"/>
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="C31:D31"/>
-    <mergeCell ref="B35:I35"/>
-    <mergeCell ref="B13:I13"/>
-    <mergeCell ref="C21:I21"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:I30"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="B14:I14"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="C26:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="E32:I32"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="C6:I6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{C9E9977D-5134-FE4B-852F-8DEBDCB543E0}"/>
@@ -3802,12 +3802,12 @@
   </cols>
   <sheetData>
     <row r="4" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B4" s="70" t="s">
+      <c r="B4" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="C4" s="70"/>
-      <c r="D4" s="70"/>
-      <c r="E4" s="70"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
     </row>
     <row r="5" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="11" t="s">
@@ -4078,256 +4078,256 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="89" t="s">
+      <c r="C3" s="71" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
-      <c r="I3" s="90"/>
+      <c r="D3" s="72"/>
+      <c r="E3" s="72"/>
+      <c r="F3" s="72"/>
+      <c r="G3" s="72"/>
+      <c r="H3" s="72"/>
+      <c r="I3" s="72"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="63" t="s">
+      <c r="C4" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="63"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
-      <c r="G4" s="63"/>
-      <c r="H4" s="63"/>
-      <c r="I4" s="63"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="63">
+      <c r="C5" s="19">
         <v>2020</v>
       </c>
-      <c r="D5" s="63"/>
-      <c r="E5" s="63"/>
-      <c r="F5" s="63"/>
-      <c r="G5" s="63"/>
-      <c r="H5" s="63"/>
-      <c r="I5" s="63"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
     </row>
     <row r="6" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="65" t="s">
+      <c r="C6" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="65"/>
-      <c r="E6" s="65"/>
-      <c r="F6" s="65"/>
-      <c r="G6" s="65"/>
-      <c r="H6" s="65"/>
-      <c r="I6" s="65"/>
+      <c r="D6" s="31"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="68" t="s">
+      <c r="C7" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="D7" s="63"/>
-      <c r="E7" s="63"/>
-      <c r="F7" s="63"/>
-      <c r="G7" s="63"/>
-      <c r="H7" s="63"/>
-      <c r="I7" s="63"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="34"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="34"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="55" t="s">
+      <c r="B9" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="55"/>
-      <c r="D9" s="55"/>
-      <c r="E9" s="55"/>
-      <c r="F9" s="55"/>
-      <c r="G9" s="55"/>
-      <c r="H9" s="55"/>
-      <c r="I9" s="55"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
     </row>
     <row r="10" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="60" t="s">
+      <c r="B10" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="60"/>
-      <c r="D10" s="60"/>
-      <c r="E10" s="60"/>
-      <c r="F10" s="60"/>
-      <c r="G10" s="60"/>
-      <c r="H10" s="60"/>
-      <c r="I10" s="60"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
     </row>
     <row r="11" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="60"/>
-      <c r="C11" s="60"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="60"/>
-      <c r="H11" s="60"/>
-      <c r="I11" s="60"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
     </row>
     <row r="12" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="60"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="60"/>
-      <c r="H12" s="60"/>
-      <c r="I12" s="60"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="34"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="34"/>
-      <c r="I13" s="34"/>
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="55" t="s">
+      <c r="B14" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="55"/>
-      <c r="D14" s="55"/>
-      <c r="E14" s="55"/>
-      <c r="F14" s="55"/>
-      <c r="G14" s="55"/>
-      <c r="H14" s="55"/>
-      <c r="I14" s="55"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="20"/>
+      <c r="I14" s="20"/>
     </row>
     <row r="15" spans="2:9" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="62" t="s">
+      <c r="C15" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="63"/>
-      <c r="E15" s="63"/>
-      <c r="F15" s="63"/>
-      <c r="G15" s="63"/>
-      <c r="H15" s="63"/>
-      <c r="I15" s="63"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="19"/>
+      <c r="I15" s="19"/>
     </row>
     <row r="16" spans="2:9" ht="98" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="80" t="s">
+      <c r="C16" s="73" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="81"/>
-      <c r="E16" s="81"/>
-      <c r="F16" s="81"/>
-      <c r="G16" s="81"/>
-      <c r="H16" s="81"/>
-      <c r="I16" s="82"/>
+      <c r="D16" s="74"/>
+      <c r="E16" s="74"/>
+      <c r="F16" s="74"/>
+      <c r="G16" s="74"/>
+      <c r="H16" s="74"/>
+      <c r="I16" s="75"/>
     </row>
     <row r="17" spans="2:9" ht="98" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="45"/>
-      <c r="C17" s="83"/>
-      <c r="D17" s="84"/>
-      <c r="E17" s="84"/>
-      <c r="F17" s="84"/>
-      <c r="G17" s="84"/>
-      <c r="H17" s="84"/>
-      <c r="I17" s="85"/>
+      <c r="C17" s="76"/>
+      <c r="D17" s="77"/>
+      <c r="E17" s="77"/>
+      <c r="F17" s="77"/>
+      <c r="G17" s="77"/>
+      <c r="H17" s="77"/>
+      <c r="I17" s="78"/>
     </row>
     <row r="18" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="62" t="s">
+      <c r="C18" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="D18" s="63"/>
-      <c r="E18" s="63"/>
-      <c r="F18" s="63"/>
-      <c r="G18" s="63"/>
-      <c r="H18" s="63"/>
-      <c r="I18" s="63"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="19"/>
+      <c r="H18" s="19"/>
+      <c r="I18" s="19"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="34"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="34"/>
-      <c r="I19" s="34"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="26"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="55" t="s">
+      <c r="B20" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="55"/>
-      <c r="D20" s="55"/>
-      <c r="E20" s="55"/>
-      <c r="F20" s="55"/>
-      <c r="G20" s="55"/>
-      <c r="H20" s="55"/>
-      <c r="I20" s="55"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="20"/>
+      <c r="I20" s="20"/>
     </row>
     <row r="21" spans="2:9" ht="160" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="86" t="s">
+      <c r="C21" s="79" t="s">
         <v>57</v>
       </c>
-      <c r="D21" s="87"/>
-      <c r="E21" s="87"/>
-      <c r="F21" s="87"/>
-      <c r="G21" s="87"/>
-      <c r="H21" s="87"/>
-      <c r="I21" s="88"/>
+      <c r="D21" s="80"/>
+      <c r="E21" s="80"/>
+      <c r="F21" s="80"/>
+      <c r="G21" s="80"/>
+      <c r="H21" s="80"/>
+      <c r="I21" s="81"/>
     </row>
     <row r="22" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="41">
+      <c r="C22" s="34">
         <v>3</v>
       </c>
       <c r="D22" s="42"/>
@@ -4354,145 +4354,166 @@
       <c r="I23" s="57"/>
     </row>
     <row r="24" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="25">
+      <c r="B24" s="60">
         <v>1</v>
       </c>
-      <c r="C24" s="71" t="s">
+      <c r="C24" s="87" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="72"/>
+      <c r="D24" s="88"/>
       <c r="E24" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="F24" s="75" t="s">
+      <c r="F24" s="89" t="s">
         <v>63</v>
       </c>
-      <c r="G24" s="75"/>
-      <c r="H24" s="75"/>
-      <c r="I24" s="76"/>
+      <c r="G24" s="89"/>
+      <c r="H24" s="89"/>
+      <c r="I24" s="90"/>
     </row>
     <row r="25" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="26"/>
-      <c r="C25" s="73"/>
-      <c r="D25" s="74"/>
+      <c r="B25" s="61"/>
+      <c r="C25" s="85"/>
+      <c r="D25" s="86"/>
       <c r="E25" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="F25" s="22" t="s">
+      <c r="F25" s="70" t="s">
         <v>64</v>
       </c>
-      <c r="G25" s="22"/>
-      <c r="H25" s="22"/>
-      <c r="I25" s="23"/>
+      <c r="G25" s="70"/>
+      <c r="H25" s="70"/>
+      <c r="I25" s="55"/>
     </row>
     <row r="26" spans="2:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="8">
         <v>2</v>
       </c>
-      <c r="C26" s="78" t="s">
+      <c r="C26" s="83" t="s">
         <v>59</v>
       </c>
-      <c r="D26" s="79"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="20"/>
-      <c r="H26" s="20"/>
-      <c r="I26" s="19"/>
+      <c r="D26" s="84"/>
+      <c r="E26" s="32"/>
+      <c r="F26" s="69"/>
+      <c r="G26" s="69"/>
+      <c r="H26" s="69"/>
+      <c r="I26" s="33"/>
     </row>
     <row r="27" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="8">
         <v>3</v>
       </c>
-      <c r="C27" s="73" t="s">
+      <c r="C27" s="85" t="s">
         <v>60</v>
       </c>
-      <c r="D27" s="74"/>
-      <c r="E27" s="18"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="20"/>
-      <c r="H27" s="20"/>
-      <c r="I27" s="19"/>
+      <c r="D27" s="86"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="69"/>
+      <c r="G27" s="69"/>
+      <c r="H27" s="69"/>
+      <c r="I27" s="33"/>
     </row>
     <row r="28" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B28" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C28" s="64" t="s">
+      <c r="C28" s="30" t="s">
         <v>65</v>
       </c>
-      <c r="D28" s="64"/>
-      <c r="E28" s="64"/>
-      <c r="F28" s="64"/>
-      <c r="G28" s="64"/>
-      <c r="H28" s="64"/>
-      <c r="I28" s="64"/>
+      <c r="D28" s="30"/>
+      <c r="E28" s="30"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="H28" s="30"/>
+      <c r="I28" s="30"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B29" s="35"/>
-      <c r="C29" s="36"/>
-      <c r="D29" s="36"/>
-      <c r="E29" s="36"/>
-      <c r="F29" s="36"/>
-      <c r="G29" s="36"/>
-      <c r="H29" s="36"/>
-      <c r="I29" s="37"/>
+      <c r="B29" s="38"/>
+      <c r="C29" s="39"/>
+      <c r="D29" s="39"/>
+      <c r="E29" s="39"/>
+      <c r="F29" s="39"/>
+      <c r="G29" s="39"/>
+      <c r="H29" s="39"/>
+      <c r="I29" s="40"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B30" s="55" t="s">
+      <c r="B30" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="C30" s="55"/>
-      <c r="D30" s="55"/>
-      <c r="E30" s="55"/>
-      <c r="F30" s="55"/>
-      <c r="G30" s="55"/>
-      <c r="H30" s="55"/>
-      <c r="I30" s="55"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="20"/>
+      <c r="H30" s="20"/>
+      <c r="I30" s="20"/>
     </row>
     <row r="31" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="77" t="s">
+      <c r="B31" s="82" t="s">
         <v>66</v>
       </c>
-      <c r="C31" s="61"/>
-      <c r="D31" s="61"/>
-      <c r="E31" s="61"/>
-      <c r="F31" s="61"/>
-      <c r="G31" s="61"/>
-      <c r="H31" s="61"/>
-      <c r="I31" s="61"/>
+      <c r="C31" s="24"/>
+      <c r="D31" s="24"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="24"/>
+      <c r="H31" s="24"/>
+      <c r="I31" s="24"/>
     </row>
     <row r="32" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="61"/>
-      <c r="C32" s="61"/>
-      <c r="D32" s="61"/>
-      <c r="E32" s="61"/>
-      <c r="F32" s="61"/>
-      <c r="G32" s="61"/>
-      <c r="H32" s="61"/>
-      <c r="I32" s="61"/>
+      <c r="B32" s="24"/>
+      <c r="C32" s="24"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="24"/>
     </row>
     <row r="33" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="61"/>
-      <c r="C33" s="61"/>
-      <c r="D33" s="61"/>
-      <c r="E33" s="61"/>
-      <c r="F33" s="61"/>
-      <c r="G33" s="61"/>
-      <c r="H33" s="61"/>
-      <c r="I33" s="61"/>
+      <c r="B33" s="24"/>
+      <c r="C33" s="24"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="24"/>
+      <c r="G33" s="24"/>
+      <c r="H33" s="24"/>
+      <c r="I33" s="24"/>
     </row>
     <row r="34" spans="2:9" ht="254" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="61"/>
-      <c r="C34" s="61"/>
-      <c r="D34" s="61"/>
-      <c r="E34" s="61"/>
-      <c r="F34" s="61"/>
-      <c r="G34" s="61"/>
-      <c r="H34" s="61"/>
-      <c r="I34" s="61"/>
+      <c r="B34" s="24"/>
+      <c r="C34" s="24"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="24"/>
+      <c r="I34" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:D25"/>
+    <mergeCell ref="F24:I24"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="C28:I28"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="B31:I34"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="C21:I21"/>
     <mergeCell ref="C15:I15"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -4505,27 +4526,6 @@
     <mergeCell ref="B10:I12"/>
     <mergeCell ref="B13:I13"/>
     <mergeCell ref="B14:I14"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="C21:I21"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="B31:I34"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:I27"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:D25"/>
-    <mergeCell ref="F24:I24"/>
-    <mergeCell ref="F25:I25"/>
-    <mergeCell ref="C28:I28"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{4DBC988E-4FF2-2C49-AA18-DD92CA6A87E8}"/>
@@ -4558,254 +4558,254 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="89" t="s">
+      <c r="C3" s="71" t="s">
         <v>67</v>
       </c>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
-      <c r="I3" s="90"/>
+      <c r="D3" s="72"/>
+      <c r="E3" s="72"/>
+      <c r="F3" s="72"/>
+      <c r="G3" s="72"/>
+      <c r="H3" s="72"/>
+      <c r="I3" s="72"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="63" t="s">
+      <c r="C4" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="D4" s="63"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
-      <c r="G4" s="63"/>
-      <c r="H4" s="63"/>
-      <c r="I4" s="63"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="63">
+      <c r="C5" s="19">
         <v>2022</v>
       </c>
-      <c r="D5" s="63"/>
-      <c r="E5" s="63"/>
-      <c r="F5" s="63"/>
-      <c r="G5" s="63"/>
-      <c r="H5" s="63"/>
-      <c r="I5" s="63"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
     </row>
     <row r="6" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="65" t="s">
+      <c r="C6" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="D6" s="65"/>
-      <c r="E6" s="65"/>
-      <c r="F6" s="65"/>
-      <c r="G6" s="65"/>
-      <c r="H6" s="65"/>
-      <c r="I6" s="65"/>
+      <c r="D6" s="31"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="68" t="s">
+      <c r="C7" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D7" s="63"/>
-      <c r="E7" s="63"/>
-      <c r="F7" s="63"/>
-      <c r="G7" s="63"/>
-      <c r="H7" s="63"/>
-      <c r="I7" s="63"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="34"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="34"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="55" t="s">
+      <c r="B9" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="55"/>
-      <c r="D9" s="55"/>
-      <c r="E9" s="55"/>
-      <c r="F9" s="55"/>
-      <c r="G9" s="55"/>
-      <c r="H9" s="55"/>
-      <c r="I9" s="55"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
     </row>
     <row r="10" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="60" t="s">
+      <c r="B10" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="C10" s="60"/>
-      <c r="D10" s="60"/>
-      <c r="E10" s="60"/>
-      <c r="F10" s="60"/>
-      <c r="G10" s="60"/>
-      <c r="H10" s="60"/>
-      <c r="I10" s="60"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
     </row>
     <row r="11" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="60"/>
-      <c r="C11" s="60"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="60"/>
-      <c r="H11" s="60"/>
-      <c r="I11" s="60"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
     </row>
     <row r="12" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="60"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="60"/>
-      <c r="H12" s="60"/>
-      <c r="I12" s="60"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="34"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="34"/>
-      <c r="I13" s="34"/>
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="55" t="s">
+      <c r="B14" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="55"/>
-      <c r="D14" s="55"/>
-      <c r="E14" s="55"/>
-      <c r="F14" s="55"/>
-      <c r="G14" s="55"/>
-      <c r="H14" s="55"/>
-      <c r="I14" s="55"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="20"/>
+      <c r="I14" s="20"/>
     </row>
     <row r="15" spans="2:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="62" t="s">
+      <c r="C15" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="D15" s="63"/>
-      <c r="E15" s="63"/>
-      <c r="F15" s="63"/>
-      <c r="G15" s="63"/>
-      <c r="H15" s="63"/>
-      <c r="I15" s="63"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="19"/>
+      <c r="I15" s="19"/>
     </row>
     <row r="16" spans="2:9" ht="247" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="80" t="s">
+      <c r="C16" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="D16" s="81"/>
-      <c r="E16" s="81"/>
-      <c r="F16" s="81"/>
-      <c r="G16" s="81"/>
-      <c r="H16" s="81"/>
-      <c r="I16" s="82"/>
+      <c r="D16" s="74"/>
+      <c r="E16" s="74"/>
+      <c r="F16" s="74"/>
+      <c r="G16" s="74"/>
+      <c r="H16" s="74"/>
+      <c r="I16" s="75"/>
     </row>
     <row r="17" spans="2:9" ht="247" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="45"/>
-      <c r="C17" s="83"/>
-      <c r="D17" s="84"/>
-      <c r="E17" s="84"/>
-      <c r="F17" s="84"/>
-      <c r="G17" s="84"/>
-      <c r="H17" s="84"/>
-      <c r="I17" s="85"/>
+      <c r="C17" s="76"/>
+      <c r="D17" s="77"/>
+      <c r="E17" s="77"/>
+      <c r="F17" s="77"/>
+      <c r="G17" s="77"/>
+      <c r="H17" s="77"/>
+      <c r="I17" s="78"/>
     </row>
     <row r="18" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="94"/>
-      <c r="D18" s="95"/>
-      <c r="E18" s="95"/>
-      <c r="F18" s="95"/>
-      <c r="G18" s="95"/>
-      <c r="H18" s="95"/>
-      <c r="I18" s="95"/>
+      <c r="C18" s="91"/>
+      <c r="D18" s="92"/>
+      <c r="E18" s="92"/>
+      <c r="F18" s="92"/>
+      <c r="G18" s="92"/>
+      <c r="H18" s="92"/>
+      <c r="I18" s="92"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="34"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="34"/>
-      <c r="I19" s="34"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="26"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="55" t="s">
+      <c r="B20" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="C20" s="55"/>
-      <c r="D20" s="55"/>
-      <c r="E20" s="55"/>
-      <c r="F20" s="55"/>
-      <c r="G20" s="55"/>
-      <c r="H20" s="55"/>
-      <c r="I20" s="55"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="20"/>
+      <c r="I20" s="20"/>
     </row>
     <row r="21" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="86" t="s">
+      <c r="C21" s="79" t="s">
         <v>74</v>
       </c>
-      <c r="D21" s="87"/>
-      <c r="E21" s="87"/>
-      <c r="F21" s="87"/>
-      <c r="G21" s="87"/>
-      <c r="H21" s="87"/>
-      <c r="I21" s="88"/>
+      <c r="D21" s="80"/>
+      <c r="E21" s="80"/>
+      <c r="F21" s="80"/>
+      <c r="G21" s="80"/>
+      <c r="H21" s="80"/>
+      <c r="I21" s="81"/>
     </row>
     <row r="22" spans="2:9" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="41" t="s">
+      <c r="C22" s="34" t="s">
         <v>79</v>
       </c>
       <c r="D22" s="42"/>
@@ -4835,10 +4835,10 @@
       <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="93" t="s">
+      <c r="C24" s="95" t="s">
         <v>75</v>
       </c>
-      <c r="D24" s="93"/>
+      <c r="D24" s="95"/>
       <c r="E24" s="56" t="s">
         <v>80</v>
       </c>
@@ -4851,10 +4851,10 @@
       <c r="B25" s="8">
         <v>2</v>
       </c>
-      <c r="C25" s="93" t="s">
+      <c r="C25" s="95" t="s">
         <v>76</v>
       </c>
-      <c r="D25" s="93"/>
+      <c r="D25" s="95"/>
       <c r="E25" s="56"/>
       <c r="F25" s="56"/>
       <c r="G25" s="56"/>
@@ -4865,94 +4865,113 @@
       <c r="B26" s="8">
         <v>3</v>
       </c>
-      <c r="C26" s="78" t="s">
+      <c r="C26" s="83" t="s">
         <v>77</v>
       </c>
-      <c r="D26" s="79"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="20"/>
-      <c r="H26" s="20"/>
-      <c r="I26" s="19"/>
+      <c r="D26" s="84"/>
+      <c r="E26" s="32"/>
+      <c r="F26" s="69"/>
+      <c r="G26" s="69"/>
+      <c r="H26" s="69"/>
+      <c r="I26" s="33"/>
     </row>
     <row r="27" spans="2:9" ht="68" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="64" t="s">
+      <c r="C27" s="30" t="s">
         <v>78</v>
       </c>
-      <c r="D27" s="64"/>
-      <c r="E27" s="64"/>
-      <c r="F27" s="64"/>
-      <c r="G27" s="64"/>
-      <c r="H27" s="64"/>
-      <c r="I27" s="64"/>
+      <c r="D27" s="30"/>
+      <c r="E27" s="30"/>
+      <c r="F27" s="30"/>
+      <c r="G27" s="30"/>
+      <c r="H27" s="30"/>
+      <c r="I27" s="30"/>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B28" s="35"/>
-      <c r="C28" s="36"/>
-      <c r="D28" s="36"/>
-      <c r="E28" s="36"/>
-      <c r="F28" s="36"/>
-      <c r="G28" s="36"/>
-      <c r="H28" s="36"/>
-      <c r="I28" s="37"/>
+      <c r="B28" s="38"/>
+      <c r="C28" s="39"/>
+      <c r="D28" s="39"/>
+      <c r="E28" s="39"/>
+      <c r="F28" s="39"/>
+      <c r="G28" s="39"/>
+      <c r="H28" s="39"/>
+      <c r="I28" s="40"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B29" s="55" t="s">
+      <c r="B29" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="C29" s="55"/>
-      <c r="D29" s="55"/>
-      <c r="E29" s="55"/>
-      <c r="F29" s="55"/>
-      <c r="G29" s="55"/>
-      <c r="H29" s="55"/>
-      <c r="I29" s="55"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
+      <c r="F29" s="20"/>
+      <c r="G29" s="20"/>
+      <c r="H29" s="20"/>
+      <c r="I29" s="20"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B30" s="91"/>
-      <c r="C30" s="92"/>
-      <c r="D30" s="92"/>
-      <c r="E30" s="92"/>
-      <c r="F30" s="92"/>
-      <c r="G30" s="92"/>
-      <c r="H30" s="92"/>
-      <c r="I30" s="92"/>
+      <c r="B30" s="93"/>
+      <c r="C30" s="94"/>
+      <c r="D30" s="94"/>
+      <c r="E30" s="94"/>
+      <c r="F30" s="94"/>
+      <c r="G30" s="94"/>
+      <c r="H30" s="94"/>
+      <c r="I30" s="94"/>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B31" s="92"/>
-      <c r="C31" s="92"/>
-      <c r="D31" s="92"/>
-      <c r="E31" s="92"/>
-      <c r="F31" s="92"/>
-      <c r="G31" s="92"/>
-      <c r="H31" s="92"/>
-      <c r="I31" s="92"/>
+      <c r="B31" s="94"/>
+      <c r="C31" s="94"/>
+      <c r="D31" s="94"/>
+      <c r="E31" s="94"/>
+      <c r="F31" s="94"/>
+      <c r="G31" s="94"/>
+      <c r="H31" s="94"/>
+      <c r="I31" s="94"/>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B32" s="92"/>
-      <c r="C32" s="92"/>
-      <c r="D32" s="92"/>
-      <c r="E32" s="92"/>
-      <c r="F32" s="92"/>
-      <c r="G32" s="92"/>
-      <c r="H32" s="92"/>
-      <c r="I32" s="92"/>
+      <c r="B32" s="94"/>
+      <c r="C32" s="94"/>
+      <c r="D32" s="94"/>
+      <c r="E32" s="94"/>
+      <c r="F32" s="94"/>
+      <c r="G32" s="94"/>
+      <c r="H32" s="94"/>
+      <c r="I32" s="94"/>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B33" s="92"/>
-      <c r="C33" s="92"/>
-      <c r="D33" s="92"/>
-      <c r="E33" s="92"/>
-      <c r="F33" s="92"/>
-      <c r="G33" s="92"/>
-      <c r="H33" s="92"/>
-      <c r="I33" s="92"/>
+      <c r="B33" s="94"/>
+      <c r="C33" s="94"/>
+      <c r="D33" s="94"/>
+      <c r="E33" s="94"/>
+      <c r="F33" s="94"/>
+      <c r="G33" s="94"/>
+      <c r="H33" s="94"/>
+      <c r="I33" s="94"/>
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:I33"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="C27:I27"/>
+    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="C21:I21"/>
     <mergeCell ref="C15:I15"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -4965,25 +4984,6 @@
     <mergeCell ref="B10:I12"/>
     <mergeCell ref="B13:I13"/>
     <mergeCell ref="B14:I14"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="C21:I21"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:I33"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="C27:I27"/>
-    <mergeCell ref="B28:I28"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{60ABBC95-3763-1140-8147-BC4DA0DFC780}"/>
@@ -5138,6 +5138,7 @@
   <dimension ref="B2:I38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" style="1" customWidth="1"/>
     <col min="3" max="3" width="14.5" style="1" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" style="1" customWidth="1"/>
@@ -5146,256 +5147,256 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="89" t="s">
+      <c r="C3" s="71" t="s">
         <v>82</v>
       </c>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
-      <c r="I3" s="90"/>
+      <c r="D3" s="72"/>
+      <c r="E3" s="72"/>
+      <c r="F3" s="72"/>
+      <c r="G3" s="72"/>
+      <c r="H3" s="72"/>
+      <c r="I3" s="72"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="63" t="s">
+      <c r="C4" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="63"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
-      <c r="G4" s="63"/>
-      <c r="H4" s="63"/>
-      <c r="I4" s="63"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="63">
+      <c r="C5" s="19">
         <v>2025</v>
       </c>
-      <c r="D5" s="63"/>
-      <c r="E5" s="63"/>
-      <c r="F5" s="63"/>
-      <c r="G5" s="63"/>
-      <c r="H5" s="63"/>
-      <c r="I5" s="63"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
     </row>
     <row r="6" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="65" t="s">
+      <c r="C6" s="31" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="65"/>
-      <c r="E6" s="65"/>
-      <c r="F6" s="65"/>
-      <c r="G6" s="65"/>
-      <c r="H6" s="65"/>
-      <c r="I6" s="65"/>
+      <c r="D6" s="31"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="68" t="s">
+      <c r="C7" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="D7" s="63"/>
-      <c r="E7" s="63"/>
-      <c r="F7" s="63"/>
-      <c r="G7" s="63"/>
-      <c r="H7" s="63"/>
-      <c r="I7" s="63"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="34"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="34"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="55" t="s">
+      <c r="B9" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="55"/>
-      <c r="D9" s="55"/>
-      <c r="E9" s="55"/>
-      <c r="F9" s="55"/>
-      <c r="G9" s="55"/>
-      <c r="H9" s="55"/>
-      <c r="I9" s="55"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B10" s="60" t="s">
+      <c r="B10" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="60"/>
-      <c r="D10" s="60"/>
-      <c r="E10" s="60"/>
-      <c r="F10" s="60"/>
-      <c r="G10" s="60"/>
-      <c r="H10" s="60"/>
-      <c r="I10" s="60"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B11" s="60"/>
-      <c r="C11" s="60"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="60"/>
-      <c r="H11" s="60"/>
-      <c r="I11" s="60"/>
-    </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B12" s="60"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="60"/>
-      <c r="H12" s="60"/>
-      <c r="I12" s="60"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+    </row>
+    <row r="12" spans="2:9" ht="92" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="34"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="34"/>
-      <c r="I13" s="34"/>
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="55" t="s">
+      <c r="B14" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="55"/>
-      <c r="D14" s="55"/>
-      <c r="E14" s="55"/>
-      <c r="F14" s="55"/>
-      <c r="G14" s="55"/>
-      <c r="H14" s="55"/>
-      <c r="I14" s="55"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="20"/>
+      <c r="I14" s="20"/>
     </row>
     <row r="15" spans="2:9" ht="46" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="64" t="s">
+      <c r="C15" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="D15" s="65"/>
-      <c r="E15" s="65"/>
-      <c r="F15" s="65"/>
-      <c r="G15" s="65"/>
-      <c r="H15" s="65"/>
-      <c r="I15" s="65"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="31"/>
+      <c r="G15" s="31"/>
+      <c r="H15" s="31"/>
+      <c r="I15" s="31"/>
     </row>
     <row r="16" spans="2:9" ht="59" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="80" t="s">
+      <c r="C16" s="73" t="s">
         <v>88</v>
       </c>
-      <c r="D16" s="81"/>
-      <c r="E16" s="81"/>
-      <c r="F16" s="81"/>
-      <c r="G16" s="81"/>
-      <c r="H16" s="81"/>
-      <c r="I16" s="82"/>
+      <c r="D16" s="74"/>
+      <c r="E16" s="74"/>
+      <c r="F16" s="74"/>
+      <c r="G16" s="74"/>
+      <c r="H16" s="74"/>
+      <c r="I16" s="75"/>
     </row>
     <row r="17" spans="2:9" ht="92" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="45"/>
-      <c r="C17" s="83"/>
-      <c r="D17" s="84"/>
-      <c r="E17" s="84"/>
-      <c r="F17" s="84"/>
-      <c r="G17" s="84"/>
-      <c r="H17" s="84"/>
-      <c r="I17" s="85"/>
+      <c r="C17" s="76"/>
+      <c r="D17" s="77"/>
+      <c r="E17" s="77"/>
+      <c r="F17" s="77"/>
+      <c r="G17" s="77"/>
+      <c r="H17" s="77"/>
+      <c r="I17" s="78"/>
     </row>
     <row r="18" spans="2:9" ht="256" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="89" t="s">
+      <c r="C18" s="71" t="s">
         <v>89</v>
       </c>
-      <c r="D18" s="63"/>
-      <c r="E18" s="63"/>
-      <c r="F18" s="63"/>
-      <c r="G18" s="63"/>
-      <c r="H18" s="63"/>
-      <c r="I18" s="63"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="19"/>
+      <c r="H18" s="19"/>
+      <c r="I18" s="19"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="34"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="34"/>
-      <c r="I19" s="34"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="26"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="55" t="s">
+      <c r="B20" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="C20" s="55"/>
-      <c r="D20" s="55"/>
-      <c r="E20" s="55"/>
-      <c r="F20" s="55"/>
-      <c r="G20" s="55"/>
-      <c r="H20" s="55"/>
-      <c r="I20" s="55"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="20"/>
+      <c r="I20" s="20"/>
     </row>
     <row r="21" spans="2:9" ht="246" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="86" t="s">
+      <c r="C21" s="79" t="s">
         <v>90</v>
       </c>
-      <c r="D21" s="87"/>
-      <c r="E21" s="87"/>
-      <c r="F21" s="87"/>
-      <c r="G21" s="87"/>
-      <c r="H21" s="87"/>
-      <c r="I21" s="88"/>
+      <c r="D21" s="80"/>
+      <c r="E21" s="80"/>
+      <c r="F21" s="80"/>
+      <c r="G21" s="80"/>
+      <c r="H21" s="80"/>
+      <c r="I21" s="81"/>
     </row>
     <row r="22" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="41">
+      <c r="C22" s="34">
         <v>8</v>
       </c>
       <c r="D22" s="42"/>
@@ -5425,210 +5426,235 @@
       <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="99" t="s">
+      <c r="C24" s="96" t="s">
         <v>92</v>
       </c>
-      <c r="D24" s="100"/>
-      <c r="E24" s="89" t="s">
+      <c r="D24" s="97"/>
+      <c r="E24" s="71" t="s">
         <v>107</v>
       </c>
-      <c r="F24" s="89"/>
-      <c r="G24" s="89"/>
-      <c r="H24" s="89"/>
-      <c r="I24" s="89"/>
+      <c r="F24" s="71"/>
+      <c r="G24" s="71"/>
+      <c r="H24" s="71"/>
+      <c r="I24" s="71"/>
     </row>
     <row r="25" spans="2:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="8">
         <v>2</v>
       </c>
-      <c r="C25" s="97" t="s">
+      <c r="C25" s="98" t="s">
         <v>93</v>
       </c>
-      <c r="D25" s="98"/>
-      <c r="E25" s="89" t="s">
+      <c r="D25" s="99"/>
+      <c r="E25" s="71" t="s">
         <v>108</v>
       </c>
-      <c r="F25" s="89"/>
-      <c r="G25" s="89"/>
-      <c r="H25" s="89"/>
-      <c r="I25" s="89"/>
+      <c r="F25" s="71"/>
+      <c r="G25" s="71"/>
+      <c r="H25" s="71"/>
+      <c r="I25" s="71"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B26" s="8">
         <v>3</v>
       </c>
-      <c r="C26" s="97" t="s">
+      <c r="C26" s="98" t="s">
         <v>94</v>
       </c>
-      <c r="D26" s="98"/>
-      <c r="E26" s="89" t="s">
+      <c r="D26" s="99"/>
+      <c r="E26" s="71" t="s">
         <v>106</v>
       </c>
-      <c r="F26" s="89"/>
-      <c r="G26" s="89"/>
-      <c r="H26" s="89"/>
-      <c r="I26" s="89"/>
+      <c r="F26" s="71"/>
+      <c r="G26" s="71"/>
+      <c r="H26" s="71"/>
+      <c r="I26" s="71"/>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B27" s="8">
         <v>4</v>
       </c>
-      <c r="C27" s="97" t="s">
+      <c r="C27" s="98" t="s">
         <v>95</v>
       </c>
-      <c r="D27" s="98"/>
-      <c r="E27" s="89" t="s">
+      <c r="D27" s="99"/>
+      <c r="E27" s="71" t="s">
         <v>105</v>
       </c>
-      <c r="F27" s="89"/>
-      <c r="G27" s="89"/>
-      <c r="H27" s="89"/>
-      <c r="I27" s="89"/>
+      <c r="F27" s="71"/>
+      <c r="G27" s="71"/>
+      <c r="H27" s="71"/>
+      <c r="I27" s="71"/>
     </row>
     <row r="28" spans="2:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="8">
         <v>5</v>
       </c>
-      <c r="C28" s="97" t="s">
+      <c r="C28" s="98" t="s">
         <v>96</v>
       </c>
-      <c r="D28" s="98"/>
-      <c r="E28" s="89" t="s">
+      <c r="D28" s="99"/>
+      <c r="E28" s="71" t="s">
         <v>104</v>
       </c>
-      <c r="F28" s="89"/>
-      <c r="G28" s="89"/>
-      <c r="H28" s="89"/>
-      <c r="I28" s="89"/>
+      <c r="F28" s="71"/>
+      <c r="G28" s="71"/>
+      <c r="H28" s="71"/>
+      <c r="I28" s="71"/>
     </row>
     <row r="29" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="8">
         <v>6</v>
       </c>
-      <c r="C29" s="93" t="s">
+      <c r="C29" s="95" t="s">
         <v>97</v>
       </c>
-      <c r="D29" s="93"/>
-      <c r="E29" s="89" t="s">
+      <c r="D29" s="95"/>
+      <c r="E29" s="71" t="s">
         <v>103</v>
       </c>
-      <c r="F29" s="89"/>
-      <c r="G29" s="89"/>
-      <c r="H29" s="89"/>
-      <c r="I29" s="89"/>
+      <c r="F29" s="71"/>
+      <c r="G29" s="71"/>
+      <c r="H29" s="71"/>
+      <c r="I29" s="71"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B30" s="8">
         <v>7</v>
       </c>
-      <c r="C30" s="93" t="s">
+      <c r="C30" s="95" t="s">
         <v>98</v>
       </c>
-      <c r="D30" s="93"/>
-      <c r="E30" s="89" t="s">
+      <c r="D30" s="95"/>
+      <c r="E30" s="71" t="s">
         <v>102</v>
       </c>
-      <c r="F30" s="96"/>
-      <c r="G30" s="96"/>
-      <c r="H30" s="96"/>
-      <c r="I30" s="96"/>
+      <c r="F30" s="100"/>
+      <c r="G30" s="100"/>
+      <c r="H30" s="100"/>
+      <c r="I30" s="100"/>
     </row>
     <row r="31" spans="2:9" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="8">
         <v>8</v>
       </c>
-      <c r="C31" s="97" t="s">
+      <c r="C31" s="98" t="s">
         <v>99</v>
       </c>
-      <c r="D31" s="98"/>
-      <c r="E31" s="41" t="s">
+      <c r="D31" s="99"/>
+      <c r="E31" s="34" t="s">
         <v>100</v>
       </c>
-      <c r="F31" s="66"/>
-      <c r="G31" s="66"/>
-      <c r="H31" s="66"/>
-      <c r="I31" s="67"/>
+      <c r="F31" s="35"/>
+      <c r="G31" s="35"/>
+      <c r="H31" s="35"/>
+      <c r="I31" s="36"/>
     </row>
     <row r="32" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B32" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C32" s="64" t="s">
+      <c r="C32" s="30" t="s">
         <v>91</v>
       </c>
-      <c r="D32" s="64"/>
-      <c r="E32" s="64"/>
-      <c r="F32" s="64"/>
-      <c r="G32" s="64"/>
-      <c r="H32" s="64"/>
-      <c r="I32" s="64"/>
+      <c r="D32" s="30"/>
+      <c r="E32" s="30"/>
+      <c r="F32" s="30"/>
+      <c r="G32" s="30"/>
+      <c r="H32" s="30"/>
+      <c r="I32" s="30"/>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B33" s="35"/>
-      <c r="C33" s="36"/>
-      <c r="D33" s="36"/>
-      <c r="E33" s="36"/>
-      <c r="F33" s="36"/>
-      <c r="G33" s="36"/>
-      <c r="H33" s="36"/>
-      <c r="I33" s="37"/>
+      <c r="B33" s="38"/>
+      <c r="C33" s="39"/>
+      <c r="D33" s="39"/>
+      <c r="E33" s="39"/>
+      <c r="F33" s="39"/>
+      <c r="G33" s="39"/>
+      <c r="H33" s="39"/>
+      <c r="I33" s="40"/>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B34" s="55" t="s">
+      <c r="B34" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="C34" s="55"/>
-      <c r="D34" s="55"/>
-      <c r="E34" s="55"/>
-      <c r="F34" s="55"/>
-      <c r="G34" s="55"/>
-      <c r="H34" s="55"/>
-      <c r="I34" s="55"/>
+      <c r="C34" s="20"/>
+      <c r="D34" s="20"/>
+      <c r="E34" s="20"/>
+      <c r="F34" s="20"/>
+      <c r="G34" s="20"/>
+      <c r="H34" s="20"/>
+      <c r="I34" s="20"/>
     </row>
     <row r="35" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="77" t="s">
+      <c r="B35" s="82" t="s">
         <v>109</v>
       </c>
-      <c r="C35" s="61"/>
-      <c r="D35" s="61"/>
-      <c r="E35" s="61"/>
-      <c r="F35" s="61"/>
-      <c r="G35" s="61"/>
-      <c r="H35" s="61"/>
-      <c r="I35" s="61"/>
+      <c r="C35" s="24"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="24"/>
+      <c r="H35" s="24"/>
+      <c r="I35" s="24"/>
     </row>
     <row r="36" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="61"/>
-      <c r="C36" s="61"/>
-      <c r="D36" s="61"/>
-      <c r="E36" s="61"/>
-      <c r="F36" s="61"/>
-      <c r="G36" s="61"/>
-      <c r="H36" s="61"/>
-      <c r="I36" s="61"/>
+      <c r="B36" s="24"/>
+      <c r="C36" s="24"/>
+      <c r="D36" s="24"/>
+      <c r="E36" s="24"/>
+      <c r="F36" s="24"/>
+      <c r="G36" s="24"/>
+      <c r="H36" s="24"/>
+      <c r="I36" s="24"/>
     </row>
     <row r="37" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="61"/>
-      <c r="C37" s="61"/>
-      <c r="D37" s="61"/>
-      <c r="E37" s="61"/>
-      <c r="F37" s="61"/>
-      <c r="G37" s="61"/>
-      <c r="H37" s="61"/>
-      <c r="I37" s="61"/>
+      <c r="B37" s="24"/>
+      <c r="C37" s="24"/>
+      <c r="D37" s="24"/>
+      <c r="E37" s="24"/>
+      <c r="F37" s="24"/>
+      <c r="G37" s="24"/>
+      <c r="H37" s="24"/>
+      <c r="I37" s="24"/>
     </row>
     <row r="38" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="61"/>
-      <c r="C38" s="61"/>
-      <c r="D38" s="61"/>
-      <c r="E38" s="61"/>
-      <c r="F38" s="61"/>
-      <c r="G38" s="61"/>
-      <c r="H38" s="61"/>
-      <c r="I38" s="61"/>
+      <c r="B38" s="24"/>
+      <c r="C38" s="24"/>
+      <c r="D38" s="24"/>
+      <c r="E38" s="24"/>
+      <c r="F38" s="24"/>
+      <c r="G38" s="24"/>
+      <c r="H38" s="24"/>
+      <c r="I38" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="41">
+    <mergeCell ref="B35:I38"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="E29:I29"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:I28"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:I31"/>
+    <mergeCell ref="C32:I32"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="B34:I34"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="C6:I6"/>
     <mergeCell ref="C7:I7"/>
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="C25:D25"/>
@@ -5645,31 +5671,6 @@
     <mergeCell ref="B13:I13"/>
     <mergeCell ref="B14:I14"/>
     <mergeCell ref="C15:I15"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="C3:I3"/>
-    <mergeCell ref="C4:I4"/>
-    <mergeCell ref="C5:I5"/>
-    <mergeCell ref="C6:I6"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="B35:I38"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="E29:I29"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:I30"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E28:I28"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:I31"/>
-    <mergeCell ref="C32:I32"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="B34:I34"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{69FD07AD-7FCA-E141-8126-AFB63E0A1511}"/>

</xml_diff>

<commit_message>
created all the prompts
</commit_message>
<xml_diff>
--- a/Papers/Resumen Papers.xlsx
+++ b/Papers/Resumen Papers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sophiaaristizabal/Documents/GitHub/LLMS_Project/Papers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AEFC2EB-2F32-6648-AAC1-0337E8C17ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3E2B5D5-32A3-3646-8458-7D83021BEA29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" firstSheet="2" activeTab="4" xr2:uid="{400AC57E-08F9-B346-9132-4F74AEBC2D15}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="20520" windowHeight="13540" xr2:uid="{400AC57E-08F9-B346-9132-4F74AEBC2D15}"/>
   </bookViews>
   <sheets>
     <sheet name="MANAGERIAL LEADERSHIP" sheetId="1" r:id="rId1"/>
@@ -115,7 +115,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="178">
   <si>
     <t>Autores</t>
   </si>
@@ -1602,20 +1602,8 @@
     <t xml:space="preserve"> “Promise,”</t>
   </si>
   <si>
-    <t>“Other Content,”</t>
-  </si>
-  <si>
-    <t>“No Message.”</t>
-  </si>
-  <si>
     <t>Two ­ hypothesis-blind research assistants classified the messages independently. received a monetary incentive for indicating the same categories as the other coder.
 The correlation between the two research assistants was high (for the Promise category, Pearson correlation is 0.87 and Cronbach’s α = 0.93).</t>
-  </si>
-  <si>
-    <t>3  We allowed three levels for the coding: 0 (category not present in message); 1 (category somewhat present in message); 2 (category strongly present in message).</t>
-  </si>
-  <si>
-    <t>We classified a message as a promise if both assistants coded the message as such</t>
   </si>
   <si>
     <t xml:space="preserve">Sistema de clasificación humana (gold standard) APPENDIX </t>
@@ -1918,10 +1906,6 @@
     <t>students are unaware of other students’ actual AI adoption</t>
   </si>
   <si>
-    <t>A varied range of sources of social desirability associated with reporting AI usage are provided by the respondents
-as well. Academic integrity concerns, such as casting AI usage as cheating or dishonest, is most frequently mentioned</t>
-  </si>
-  <si>
     <t>The reporting gap is overestimation of others’ usage (22/71). Among these participants, multiple respondents suggest that this overestimation could come from biased perception: students are “primed” by AI reliance in certain groups and overgeneralize it to all other students</t>
   </si>
   <si>
@@ -2099,9 +2083,6 @@
     <t>academic integrity</t>
   </si>
   <si>
-    <t>T, F or F?</t>
-  </si>
-  <si>
     <t>info asymmetry</t>
   </si>
   <si>
@@ -2127,6 +2108,37 @@
   </si>
   <si>
     <t>0          . . .             *</t>
+  </si>
+  <si>
+    <t>T, F or F?
+si es T, los demás tags se vuelven automáticamente FALSE</t>
+  </si>
+  <si>
+    <t>A varied range of sources of social desirability associated with reporting AI usage are provided by the respondents as well. Academic integrity concerns, such as casting AI usage as cheating or dishonest, is most frequently mentioned</t>
+  </si>
+  <si>
+    <t>“Is efficiency” (“other content”)</t>
+  </si>
+  <si>
+    <t>"is ethics"  (“other content”)</t>
+  </si>
+  <si>
+    <t>3  We allowed three levels for the coding: 0 (category not present in message); 1 (category somewhat present in message); 2 (category strongly present in message).
+29After sighting the messages, we decided to break down the “Other Content” category into “Appeal to Efficiency,”
+“Appeal to Fairness,” and “Other Content.” We did this because we realized that some participants seemed to use
+other, non-promise, types of arguments to convince the trustor to choose IN. The same message could be classified
+into more than one category (e.g., both as Promise and as an Appeal to Efficiency). Only 13 messages (8 percent)
+contain an appeal to fairness but 84 messages (49 percent) contain an appeal to efficiency. The latter is highly
+correlated with the presence of a promise (Pearson correlation 0.75).</t>
+  </si>
+  <si>
+    <t>This type of argument emphasizes that a decision or action is just, equitable, or morally right based on principles of fairness. In the context of the experiment, it refers to messages or arguments that invoke fairness considerations to persuade the trustor to choose the cooperative option, suggesting that such a choice is morally or ethically justified</t>
+  </si>
+  <si>
+    <t>This argument appeals to the practical benefits of efficiency, emphasizing that a decision promotes optimal use of resources or maximizes overall welfare. In this context, messages containing an appeal to efficiency aim to convince the trustor to cooperate because it leads to better resource allocation or more favorable outcomes for all parties involved. The experiments found that appeals to efficiency are highly correlated with promises</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We classified a message as a promise if both assistants coded the message as such. The category of promise is defined as a message in which the sender (trustee) explicitly or implicitly commits to a specific future action, such as choosing to ROLL. </t>
   </si>
 </sst>
 </file>
@@ -2367,7 +2379,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2418,164 +2430,221 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -2583,59 +2652,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -2643,13 +2667,13 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2658,14 +2682,17 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2698,7 +2725,7 @@
       <xdr:col>6</xdr:col>
       <xdr:colOff>70790</xdr:colOff>
       <xdr:row>38</xdr:row>
-      <xdr:rowOff>1110825</xdr:rowOff>
+      <xdr:rowOff>1110824</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2741,7 +2768,7 @@
       <xdr:col>8</xdr:col>
       <xdr:colOff>3663820</xdr:colOff>
       <xdr:row>39</xdr:row>
-      <xdr:rowOff>609600</xdr:rowOff>
+      <xdr:rowOff>609599</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3216,384 +3243,384 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="21"/>
+      <c r="D3" s="70"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="70"/>
+      <c r="H3" s="70"/>
+      <c r="I3" s="70"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="71" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
+      <c r="D4" s="71"/>
+      <c r="E4" s="71"/>
+      <c r="F4" s="71"/>
+      <c r="G4" s="71"/>
+      <c r="H4" s="71"/>
+      <c r="I4" s="71"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="64">
         <v>2025</v>
       </c>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="64"/>
     </row>
     <row r="6" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
+      <c r="D6" s="64"/>
+      <c r="E6" s="64"/>
+      <c r="F6" s="64"/>
+      <c r="G6" s="64"/>
+      <c r="H6" s="64"/>
+      <c r="I6" s="64"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="69" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
+      <c r="D7" s="64"/>
+      <c r="E7" s="64"/>
+      <c r="F7" s="64"/>
+      <c r="G7" s="64"/>
+      <c r="H7" s="64"/>
+      <c r="I7" s="64"/>
     </row>
     <row r="8" spans="2:9" ht="9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="28"/>
     </row>
     <row r="9" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="20"/>
+      <c r="C9" s="54"/>
+      <c r="D9" s="54"/>
+      <c r="E9" s="54"/>
+      <c r="F9" s="54"/>
+      <c r="G9" s="54"/>
+      <c r="H9" s="54"/>
+      <c r="I9" s="54"/>
     </row>
     <row r="10" spans="2:9" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="61" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
+      <c r="C10" s="61"/>
+      <c r="D10" s="61"/>
+      <c r="E10" s="61"/>
+      <c r="F10" s="61"/>
+      <c r="G10" s="61"/>
+      <c r="H10" s="61"/>
+      <c r="I10" s="61"/>
     </row>
     <row r="11" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="23"/>
+      <c r="B11" s="61"/>
+      <c r="C11" s="61"/>
+      <c r="D11" s="61"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="61"/>
+      <c r="I11" s="61"/>
     </row>
     <row r="12" spans="2:9" ht="11" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
-      <c r="H12" s="23"/>
-      <c r="I12" s="23"/>
+      <c r="B12" s="61"/>
+      <c r="C12" s="61"/>
+      <c r="D12" s="61"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
+      <c r="G12" s="61"/>
+      <c r="H12" s="61"/>
+      <c r="I12" s="61"/>
     </row>
     <row r="13" spans="2:9" ht="9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="26"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="28"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="54" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="20"/>
+      <c r="C14" s="54"/>
+      <c r="D14" s="54"/>
+      <c r="E14" s="54"/>
+      <c r="F14" s="54"/>
+      <c r="G14" s="54"/>
+      <c r="H14" s="54"/>
+      <c r="I14" s="54"/>
     </row>
     <row r="15" spans="2:9" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="19"/>
-    </row>
-    <row r="16" spans="2:9" ht="125" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="44" t="s">
+      <c r="D15" s="64"/>
+      <c r="E15" s="64"/>
+      <c r="F15" s="64"/>
+      <c r="G15" s="64"/>
+      <c r="H15" s="64"/>
+      <c r="I15" s="64"/>
+    </row>
+    <row r="16" spans="2:9" ht="136" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="46" t="s">
+      <c r="C16" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="D16" s="47"/>
-      <c r="E16" s="47"/>
-      <c r="F16" s="47"/>
-      <c r="G16" s="47"/>
-      <c r="H16" s="47"/>
-      <c r="I16" s="48"/>
+      <c r="D16" s="46"/>
+      <c r="E16" s="46"/>
+      <c r="F16" s="46"/>
+      <c r="G16" s="46"/>
+      <c r="H16" s="46"/>
+      <c r="I16" s="47"/>
     </row>
     <row r="17" spans="2:9" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="45"/>
-      <c r="C17" s="49"/>
-      <c r="D17" s="50"/>
-      <c r="E17" s="50"/>
-      <c r="F17" s="50"/>
-      <c r="G17" s="50"/>
-      <c r="H17" s="50"/>
-      <c r="I17" s="51"/>
+      <c r="B17" s="44"/>
+      <c r="C17" s="48"/>
+      <c r="D17" s="49"/>
+      <c r="E17" s="49"/>
+      <c r="F17" s="49"/>
+      <c r="G17" s="49"/>
+      <c r="H17" s="49"/>
+      <c r="I17" s="50"/>
     </row>
     <row r="18" spans="2:9" ht="67" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="25" t="s">
+      <c r="C18" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
+      <c r="D18" s="64"/>
+      <c r="E18" s="64"/>
+      <c r="F18" s="64"/>
+      <c r="G18" s="64"/>
+      <c r="H18" s="64"/>
+      <c r="I18" s="64"/>
     </row>
     <row r="19" spans="2:9" ht="7" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="28"/>
+      <c r="I19" s="28"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20"/>
-      <c r="I20" s="20"/>
+      <c r="C20" s="54"/>
+      <c r="D20" s="54"/>
+      <c r="E20" s="54"/>
+      <c r="F20" s="54"/>
+      <c r="G20" s="54"/>
+      <c r="H20" s="54"/>
+      <c r="I20" s="54"/>
     </row>
     <row r="21" spans="2:9" ht="43" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="41" t="s">
+      <c r="C21" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="28"/>
-      <c r="H21" s="28"/>
-      <c r="I21" s="29"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="38"/>
+      <c r="F21" s="38"/>
+      <c r="G21" s="38"/>
+      <c r="H21" s="38"/>
+      <c r="I21" s="39"/>
     </row>
     <row r="22" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B22" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="34">
+      <c r="C22" s="40">
         <v>9</v>
       </c>
-      <c r="D22" s="42"/>
-      <c r="E22" s="42"/>
-      <c r="F22" s="42"/>
-      <c r="G22" s="42"/>
-      <c r="H22" s="42"/>
-      <c r="I22" s="43"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="41"/>
+      <c r="F22" s="41"/>
+      <c r="G22" s="41"/>
+      <c r="H22" s="41"/>
+      <c r="I22" s="42"/>
     </row>
     <row r="23" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="56" t="s">
+      <c r="C23" s="55" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="56"/>
-      <c r="E23" s="57" t="s">
+      <c r="D23" s="55"/>
+      <c r="E23" s="56" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="57"/>
-      <c r="G23" s="57"/>
-      <c r="H23" s="57"/>
-      <c r="I23" s="57"/>
+      <c r="F23" s="56"/>
+      <c r="G23" s="56"/>
+      <c r="H23" s="56"/>
+      <c r="I23" s="56"/>
     </row>
     <row r="24" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="54" t="s">
+      <c r="C24" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="D24" s="55"/>
-      <c r="E24" s="41" t="s">
+      <c r="D24" s="32"/>
+      <c r="E24" s="37" t="s">
         <v>37</v>
       </c>
-      <c r="F24" s="58"/>
-      <c r="G24" s="58"/>
-      <c r="H24" s="58"/>
-      <c r="I24" s="59"/>
+      <c r="F24" s="57"/>
+      <c r="G24" s="57"/>
+      <c r="H24" s="57"/>
+      <c r="I24" s="58"/>
     </row>
     <row r="25" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="8">
         <v>2</v>
       </c>
-      <c r="C25" s="54" t="s">
+      <c r="C25" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="D25" s="55"/>
-      <c r="E25" s="54"/>
-      <c r="F25" s="70"/>
-      <c r="G25" s="70"/>
-      <c r="H25" s="70"/>
-      <c r="I25" s="55"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="30"/>
+      <c r="F25" s="31"/>
+      <c r="G25" s="31"/>
+      <c r="H25" s="31"/>
+      <c r="I25" s="32"/>
     </row>
     <row r="26" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="60">
+      <c r="B26" s="59">
         <v>3</v>
       </c>
-      <c r="C26" s="62" t="s">
+      <c r="C26" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="D26" s="63"/>
-      <c r="E26" s="37" t="s">
+      <c r="D26" s="20"/>
+      <c r="E26" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="F26" s="37"/>
-      <c r="G26" s="70" t="s">
+      <c r="F26" s="33"/>
+      <c r="G26" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="H26" s="70"/>
-      <c r="I26" s="55"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="32"/>
     </row>
     <row r="27" spans="2:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="61"/>
-      <c r="C27" s="64"/>
-      <c r="D27" s="65"/>
-      <c r="E27" s="32" t="s">
+      <c r="B27" s="60"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="F27" s="33"/>
-      <c r="G27" s="66" t="s">
+      <c r="F27" s="24"/>
+      <c r="G27" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="H27" s="67"/>
-      <c r="I27" s="68"/>
+      <c r="H27" s="26"/>
+      <c r="I27" s="27"/>
     </row>
     <row r="28" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="8">
         <v>4</v>
       </c>
-      <c r="C28" s="32" t="s">
+      <c r="C28" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="D28" s="33"/>
-      <c r="E28" s="27" t="s">
+      <c r="D28" s="24"/>
+      <c r="E28" s="51" t="s">
         <v>32</v>
       </c>
-      <c r="F28" s="28"/>
-      <c r="G28" s="28"/>
-      <c r="H28" s="28"/>
-      <c r="I28" s="29"/>
+      <c r="F28" s="38"/>
+      <c r="G28" s="38"/>
+      <c r="H28" s="38"/>
+      <c r="I28" s="39"/>
     </row>
     <row r="29" spans="2:9" ht="43" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="8">
         <v>5</v>
       </c>
-      <c r="C29" s="37" t="s">
+      <c r="C29" s="33" t="s">
         <v>27</v>
       </c>
-      <c r="D29" s="37"/>
-      <c r="E29" s="30" t="s">
+      <c r="D29" s="33"/>
+      <c r="E29" s="65" t="s">
         <v>33</v>
       </c>
-      <c r="F29" s="30"/>
-      <c r="G29" s="30"/>
-      <c r="H29" s="30"/>
-      <c r="I29" s="30"/>
+      <c r="F29" s="65"/>
+      <c r="G29" s="65"/>
+      <c r="H29" s="65"/>
+      <c r="I29" s="65"/>
     </row>
     <row r="30" spans="2:9" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="8">
         <v>6</v>
       </c>
-      <c r="C30" s="32" t="s">
+      <c r="C30" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="D30" s="33"/>
-      <c r="E30" s="27" t="s">
+      <c r="D30" s="24"/>
+      <c r="E30" s="51" t="s">
         <v>34</v>
       </c>
       <c r="F30" s="52"/>
@@ -3605,137 +3632,150 @@
       <c r="B31" s="8">
         <v>7</v>
       </c>
-      <c r="C31" s="37" t="s">
+      <c r="C31" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="D31" s="37"/>
-      <c r="E31" s="30" t="s">
+      <c r="D31" s="33"/>
+      <c r="E31" s="65" t="s">
         <v>35</v>
       </c>
-      <c r="F31" s="31"/>
-      <c r="G31" s="31"/>
-      <c r="H31" s="31"/>
-      <c r="I31" s="31"/>
+      <c r="F31" s="66"/>
+      <c r="G31" s="66"/>
+      <c r="H31" s="66"/>
+      <c r="I31" s="66"/>
     </row>
     <row r="32" spans="2:9" ht="53" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="8">
         <v>8</v>
       </c>
-      <c r="C32" s="32" t="s">
+      <c r="C32" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="D32" s="33"/>
-      <c r="E32" s="32"/>
-      <c r="F32" s="69"/>
-      <c r="G32" s="69"/>
-      <c r="H32" s="69"/>
-      <c r="I32" s="33"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="29"/>
+      <c r="H32" s="29"/>
+      <c r="I32" s="24"/>
     </row>
     <row r="33" spans="2:9" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="8">
         <v>9</v>
       </c>
-      <c r="C33" s="32" t="s">
+      <c r="C33" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="D33" s="33"/>
-      <c r="E33" s="34" t="s">
+      <c r="D33" s="24"/>
+      <c r="E33" s="40" t="s">
         <v>46</v>
       </c>
-      <c r="F33" s="35"/>
-      <c r="G33" s="35"/>
-      <c r="H33" s="35"/>
-      <c r="I33" s="36"/>
+      <c r="F33" s="67"/>
+      <c r="G33" s="67"/>
+      <c r="H33" s="67"/>
+      <c r="I33" s="68"/>
     </row>
     <row r="34" spans="2:9" ht="190" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C34" s="30" t="s">
+      <c r="C34" s="65" t="s">
         <v>31</v>
       </c>
-      <c r="D34" s="30"/>
-      <c r="E34" s="30"/>
-      <c r="F34" s="30"/>
-      <c r="G34" s="30"/>
-      <c r="H34" s="30"/>
-      <c r="I34" s="30"/>
+      <c r="D34" s="65"/>
+      <c r="E34" s="65"/>
+      <c r="F34" s="65"/>
+      <c r="G34" s="65"/>
+      <c r="H34" s="65"/>
+      <c r="I34" s="65"/>
     </row>
     <row r="35" spans="2:9" ht="10" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="38"/>
-      <c r="C35" s="39"/>
-      <c r="D35" s="39"/>
-      <c r="E35" s="39"/>
-      <c r="F35" s="39"/>
-      <c r="G35" s="39"/>
-      <c r="H35" s="39"/>
-      <c r="I35" s="40"/>
+      <c r="B35" s="34"/>
+      <c r="C35" s="35"/>
+      <c r="D35" s="35"/>
+      <c r="E35" s="35"/>
+      <c r="F35" s="35"/>
+      <c r="G35" s="35"/>
+      <c r="H35" s="35"/>
+      <c r="I35" s="36"/>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B36" s="20" t="s">
+      <c r="B36" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="C36" s="20"/>
-      <c r="D36" s="20"/>
-      <c r="E36" s="20"/>
-      <c r="F36" s="20"/>
-      <c r="G36" s="20"/>
-      <c r="H36" s="20"/>
-      <c r="I36" s="20"/>
+      <c r="C36" s="54"/>
+      <c r="D36" s="54"/>
+      <c r="E36" s="54"/>
+      <c r="F36" s="54"/>
+      <c r="G36" s="54"/>
+      <c r="H36" s="54"/>
+      <c r="I36" s="54"/>
     </row>
     <row r="37" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="24" t="s">
+      <c r="B37" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="C37" s="24"/>
-      <c r="D37" s="24"/>
-      <c r="E37" s="24"/>
-      <c r="F37" s="24"/>
-      <c r="G37" s="24"/>
-      <c r="H37" s="24"/>
-      <c r="I37" s="24"/>
+      <c r="C37" s="62"/>
+      <c r="D37" s="62"/>
+      <c r="E37" s="62"/>
+      <c r="F37" s="62"/>
+      <c r="G37" s="62"/>
+      <c r="H37" s="62"/>
+      <c r="I37" s="62"/>
     </row>
     <row r="38" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="24"/>
-      <c r="C38" s="24"/>
-      <c r="D38" s="24"/>
-      <c r="E38" s="24"/>
-      <c r="F38" s="24"/>
-      <c r="G38" s="24"/>
-      <c r="H38" s="24"/>
-      <c r="I38" s="24"/>
+      <c r="B38" s="62"/>
+      <c r="C38" s="62"/>
+      <c r="D38" s="62"/>
+      <c r="E38" s="62"/>
+      <c r="F38" s="62"/>
+      <c r="G38" s="62"/>
+      <c r="H38" s="62"/>
+      <c r="I38" s="62"/>
     </row>
     <row r="39" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="24"/>
-      <c r="C39" s="24"/>
-      <c r="D39" s="24"/>
-      <c r="E39" s="24"/>
-      <c r="F39" s="24"/>
-      <c r="G39" s="24"/>
-      <c r="H39" s="24"/>
-      <c r="I39" s="24"/>
+      <c r="B39" s="62"/>
+      <c r="C39" s="62"/>
+      <c r="D39" s="62"/>
+      <c r="E39" s="62"/>
+      <c r="F39" s="62"/>
+      <c r="G39" s="62"/>
+      <c r="H39" s="62"/>
+      <c r="I39" s="62"/>
     </row>
     <row r="40" spans="2:9" ht="76" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B40" s="24"/>
-      <c r="C40" s="24"/>
-      <c r="D40" s="24"/>
-      <c r="E40" s="24"/>
-      <c r="F40" s="24"/>
-      <c r="G40" s="24"/>
-      <c r="H40" s="24"/>
-      <c r="I40" s="24"/>
+      <c r="B40" s="62"/>
+      <c r="C40" s="62"/>
+      <c r="D40" s="62"/>
+      <c r="E40" s="62"/>
+      <c r="F40" s="62"/>
+      <c r="G40" s="62"/>
+      <c r="H40" s="62"/>
+      <c r="I40" s="62"/>
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="C26:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="E32:I32"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="B36:I36"/>
+    <mergeCell ref="B10:I12"/>
+    <mergeCell ref="B9:I9"/>
+    <mergeCell ref="B37:I40"/>
+    <mergeCell ref="C15:I15"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="E28:I28"/>
+    <mergeCell ref="E29:I29"/>
+    <mergeCell ref="E31:I31"/>
+    <mergeCell ref="C34:I34"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="E33:I33"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C31:D31"/>
     <mergeCell ref="B35:I35"/>
     <mergeCell ref="B13:I13"/>
     <mergeCell ref="C21:I21"/>
@@ -3752,28 +3792,15 @@
     <mergeCell ref="E24:I24"/>
     <mergeCell ref="C25:D25"/>
     <mergeCell ref="B26:B27"/>
-    <mergeCell ref="B36:I36"/>
-    <mergeCell ref="B10:I12"/>
-    <mergeCell ref="B9:I9"/>
-    <mergeCell ref="B37:I40"/>
-    <mergeCell ref="C15:I15"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="E28:I28"/>
-    <mergeCell ref="E29:I29"/>
-    <mergeCell ref="E31:I31"/>
-    <mergeCell ref="C34:I34"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="E33:I33"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C7:I7"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="C3:I3"/>
-    <mergeCell ref="C4:I4"/>
-    <mergeCell ref="C5:I5"/>
-    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="C26:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="E32:I32"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="G26:I26"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{C9E9977D-5134-FE4B-852F-8DEBDCB543E0}"/>
@@ -3802,254 +3829,254 @@
   </cols>
   <sheetData>
     <row r="4" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B4" s="22" t="s">
-        <v>133</v>
-      </c>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
+      <c r="B4" s="71" t="s">
+        <v>128</v>
+      </c>
+      <c r="C4" s="71"/>
+      <c r="D4" s="71"/>
+      <c r="E4" s="71"/>
     </row>
     <row r="5" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="11" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="6" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="11" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
     </row>
     <row r="7" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="11" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="8" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="11" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="11" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="10" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="11" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="11" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="11" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="12" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="11" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="13" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="11" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="14" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="11" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="15" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>128</v>
-      </c>
       <c r="E15" s="10" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="16" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="11" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="11" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="18" spans="2:5" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="11" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="19" spans="2:5" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="11" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="20" spans="2:5" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="11" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C20" s="10"/>
       <c r="D20" s="2" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B21" s="11" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="2" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.2">
@@ -4078,442 +4105,421 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="71" t="s">
+      <c r="C3" s="90" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="72"/>
-      <c r="E3" s="72"/>
-      <c r="F3" s="72"/>
-      <c r="G3" s="72"/>
-      <c r="H3" s="72"/>
-      <c r="I3" s="72"/>
+      <c r="D3" s="91"/>
+      <c r="E3" s="91"/>
+      <c r="F3" s="91"/>
+      <c r="G3" s="91"/>
+      <c r="H3" s="91"/>
+      <c r="I3" s="91"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="64" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
+      <c r="D4" s="64"/>
+      <c r="E4" s="64"/>
+      <c r="F4" s="64"/>
+      <c r="G4" s="64"/>
+      <c r="H4" s="64"/>
+      <c r="I4" s="64"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="64">
         <v>2020</v>
       </c>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="64"/>
     </row>
     <row r="6" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="31" t="s">
+      <c r="C6" s="66" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="31"/>
-      <c r="H6" s="31"/>
-      <c r="I6" s="31"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
+      <c r="G6" s="66"/>
+      <c r="H6" s="66"/>
+      <c r="I6" s="66"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="69" t="s">
         <v>51</v>
       </c>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
+      <c r="D7" s="64"/>
+      <c r="E7" s="64"/>
+      <c r="F7" s="64"/>
+      <c r="G7" s="64"/>
+      <c r="H7" s="64"/>
+      <c r="I7" s="64"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="28"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="20"/>
+      <c r="C9" s="54"/>
+      <c r="D9" s="54"/>
+      <c r="E9" s="54"/>
+      <c r="F9" s="54"/>
+      <c r="G9" s="54"/>
+      <c r="H9" s="54"/>
+      <c r="I9" s="54"/>
     </row>
     <row r="10" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="61" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
+      <c r="C10" s="61"/>
+      <c r="D10" s="61"/>
+      <c r="E10" s="61"/>
+      <c r="F10" s="61"/>
+      <c r="G10" s="61"/>
+      <c r="H10" s="61"/>
+      <c r="I10" s="61"/>
     </row>
     <row r="11" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="23"/>
+      <c r="B11" s="61"/>
+      <c r="C11" s="61"/>
+      <c r="D11" s="61"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="61"/>
+      <c r="I11" s="61"/>
     </row>
     <row r="12" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
-      <c r="H12" s="23"/>
-      <c r="I12" s="23"/>
+      <c r="B12" s="61"/>
+      <c r="C12" s="61"/>
+      <c r="D12" s="61"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
+      <c r="G12" s="61"/>
+      <c r="H12" s="61"/>
+      <c r="I12" s="61"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="26"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="28"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="54" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="20"/>
+      <c r="C14" s="54"/>
+      <c r="D14" s="54"/>
+      <c r="E14" s="54"/>
+      <c r="F14" s="54"/>
+      <c r="G14" s="54"/>
+      <c r="H14" s="54"/>
+      <c r="I14" s="54"/>
     </row>
     <row r="15" spans="2:9" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="63" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="19"/>
+      <c r="D15" s="64"/>
+      <c r="E15" s="64"/>
+      <c r="F15" s="64"/>
+      <c r="G15" s="64"/>
+      <c r="H15" s="64"/>
+      <c r="I15" s="64"/>
     </row>
     <row r="16" spans="2:9" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="44" t="s">
+      <c r="B16" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="73" t="s">
+      <c r="C16" s="81" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="74"/>
-      <c r="E16" s="74"/>
-      <c r="F16" s="74"/>
-      <c r="G16" s="74"/>
-      <c r="H16" s="74"/>
-      <c r="I16" s="75"/>
+      <c r="D16" s="82"/>
+      <c r="E16" s="82"/>
+      <c r="F16" s="82"/>
+      <c r="G16" s="82"/>
+      <c r="H16" s="82"/>
+      <c r="I16" s="83"/>
     </row>
     <row r="17" spans="2:9" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="45"/>
-      <c r="C17" s="76"/>
-      <c r="D17" s="77"/>
-      <c r="E17" s="77"/>
-      <c r="F17" s="77"/>
-      <c r="G17" s="77"/>
-      <c r="H17" s="77"/>
-      <c r="I17" s="78"/>
+      <c r="B17" s="44"/>
+      <c r="C17" s="84"/>
+      <c r="D17" s="85"/>
+      <c r="E17" s="85"/>
+      <c r="F17" s="85"/>
+      <c r="G17" s="85"/>
+      <c r="H17" s="85"/>
+      <c r="I17" s="86"/>
     </row>
     <row r="18" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="25" t="s">
+      <c r="C18" s="63" t="s">
         <v>56</v>
       </c>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
+      <c r="D18" s="64"/>
+      <c r="E18" s="64"/>
+      <c r="F18" s="64"/>
+      <c r="G18" s="64"/>
+      <c r="H18" s="64"/>
+      <c r="I18" s="64"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="28"/>
+      <c r="I19" s="28"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20"/>
-      <c r="I20" s="20"/>
+      <c r="C20" s="54"/>
+      <c r="D20" s="54"/>
+      <c r="E20" s="54"/>
+      <c r="F20" s="54"/>
+      <c r="G20" s="54"/>
+      <c r="H20" s="54"/>
+      <c r="I20" s="54"/>
     </row>
     <row r="21" spans="2:9" ht="160" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="79" t="s">
+      <c r="C21" s="87" t="s">
         <v>57</v>
       </c>
-      <c r="D21" s="80"/>
-      <c r="E21" s="80"/>
-      <c r="F21" s="80"/>
-      <c r="G21" s="80"/>
-      <c r="H21" s="80"/>
-      <c r="I21" s="81"/>
+      <c r="D21" s="88"/>
+      <c r="E21" s="88"/>
+      <c r="F21" s="88"/>
+      <c r="G21" s="88"/>
+      <c r="H21" s="88"/>
+      <c r="I21" s="89"/>
     </row>
     <row r="22" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="34">
+      <c r="C22" s="40">
         <v>3</v>
       </c>
-      <c r="D22" s="42"/>
-      <c r="E22" s="42"/>
-      <c r="F22" s="42"/>
-      <c r="G22" s="42"/>
-      <c r="H22" s="42"/>
-      <c r="I22" s="43"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="41"/>
+      <c r="F22" s="41"/>
+      <c r="G22" s="41"/>
+      <c r="H22" s="41"/>
+      <c r="I22" s="42"/>
     </row>
     <row r="23" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="56" t="s">
+      <c r="C23" s="55" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="56"/>
-      <c r="E23" s="57" t="s">
+      <c r="D23" s="55"/>
+      <c r="E23" s="56" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="57"/>
-      <c r="G23" s="57"/>
-      <c r="H23" s="57"/>
-      <c r="I23" s="57"/>
+      <c r="F23" s="56"/>
+      <c r="G23" s="56"/>
+      <c r="H23" s="56"/>
+      <c r="I23" s="56"/>
     </row>
     <row r="24" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="60">
+      <c r="B24" s="59">
         <v>1</v>
       </c>
-      <c r="C24" s="87" t="s">
+      <c r="C24" s="72" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="88"/>
+      <c r="D24" s="73"/>
       <c r="E24" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="F24" s="89" t="s">
+      <c r="F24" s="76" t="s">
         <v>63</v>
       </c>
-      <c r="G24" s="89"/>
-      <c r="H24" s="89"/>
-      <c r="I24" s="90"/>
+      <c r="G24" s="76"/>
+      <c r="H24" s="76"/>
+      <c r="I24" s="77"/>
     </row>
     <row r="25" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="61"/>
-      <c r="C25" s="85"/>
-      <c r="D25" s="86"/>
+      <c r="B25" s="60"/>
+      <c r="C25" s="74"/>
+      <c r="D25" s="75"/>
       <c r="E25" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="F25" s="70" t="s">
+      <c r="F25" s="31" t="s">
         <v>64</v>
       </c>
-      <c r="G25" s="70"/>
-      <c r="H25" s="70"/>
-      <c r="I25" s="55"/>
+      <c r="G25" s="31"/>
+      <c r="H25" s="31"/>
+      <c r="I25" s="32"/>
     </row>
     <row r="26" spans="2:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="8">
         <v>2</v>
       </c>
-      <c r="C26" s="83" t="s">
+      <c r="C26" s="79" t="s">
         <v>59</v>
       </c>
-      <c r="D26" s="84"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="69"/>
-      <c r="G26" s="69"/>
-      <c r="H26" s="69"/>
-      <c r="I26" s="33"/>
+      <c r="D26" s="80"/>
+      <c r="E26" s="23"/>
+      <c r="F26" s="29"/>
+      <c r="G26" s="29"/>
+      <c r="H26" s="29"/>
+      <c r="I26" s="24"/>
     </row>
     <row r="27" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="8">
         <v>3</v>
       </c>
-      <c r="C27" s="85" t="s">
+      <c r="C27" s="74" t="s">
         <v>60</v>
       </c>
-      <c r="D27" s="86"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="69"/>
-      <c r="G27" s="69"/>
-      <c r="H27" s="69"/>
-      <c r="I27" s="33"/>
+      <c r="D27" s="75"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="29"/>
+      <c r="G27" s="29"/>
+      <c r="H27" s="29"/>
+      <c r="I27" s="24"/>
     </row>
     <row r="28" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B28" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C28" s="30" t="s">
+      <c r="C28" s="65" t="s">
         <v>65</v>
       </c>
-      <c r="D28" s="30"/>
-      <c r="E28" s="30"/>
-      <c r="F28" s="30"/>
-      <c r="G28" s="30"/>
-      <c r="H28" s="30"/>
-      <c r="I28" s="30"/>
+      <c r="D28" s="65"/>
+      <c r="E28" s="65"/>
+      <c r="F28" s="65"/>
+      <c r="G28" s="65"/>
+      <c r="H28" s="65"/>
+      <c r="I28" s="65"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B29" s="38"/>
-      <c r="C29" s="39"/>
-      <c r="D29" s="39"/>
-      <c r="E29" s="39"/>
-      <c r="F29" s="39"/>
-      <c r="G29" s="39"/>
-      <c r="H29" s="39"/>
-      <c r="I29" s="40"/>
+      <c r="B29" s="34"/>
+      <c r="C29" s="35"/>
+      <c r="D29" s="35"/>
+      <c r="E29" s="35"/>
+      <c r="F29" s="35"/>
+      <c r="G29" s="35"/>
+      <c r="H29" s="35"/>
+      <c r="I29" s="36"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B30" s="20" t="s">
+      <c r="B30" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
-      <c r="E30" s="20"/>
-      <c r="F30" s="20"/>
-      <c r="G30" s="20"/>
-      <c r="H30" s="20"/>
-      <c r="I30" s="20"/>
+      <c r="C30" s="54"/>
+      <c r="D30" s="54"/>
+      <c r="E30" s="54"/>
+      <c r="F30" s="54"/>
+      <c r="G30" s="54"/>
+      <c r="H30" s="54"/>
+      <c r="I30" s="54"/>
     </row>
     <row r="31" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="82" t="s">
+      <c r="B31" s="78" t="s">
         <v>66</v>
       </c>
-      <c r="C31" s="24"/>
-      <c r="D31" s="24"/>
-      <c r="E31" s="24"/>
-      <c r="F31" s="24"/>
-      <c r="G31" s="24"/>
-      <c r="H31" s="24"/>
-      <c r="I31" s="24"/>
+      <c r="C31" s="62"/>
+      <c r="D31" s="62"/>
+      <c r="E31" s="62"/>
+      <c r="F31" s="62"/>
+      <c r="G31" s="62"/>
+      <c r="H31" s="62"/>
+      <c r="I31" s="62"/>
     </row>
     <row r="32" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="24"/>
-      <c r="C32" s="24"/>
-      <c r="D32" s="24"/>
-      <c r="E32" s="24"/>
-      <c r="F32" s="24"/>
-      <c r="G32" s="24"/>
-      <c r="H32" s="24"/>
-      <c r="I32" s="24"/>
+      <c r="B32" s="62"/>
+      <c r="C32" s="62"/>
+      <c r="D32" s="62"/>
+      <c r="E32" s="62"/>
+      <c r="F32" s="62"/>
+      <c r="G32" s="62"/>
+      <c r="H32" s="62"/>
+      <c r="I32" s="62"/>
     </row>
     <row r="33" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="24"/>
-      <c r="C33" s="24"/>
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="24"/>
-      <c r="G33" s="24"/>
-      <c r="H33" s="24"/>
-      <c r="I33" s="24"/>
+      <c r="B33" s="62"/>
+      <c r="C33" s="62"/>
+      <c r="D33" s="62"/>
+      <c r="E33" s="62"/>
+      <c r="F33" s="62"/>
+      <c r="G33" s="62"/>
+      <c r="H33" s="62"/>
+      <c r="I33" s="62"/>
     </row>
     <row r="34" spans="2:9" ht="254" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="24"/>
-      <c r="C34" s="24"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="24"/>
-      <c r="F34" s="24"/>
-      <c r="G34" s="24"/>
-      <c r="H34" s="24"/>
-      <c r="I34" s="24"/>
+      <c r="B34" s="62"/>
+      <c r="C34" s="62"/>
+      <c r="D34" s="62"/>
+      <c r="E34" s="62"/>
+      <c r="F34" s="62"/>
+      <c r="G34" s="62"/>
+      <c r="H34" s="62"/>
+      <c r="I34" s="62"/>
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:D25"/>
-    <mergeCell ref="F24:I24"/>
-    <mergeCell ref="F25:I25"/>
-    <mergeCell ref="C28:I28"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="B31:I34"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:I27"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="C21:I21"/>
     <mergeCell ref="C15:I15"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -4526,6 +4532,27 @@
     <mergeCell ref="B10:I12"/>
     <mergeCell ref="B13:I13"/>
     <mergeCell ref="B14:I14"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="B31:I34"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:D25"/>
+    <mergeCell ref="F24:I24"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="C28:I28"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{4DBC988E-4FF2-2C49-AA18-DD92CA6A87E8}"/>
@@ -4552,426 +4579,411 @@
   <cols>
     <col min="2" max="2" width="23.33203125" style="1" customWidth="1"/>
     <col min="3" max="3" width="14.5" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1640625" style="1" customWidth="1"/>
     <col min="8" max="8" width="18.33203125" customWidth="1"/>
     <col min="9" max="9" width="49.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="71" t="s">
+      <c r="C3" s="90" t="s">
         <v>67</v>
       </c>
-      <c r="D3" s="72"/>
-      <c r="E3" s="72"/>
-      <c r="F3" s="72"/>
-      <c r="G3" s="72"/>
-      <c r="H3" s="72"/>
-      <c r="I3" s="72"/>
+      <c r="D3" s="91"/>
+      <c r="E3" s="91"/>
+      <c r="F3" s="91"/>
+      <c r="G3" s="91"/>
+      <c r="H3" s="91"/>
+      <c r="I3" s="91"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="64" t="s">
         <v>68</v>
       </c>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
+      <c r="D4" s="64"/>
+      <c r="E4" s="64"/>
+      <c r="F4" s="64"/>
+      <c r="G4" s="64"/>
+      <c r="H4" s="64"/>
+      <c r="I4" s="64"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="64">
         <v>2022</v>
       </c>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="64"/>
     </row>
     <row r="6" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="31" t="s">
+      <c r="C6" s="66" t="s">
         <v>69</v>
       </c>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="31"/>
-      <c r="H6" s="31"/>
-      <c r="I6" s="31"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
+      <c r="G6" s="66"/>
+      <c r="H6" s="66"/>
+      <c r="I6" s="66"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="69" t="s">
         <v>70</v>
       </c>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
+      <c r="D7" s="64"/>
+      <c r="E7" s="64"/>
+      <c r="F7" s="64"/>
+      <c r="G7" s="64"/>
+      <c r="H7" s="64"/>
+      <c r="I7" s="64"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="28"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="20"/>
+      <c r="C9" s="54"/>
+      <c r="D9" s="54"/>
+      <c r="E9" s="54"/>
+      <c r="F9" s="54"/>
+      <c r="G9" s="54"/>
+      <c r="H9" s="54"/>
+      <c r="I9" s="54"/>
     </row>
     <row r="10" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="61" t="s">
         <v>71</v>
       </c>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
+      <c r="C10" s="61"/>
+      <c r="D10" s="61"/>
+      <c r="E10" s="61"/>
+      <c r="F10" s="61"/>
+      <c r="G10" s="61"/>
+      <c r="H10" s="61"/>
+      <c r="I10" s="61"/>
     </row>
     <row r="11" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="23"/>
+      <c r="B11" s="61"/>
+      <c r="C11" s="61"/>
+      <c r="D11" s="61"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="61"/>
+      <c r="I11" s="61"/>
     </row>
     <row r="12" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
-      <c r="H12" s="23"/>
-      <c r="I12" s="23"/>
+      <c r="B12" s="61"/>
+      <c r="C12" s="61"/>
+      <c r="D12" s="61"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
+      <c r="G12" s="61"/>
+      <c r="H12" s="61"/>
+      <c r="I12" s="61"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="26"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="28"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="54" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="20"/>
+      <c r="C14" s="54"/>
+      <c r="D14" s="54"/>
+      <c r="E14" s="54"/>
+      <c r="F14" s="54"/>
+      <c r="G14" s="54"/>
+      <c r="H14" s="54"/>
+      <c r="I14" s="54"/>
     </row>
     <row r="15" spans="2:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="63" t="s">
         <v>73</v>
       </c>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="19"/>
+      <c r="D15" s="64"/>
+      <c r="E15" s="64"/>
+      <c r="F15" s="64"/>
+      <c r="G15" s="64"/>
+      <c r="H15" s="64"/>
+      <c r="I15" s="64"/>
     </row>
     <row r="16" spans="2:9" ht="247" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="44" t="s">
+      <c r="B16" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="73" t="s">
+      <c r="C16" s="81" t="s">
         <v>72</v>
       </c>
-      <c r="D16" s="74"/>
-      <c r="E16" s="74"/>
-      <c r="F16" s="74"/>
-      <c r="G16" s="74"/>
-      <c r="H16" s="74"/>
-      <c r="I16" s="75"/>
+      <c r="D16" s="82"/>
+      <c r="E16" s="82"/>
+      <c r="F16" s="82"/>
+      <c r="G16" s="82"/>
+      <c r="H16" s="82"/>
+      <c r="I16" s="83"/>
     </row>
     <row r="17" spans="2:9" ht="247" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="45"/>
-      <c r="C17" s="76"/>
-      <c r="D17" s="77"/>
-      <c r="E17" s="77"/>
-      <c r="F17" s="77"/>
-      <c r="G17" s="77"/>
-      <c r="H17" s="77"/>
-      <c r="I17" s="78"/>
+      <c r="B17" s="44"/>
+      <c r="C17" s="84"/>
+      <c r="D17" s="85"/>
+      <c r="E17" s="85"/>
+      <c r="F17" s="85"/>
+      <c r="G17" s="85"/>
+      <c r="H17" s="85"/>
+      <c r="I17" s="86"/>
     </row>
     <row r="18" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="91"/>
-      <c r="D18" s="92"/>
-      <c r="E18" s="92"/>
-      <c r="F18" s="92"/>
-      <c r="G18" s="92"/>
-      <c r="H18" s="92"/>
-      <c r="I18" s="92"/>
+      <c r="C18" s="95"/>
+      <c r="D18" s="96"/>
+      <c r="E18" s="96"/>
+      <c r="F18" s="96"/>
+      <c r="G18" s="96"/>
+      <c r="H18" s="96"/>
+      <c r="I18" s="96"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="28"/>
+      <c r="I19" s="28"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20"/>
-      <c r="I20" s="20"/>
+      <c r="B20" s="54" t="s">
+        <v>77</v>
+      </c>
+      <c r="C20" s="54"/>
+      <c r="D20" s="54"/>
+      <c r="E20" s="54"/>
+      <c r="F20" s="54"/>
+      <c r="G20" s="54"/>
+      <c r="H20" s="54"/>
+      <c r="I20" s="54"/>
     </row>
     <row r="21" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="79" t="s">
+      <c r="C21" s="87" t="s">
         <v>74</v>
       </c>
-      <c r="D21" s="80"/>
-      <c r="E21" s="80"/>
-      <c r="F21" s="80"/>
-      <c r="G21" s="80"/>
-      <c r="H21" s="80"/>
-      <c r="I21" s="81"/>
-    </row>
-    <row r="22" spans="2:9" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D21" s="88"/>
+      <c r="E21" s="88"/>
+      <c r="F21" s="88"/>
+      <c r="G21" s="88"/>
+      <c r="H21" s="88"/>
+      <c r="I21" s="89"/>
+    </row>
+    <row r="22" spans="2:9" ht="165" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="34" t="s">
-        <v>79</v>
-      </c>
-      <c r="D22" s="42"/>
-      <c r="E22" s="42"/>
-      <c r="F22" s="42"/>
-      <c r="G22" s="42"/>
-      <c r="H22" s="42"/>
-      <c r="I22" s="43"/>
+      <c r="C22" s="40" t="s">
+        <v>174</v>
+      </c>
+      <c r="D22" s="41"/>
+      <c r="E22" s="41"/>
+      <c r="F22" s="41"/>
+      <c r="G22" s="41"/>
+      <c r="H22" s="41"/>
+      <c r="I22" s="42"/>
     </row>
     <row r="23" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="56" t="s">
+      <c r="C23" s="55" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="56"/>
-      <c r="E23" s="57" t="s">
+      <c r="D23" s="55"/>
+      <c r="E23" s="56" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="57"/>
-      <c r="G23" s="57"/>
-      <c r="H23" s="57"/>
-      <c r="I23" s="57"/>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="F23" s="56"/>
+      <c r="G23" s="56"/>
+      <c r="H23" s="56"/>
+      <c r="I23" s="56"/>
+    </row>
+    <row r="24" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="95" t="s">
+      <c r="C24" s="94" t="s">
         <v>75</v>
       </c>
-      <c r="D24" s="95"/>
-      <c r="E24" s="56" t="s">
-        <v>80</v>
-      </c>
-      <c r="F24" s="56"/>
-      <c r="G24" s="56"/>
-      <c r="H24" s="56"/>
-      <c r="I24" s="56"/>
-    </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="D24" s="94"/>
+      <c r="E24" s="105" t="s">
+        <v>177</v>
+      </c>
+      <c r="F24" s="105"/>
+      <c r="G24" s="105"/>
+      <c r="H24" s="105"/>
+      <c r="I24" s="105"/>
+    </row>
+    <row r="25" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="8">
         <v>2</v>
       </c>
-      <c r="C25" s="95" t="s">
-        <v>76</v>
-      </c>
-      <c r="D25" s="95"/>
-      <c r="E25" s="56"/>
-      <c r="F25" s="56"/>
-      <c r="G25" s="56"/>
-      <c r="H25" s="56"/>
-      <c r="I25" s="56"/>
-    </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="C25" s="94" t="s">
+        <v>172</v>
+      </c>
+      <c r="D25" s="94"/>
+      <c r="E25" s="90" t="s">
+        <v>175</v>
+      </c>
+      <c r="F25" s="90"/>
+      <c r="G25" s="90"/>
+      <c r="H25" s="90"/>
+      <c r="I25" s="90"/>
+    </row>
+    <row r="26" spans="2:9" ht="71" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="8">
         <v>3</v>
       </c>
-      <c r="C26" s="83" t="s">
-        <v>77</v>
-      </c>
-      <c r="D26" s="84"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="69"/>
-      <c r="G26" s="69"/>
-      <c r="H26" s="69"/>
-      <c r="I26" s="33"/>
+      <c r="C26" s="98" t="s">
+        <v>173</v>
+      </c>
+      <c r="D26" s="99"/>
+      <c r="E26" s="37" t="s">
+        <v>176</v>
+      </c>
+      <c r="F26" s="76"/>
+      <c r="G26" s="76"/>
+      <c r="H26" s="76"/>
+      <c r="I26" s="77"/>
     </row>
     <row r="27" spans="2:9" ht="68" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="30" t="s">
-        <v>78</v>
-      </c>
-      <c r="D27" s="30"/>
-      <c r="E27" s="30"/>
-      <c r="F27" s="30"/>
-      <c r="G27" s="30"/>
-      <c r="H27" s="30"/>
-      <c r="I27" s="30"/>
+      <c r="C27" s="65" t="s">
+        <v>76</v>
+      </c>
+      <c r="D27" s="65"/>
+      <c r="E27" s="65"/>
+      <c r="F27" s="65"/>
+      <c r="G27" s="65"/>
+      <c r="H27" s="65"/>
+      <c r="I27" s="65"/>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B28" s="38"/>
-      <c r="C28" s="39"/>
-      <c r="D28" s="39"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="39"/>
-      <c r="G28" s="39"/>
-      <c r="H28" s="39"/>
-      <c r="I28" s="40"/>
+      <c r="B28" s="34"/>
+      <c r="C28" s="35"/>
+      <c r="D28" s="35"/>
+      <c r="E28" s="35"/>
+      <c r="F28" s="35"/>
+      <c r="G28" s="35"/>
+      <c r="H28" s="35"/>
+      <c r="I28" s="36"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B29" s="20" t="s">
+      <c r="B29" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="C29" s="20"/>
-      <c r="D29" s="20"/>
-      <c r="E29" s="20"/>
-      <c r="F29" s="20"/>
-      <c r="G29" s="20"/>
-      <c r="H29" s="20"/>
-      <c r="I29" s="20"/>
+      <c r="C29" s="54"/>
+      <c r="D29" s="54"/>
+      <c r="E29" s="54"/>
+      <c r="F29" s="54"/>
+      <c r="G29" s="54"/>
+      <c r="H29" s="54"/>
+      <c r="I29" s="54"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B30" s="93"/>
-      <c r="C30" s="94"/>
-      <c r="D30" s="94"/>
-      <c r="E30" s="94"/>
-      <c r="F30" s="94"/>
-      <c r="G30" s="94"/>
-      <c r="H30" s="94"/>
-      <c r="I30" s="94"/>
+      <c r="B30" s="92"/>
+      <c r="C30" s="93"/>
+      <c r="D30" s="93"/>
+      <c r="E30" s="93"/>
+      <c r="F30" s="93"/>
+      <c r="G30" s="93"/>
+      <c r="H30" s="93"/>
+      <c r="I30" s="93"/>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B31" s="94"/>
-      <c r="C31" s="94"/>
-      <c r="D31" s="94"/>
-      <c r="E31" s="94"/>
-      <c r="F31" s="94"/>
-      <c r="G31" s="94"/>
-      <c r="H31" s="94"/>
-      <c r="I31" s="94"/>
+      <c r="B31" s="93"/>
+      <c r="C31" s="93"/>
+      <c r="D31" s="93"/>
+      <c r="E31" s="93"/>
+      <c r="F31" s="93"/>
+      <c r="G31" s="93"/>
+      <c r="H31" s="93"/>
+      <c r="I31" s="93"/>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B32" s="94"/>
-      <c r="C32" s="94"/>
-      <c r="D32" s="94"/>
-      <c r="E32" s="94"/>
-      <c r="F32" s="94"/>
-      <c r="G32" s="94"/>
-      <c r="H32" s="94"/>
-      <c r="I32" s="94"/>
+      <c r="B32" s="93"/>
+      <c r="C32" s="93"/>
+      <c r="D32" s="93"/>
+      <c r="E32" s="93"/>
+      <c r="F32" s="93"/>
+      <c r="G32" s="93"/>
+      <c r="H32" s="93"/>
+      <c r="I32" s="93"/>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B33" s="94"/>
-      <c r="C33" s="94"/>
-      <c r="D33" s="94"/>
-      <c r="E33" s="94"/>
-      <c r="F33" s="94"/>
-      <c r="G33" s="94"/>
-      <c r="H33" s="94"/>
-      <c r="I33" s="94"/>
+      <c r="B33" s="93"/>
+      <c r="C33" s="93"/>
+      <c r="D33" s="93"/>
+      <c r="E33" s="93"/>
+      <c r="F33" s="93"/>
+      <c r="G33" s="93"/>
+      <c r="H33" s="93"/>
+      <c r="I33" s="93"/>
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:I33"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="C27:I27"/>
-    <mergeCell ref="B28:I28"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="C21:I21"/>
     <mergeCell ref="C15:I15"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -4984,6 +4996,25 @@
     <mergeCell ref="B10:I12"/>
     <mergeCell ref="B13:I13"/>
     <mergeCell ref="B14:I14"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:I33"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="C27:I27"/>
+    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:I26"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{60ABBC95-3763-1140-8147-BC4DA0DFC780}"/>
@@ -5005,79 +5036,79 @@
   <sheetData>
     <row r="4" spans="3:5" x14ac:dyDescent="0.2">
       <c r="C4" s="11" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="3:5" ht="17" x14ac:dyDescent="0.2">
       <c r="C5" s="11" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6" spans="3:5" x14ac:dyDescent="0.2">
       <c r="C6" s="11" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7" spans="3:5" x14ac:dyDescent="0.2">
       <c r="C7" s="11" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" spans="3:5" x14ac:dyDescent="0.2">
       <c r="C8" s="11" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="9" spans="3:5" x14ac:dyDescent="0.2">
       <c r="C9" s="11" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10" spans="3:5" x14ac:dyDescent="0.2">
       <c r="C10" s="12" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" spans="3:5" x14ac:dyDescent="0.2">
@@ -5135,526 +5166,510 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{625A714D-2F1D-8548-AF4D-43E8CCED86F0}">
-  <dimension ref="B2:I38"/>
+  <dimension ref="B1:I38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="18.33203125" customWidth="1"/>
-    <col min="9" max="9" width="49.5" customWidth="1"/>
+    <col min="3" max="4" width="15.1640625" style="1" customWidth="1"/>
+    <col min="5" max="9" width="15.1640625" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B1" s="104"/>
+      <c r="C1" s="104"/>
+      <c r="D1" s="104"/>
+      <c r="E1" s="104"/>
+      <c r="F1" s="104"/>
+      <c r="G1" s="104"/>
+      <c r="H1" s="104"/>
+      <c r="I1" s="104"/>
+    </row>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="71" t="s">
-        <v>82</v>
-      </c>
-      <c r="D3" s="72"/>
-      <c r="E3" s="72"/>
-      <c r="F3" s="72"/>
-      <c r="G3" s="72"/>
-      <c r="H3" s="72"/>
-      <c r="I3" s="72"/>
+      <c r="C3" s="90" t="s">
+        <v>78</v>
+      </c>
+      <c r="D3" s="91"/>
+      <c r="E3" s="91"/>
+      <c r="F3" s="91"/>
+      <c r="G3" s="91"/>
+      <c r="H3" s="91"/>
+      <c r="I3" s="91"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
+      <c r="C4" s="64" t="s">
+        <v>79</v>
+      </c>
+      <c r="D4" s="64"/>
+      <c r="E4" s="64"/>
+      <c r="F4" s="64"/>
+      <c r="G4" s="64"/>
+      <c r="H4" s="64"/>
+      <c r="I4" s="64"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="64">
         <v>2025</v>
       </c>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="64"/>
     </row>
     <row r="6" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="31" t="s">
-        <v>85</v>
-      </c>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="31"/>
-      <c r="H6" s="31"/>
-      <c r="I6" s="31"/>
+      <c r="C6" s="66" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
+      <c r="G6" s="66"/>
+      <c r="H6" s="66"/>
+      <c r="I6" s="66"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
+      <c r="C7" s="69" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="64"/>
+      <c r="E7" s="64"/>
+      <c r="F7" s="64"/>
+      <c r="G7" s="64"/>
+      <c r="H7" s="64"/>
+      <c r="I7" s="64"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="28"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="20"/>
+      <c r="C9" s="54"/>
+      <c r="D9" s="54"/>
+      <c r="E9" s="54"/>
+      <c r="F9" s="54"/>
+      <c r="G9" s="54"/>
+      <c r="H9" s="54"/>
+      <c r="I9" s="54"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B10" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
+      <c r="B10" s="61" t="s">
+        <v>82</v>
+      </c>
+      <c r="C10" s="61"/>
+      <c r="D10" s="61"/>
+      <c r="E10" s="61"/>
+      <c r="F10" s="61"/>
+      <c r="G10" s="61"/>
+      <c r="H10" s="61"/>
+      <c r="I10" s="61"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="23"/>
+      <c r="B11" s="61"/>
+      <c r="C11" s="61"/>
+      <c r="D11" s="61"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="61"/>
+      <c r="I11" s="61"/>
     </row>
     <row r="12" spans="2:9" ht="92" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
-      <c r="H12" s="23"/>
-      <c r="I12" s="23"/>
+      <c r="B12" s="61"/>
+      <c r="C12" s="61"/>
+      <c r="D12" s="61"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
+      <c r="G12" s="61"/>
+      <c r="H12" s="61"/>
+      <c r="I12" s="61"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="26"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="28"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="54" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="20"/>
-    </row>
-    <row r="15" spans="2:9" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C14" s="54"/>
+      <c r="D14" s="54"/>
+      <c r="E14" s="54"/>
+      <c r="F14" s="54"/>
+      <c r="G14" s="54"/>
+      <c r="H14" s="54"/>
+      <c r="I14" s="54"/>
+    </row>
+    <row r="15" spans="2:9" ht="59" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="D15" s="31"/>
-      <c r="E15" s="31"/>
-      <c r="F15" s="31"/>
-      <c r="G15" s="31"/>
-      <c r="H15" s="31"/>
-      <c r="I15" s="31"/>
+      <c r="C15" s="65" t="s">
+        <v>83</v>
+      </c>
+      <c r="D15" s="66"/>
+      <c r="E15" s="66"/>
+      <c r="F15" s="66"/>
+      <c r="G15" s="66"/>
+      <c r="H15" s="66"/>
+      <c r="I15" s="66"/>
     </row>
     <row r="16" spans="2:9" ht="59" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="44" t="s">
+      <c r="B16" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="73" t="s">
-        <v>88</v>
-      </c>
-      <c r="D16" s="74"/>
-      <c r="E16" s="74"/>
-      <c r="F16" s="74"/>
-      <c r="G16" s="74"/>
-      <c r="H16" s="74"/>
-      <c r="I16" s="75"/>
-    </row>
-    <row r="17" spans="2:9" ht="92" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="45"/>
-      <c r="C17" s="76"/>
-      <c r="D17" s="77"/>
-      <c r="E17" s="77"/>
-      <c r="F17" s="77"/>
-      <c r="G17" s="77"/>
-      <c r="H17" s="77"/>
-      <c r="I17" s="78"/>
-    </row>
-    <row r="18" spans="2:9" ht="256" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C16" s="81" t="s">
+        <v>84</v>
+      </c>
+      <c r="D16" s="82"/>
+      <c r="E16" s="82"/>
+      <c r="F16" s="82"/>
+      <c r="G16" s="82"/>
+      <c r="H16" s="82"/>
+      <c r="I16" s="83"/>
+    </row>
+    <row r="17" spans="2:9" ht="113" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="44"/>
+      <c r="C17" s="84"/>
+      <c r="D17" s="85"/>
+      <c r="E17" s="85"/>
+      <c r="F17" s="85"/>
+      <c r="G17" s="85"/>
+      <c r="H17" s="85"/>
+      <c r="I17" s="86"/>
+    </row>
+    <row r="18" spans="2:9" ht="358" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="71" t="s">
-        <v>89</v>
-      </c>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
+      <c r="C18" s="61" t="s">
+        <v>85</v>
+      </c>
+      <c r="D18" s="66"/>
+      <c r="E18" s="66"/>
+      <c r="F18" s="66"/>
+      <c r="G18" s="66"/>
+      <c r="H18" s="66"/>
+      <c r="I18" s="66"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="28"/>
+      <c r="I19" s="28"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20"/>
-      <c r="I20" s="20"/>
-    </row>
-    <row r="21" spans="2:9" ht="246" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="54" t="s">
+        <v>77</v>
+      </c>
+      <c r="C20" s="54"/>
+      <c r="D20" s="54"/>
+      <c r="E20" s="54"/>
+      <c r="F20" s="54"/>
+      <c r="G20" s="54"/>
+      <c r="H20" s="54"/>
+      <c r="I20" s="54"/>
+    </row>
+    <row r="21" spans="2:9" ht="332" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="79" t="s">
-        <v>90</v>
-      </c>
-      <c r="D21" s="80"/>
-      <c r="E21" s="80"/>
-      <c r="F21" s="80"/>
-      <c r="G21" s="80"/>
-      <c r="H21" s="80"/>
-      <c r="I21" s="81"/>
+      <c r="C21" s="87" t="s">
+        <v>86</v>
+      </c>
+      <c r="D21" s="88"/>
+      <c r="E21" s="88"/>
+      <c r="F21" s="88"/>
+      <c r="G21" s="88"/>
+      <c r="H21" s="88"/>
+      <c r="I21" s="89"/>
     </row>
     <row r="22" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="34">
+      <c r="C22" s="40">
         <v>8</v>
       </c>
-      <c r="D22" s="42"/>
-      <c r="E22" s="42"/>
-      <c r="F22" s="42"/>
-      <c r="G22" s="42"/>
-      <c r="H22" s="42"/>
-      <c r="I22" s="43"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="41"/>
+      <c r="F22" s="41"/>
+      <c r="G22" s="41"/>
+      <c r="H22" s="41"/>
+      <c r="I22" s="42"/>
     </row>
     <row r="23" spans="2:9" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="56" t="s">
+      <c r="C23" s="55" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="56"/>
-      <c r="E23" s="57" t="s">
-        <v>101</v>
-      </c>
-      <c r="F23" s="57"/>
-      <c r="G23" s="57"/>
-      <c r="H23" s="57"/>
-      <c r="I23" s="57"/>
-    </row>
-    <row r="24" spans="2:9" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D23" s="55"/>
+      <c r="E23" s="56" t="s">
+        <v>97</v>
+      </c>
+      <c r="F23" s="56"/>
+      <c r="G23" s="56"/>
+      <c r="H23" s="56"/>
+      <c r="I23" s="56"/>
+    </row>
+    <row r="24" spans="2:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="96" t="s">
-        <v>92</v>
-      </c>
-      <c r="D24" s="97"/>
-      <c r="E24" s="71" t="s">
-        <v>107</v>
-      </c>
-      <c r="F24" s="71"/>
-      <c r="G24" s="71"/>
-      <c r="H24" s="71"/>
-      <c r="I24" s="71"/>
+      <c r="C24" s="100" t="s">
+        <v>88</v>
+      </c>
+      <c r="D24" s="101"/>
+      <c r="E24" s="90" t="s">
+        <v>171</v>
+      </c>
+      <c r="F24" s="90"/>
+      <c r="G24" s="90"/>
+      <c r="H24" s="90"/>
+      <c r="I24" s="90"/>
     </row>
     <row r="25" spans="2:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="8">
         <v>2</v>
       </c>
       <c r="C25" s="98" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="D25" s="99"/>
-      <c r="E25" s="71" t="s">
-        <v>108</v>
-      </c>
-      <c r="F25" s="71"/>
-      <c r="G25" s="71"/>
-      <c r="H25" s="71"/>
-      <c r="I25" s="71"/>
+      <c r="E25" s="90" t="s">
+        <v>103</v>
+      </c>
+      <c r="F25" s="90"/>
+      <c r="G25" s="90"/>
+      <c r="H25" s="90"/>
+      <c r="I25" s="90"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B26" s="8">
         <v>3</v>
       </c>
       <c r="C26" s="98" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D26" s="99"/>
-      <c r="E26" s="71" t="s">
-        <v>106</v>
-      </c>
-      <c r="F26" s="71"/>
-      <c r="G26" s="71"/>
-      <c r="H26" s="71"/>
-      <c r="I26" s="71"/>
+      <c r="E26" s="90" t="s">
+        <v>102</v>
+      </c>
+      <c r="F26" s="90"/>
+      <c r="G26" s="90"/>
+      <c r="H26" s="90"/>
+      <c r="I26" s="90"/>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B27" s="8">
         <v>4</v>
       </c>
       <c r="C27" s="98" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="D27" s="99"/>
-      <c r="E27" s="71" t="s">
-        <v>105</v>
-      </c>
-      <c r="F27" s="71"/>
-      <c r="G27" s="71"/>
-      <c r="H27" s="71"/>
-      <c r="I27" s="71"/>
+      <c r="E27" s="90" t="s">
+        <v>101</v>
+      </c>
+      <c r="F27" s="90"/>
+      <c r="G27" s="90"/>
+      <c r="H27" s="90"/>
+      <c r="I27" s="90"/>
     </row>
     <row r="28" spans="2:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="8">
         <v>5</v>
       </c>
       <c r="C28" s="98" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D28" s="99"/>
-      <c r="E28" s="71" t="s">
-        <v>104</v>
-      </c>
-      <c r="F28" s="71"/>
-      <c r="G28" s="71"/>
-      <c r="H28" s="71"/>
-      <c r="I28" s="71"/>
+      <c r="E28" s="90" t="s">
+        <v>100</v>
+      </c>
+      <c r="F28" s="90"/>
+      <c r="G28" s="90"/>
+      <c r="H28" s="90"/>
+      <c r="I28" s="90"/>
     </row>
     <row r="29" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="8">
         <v>6</v>
       </c>
-      <c r="C29" s="95" t="s">
-        <v>97</v>
-      </c>
-      <c r="D29" s="95"/>
-      <c r="E29" s="71" t="s">
-        <v>103</v>
-      </c>
-      <c r="F29" s="71"/>
-      <c r="G29" s="71"/>
-      <c r="H29" s="71"/>
-      <c r="I29" s="71"/>
+      <c r="C29" s="94" t="s">
+        <v>93</v>
+      </c>
+      <c r="D29" s="94"/>
+      <c r="E29" s="90" t="s">
+        <v>99</v>
+      </c>
+      <c r="F29" s="90"/>
+      <c r="G29" s="90"/>
+      <c r="H29" s="90"/>
+      <c r="I29" s="90"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B30" s="8">
         <v>7</v>
       </c>
-      <c r="C30" s="95" t="s">
+      <c r="C30" s="94" t="s">
+        <v>94</v>
+      </c>
+      <c r="D30" s="94"/>
+      <c r="E30" s="90" t="s">
         <v>98</v>
       </c>
-      <c r="D30" s="95"/>
-      <c r="E30" s="71" t="s">
-        <v>102</v>
-      </c>
-      <c r="F30" s="100"/>
-      <c r="G30" s="100"/>
-      <c r="H30" s="100"/>
-      <c r="I30" s="100"/>
+      <c r="F30" s="97"/>
+      <c r="G30" s="97"/>
+      <c r="H30" s="97"/>
+      <c r="I30" s="97"/>
     </row>
     <row r="31" spans="2:9" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="8">
         <v>8</v>
       </c>
       <c r="C31" s="98" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D31" s="99"/>
-      <c r="E31" s="34" t="s">
-        <v>100</v>
-      </c>
-      <c r="F31" s="35"/>
-      <c r="G31" s="35"/>
-      <c r="H31" s="35"/>
-      <c r="I31" s="36"/>
+      <c r="E31" s="40" t="s">
+        <v>96</v>
+      </c>
+      <c r="F31" s="67"/>
+      <c r="G31" s="67"/>
+      <c r="H31" s="67"/>
+      <c r="I31" s="68"/>
     </row>
     <row r="32" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B32" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C32" s="30" t="s">
-        <v>91</v>
-      </c>
-      <c r="D32" s="30"/>
-      <c r="E32" s="30"/>
-      <c r="F32" s="30"/>
-      <c r="G32" s="30"/>
-      <c r="H32" s="30"/>
-      <c r="I32" s="30"/>
+      <c r="C32" s="65" t="s">
+        <v>87</v>
+      </c>
+      <c r="D32" s="65"/>
+      <c r="E32" s="65"/>
+      <c r="F32" s="65"/>
+      <c r="G32" s="65"/>
+      <c r="H32" s="65"/>
+      <c r="I32" s="65"/>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B33" s="38"/>
-      <c r="C33" s="39"/>
-      <c r="D33" s="39"/>
-      <c r="E33" s="39"/>
-      <c r="F33" s="39"/>
-      <c r="G33" s="39"/>
-      <c r="H33" s="39"/>
-      <c r="I33" s="40"/>
+      <c r="B33" s="34"/>
+      <c r="C33" s="35"/>
+      <c r="D33" s="35"/>
+      <c r="E33" s="35"/>
+      <c r="F33" s="35"/>
+      <c r="G33" s="35"/>
+      <c r="H33" s="35"/>
+      <c r="I33" s="36"/>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B34" s="20" t="s">
+      <c r="B34" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="C34" s="20"/>
-      <c r="D34" s="20"/>
-      <c r="E34" s="20"/>
-      <c r="F34" s="20"/>
-      <c r="G34" s="20"/>
-      <c r="H34" s="20"/>
-      <c r="I34" s="20"/>
+      <c r="C34" s="54"/>
+      <c r="D34" s="54"/>
+      <c r="E34" s="54"/>
+      <c r="F34" s="54"/>
+      <c r="G34" s="54"/>
+      <c r="H34" s="54"/>
+      <c r="I34" s="54"/>
     </row>
     <row r="35" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="82" t="s">
-        <v>109</v>
-      </c>
-      <c r="C35" s="24"/>
-      <c r="D35" s="24"/>
-      <c r="E35" s="24"/>
-      <c r="F35" s="24"/>
-      <c r="G35" s="24"/>
-      <c r="H35" s="24"/>
-      <c r="I35" s="24"/>
+      <c r="B35" s="78" t="s">
+        <v>104</v>
+      </c>
+      <c r="C35" s="62"/>
+      <c r="D35" s="62"/>
+      <c r="E35" s="62"/>
+      <c r="F35" s="62"/>
+      <c r="G35" s="62"/>
+      <c r="H35" s="62"/>
+      <c r="I35" s="62"/>
     </row>
     <row r="36" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="24"/>
-      <c r="C36" s="24"/>
-      <c r="D36" s="24"/>
-      <c r="E36" s="24"/>
-      <c r="F36" s="24"/>
-      <c r="G36" s="24"/>
-      <c r="H36" s="24"/>
-      <c r="I36" s="24"/>
+      <c r="B36" s="62"/>
+      <c r="C36" s="62"/>
+      <c r="D36" s="62"/>
+      <c r="E36" s="62"/>
+      <c r="F36" s="62"/>
+      <c r="G36" s="62"/>
+      <c r="H36" s="62"/>
+      <c r="I36" s="62"/>
     </row>
     <row r="37" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="24"/>
-      <c r="C37" s="24"/>
-      <c r="D37" s="24"/>
-      <c r="E37" s="24"/>
-      <c r="F37" s="24"/>
-      <c r="G37" s="24"/>
-      <c r="H37" s="24"/>
-      <c r="I37" s="24"/>
+      <c r="B37" s="62"/>
+      <c r="C37" s="62"/>
+      <c r="D37" s="62"/>
+      <c r="E37" s="62"/>
+      <c r="F37" s="62"/>
+      <c r="G37" s="62"/>
+      <c r="H37" s="62"/>
+      <c r="I37" s="62"/>
     </row>
     <row r="38" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="24"/>
-      <c r="C38" s="24"/>
-      <c r="D38" s="24"/>
-      <c r="E38" s="24"/>
-      <c r="F38" s="24"/>
-      <c r="G38" s="24"/>
-      <c r="H38" s="24"/>
-      <c r="I38" s="24"/>
+      <c r="B38" s="62"/>
+      <c r="C38" s="62"/>
+      <c r="D38" s="62"/>
+      <c r="E38" s="62"/>
+      <c r="F38" s="62"/>
+      <c r="G38" s="62"/>
+      <c r="H38" s="62"/>
+      <c r="I38" s="62"/>
     </row>
   </sheetData>
-  <mergeCells count="41">
-    <mergeCell ref="B35:I38"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="E29:I29"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:I30"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E28:I28"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:I31"/>
-    <mergeCell ref="C32:I32"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="B34:I34"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="C3:I3"/>
-    <mergeCell ref="C4:I4"/>
-    <mergeCell ref="C5:I5"/>
-    <mergeCell ref="C6:I6"/>
+  <mergeCells count="42">
+    <mergeCell ref="B1:I1"/>
     <mergeCell ref="C7:I7"/>
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="C25:D25"/>
@@ -5671,6 +5686,31 @@
     <mergeCell ref="B13:I13"/>
     <mergeCell ref="B14:I14"/>
     <mergeCell ref="C15:I15"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="B35:I38"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="E29:I29"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:I28"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:I31"/>
+    <mergeCell ref="C32:I32"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="B34:I34"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{69FD07AD-7FCA-E141-8126-AFB63E0A1511}"/>
@@ -5692,167 +5732,167 @@
   <sheetData>
     <row r="3" spans="3:5" x14ac:dyDescent="0.2">
       <c r="C3" s="11" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="4" spans="3:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="C4" s="11" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="3:5" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C4" s="103" t="s">
+        <v>156</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="E4" s="102" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C5" s="103" t="s">
+        <v>157</v>
+      </c>
+      <c r="D5" s="102" t="s">
+        <v>167</v>
+      </c>
+      <c r="E5" s="102" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="6" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C6" s="103" t="s">
+        <v>158</v>
+      </c>
+      <c r="D6" s="102" t="s">
+        <v>167</v>
+      </c>
+      <c r="E6" s="102" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="7" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C7" s="103" t="s">
+        <v>159</v>
+      </c>
+      <c r="D7" s="102" t="s">
+        <v>167</v>
+      </c>
+      <c r="E7" s="102" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="8" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C8" s="103" t="s">
+        <v>160</v>
+      </c>
+      <c r="D8" s="102" t="s">
+        <v>167</v>
+      </c>
+      <c r="E8" s="102" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="9" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C9" s="103" t="s">
         <v>161</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D9" s="102" t="s">
+        <v>167</v>
+      </c>
+      <c r="E9" s="102" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="10" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C10" s="103" t="s">
+        <v>162</v>
+      </c>
+      <c r="D10" s="102" t="s">
+        <v>167</v>
+      </c>
+      <c r="E10" s="102" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="11" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C11" s="103" t="s">
+        <v>163</v>
+      </c>
+      <c r="D11" s="102" t="s">
+        <v>167</v>
+      </c>
+      <c r="E11" s="102" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="12" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C12" s="103" t="s">
+        <v>163</v>
+      </c>
+      <c r="D12" s="102" t="s">
+        <v>167</v>
+      </c>
+      <c r="E12" s="102" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="13" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C13" s="103" t="s">
+        <v>164</v>
+      </c>
+      <c r="D13" s="102" t="s">
+        <v>167</v>
+      </c>
+      <c r="E13" s="102" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="14" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C14" s="103" t="s">
+        <v>163</v>
+      </c>
+      <c r="D14" s="102" t="s">
+        <v>167</v>
+      </c>
+      <c r="E14" s="102" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="15" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C15" s="103" t="s">
+        <v>165</v>
+      </c>
+      <c r="D15" s="102" t="s">
+        <v>167</v>
+      </c>
+      <c r="E15" s="102" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="16" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C16" s="103" t="s">
         <v>166</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="5" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C5" s="11" t="s">
-        <v>162</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="6" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C6" s="11" t="s">
-        <v>163</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="7" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C7" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="8" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C8" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="9" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C9" s="11" t="s">
+      <c r="D16" s="102" t="s">
         <v>167</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="10" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C10" s="11" t="s">
-        <v>168</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="11" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C11" s="11" t="s">
-        <v>169</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="12" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C12" s="11" t="s">
-        <v>169</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="13" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C13" s="11" t="s">
-        <v>170</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="14" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C14" s="11" t="s">
-        <v>169</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="15" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C15" s="11" t="s">
-        <v>171</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="16" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C16" s="11" t="s">
-        <v>172</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>160</v>
+      <c r="E16" s="102" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="17" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C17" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>160</v>
+      <c r="C17" s="103" t="s">
+        <v>120</v>
+      </c>
+      <c r="D17" s="102" t="s">
+        <v>167</v>
+      </c>
+      <c r="E17" s="102" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
did the basic interface for the main code
</commit_message>
<xml_diff>
--- a/Papers/Resumen Papers.xlsx
+++ b/Papers/Resumen Papers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sophiaaristizabal/Documents/GitHub/LLMS_Project/Papers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3E2B5D5-32A3-3646-8458-7D83021BEA29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB359F70-9C83-E241-BD1C-98DABD7B1BF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="20520" windowHeight="13540" xr2:uid="{400AC57E-08F9-B346-9132-4F74AEBC2D15}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="20520" windowHeight="13540" firstSheet="3" activeTab="6" xr2:uid="{400AC57E-08F9-B346-9132-4F74AEBC2D15}"/>
   </bookViews>
   <sheets>
     <sheet name="MANAGERIAL LEADERSHIP" sheetId="1" r:id="rId1"/>
@@ -2433,6 +2433,144 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2446,12 +2584,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2460,137 +2592,59 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2598,58 +2652,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2661,38 +2673,26 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3243,523 +3243,542 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="54" t="s">
+      <c r="B2" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="70" t="s">
+      <c r="C3" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="70"/>
-      <c r="E3" s="70"/>
-      <c r="F3" s="70"/>
-      <c r="G3" s="70"/>
-      <c r="H3" s="70"/>
-      <c r="I3" s="70"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="71" t="s">
+      <c r="C4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="71"/>
-      <c r="E4" s="71"/>
-      <c r="F4" s="71"/>
-      <c r="G4" s="71"/>
-      <c r="H4" s="71"/>
-      <c r="I4" s="71"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="25"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="64">
+      <c r="C5" s="22">
         <v>2025</v>
       </c>
-      <c r="D5" s="64"/>
-      <c r="E5" s="64"/>
-      <c r="F5" s="64"/>
-      <c r="G5" s="64"/>
-      <c r="H5" s="64"/>
-      <c r="I5" s="64"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
     </row>
     <row r="6" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="64" t="s">
+      <c r="C6" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="64"/>
-      <c r="E6" s="64"/>
-      <c r="F6" s="64"/>
-      <c r="G6" s="64"/>
-      <c r="H6" s="64"/>
-      <c r="I6" s="64"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="22"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="69" t="s">
+      <c r="C7" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="64"/>
-      <c r="E7" s="64"/>
-      <c r="F7" s="64"/>
-      <c r="G7" s="64"/>
-      <c r="H7" s="64"/>
-      <c r="I7" s="64"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="22"/>
     </row>
     <row r="8" spans="2:9" ht="9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="28"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="28"/>
-      <c r="I8" s="28"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="29"/>
+      <c r="I8" s="29"/>
     </row>
     <row r="9" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="54" t="s">
+      <c r="B9" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="54"/>
-      <c r="D9" s="54"/>
-      <c r="E9" s="54"/>
-      <c r="F9" s="54"/>
-      <c r="G9" s="54"/>
-      <c r="H9" s="54"/>
-      <c r="I9" s="54"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
     </row>
     <row r="10" spans="2:9" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="61" t="s">
+      <c r="B10" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="61"/>
-      <c r="D10" s="61"/>
-      <c r="E10" s="61"/>
-      <c r="F10" s="61"/>
-      <c r="G10" s="61"/>
-      <c r="H10" s="61"/>
-      <c r="I10" s="61"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="26"/>
     </row>
     <row r="11" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="61"/>
-      <c r="C11" s="61"/>
-      <c r="D11" s="61"/>
-      <c r="E11" s="61"/>
-      <c r="F11" s="61"/>
-      <c r="G11" s="61"/>
-      <c r="H11" s="61"/>
-      <c r="I11" s="61"/>
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="26"/>
     </row>
     <row r="12" spans="2:9" ht="11" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="61"/>
-      <c r="C12" s="61"/>
-      <c r="D12" s="61"/>
-      <c r="E12" s="61"/>
-      <c r="F12" s="61"/>
-      <c r="G12" s="61"/>
-      <c r="H12" s="61"/>
-      <c r="I12" s="61"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="26"/>
     </row>
     <row r="13" spans="2:9" ht="9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="28"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="28"/>
-      <c r="G13" s="28"/>
-      <c r="H13" s="28"/>
-      <c r="I13" s="28"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
+      <c r="I13" s="29"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="54" t="s">
+      <c r="B14" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="54"/>
-      <c r="D14" s="54"/>
-      <c r="E14" s="54"/>
-      <c r="F14" s="54"/>
-      <c r="G14" s="54"/>
-      <c r="H14" s="54"/>
-      <c r="I14" s="54"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="23"/>
     </row>
     <row r="15" spans="2:9" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="63" t="s">
+      <c r="C15" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="64"/>
-      <c r="E15" s="64"/>
-      <c r="F15" s="64"/>
-      <c r="G15" s="64"/>
-      <c r="H15" s="64"/>
-      <c r="I15" s="64"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
+      <c r="I15" s="22"/>
     </row>
     <row r="16" spans="2:9" ht="136" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="43" t="s">
+      <c r="B16" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="45" t="s">
+      <c r="C16" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="D16" s="46"/>
-      <c r="E16" s="46"/>
-      <c r="F16" s="46"/>
-      <c r="G16" s="46"/>
-      <c r="H16" s="46"/>
-      <c r="I16" s="47"/>
+      <c r="D16" s="50"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="50"/>
+      <c r="G16" s="50"/>
+      <c r="H16" s="50"/>
+      <c r="I16" s="51"/>
     </row>
     <row r="17" spans="2:9" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="44"/>
-      <c r="C17" s="48"/>
-      <c r="D17" s="49"/>
-      <c r="E17" s="49"/>
-      <c r="F17" s="49"/>
-      <c r="G17" s="49"/>
-      <c r="H17" s="49"/>
-      <c r="I17" s="50"/>
+      <c r="B17" s="48"/>
+      <c r="C17" s="52"/>
+      <c r="D17" s="53"/>
+      <c r="E17" s="53"/>
+      <c r="F17" s="53"/>
+      <c r="G17" s="53"/>
+      <c r="H17" s="53"/>
+      <c r="I17" s="54"/>
     </row>
     <row r="18" spans="2:9" ht="67" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="63" t="s">
+      <c r="C18" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="64"/>
-      <c r="E18" s="64"/>
-      <c r="F18" s="64"/>
-      <c r="G18" s="64"/>
-      <c r="H18" s="64"/>
-      <c r="I18" s="64"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="22"/>
     </row>
     <row r="19" spans="2:9" ht="7" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="28"/>
-      <c r="I19" s="28"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="29"/>
+      <c r="I19" s="29"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="54" t="s">
+      <c r="B20" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="54"/>
-      <c r="D20" s="54"/>
-      <c r="E20" s="54"/>
-      <c r="F20" s="54"/>
-      <c r="G20" s="54"/>
-      <c r="H20" s="54"/>
-      <c r="I20" s="54"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="23"/>
+      <c r="I20" s="23"/>
     </row>
     <row r="21" spans="2:9" ht="43" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="37" t="s">
+      <c r="C21" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="38"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="38"/>
-      <c r="G21" s="38"/>
-      <c r="H21" s="38"/>
-      <c r="I21" s="39"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="31"/>
+      <c r="G21" s="31"/>
+      <c r="H21" s="31"/>
+      <c r="I21" s="32"/>
     </row>
     <row r="22" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B22" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="40">
+      <c r="C22" s="37">
         <v>9</v>
       </c>
-      <c r="D22" s="41"/>
-      <c r="E22" s="41"/>
-      <c r="F22" s="41"/>
-      <c r="G22" s="41"/>
-      <c r="H22" s="41"/>
-      <c r="I22" s="42"/>
+      <c r="D22" s="45"/>
+      <c r="E22" s="45"/>
+      <c r="F22" s="45"/>
+      <c r="G22" s="45"/>
+      <c r="H22" s="45"/>
+      <c r="I22" s="46"/>
     </row>
     <row r="23" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="55" t="s">
+      <c r="C23" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="55"/>
-      <c r="E23" s="56" t="s">
+      <c r="D23" s="59"/>
+      <c r="E23" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="56"/>
-      <c r="G23" s="56"/>
-      <c r="H23" s="56"/>
-      <c r="I23" s="56"/>
+      <c r="F23" s="60"/>
+      <c r="G23" s="60"/>
+      <c r="H23" s="60"/>
+      <c r="I23" s="60"/>
     </row>
     <row r="24" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="30" t="s">
+      <c r="C24" s="57" t="s">
         <v>38</v>
       </c>
-      <c r="D24" s="32"/>
-      <c r="E24" s="37" t="s">
+      <c r="D24" s="58"/>
+      <c r="E24" s="44" t="s">
         <v>37</v>
       </c>
-      <c r="F24" s="57"/>
-      <c r="G24" s="57"/>
-      <c r="H24" s="57"/>
-      <c r="I24" s="58"/>
+      <c r="F24" s="61"/>
+      <c r="G24" s="61"/>
+      <c r="H24" s="61"/>
+      <c r="I24" s="62"/>
     </row>
     <row r="25" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="8">
         <v>2</v>
       </c>
-      <c r="C25" s="30" t="s">
+      <c r="C25" s="57" t="s">
         <v>39</v>
       </c>
-      <c r="D25" s="32"/>
-      <c r="E25" s="30"/>
-      <c r="F25" s="31"/>
-      <c r="G25" s="31"/>
-      <c r="H25" s="31"/>
-      <c r="I25" s="32"/>
+      <c r="D25" s="58"/>
+      <c r="E25" s="57"/>
+      <c r="F25" s="73"/>
+      <c r="G25" s="73"/>
+      <c r="H25" s="73"/>
+      <c r="I25" s="58"/>
     </row>
     <row r="26" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="59">
+      <c r="B26" s="63">
         <v>3</v>
       </c>
-      <c r="C26" s="19" t="s">
+      <c r="C26" s="65" t="s">
         <v>40</v>
       </c>
-      <c r="D26" s="20"/>
-      <c r="E26" s="33" t="s">
+      <c r="D26" s="66"/>
+      <c r="E26" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="F26" s="33"/>
-      <c r="G26" s="31" t="s">
+      <c r="F26" s="40"/>
+      <c r="G26" s="73" t="s">
         <v>41</v>
       </c>
-      <c r="H26" s="31"/>
-      <c r="I26" s="32"/>
+      <c r="H26" s="73"/>
+      <c r="I26" s="58"/>
     </row>
     <row r="27" spans="2:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="60"/>
-      <c r="C27" s="21"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="23" t="s">
+      <c r="B27" s="64"/>
+      <c r="C27" s="67"/>
+      <c r="D27" s="68"/>
+      <c r="E27" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="F27" s="24"/>
-      <c r="G27" s="25" t="s">
+      <c r="F27" s="36"/>
+      <c r="G27" s="69" t="s">
         <v>43</v>
       </c>
-      <c r="H27" s="26"/>
-      <c r="I27" s="27"/>
+      <c r="H27" s="70"/>
+      <c r="I27" s="71"/>
     </row>
     <row r="28" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="8">
         <v>4</v>
       </c>
-      <c r="C28" s="23" t="s">
+      <c r="C28" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="D28" s="24"/>
-      <c r="E28" s="51" t="s">
+      <c r="D28" s="36"/>
+      <c r="E28" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="F28" s="38"/>
-      <c r="G28" s="38"/>
-      <c r="H28" s="38"/>
-      <c r="I28" s="39"/>
+      <c r="F28" s="31"/>
+      <c r="G28" s="31"/>
+      <c r="H28" s="31"/>
+      <c r="I28" s="32"/>
     </row>
     <row r="29" spans="2:9" ht="43" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="8">
         <v>5</v>
       </c>
-      <c r="C29" s="33" t="s">
+      <c r="C29" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="D29" s="33"/>
-      <c r="E29" s="65" t="s">
+      <c r="D29" s="40"/>
+      <c r="E29" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="F29" s="65"/>
-      <c r="G29" s="65"/>
-      <c r="H29" s="65"/>
-      <c r="I29" s="65"/>
+      <c r="F29" s="33"/>
+      <c r="G29" s="33"/>
+      <c r="H29" s="33"/>
+      <c r="I29" s="33"/>
     </row>
     <row r="30" spans="2:9" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="8">
         <v>6</v>
       </c>
-      <c r="C30" s="23" t="s">
+      <c r="C30" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="D30" s="24"/>
-      <c r="E30" s="51" t="s">
+      <c r="D30" s="36"/>
+      <c r="E30" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="F30" s="52"/>
-      <c r="G30" s="52"/>
-      <c r="H30" s="52"/>
-      <c r="I30" s="53"/>
+      <c r="F30" s="55"/>
+      <c r="G30" s="55"/>
+      <c r="H30" s="55"/>
+      <c r="I30" s="56"/>
     </row>
     <row r="31" spans="2:9" ht="53" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="8">
         <v>7</v>
       </c>
-      <c r="C31" s="33" t="s">
+      <c r="C31" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="D31" s="33"/>
-      <c r="E31" s="65" t="s">
+      <c r="D31" s="40"/>
+      <c r="E31" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="F31" s="66"/>
-      <c r="G31" s="66"/>
-      <c r="H31" s="66"/>
-      <c r="I31" s="66"/>
+      <c r="F31" s="34"/>
+      <c r="G31" s="34"/>
+      <c r="H31" s="34"/>
+      <c r="I31" s="34"/>
     </row>
     <row r="32" spans="2:9" ht="53" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="8">
         <v>8</v>
       </c>
-      <c r="C32" s="23" t="s">
+      <c r="C32" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="D32" s="24"/>
-      <c r="E32" s="23"/>
-      <c r="F32" s="29"/>
-      <c r="G32" s="29"/>
-      <c r="H32" s="29"/>
-      <c r="I32" s="24"/>
+      <c r="D32" s="36"/>
+      <c r="E32" s="35"/>
+      <c r="F32" s="72"/>
+      <c r="G32" s="72"/>
+      <c r="H32" s="72"/>
+      <c r="I32" s="36"/>
     </row>
     <row r="33" spans="2:9" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="8">
         <v>9</v>
       </c>
-      <c r="C33" s="23" t="s">
+      <c r="C33" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="D33" s="24"/>
-      <c r="E33" s="40" t="s">
+      <c r="D33" s="36"/>
+      <c r="E33" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="F33" s="67"/>
-      <c r="G33" s="67"/>
-      <c r="H33" s="67"/>
-      <c r="I33" s="68"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="38"/>
+      <c r="H33" s="38"/>
+      <c r="I33" s="39"/>
     </row>
     <row r="34" spans="2:9" ht="190" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C34" s="65" t="s">
+      <c r="C34" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="D34" s="65"/>
-      <c r="E34" s="65"/>
-      <c r="F34" s="65"/>
-      <c r="G34" s="65"/>
-      <c r="H34" s="65"/>
-      <c r="I34" s="65"/>
+      <c r="D34" s="33"/>
+      <c r="E34" s="33"/>
+      <c r="F34" s="33"/>
+      <c r="G34" s="33"/>
+      <c r="H34" s="33"/>
+      <c r="I34" s="33"/>
     </row>
     <row r="35" spans="2:9" ht="10" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="34"/>
-      <c r="C35" s="35"/>
-      <c r="D35" s="35"/>
-      <c r="E35" s="35"/>
-      <c r="F35" s="35"/>
-      <c r="G35" s="35"/>
-      <c r="H35" s="35"/>
-      <c r="I35" s="36"/>
+      <c r="B35" s="41"/>
+      <c r="C35" s="42"/>
+      <c r="D35" s="42"/>
+      <c r="E35" s="42"/>
+      <c r="F35" s="42"/>
+      <c r="G35" s="42"/>
+      <c r="H35" s="42"/>
+      <c r="I35" s="43"/>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B36" s="54" t="s">
+      <c r="B36" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="C36" s="54"/>
-      <c r="D36" s="54"/>
-      <c r="E36" s="54"/>
-      <c r="F36" s="54"/>
-      <c r="G36" s="54"/>
-      <c r="H36" s="54"/>
-      <c r="I36" s="54"/>
+      <c r="C36" s="23"/>
+      <c r="D36" s="23"/>
+      <c r="E36" s="23"/>
+      <c r="F36" s="23"/>
+      <c r="G36" s="23"/>
+      <c r="H36" s="23"/>
+      <c r="I36" s="23"/>
     </row>
     <row r="37" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="62" t="s">
+      <c r="B37" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="C37" s="62"/>
-      <c r="D37" s="62"/>
-      <c r="E37" s="62"/>
-      <c r="F37" s="62"/>
-      <c r="G37" s="62"/>
-      <c r="H37" s="62"/>
-      <c r="I37" s="62"/>
+      <c r="C37" s="27"/>
+      <c r="D37" s="27"/>
+      <c r="E37" s="27"/>
+      <c r="F37" s="27"/>
+      <c r="G37" s="27"/>
+      <c r="H37" s="27"/>
+      <c r="I37" s="27"/>
     </row>
     <row r="38" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="62"/>
-      <c r="C38" s="62"/>
-      <c r="D38" s="62"/>
-      <c r="E38" s="62"/>
-      <c r="F38" s="62"/>
-      <c r="G38" s="62"/>
-      <c r="H38" s="62"/>
-      <c r="I38" s="62"/>
+      <c r="B38" s="27"/>
+      <c r="C38" s="27"/>
+      <c r="D38" s="27"/>
+      <c r="E38" s="27"/>
+      <c r="F38" s="27"/>
+      <c r="G38" s="27"/>
+      <c r="H38" s="27"/>
+      <c r="I38" s="27"/>
     </row>
     <row r="39" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="62"/>
-      <c r="C39" s="62"/>
-      <c r="D39" s="62"/>
-      <c r="E39" s="62"/>
-      <c r="F39" s="62"/>
-      <c r="G39" s="62"/>
-      <c r="H39" s="62"/>
-      <c r="I39" s="62"/>
+      <c r="B39" s="27"/>
+      <c r="C39" s="27"/>
+      <c r="D39" s="27"/>
+      <c r="E39" s="27"/>
+      <c r="F39" s="27"/>
+      <c r="G39" s="27"/>
+      <c r="H39" s="27"/>
+      <c r="I39" s="27"/>
     </row>
     <row r="40" spans="2:9" ht="76" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B40" s="62"/>
-      <c r="C40" s="62"/>
-      <c r="D40" s="62"/>
-      <c r="E40" s="62"/>
-      <c r="F40" s="62"/>
-      <c r="G40" s="62"/>
-      <c r="H40" s="62"/>
-      <c r="I40" s="62"/>
+      <c r="B40" s="27"/>
+      <c r="C40" s="27"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="27"/>
+      <c r="F40" s="27"/>
+      <c r="G40" s="27"/>
+      <c r="H40" s="27"/>
+      <c r="I40" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="C7:I7"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="C3:I3"/>
-    <mergeCell ref="C4:I4"/>
-    <mergeCell ref="C5:I5"/>
-    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="C26:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="E32:I32"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="B26:B27"/>
     <mergeCell ref="B36:I36"/>
     <mergeCell ref="B10:I12"/>
     <mergeCell ref="B9:I9"/>
@@ -3776,31 +3795,12 @@
     <mergeCell ref="C28:D28"/>
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="C31:D31"/>
-    <mergeCell ref="B35:I35"/>
-    <mergeCell ref="B13:I13"/>
-    <mergeCell ref="C21:I21"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:I30"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="B14:I14"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="C26:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="E32:I32"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="C6:I6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{C9E9977D-5134-FE4B-852F-8DEBDCB543E0}"/>
@@ -3829,12 +3829,12 @@
   </cols>
   <sheetData>
     <row r="4" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B4" s="71" t="s">
+      <c r="B4" s="25" t="s">
         <v>128</v>
       </c>
-      <c r="C4" s="71"/>
-      <c r="D4" s="71"/>
-      <c r="E4" s="71"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
     </row>
     <row r="5" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="11" t="s">
@@ -4105,421 +4105,442 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="54" t="s">
+      <c r="B2" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="90" t="s">
+      <c r="C3" s="74" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="91"/>
-      <c r="E3" s="91"/>
-      <c r="F3" s="91"/>
-      <c r="G3" s="91"/>
-      <c r="H3" s="91"/>
-      <c r="I3" s="91"/>
+      <c r="D3" s="75"/>
+      <c r="E3" s="75"/>
+      <c r="F3" s="75"/>
+      <c r="G3" s="75"/>
+      <c r="H3" s="75"/>
+      <c r="I3" s="75"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="64" t="s">
+      <c r="C4" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="64"/>
-      <c r="E4" s="64"/>
-      <c r="F4" s="64"/>
-      <c r="G4" s="64"/>
-      <c r="H4" s="64"/>
-      <c r="I4" s="64"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="64">
+      <c r="C5" s="22">
         <v>2020</v>
       </c>
-      <c r="D5" s="64"/>
-      <c r="E5" s="64"/>
-      <c r="F5" s="64"/>
-      <c r="G5" s="64"/>
-      <c r="H5" s="64"/>
-      <c r="I5" s="64"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
     </row>
     <row r="6" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="66" t="s">
+      <c r="C6" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="66"/>
-      <c r="E6" s="66"/>
-      <c r="F6" s="66"/>
-      <c r="G6" s="66"/>
-      <c r="H6" s="66"/>
-      <c r="I6" s="66"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="34"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="69" t="s">
+      <c r="C7" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="D7" s="64"/>
-      <c r="E7" s="64"/>
-      <c r="F7" s="64"/>
-      <c r="G7" s="64"/>
-      <c r="H7" s="64"/>
-      <c r="I7" s="64"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="22"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="28"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="28"/>
-      <c r="I8" s="28"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="29"/>
+      <c r="I8" s="29"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="54" t="s">
+      <c r="B9" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="54"/>
-      <c r="D9" s="54"/>
-      <c r="E9" s="54"/>
-      <c r="F9" s="54"/>
-      <c r="G9" s="54"/>
-      <c r="H9" s="54"/>
-      <c r="I9" s="54"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
     </row>
     <row r="10" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="61" t="s">
+      <c r="B10" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="61"/>
-      <c r="D10" s="61"/>
-      <c r="E10" s="61"/>
-      <c r="F10" s="61"/>
-      <c r="G10" s="61"/>
-      <c r="H10" s="61"/>
-      <c r="I10" s="61"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="26"/>
     </row>
     <row r="11" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="61"/>
-      <c r="C11" s="61"/>
-      <c r="D11" s="61"/>
-      <c r="E11" s="61"/>
-      <c r="F11" s="61"/>
-      <c r="G11" s="61"/>
-      <c r="H11" s="61"/>
-      <c r="I11" s="61"/>
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="26"/>
     </row>
     <row r="12" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="61"/>
-      <c r="C12" s="61"/>
-      <c r="D12" s="61"/>
-      <c r="E12" s="61"/>
-      <c r="F12" s="61"/>
-      <c r="G12" s="61"/>
-      <c r="H12" s="61"/>
-      <c r="I12" s="61"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="26"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="28"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="28"/>
-      <c r="G13" s="28"/>
-      <c r="H13" s="28"/>
-      <c r="I13" s="28"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
+      <c r="I13" s="29"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="54" t="s">
+      <c r="B14" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="54"/>
-      <c r="D14" s="54"/>
-      <c r="E14" s="54"/>
-      <c r="F14" s="54"/>
-      <c r="G14" s="54"/>
-      <c r="H14" s="54"/>
-      <c r="I14" s="54"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="23"/>
     </row>
     <row r="15" spans="2:9" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="63" t="s">
+      <c r="C15" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="64"/>
-      <c r="E15" s="64"/>
-      <c r="F15" s="64"/>
-      <c r="G15" s="64"/>
-      <c r="H15" s="64"/>
-      <c r="I15" s="64"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
+      <c r="I15" s="22"/>
     </row>
     <row r="16" spans="2:9" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="43" t="s">
+      <c r="B16" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="81" t="s">
+      <c r="C16" s="76" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="82"/>
-      <c r="E16" s="82"/>
-      <c r="F16" s="82"/>
-      <c r="G16" s="82"/>
-      <c r="H16" s="82"/>
-      <c r="I16" s="83"/>
+      <c r="D16" s="77"/>
+      <c r="E16" s="77"/>
+      <c r="F16" s="77"/>
+      <c r="G16" s="77"/>
+      <c r="H16" s="77"/>
+      <c r="I16" s="78"/>
     </row>
     <row r="17" spans="2:9" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="44"/>
-      <c r="C17" s="84"/>
-      <c r="D17" s="85"/>
-      <c r="E17" s="85"/>
-      <c r="F17" s="85"/>
-      <c r="G17" s="85"/>
-      <c r="H17" s="85"/>
-      <c r="I17" s="86"/>
+      <c r="B17" s="48"/>
+      <c r="C17" s="79"/>
+      <c r="D17" s="80"/>
+      <c r="E17" s="80"/>
+      <c r="F17" s="80"/>
+      <c r="G17" s="80"/>
+      <c r="H17" s="80"/>
+      <c r="I17" s="81"/>
     </row>
     <row r="18" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="63" t="s">
+      <c r="C18" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="D18" s="64"/>
-      <c r="E18" s="64"/>
-      <c r="F18" s="64"/>
-      <c r="G18" s="64"/>
-      <c r="H18" s="64"/>
-      <c r="I18" s="64"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="22"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="28"/>
-      <c r="I19" s="28"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="29"/>
+      <c r="I19" s="29"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="54" t="s">
+      <c r="B20" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="54"/>
-      <c r="D20" s="54"/>
-      <c r="E20" s="54"/>
-      <c r="F20" s="54"/>
-      <c r="G20" s="54"/>
-      <c r="H20" s="54"/>
-      <c r="I20" s="54"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="23"/>
+      <c r="I20" s="23"/>
     </row>
     <row r="21" spans="2:9" ht="160" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="87" t="s">
+      <c r="C21" s="82" t="s">
         <v>57</v>
       </c>
-      <c r="D21" s="88"/>
-      <c r="E21" s="88"/>
-      <c r="F21" s="88"/>
-      <c r="G21" s="88"/>
-      <c r="H21" s="88"/>
-      <c r="I21" s="89"/>
+      <c r="D21" s="83"/>
+      <c r="E21" s="83"/>
+      <c r="F21" s="83"/>
+      <c r="G21" s="83"/>
+      <c r="H21" s="83"/>
+      <c r="I21" s="84"/>
     </row>
     <row r="22" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="40">
+      <c r="C22" s="37">
         <v>3</v>
       </c>
-      <c r="D22" s="41"/>
-      <c r="E22" s="41"/>
-      <c r="F22" s="41"/>
-      <c r="G22" s="41"/>
-      <c r="H22" s="41"/>
-      <c r="I22" s="42"/>
+      <c r="D22" s="45"/>
+      <c r="E22" s="45"/>
+      <c r="F22" s="45"/>
+      <c r="G22" s="45"/>
+      <c r="H22" s="45"/>
+      <c r="I22" s="46"/>
     </row>
     <row r="23" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="55" t="s">
+      <c r="C23" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="55"/>
-      <c r="E23" s="56" t="s">
+      <c r="D23" s="59"/>
+      <c r="E23" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="56"/>
-      <c r="G23" s="56"/>
-      <c r="H23" s="56"/>
-      <c r="I23" s="56"/>
+      <c r="F23" s="60"/>
+      <c r="G23" s="60"/>
+      <c r="H23" s="60"/>
+      <c r="I23" s="60"/>
     </row>
     <row r="24" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="59">
+      <c r="B24" s="63">
         <v>1</v>
       </c>
-      <c r="C24" s="72" t="s">
+      <c r="C24" s="90" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="73"/>
+      <c r="D24" s="91"/>
       <c r="E24" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="F24" s="76" t="s">
+      <c r="F24" s="92" t="s">
         <v>63</v>
       </c>
-      <c r="G24" s="76"/>
-      <c r="H24" s="76"/>
-      <c r="I24" s="77"/>
+      <c r="G24" s="92"/>
+      <c r="H24" s="92"/>
+      <c r="I24" s="93"/>
     </row>
     <row r="25" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="60"/>
-      <c r="C25" s="74"/>
-      <c r="D25" s="75"/>
+      <c r="B25" s="64"/>
+      <c r="C25" s="88"/>
+      <c r="D25" s="89"/>
       <c r="E25" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="F25" s="31" t="s">
+      <c r="F25" s="73" t="s">
         <v>64</v>
       </c>
-      <c r="G25" s="31"/>
-      <c r="H25" s="31"/>
-      <c r="I25" s="32"/>
+      <c r="G25" s="73"/>
+      <c r="H25" s="73"/>
+      <c r="I25" s="58"/>
     </row>
     <row r="26" spans="2:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="8">
         <v>2</v>
       </c>
-      <c r="C26" s="79" t="s">
+      <c r="C26" s="86" t="s">
         <v>59</v>
       </c>
-      <c r="D26" s="80"/>
-      <c r="E26" s="23"/>
-      <c r="F26" s="29"/>
-      <c r="G26" s="29"/>
-      <c r="H26" s="29"/>
-      <c r="I26" s="24"/>
+      <c r="D26" s="87"/>
+      <c r="E26" s="35"/>
+      <c r="F26" s="72"/>
+      <c r="G26" s="72"/>
+      <c r="H26" s="72"/>
+      <c r="I26" s="36"/>
     </row>
     <row r="27" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="8">
         <v>3</v>
       </c>
-      <c r="C27" s="74" t="s">
+      <c r="C27" s="88" t="s">
         <v>60</v>
       </c>
-      <c r="D27" s="75"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="29"/>
-      <c r="H27" s="29"/>
-      <c r="I27" s="24"/>
+      <c r="D27" s="89"/>
+      <c r="E27" s="35"/>
+      <c r="F27" s="72"/>
+      <c r="G27" s="72"/>
+      <c r="H27" s="72"/>
+      <c r="I27" s="36"/>
     </row>
     <row r="28" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B28" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C28" s="65" t="s">
+      <c r="C28" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="D28" s="65"/>
-      <c r="E28" s="65"/>
-      <c r="F28" s="65"/>
-      <c r="G28" s="65"/>
-      <c r="H28" s="65"/>
-      <c r="I28" s="65"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
+      <c r="H28" s="33"/>
+      <c r="I28" s="33"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B29" s="34"/>
-      <c r="C29" s="35"/>
-      <c r="D29" s="35"/>
-      <c r="E29" s="35"/>
-      <c r="F29" s="35"/>
-      <c r="G29" s="35"/>
-      <c r="H29" s="35"/>
-      <c r="I29" s="36"/>
+      <c r="B29" s="41"/>
+      <c r="C29" s="42"/>
+      <c r="D29" s="42"/>
+      <c r="E29" s="42"/>
+      <c r="F29" s="42"/>
+      <c r="G29" s="42"/>
+      <c r="H29" s="42"/>
+      <c r="I29" s="43"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B30" s="54" t="s">
+      <c r="B30" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="C30" s="54"/>
-      <c r="D30" s="54"/>
-      <c r="E30" s="54"/>
-      <c r="F30" s="54"/>
-      <c r="G30" s="54"/>
-      <c r="H30" s="54"/>
-      <c r="I30" s="54"/>
+      <c r="C30" s="23"/>
+      <c r="D30" s="23"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="23"/>
+      <c r="G30" s="23"/>
+      <c r="H30" s="23"/>
+      <c r="I30" s="23"/>
     </row>
     <row r="31" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="78" t="s">
+      <c r="B31" s="85" t="s">
         <v>66</v>
       </c>
-      <c r="C31" s="62"/>
-      <c r="D31" s="62"/>
-      <c r="E31" s="62"/>
-      <c r="F31" s="62"/>
-      <c r="G31" s="62"/>
-      <c r="H31" s="62"/>
-      <c r="I31" s="62"/>
+      <c r="C31" s="27"/>
+      <c r="D31" s="27"/>
+      <c r="E31" s="27"/>
+      <c r="F31" s="27"/>
+      <c r="G31" s="27"/>
+      <c r="H31" s="27"/>
+      <c r="I31" s="27"/>
     </row>
     <row r="32" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="62"/>
-      <c r="C32" s="62"/>
-      <c r="D32" s="62"/>
-      <c r="E32" s="62"/>
-      <c r="F32" s="62"/>
-      <c r="G32" s="62"/>
-      <c r="H32" s="62"/>
-      <c r="I32" s="62"/>
+      <c r="B32" s="27"/>
+      <c r="C32" s="27"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="27"/>
+      <c r="F32" s="27"/>
+      <c r="G32" s="27"/>
+      <c r="H32" s="27"/>
+      <c r="I32" s="27"/>
     </row>
     <row r="33" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="62"/>
-      <c r="C33" s="62"/>
-      <c r="D33" s="62"/>
-      <c r="E33" s="62"/>
-      <c r="F33" s="62"/>
-      <c r="G33" s="62"/>
-      <c r="H33" s="62"/>
-      <c r="I33" s="62"/>
+      <c r="B33" s="27"/>
+      <c r="C33" s="27"/>
+      <c r="D33" s="27"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="27"/>
+      <c r="G33" s="27"/>
+      <c r="H33" s="27"/>
+      <c r="I33" s="27"/>
     </row>
     <row r="34" spans="2:9" ht="254" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="62"/>
-      <c r="C34" s="62"/>
-      <c r="D34" s="62"/>
-      <c r="E34" s="62"/>
-      <c r="F34" s="62"/>
-      <c r="G34" s="62"/>
-      <c r="H34" s="62"/>
-      <c r="I34" s="62"/>
+      <c r="B34" s="27"/>
+      <c r="C34" s="27"/>
+      <c r="D34" s="27"/>
+      <c r="E34" s="27"/>
+      <c r="F34" s="27"/>
+      <c r="G34" s="27"/>
+      <c r="H34" s="27"/>
+      <c r="I34" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:D25"/>
+    <mergeCell ref="F24:I24"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="C28:I28"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="B31:I34"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="C21:I21"/>
     <mergeCell ref="C15:I15"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -4532,32 +4553,12 @@
     <mergeCell ref="B10:I12"/>
     <mergeCell ref="B13:I13"/>
     <mergeCell ref="B14:I14"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="C21:I21"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="B31:I34"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:I27"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:D25"/>
-    <mergeCell ref="F24:I24"/>
-    <mergeCell ref="F25:I25"/>
-    <mergeCell ref="C28:I28"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{4DBC988E-4FF2-2C49-AA18-DD92CA6A87E8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
 </worksheet>
@@ -4585,405 +4586,424 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="54" t="s">
+      <c r="B2" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="90" t="s">
+      <c r="C3" s="74" t="s">
         <v>67</v>
       </c>
-      <c r="D3" s="91"/>
-      <c r="E3" s="91"/>
-      <c r="F3" s="91"/>
-      <c r="G3" s="91"/>
-      <c r="H3" s="91"/>
-      <c r="I3" s="91"/>
+      <c r="D3" s="75"/>
+      <c r="E3" s="75"/>
+      <c r="F3" s="75"/>
+      <c r="G3" s="75"/>
+      <c r="H3" s="75"/>
+      <c r="I3" s="75"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="64" t="s">
+      <c r="C4" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="D4" s="64"/>
-      <c r="E4" s="64"/>
-      <c r="F4" s="64"/>
-      <c r="G4" s="64"/>
-      <c r="H4" s="64"/>
-      <c r="I4" s="64"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="64">
+      <c r="C5" s="22">
         <v>2022</v>
       </c>
-      <c r="D5" s="64"/>
-      <c r="E5" s="64"/>
-      <c r="F5" s="64"/>
-      <c r="G5" s="64"/>
-      <c r="H5" s="64"/>
-      <c r="I5" s="64"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
     </row>
     <row r="6" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="66" t="s">
+      <c r="C6" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="D6" s="66"/>
-      <c r="E6" s="66"/>
-      <c r="F6" s="66"/>
-      <c r="G6" s="66"/>
-      <c r="H6" s="66"/>
-      <c r="I6" s="66"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="34"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="69" t="s">
+      <c r="C7" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="D7" s="64"/>
-      <c r="E7" s="64"/>
-      <c r="F7" s="64"/>
-      <c r="G7" s="64"/>
-      <c r="H7" s="64"/>
-      <c r="I7" s="64"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="22"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="28"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="28"/>
-      <c r="I8" s="28"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="29"/>
+      <c r="I8" s="29"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="54" t="s">
+      <c r="B9" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="54"/>
-      <c r="D9" s="54"/>
-      <c r="E9" s="54"/>
-      <c r="F9" s="54"/>
-      <c r="G9" s="54"/>
-      <c r="H9" s="54"/>
-      <c r="I9" s="54"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
     </row>
     <row r="10" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="61" t="s">
+      <c r="B10" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="C10" s="61"/>
-      <c r="D10" s="61"/>
-      <c r="E10" s="61"/>
-      <c r="F10" s="61"/>
-      <c r="G10" s="61"/>
-      <c r="H10" s="61"/>
-      <c r="I10" s="61"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="26"/>
     </row>
     <row r="11" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="61"/>
-      <c r="C11" s="61"/>
-      <c r="D11" s="61"/>
-      <c r="E11" s="61"/>
-      <c r="F11" s="61"/>
-      <c r="G11" s="61"/>
-      <c r="H11" s="61"/>
-      <c r="I11" s="61"/>
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="26"/>
     </row>
     <row r="12" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="61"/>
-      <c r="C12" s="61"/>
-      <c r="D12" s="61"/>
-      <c r="E12" s="61"/>
-      <c r="F12" s="61"/>
-      <c r="G12" s="61"/>
-      <c r="H12" s="61"/>
-      <c r="I12" s="61"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="26"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="28"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="28"/>
-      <c r="G13" s="28"/>
-      <c r="H13" s="28"/>
-      <c r="I13" s="28"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
+      <c r="I13" s="29"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="54" t="s">
+      <c r="B14" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="54"/>
-      <c r="D14" s="54"/>
-      <c r="E14" s="54"/>
-      <c r="F14" s="54"/>
-      <c r="G14" s="54"/>
-      <c r="H14" s="54"/>
-      <c r="I14" s="54"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="23"/>
     </row>
     <row r="15" spans="2:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="63" t="s">
+      <c r="C15" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="D15" s="64"/>
-      <c r="E15" s="64"/>
-      <c r="F15" s="64"/>
-      <c r="G15" s="64"/>
-      <c r="H15" s="64"/>
-      <c r="I15" s="64"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
+      <c r="I15" s="22"/>
     </row>
     <row r="16" spans="2:9" ht="247" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="43" t="s">
+      <c r="B16" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="81" t="s">
+      <c r="C16" s="76" t="s">
         <v>72</v>
       </c>
-      <c r="D16" s="82"/>
-      <c r="E16" s="82"/>
-      <c r="F16" s="82"/>
-      <c r="G16" s="82"/>
-      <c r="H16" s="82"/>
-      <c r="I16" s="83"/>
+      <c r="D16" s="77"/>
+      <c r="E16" s="77"/>
+      <c r="F16" s="77"/>
+      <c r="G16" s="77"/>
+      <c r="H16" s="77"/>
+      <c r="I16" s="78"/>
     </row>
     <row r="17" spans="2:9" ht="247" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="44"/>
-      <c r="C17" s="84"/>
-      <c r="D17" s="85"/>
-      <c r="E17" s="85"/>
-      <c r="F17" s="85"/>
-      <c r="G17" s="85"/>
-      <c r="H17" s="85"/>
-      <c r="I17" s="86"/>
+      <c r="B17" s="48"/>
+      <c r="C17" s="79"/>
+      <c r="D17" s="80"/>
+      <c r="E17" s="80"/>
+      <c r="F17" s="80"/>
+      <c r="G17" s="80"/>
+      <c r="H17" s="80"/>
+      <c r="I17" s="81"/>
     </row>
     <row r="18" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="95"/>
-      <c r="D18" s="96"/>
-      <c r="E18" s="96"/>
-      <c r="F18" s="96"/>
-      <c r="G18" s="96"/>
-      <c r="H18" s="96"/>
-      <c r="I18" s="96"/>
+      <c r="C18" s="94"/>
+      <c r="D18" s="95"/>
+      <c r="E18" s="95"/>
+      <c r="F18" s="95"/>
+      <c r="G18" s="95"/>
+      <c r="H18" s="95"/>
+      <c r="I18" s="95"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="28"/>
-      <c r="I19" s="28"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="29"/>
+      <c r="I19" s="29"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="54" t="s">
+      <c r="B20" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="C20" s="54"/>
-      <c r="D20" s="54"/>
-      <c r="E20" s="54"/>
-      <c r="F20" s="54"/>
-      <c r="G20" s="54"/>
-      <c r="H20" s="54"/>
-      <c r="I20" s="54"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="23"/>
+      <c r="I20" s="23"/>
     </row>
     <row r="21" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="87" t="s">
+      <c r="C21" s="82" t="s">
         <v>74</v>
       </c>
-      <c r="D21" s="88"/>
-      <c r="E21" s="88"/>
-      <c r="F21" s="88"/>
-      <c r="G21" s="88"/>
-      <c r="H21" s="88"/>
-      <c r="I21" s="89"/>
+      <c r="D21" s="83"/>
+      <c r="E21" s="83"/>
+      <c r="F21" s="83"/>
+      <c r="G21" s="83"/>
+      <c r="H21" s="83"/>
+      <c r="I21" s="84"/>
     </row>
     <row r="22" spans="2:9" ht="165" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="40" t="s">
+      <c r="C22" s="37" t="s">
         <v>174</v>
       </c>
-      <c r="D22" s="41"/>
-      <c r="E22" s="41"/>
-      <c r="F22" s="41"/>
-      <c r="G22" s="41"/>
-      <c r="H22" s="41"/>
-      <c r="I22" s="42"/>
+      <c r="D22" s="45"/>
+      <c r="E22" s="45"/>
+      <c r="F22" s="45"/>
+      <c r="G22" s="45"/>
+      <c r="H22" s="45"/>
+      <c r="I22" s="46"/>
     </row>
     <row r="23" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="55" t="s">
+      <c r="C23" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="55"/>
-      <c r="E23" s="56" t="s">
+      <c r="D23" s="59"/>
+      <c r="E23" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="56"/>
-      <c r="G23" s="56"/>
-      <c r="H23" s="56"/>
-      <c r="I23" s="56"/>
+      <c r="F23" s="60"/>
+      <c r="G23" s="60"/>
+      <c r="H23" s="60"/>
+      <c r="I23" s="60"/>
     </row>
     <row r="24" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="94" t="s">
+      <c r="C24" s="98" t="s">
         <v>75</v>
       </c>
-      <c r="D24" s="94"/>
-      <c r="E24" s="105" t="s">
+      <c r="D24" s="98"/>
+      <c r="E24" s="99" t="s">
         <v>177</v>
       </c>
-      <c r="F24" s="105"/>
-      <c r="G24" s="105"/>
-      <c r="H24" s="105"/>
-      <c r="I24" s="105"/>
+      <c r="F24" s="99"/>
+      <c r="G24" s="99"/>
+      <c r="H24" s="99"/>
+      <c r="I24" s="99"/>
     </row>
     <row r="25" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="8">
         <v>2</v>
       </c>
-      <c r="C25" s="94" t="s">
+      <c r="C25" s="98" t="s">
         <v>172</v>
       </c>
-      <c r="D25" s="94"/>
-      <c r="E25" s="90" t="s">
+      <c r="D25" s="98"/>
+      <c r="E25" s="74" t="s">
         <v>175</v>
       </c>
-      <c r="F25" s="90"/>
-      <c r="G25" s="90"/>
-      <c r="H25" s="90"/>
-      <c r="I25" s="90"/>
+      <c r="F25" s="74"/>
+      <c r="G25" s="74"/>
+      <c r="H25" s="74"/>
+      <c r="I25" s="74"/>
     </row>
     <row r="26" spans="2:9" ht="71" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="8">
         <v>3</v>
       </c>
-      <c r="C26" s="98" t="s">
+      <c r="C26" s="100" t="s">
         <v>173</v>
       </c>
-      <c r="D26" s="99"/>
-      <c r="E26" s="37" t="s">
+      <c r="D26" s="101"/>
+      <c r="E26" s="44" t="s">
         <v>176</v>
       </c>
-      <c r="F26" s="76"/>
-      <c r="G26" s="76"/>
-      <c r="H26" s="76"/>
-      <c r="I26" s="77"/>
+      <c r="F26" s="92"/>
+      <c r="G26" s="92"/>
+      <c r="H26" s="92"/>
+      <c r="I26" s="93"/>
     </row>
     <row r="27" spans="2:9" ht="68" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="65" t="s">
+      <c r="C27" s="33" t="s">
         <v>76</v>
       </c>
-      <c r="D27" s="65"/>
-      <c r="E27" s="65"/>
-      <c r="F27" s="65"/>
-      <c r="G27" s="65"/>
-      <c r="H27" s="65"/>
-      <c r="I27" s="65"/>
+      <c r="D27" s="33"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
+      <c r="G27" s="33"/>
+      <c r="H27" s="33"/>
+      <c r="I27" s="33"/>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B28" s="34"/>
-      <c r="C28" s="35"/>
-      <c r="D28" s="35"/>
-      <c r="E28" s="35"/>
-      <c r="F28" s="35"/>
-      <c r="G28" s="35"/>
-      <c r="H28" s="35"/>
-      <c r="I28" s="36"/>
+      <c r="B28" s="41"/>
+      <c r="C28" s="42"/>
+      <c r="D28" s="42"/>
+      <c r="E28" s="42"/>
+      <c r="F28" s="42"/>
+      <c r="G28" s="42"/>
+      <c r="H28" s="42"/>
+      <c r="I28" s="43"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B29" s="54" t="s">
+      <c r="B29" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="C29" s="54"/>
-      <c r="D29" s="54"/>
-      <c r="E29" s="54"/>
-      <c r="F29" s="54"/>
-      <c r="G29" s="54"/>
-      <c r="H29" s="54"/>
-      <c r="I29" s="54"/>
+      <c r="C29" s="23"/>
+      <c r="D29" s="23"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="23"/>
+      <c r="H29" s="23"/>
+      <c r="I29" s="23"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B30" s="92"/>
-      <c r="C30" s="93"/>
-      <c r="D30" s="93"/>
-      <c r="E30" s="93"/>
-      <c r="F30" s="93"/>
-      <c r="G30" s="93"/>
-      <c r="H30" s="93"/>
-      <c r="I30" s="93"/>
+      <c r="B30" s="96"/>
+      <c r="C30" s="97"/>
+      <c r="D30" s="97"/>
+      <c r="E30" s="97"/>
+      <c r="F30" s="97"/>
+      <c r="G30" s="97"/>
+      <c r="H30" s="97"/>
+      <c r="I30" s="97"/>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B31" s="93"/>
-      <c r="C31" s="93"/>
-      <c r="D31" s="93"/>
-      <c r="E31" s="93"/>
-      <c r="F31" s="93"/>
-      <c r="G31" s="93"/>
-      <c r="H31" s="93"/>
-      <c r="I31" s="93"/>
+      <c r="B31" s="97"/>
+      <c r="C31" s="97"/>
+      <c r="D31" s="97"/>
+      <c r="E31" s="97"/>
+      <c r="F31" s="97"/>
+      <c r="G31" s="97"/>
+      <c r="H31" s="97"/>
+      <c r="I31" s="97"/>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B32" s="93"/>
-      <c r="C32" s="93"/>
-      <c r="D32" s="93"/>
-      <c r="E32" s="93"/>
-      <c r="F32" s="93"/>
-      <c r="G32" s="93"/>
-      <c r="H32" s="93"/>
-      <c r="I32" s="93"/>
+      <c r="B32" s="97"/>
+      <c r="C32" s="97"/>
+      <c r="D32" s="97"/>
+      <c r="E32" s="97"/>
+      <c r="F32" s="97"/>
+      <c r="G32" s="97"/>
+      <c r="H32" s="97"/>
+      <c r="I32" s="97"/>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B33" s="93"/>
-      <c r="C33" s="93"/>
-      <c r="D33" s="93"/>
-      <c r="E33" s="93"/>
-      <c r="F33" s="93"/>
-      <c r="G33" s="93"/>
-      <c r="H33" s="93"/>
-      <c r="I33" s="93"/>
+      <c r="B33" s="97"/>
+      <c r="C33" s="97"/>
+      <c r="D33" s="97"/>
+      <c r="E33" s="97"/>
+      <c r="F33" s="97"/>
+      <c r="G33" s="97"/>
+      <c r="H33" s="97"/>
+      <c r="I33" s="97"/>
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:I33"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="C27:I27"/>
+    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="C21:I21"/>
     <mergeCell ref="C15:I15"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -4996,30 +5016,12 @@
     <mergeCell ref="B10:I12"/>
     <mergeCell ref="B13:I13"/>
     <mergeCell ref="B14:I14"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="C21:I21"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:I33"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="C27:I27"/>
-    <mergeCell ref="B28:I28"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E26:I26"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{60ABBC95-3763-1140-8147-BC4DA0DFC780}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -5176,525 +5178,499 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B1" s="104"/>
-      <c r="C1" s="104"/>
-      <c r="D1" s="104"/>
-      <c r="E1" s="104"/>
-      <c r="F1" s="104"/>
-      <c r="G1" s="104"/>
-      <c r="H1" s="104"/>
-      <c r="I1" s="104"/>
+      <c r="B1" s="102"/>
+      <c r="C1" s="102"/>
+      <c r="D1" s="102"/>
+      <c r="E1" s="102"/>
+      <c r="F1" s="102"/>
+      <c r="G1" s="102"/>
+      <c r="H1" s="102"/>
+      <c r="I1" s="102"/>
     </row>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="54" t="s">
+      <c r="B2" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="90" t="s">
+      <c r="C3" s="74" t="s">
         <v>78</v>
       </c>
-      <c r="D3" s="91"/>
-      <c r="E3" s="91"/>
-      <c r="F3" s="91"/>
-      <c r="G3" s="91"/>
-      <c r="H3" s="91"/>
-      <c r="I3" s="91"/>
+      <c r="D3" s="75"/>
+      <c r="E3" s="75"/>
+      <c r="F3" s="75"/>
+      <c r="G3" s="75"/>
+      <c r="H3" s="75"/>
+      <c r="I3" s="75"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="64" t="s">
+      <c r="C4" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="D4" s="64"/>
-      <c r="E4" s="64"/>
-      <c r="F4" s="64"/>
-      <c r="G4" s="64"/>
-      <c r="H4" s="64"/>
-      <c r="I4" s="64"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="64">
+      <c r="C5" s="22">
         <v>2025</v>
       </c>
-      <c r="D5" s="64"/>
-      <c r="E5" s="64"/>
-      <c r="F5" s="64"/>
-      <c r="G5" s="64"/>
-      <c r="H5" s="64"/>
-      <c r="I5" s="64"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
     </row>
     <row r="6" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="66" t="s">
+      <c r="C6" s="34" t="s">
         <v>81</v>
       </c>
-      <c r="D6" s="66"/>
-      <c r="E6" s="66"/>
-      <c r="F6" s="66"/>
-      <c r="G6" s="66"/>
-      <c r="H6" s="66"/>
-      <c r="I6" s="66"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="34"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="69" t="s">
+      <c r="C7" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="D7" s="64"/>
-      <c r="E7" s="64"/>
-      <c r="F7" s="64"/>
-      <c r="G7" s="64"/>
-      <c r="H7" s="64"/>
-      <c r="I7" s="64"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="22"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="28"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="28"/>
-      <c r="I8" s="28"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="29"/>
+      <c r="I8" s="29"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="54" t="s">
+      <c r="B9" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="54"/>
-      <c r="D9" s="54"/>
-      <c r="E9" s="54"/>
-      <c r="F9" s="54"/>
-      <c r="G9" s="54"/>
-      <c r="H9" s="54"/>
-      <c r="I9" s="54"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B10" s="61" t="s">
+      <c r="B10" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="C10" s="61"/>
-      <c r="D10" s="61"/>
-      <c r="E10" s="61"/>
-      <c r="F10" s="61"/>
-      <c r="G10" s="61"/>
-      <c r="H10" s="61"/>
-      <c r="I10" s="61"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="26"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B11" s="61"/>
-      <c r="C11" s="61"/>
-      <c r="D11" s="61"/>
-      <c r="E11" s="61"/>
-      <c r="F11" s="61"/>
-      <c r="G11" s="61"/>
-      <c r="H11" s="61"/>
-      <c r="I11" s="61"/>
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="26"/>
     </row>
     <row r="12" spans="2:9" ht="92" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="61"/>
-      <c r="C12" s="61"/>
-      <c r="D12" s="61"/>
-      <c r="E12" s="61"/>
-      <c r="F12" s="61"/>
-      <c r="G12" s="61"/>
-      <c r="H12" s="61"/>
-      <c r="I12" s="61"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="26"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="28"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="28"/>
-      <c r="G13" s="28"/>
-      <c r="H13" s="28"/>
-      <c r="I13" s="28"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
+      <c r="I13" s="29"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="54" t="s">
+      <c r="B14" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="54"/>
-      <c r="D14" s="54"/>
-      <c r="E14" s="54"/>
-      <c r="F14" s="54"/>
-      <c r="G14" s="54"/>
-      <c r="H14" s="54"/>
-      <c r="I14" s="54"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="23"/>
     </row>
     <row r="15" spans="2:9" ht="59" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="65" t="s">
+      <c r="C15" s="33" t="s">
         <v>83</v>
       </c>
-      <c r="D15" s="66"/>
-      <c r="E15" s="66"/>
-      <c r="F15" s="66"/>
-      <c r="G15" s="66"/>
-      <c r="H15" s="66"/>
-      <c r="I15" s="66"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="34"/>
+      <c r="I15" s="34"/>
     </row>
     <row r="16" spans="2:9" ht="59" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="43" t="s">
+      <c r="B16" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="81" t="s">
+      <c r="C16" s="76" t="s">
         <v>84</v>
       </c>
-      <c r="D16" s="82"/>
-      <c r="E16" s="82"/>
-      <c r="F16" s="82"/>
-      <c r="G16" s="82"/>
-      <c r="H16" s="82"/>
-      <c r="I16" s="83"/>
+      <c r="D16" s="77"/>
+      <c r="E16" s="77"/>
+      <c r="F16" s="77"/>
+      <c r="G16" s="77"/>
+      <c r="H16" s="77"/>
+      <c r="I16" s="78"/>
     </row>
     <row r="17" spans="2:9" ht="113" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="44"/>
-      <c r="C17" s="84"/>
-      <c r="D17" s="85"/>
-      <c r="E17" s="85"/>
-      <c r="F17" s="85"/>
-      <c r="G17" s="85"/>
-      <c r="H17" s="85"/>
-      <c r="I17" s="86"/>
+      <c r="B17" s="48"/>
+      <c r="C17" s="79"/>
+      <c r="D17" s="80"/>
+      <c r="E17" s="80"/>
+      <c r="F17" s="80"/>
+      <c r="G17" s="80"/>
+      <c r="H17" s="80"/>
+      <c r="I17" s="81"/>
     </row>
     <row r="18" spans="2:9" ht="358" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="61" t="s">
+      <c r="C18" s="26" t="s">
         <v>85</v>
       </c>
-      <c r="D18" s="66"/>
-      <c r="E18" s="66"/>
-      <c r="F18" s="66"/>
-      <c r="G18" s="66"/>
-      <c r="H18" s="66"/>
-      <c r="I18" s="66"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="34"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="34"/>
+      <c r="I18" s="34"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="28"/>
-      <c r="I19" s="28"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="29"/>
+      <c r="I19" s="29"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="54" t="s">
+      <c r="B20" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="C20" s="54"/>
-      <c r="D20" s="54"/>
-      <c r="E20" s="54"/>
-      <c r="F20" s="54"/>
-      <c r="G20" s="54"/>
-      <c r="H20" s="54"/>
-      <c r="I20" s="54"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="23"/>
+      <c r="I20" s="23"/>
     </row>
     <row r="21" spans="2:9" ht="332" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="87" t="s">
+      <c r="C21" s="82" t="s">
         <v>86</v>
       </c>
-      <c r="D21" s="88"/>
-      <c r="E21" s="88"/>
-      <c r="F21" s="88"/>
-      <c r="G21" s="88"/>
-      <c r="H21" s="88"/>
-      <c r="I21" s="89"/>
+      <c r="D21" s="83"/>
+      <c r="E21" s="83"/>
+      <c r="F21" s="83"/>
+      <c r="G21" s="83"/>
+      <c r="H21" s="83"/>
+      <c r="I21" s="84"/>
     </row>
     <row r="22" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="40">
+      <c r="C22" s="37">
         <v>8</v>
       </c>
-      <c r="D22" s="41"/>
-      <c r="E22" s="41"/>
-      <c r="F22" s="41"/>
-      <c r="G22" s="41"/>
-      <c r="H22" s="41"/>
-      <c r="I22" s="42"/>
+      <c r="D22" s="45"/>
+      <c r="E22" s="45"/>
+      <c r="F22" s="45"/>
+      <c r="G22" s="45"/>
+      <c r="H22" s="45"/>
+      <c r="I22" s="46"/>
     </row>
     <row r="23" spans="2:9" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="55" t="s">
+      <c r="C23" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="55"/>
-      <c r="E23" s="56" t="s">
+      <c r="D23" s="59"/>
+      <c r="E23" s="60" t="s">
         <v>97</v>
       </c>
-      <c r="F23" s="56"/>
-      <c r="G23" s="56"/>
-      <c r="H23" s="56"/>
-      <c r="I23" s="56"/>
+      <c r="F23" s="60"/>
+      <c r="G23" s="60"/>
+      <c r="H23" s="60"/>
+      <c r="I23" s="60"/>
     </row>
     <row r="24" spans="2:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="100" t="s">
+      <c r="C24" s="103" t="s">
         <v>88</v>
       </c>
-      <c r="D24" s="101"/>
-      <c r="E24" s="90" t="s">
+      <c r="D24" s="104"/>
+      <c r="E24" s="74" t="s">
         <v>171</v>
       </c>
-      <c r="F24" s="90"/>
-      <c r="G24" s="90"/>
-      <c r="H24" s="90"/>
-      <c r="I24" s="90"/>
+      <c r="F24" s="74"/>
+      <c r="G24" s="74"/>
+      <c r="H24" s="74"/>
+      <c r="I24" s="74"/>
     </row>
     <row r="25" spans="2:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="8">
         <v>2</v>
       </c>
-      <c r="C25" s="98" t="s">
+      <c r="C25" s="100" t="s">
         <v>89</v>
       </c>
-      <c r="D25" s="99"/>
-      <c r="E25" s="90" t="s">
+      <c r="D25" s="101"/>
+      <c r="E25" s="74" t="s">
         <v>103</v>
       </c>
-      <c r="F25" s="90"/>
-      <c r="G25" s="90"/>
-      <c r="H25" s="90"/>
-      <c r="I25" s="90"/>
+      <c r="F25" s="74"/>
+      <c r="G25" s="74"/>
+      <c r="H25" s="74"/>
+      <c r="I25" s="74"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B26" s="8">
         <v>3</v>
       </c>
-      <c r="C26" s="98" t="s">
+      <c r="C26" s="100" t="s">
         <v>90</v>
       </c>
-      <c r="D26" s="99"/>
-      <c r="E26" s="90" t="s">
+      <c r="D26" s="101"/>
+      <c r="E26" s="74" t="s">
         <v>102</v>
       </c>
-      <c r="F26" s="90"/>
-      <c r="G26" s="90"/>
-      <c r="H26" s="90"/>
-      <c r="I26" s="90"/>
+      <c r="F26" s="74"/>
+      <c r="G26" s="74"/>
+      <c r="H26" s="74"/>
+      <c r="I26" s="74"/>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B27" s="8">
         <v>4</v>
       </c>
-      <c r="C27" s="98" t="s">
+      <c r="C27" s="100" t="s">
         <v>91</v>
       </c>
-      <c r="D27" s="99"/>
-      <c r="E27" s="90" t="s">
+      <c r="D27" s="101"/>
+      <c r="E27" s="74" t="s">
         <v>101</v>
       </c>
-      <c r="F27" s="90"/>
-      <c r="G27" s="90"/>
-      <c r="H27" s="90"/>
-      <c r="I27" s="90"/>
+      <c r="F27" s="74"/>
+      <c r="G27" s="74"/>
+      <c r="H27" s="74"/>
+      <c r="I27" s="74"/>
     </row>
     <row r="28" spans="2:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="8">
         <v>5</v>
       </c>
-      <c r="C28" s="98" t="s">
+      <c r="C28" s="100" t="s">
         <v>92</v>
       </c>
-      <c r="D28" s="99"/>
-      <c r="E28" s="90" t="s">
+      <c r="D28" s="101"/>
+      <c r="E28" s="74" t="s">
         <v>100</v>
       </c>
-      <c r="F28" s="90"/>
-      <c r="G28" s="90"/>
-      <c r="H28" s="90"/>
-      <c r="I28" s="90"/>
+      <c r="F28" s="74"/>
+      <c r="G28" s="74"/>
+      <c r="H28" s="74"/>
+      <c r="I28" s="74"/>
     </row>
     <row r="29" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="8">
         <v>6</v>
       </c>
-      <c r="C29" s="94" t="s">
+      <c r="C29" s="98" t="s">
         <v>93</v>
       </c>
-      <c r="D29" s="94"/>
-      <c r="E29" s="90" t="s">
+      <c r="D29" s="98"/>
+      <c r="E29" s="74" t="s">
         <v>99</v>
       </c>
-      <c r="F29" s="90"/>
-      <c r="G29" s="90"/>
-      <c r="H29" s="90"/>
-      <c r="I29" s="90"/>
+      <c r="F29" s="74"/>
+      <c r="G29" s="74"/>
+      <c r="H29" s="74"/>
+      <c r="I29" s="74"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B30" s="8">
         <v>7</v>
       </c>
-      <c r="C30" s="94" t="s">
+      <c r="C30" s="98" t="s">
         <v>94</v>
       </c>
-      <c r="D30" s="94"/>
-      <c r="E30" s="90" t="s">
+      <c r="D30" s="98"/>
+      <c r="E30" s="74" t="s">
         <v>98</v>
       </c>
-      <c r="F30" s="97"/>
-      <c r="G30" s="97"/>
-      <c r="H30" s="97"/>
-      <c r="I30" s="97"/>
+      <c r="F30" s="105"/>
+      <c r="G30" s="105"/>
+      <c r="H30" s="105"/>
+      <c r="I30" s="105"/>
     </row>
     <row r="31" spans="2:9" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="8">
         <v>8</v>
       </c>
-      <c r="C31" s="98" t="s">
+      <c r="C31" s="100" t="s">
         <v>95</v>
       </c>
-      <c r="D31" s="99"/>
-      <c r="E31" s="40" t="s">
+      <c r="D31" s="101"/>
+      <c r="E31" s="37" t="s">
         <v>96</v>
       </c>
-      <c r="F31" s="67"/>
-      <c r="G31" s="67"/>
-      <c r="H31" s="67"/>
-      <c r="I31" s="68"/>
+      <c r="F31" s="38"/>
+      <c r="G31" s="38"/>
+      <c r="H31" s="38"/>
+      <c r="I31" s="39"/>
     </row>
     <row r="32" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B32" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C32" s="65" t="s">
+      <c r="C32" s="33" t="s">
         <v>87</v>
       </c>
-      <c r="D32" s="65"/>
-      <c r="E32" s="65"/>
-      <c r="F32" s="65"/>
-      <c r="G32" s="65"/>
-      <c r="H32" s="65"/>
-      <c r="I32" s="65"/>
+      <c r="D32" s="33"/>
+      <c r="E32" s="33"/>
+      <c r="F32" s="33"/>
+      <c r="G32" s="33"/>
+      <c r="H32" s="33"/>
+      <c r="I32" s="33"/>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B33" s="34"/>
-      <c r="C33" s="35"/>
-      <c r="D33" s="35"/>
-      <c r="E33" s="35"/>
-      <c r="F33" s="35"/>
-      <c r="G33" s="35"/>
-      <c r="H33" s="35"/>
-      <c r="I33" s="36"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="42"/>
+      <c r="D33" s="42"/>
+      <c r="E33" s="42"/>
+      <c r="F33" s="42"/>
+      <c r="G33" s="42"/>
+      <c r="H33" s="42"/>
+      <c r="I33" s="43"/>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B34" s="54" t="s">
+      <c r="B34" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="C34" s="54"/>
-      <c r="D34" s="54"/>
-      <c r="E34" s="54"/>
-      <c r="F34" s="54"/>
-      <c r="G34" s="54"/>
-      <c r="H34" s="54"/>
-      <c r="I34" s="54"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="23"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="23"/>
+      <c r="G34" s="23"/>
+      <c r="H34" s="23"/>
+      <c r="I34" s="23"/>
     </row>
     <row r="35" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="78" t="s">
+      <c r="B35" s="85" t="s">
         <v>104</v>
       </c>
-      <c r="C35" s="62"/>
-      <c r="D35" s="62"/>
-      <c r="E35" s="62"/>
-      <c r="F35" s="62"/>
-      <c r="G35" s="62"/>
-      <c r="H35" s="62"/>
-      <c r="I35" s="62"/>
+      <c r="C35" s="27"/>
+      <c r="D35" s="27"/>
+      <c r="E35" s="27"/>
+      <c r="F35" s="27"/>
+      <c r="G35" s="27"/>
+      <c r="H35" s="27"/>
+      <c r="I35" s="27"/>
     </row>
     <row r="36" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="62"/>
-      <c r="C36" s="62"/>
-      <c r="D36" s="62"/>
-      <c r="E36" s="62"/>
-      <c r="F36" s="62"/>
-      <c r="G36" s="62"/>
-      <c r="H36" s="62"/>
-      <c r="I36" s="62"/>
+      <c r="B36" s="27"/>
+      <c r="C36" s="27"/>
+      <c r="D36" s="27"/>
+      <c r="E36" s="27"/>
+      <c r="F36" s="27"/>
+      <c r="G36" s="27"/>
+      <c r="H36" s="27"/>
+      <c r="I36" s="27"/>
     </row>
     <row r="37" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="62"/>
-      <c r="C37" s="62"/>
-      <c r="D37" s="62"/>
-      <c r="E37" s="62"/>
-      <c r="F37" s="62"/>
-      <c r="G37" s="62"/>
-      <c r="H37" s="62"/>
-      <c r="I37" s="62"/>
+      <c r="B37" s="27"/>
+      <c r="C37" s="27"/>
+      <c r="D37" s="27"/>
+      <c r="E37" s="27"/>
+      <c r="F37" s="27"/>
+      <c r="G37" s="27"/>
+      <c r="H37" s="27"/>
+      <c r="I37" s="27"/>
     </row>
     <row r="38" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="62"/>
-      <c r="C38" s="62"/>
-      <c r="D38" s="62"/>
-      <c r="E38" s="62"/>
-      <c r="F38" s="62"/>
-      <c r="G38" s="62"/>
-      <c r="H38" s="62"/>
-      <c r="I38" s="62"/>
+      <c r="B38" s="27"/>
+      <c r="C38" s="27"/>
+      <c r="D38" s="27"/>
+      <c r="E38" s="27"/>
+      <c r="F38" s="27"/>
+      <c r="G38" s="27"/>
+      <c r="H38" s="27"/>
+      <c r="I38" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="42">
-    <mergeCell ref="B1:I1"/>
-    <mergeCell ref="C7:I7"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="E27:I27"/>
-    <mergeCell ref="C21:I21"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="B9:I9"/>
-    <mergeCell ref="B10:I12"/>
-    <mergeCell ref="B13:I13"/>
-    <mergeCell ref="B14:I14"/>
-    <mergeCell ref="C15:I15"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="C3:I3"/>
-    <mergeCell ref="C4:I4"/>
-    <mergeCell ref="C5:I5"/>
-    <mergeCell ref="C6:I6"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
     <mergeCell ref="B20:I20"/>
     <mergeCell ref="B35:I38"/>
     <mergeCell ref="C22:I22"/>
@@ -5711,11 +5687,38 @@
     <mergeCell ref="C32:I32"/>
     <mergeCell ref="B33:I33"/>
     <mergeCell ref="B34:I34"/>
+    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B9:I9"/>
+    <mergeCell ref="B10:I12"/>
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="C15:I15"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="C5:I5"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{69FD07AD-7FCA-E141-8126-AFB63E0A1511}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -5742,156 +5745,156 @@
       </c>
     </row>
     <row r="4" spans="3:5" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C4" s="103" t="s">
+      <c r="C4" s="20" t="s">
         <v>156</v>
       </c>
       <c r="D4" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="E4" s="102" t="s">
+      <c r="E4" s="19" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="5" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C5" s="103" t="s">
+      <c r="C5" s="20" t="s">
         <v>157</v>
       </c>
-      <c r="D5" s="102" t="s">
+      <c r="D5" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="E5" s="102" t="s">
+      <c r="E5" s="19" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="6" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C6" s="103" t="s">
+      <c r="C6" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="D6" s="102" t="s">
+      <c r="D6" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="E6" s="102" t="s">
+      <c r="E6" s="19" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="7" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C7" s="103" t="s">
+      <c r="C7" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="D7" s="102" t="s">
+      <c r="D7" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="E7" s="102" t="s">
+      <c r="E7" s="19" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="8" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C8" s="103" t="s">
+      <c r="C8" s="20" t="s">
         <v>160</v>
       </c>
-      <c r="D8" s="102" t="s">
+      <c r="D8" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="E8" s="102" t="s">
+      <c r="E8" s="19" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="9" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C9" s="103" t="s">
+      <c r="C9" s="20" t="s">
         <v>161</v>
       </c>
-      <c r="D9" s="102" t="s">
+      <c r="D9" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="E9" s="102" t="s">
+      <c r="E9" s="19" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="10" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C10" s="103" t="s">
+      <c r="C10" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="D10" s="102" t="s">
+      <c r="D10" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="E10" s="102" t="s">
+      <c r="E10" s="19" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="11" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C11" s="103" t="s">
+      <c r="C11" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="D11" s="102" t="s">
+      <c r="D11" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="E11" s="102" t="s">
+      <c r="E11" s="19" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="12" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C12" s="103" t="s">
+      <c r="C12" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="D12" s="102" t="s">
+      <c r="D12" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="E12" s="102" t="s">
+      <c r="E12" s="19" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="13" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C13" s="103" t="s">
+      <c r="C13" s="20" t="s">
         <v>164</v>
       </c>
-      <c r="D13" s="102" t="s">
+      <c r="D13" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="E13" s="102" t="s">
+      <c r="E13" s="19" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="14" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C14" s="103" t="s">
+      <c r="C14" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="D14" s="102" t="s">
+      <c r="D14" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="E14" s="102" t="s">
+      <c r="E14" s="19" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="15" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C15" s="103" t="s">
+      <c r="C15" s="20" t="s">
         <v>165</v>
       </c>
-      <c r="D15" s="102" t="s">
+      <c r="D15" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="E15" s="102" t="s">
+      <c r="E15" s="19" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="16" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C16" s="103" t="s">
+      <c r="C16" s="20" t="s">
         <v>166</v>
       </c>
-      <c r="D16" s="102" t="s">
+      <c r="D16" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="E16" s="102" t="s">
+      <c r="E16" s="19" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="17" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C17" s="103" t="s">
+      <c r="C17" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="D17" s="102" t="s">
+      <c r="D17" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="E17" s="102" t="s">
+      <c r="E17" s="19" t="s">
         <v>155</v>
       </c>
     </row>

</xml_diff>

<commit_message>
did the test to connect to gemini and actually edited the main code (needs to be tested)
</commit_message>
<xml_diff>
--- a/Papers/Resumen Papers.xlsx
+++ b/Papers/Resumen Papers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sophiaaristizabal/Documents/GitHub/LLMS_Project/Papers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB359F70-9C83-E241-BD1C-98DABD7B1BF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABA4A6DB-F527-344F-912B-0AEA2E6B1646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="20520" windowHeight="13540" firstSheet="3" activeTab="6" xr2:uid="{400AC57E-08F9-B346-9132-4F74AEBC2D15}"/>
+    <workbookView xWindow="7040" yWindow="2400" windowWidth="20520" windowHeight="13540" xr2:uid="{400AC57E-08F9-B346-9132-4F74AEBC2D15}"/>
   </bookViews>
   <sheets>
     <sheet name="MANAGERIAL LEADERSHIP" sheetId="1" r:id="rId1"/>
@@ -2439,164 +2439,218 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -2604,59 +2658,23 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -2664,23 +2682,8 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -2690,9 +2693,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3243,526 +3243,539 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="72" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
+      <c r="D3" s="72"/>
+      <c r="E3" s="72"/>
+      <c r="F3" s="72"/>
+      <c r="G3" s="72"/>
+      <c r="H3" s="72"/>
+      <c r="I3" s="72"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="C4" s="73" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="25"/>
-      <c r="I4" s="25"/>
+      <c r="D4" s="73"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="73"/>
+      <c r="H4" s="73"/>
+      <c r="I4" s="73"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="22">
+      <c r="C5" s="66">
         <v>2025</v>
       </c>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
+      <c r="D5" s="66"/>
+      <c r="E5" s="66"/>
+      <c r="F5" s="66"/>
+      <c r="G5" s="66"/>
+      <c r="H5" s="66"/>
+      <c r="I5" s="66"/>
     </row>
     <row r="6" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="66" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
+      <c r="G6" s="66"/>
+      <c r="H6" s="66"/>
+      <c r="I6" s="66"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="22"/>
+      <c r="D7" s="66"/>
+      <c r="E7" s="66"/>
+      <c r="F7" s="66"/>
+      <c r="G7" s="66"/>
+      <c r="H7" s="66"/>
+      <c r="I7" s="66"/>
     </row>
     <row r="8" spans="2:9" ht="9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="29"/>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="29"/>
-      <c r="I8" s="29"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
     </row>
     <row r="9" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="56" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="23"/>
+      <c r="C9" s="56"/>
+      <c r="D9" s="56"/>
+      <c r="E9" s="56"/>
+      <c r="F9" s="56"/>
+      <c r="G9" s="56"/>
+      <c r="H9" s="56"/>
+      <c r="I9" s="56"/>
     </row>
     <row r="10" spans="2:9" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
+      <c r="C10" s="63"/>
+      <c r="D10" s="63"/>
+      <c r="E10" s="63"/>
+      <c r="F10" s="63"/>
+      <c r="G10" s="63"/>
+      <c r="H10" s="63"/>
+      <c r="I10" s="63"/>
     </row>
     <row r="11" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="26"/>
+      <c r="B11" s="63"/>
+      <c r="C11" s="63"/>
+      <c r="D11" s="63"/>
+      <c r="E11" s="63"/>
+      <c r="F11" s="63"/>
+      <c r="G11" s="63"/>
+      <c r="H11" s="63"/>
+      <c r="I11" s="63"/>
     </row>
     <row r="12" spans="2:9" ht="11" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="26"/>
+      <c r="B12" s="63"/>
+      <c r="C12" s="63"/>
+      <c r="D12" s="63"/>
+      <c r="E12" s="63"/>
+      <c r="F12" s="63"/>
+      <c r="G12" s="63"/>
+      <c r="H12" s="63"/>
+      <c r="I12" s="63"/>
     </row>
     <row r="13" spans="2:9" ht="9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="29"/>
-      <c r="C13" s="29"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="29"/>
-      <c r="F13" s="29"/>
-      <c r="G13" s="29"/>
-      <c r="H13" s="29"/>
-      <c r="I13" s="29"/>
+      <c r="B13" s="30"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="30"/>
+      <c r="I13" s="30"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="23" t="s">
+      <c r="B14" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23"/>
-      <c r="H14" s="23"/>
-      <c r="I14" s="23"/>
+      <c r="C14" s="56"/>
+      <c r="D14" s="56"/>
+      <c r="E14" s="56"/>
+      <c r="F14" s="56"/>
+      <c r="G14" s="56"/>
+      <c r="H14" s="56"/>
+      <c r="I14" s="56"/>
     </row>
     <row r="15" spans="2:9" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="28" t="s">
+      <c r="C15" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="22"/>
-      <c r="I15" s="22"/>
+      <c r="D15" s="66"/>
+      <c r="E15" s="66"/>
+      <c r="F15" s="66"/>
+      <c r="G15" s="66"/>
+      <c r="H15" s="66"/>
+      <c r="I15" s="66"/>
     </row>
     <row r="16" spans="2:9" ht="136" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="47" t="s">
+      <c r="B16" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="49" t="s">
+      <c r="C16" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="D16" s="50"/>
-      <c r="E16" s="50"/>
-      <c r="F16" s="50"/>
-      <c r="G16" s="50"/>
-      <c r="H16" s="50"/>
-      <c r="I16" s="51"/>
+      <c r="D16" s="48"/>
+      <c r="E16" s="48"/>
+      <c r="F16" s="48"/>
+      <c r="G16" s="48"/>
+      <c r="H16" s="48"/>
+      <c r="I16" s="49"/>
     </row>
     <row r="17" spans="2:9" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="48"/>
-      <c r="C17" s="52"/>
-      <c r="D17" s="53"/>
-      <c r="E17" s="53"/>
-      <c r="F17" s="53"/>
-      <c r="G17" s="53"/>
-      <c r="H17" s="53"/>
-      <c r="I17" s="54"/>
+      <c r="B17" s="46"/>
+      <c r="C17" s="50"/>
+      <c r="D17" s="51"/>
+      <c r="E17" s="51"/>
+      <c r="F17" s="51"/>
+      <c r="G17" s="51"/>
+      <c r="H17" s="51"/>
+      <c r="I17" s="52"/>
     </row>
     <row r="18" spans="2:9" ht="67" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="65" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
+      <c r="D18" s="66"/>
+      <c r="E18" s="66"/>
+      <c r="F18" s="66"/>
+      <c r="G18" s="66"/>
+      <c r="H18" s="66"/>
+      <c r="I18" s="66"/>
     </row>
     <row r="19" spans="2:9" ht="7" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="29"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="29"/>
-      <c r="G19" s="29"/>
-      <c r="H19" s="29"/>
-      <c r="I19" s="29"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="30"/>
+      <c r="I19" s="30"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="56" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="23"/>
+      <c r="C20" s="56"/>
+      <c r="D20" s="56"/>
+      <c r="E20" s="56"/>
+      <c r="F20" s="56"/>
+      <c r="G20" s="56"/>
+      <c r="H20" s="56"/>
+      <c r="I20" s="56"/>
     </row>
     <row r="21" spans="2:9" ht="43" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="44" t="s">
+      <c r="C21" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="31"/>
-      <c r="E21" s="31"/>
-      <c r="F21" s="31"/>
-      <c r="G21" s="31"/>
-      <c r="H21" s="31"/>
-      <c r="I21" s="32"/>
+      <c r="D21" s="40"/>
+      <c r="E21" s="40"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="40"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="41"/>
     </row>
     <row r="22" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B22" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="37">
+      <c r="C22" s="42">
         <v>9</v>
       </c>
-      <c r="D22" s="45"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="45"/>
-      <c r="H22" s="45"/>
-      <c r="I22" s="46"/>
+      <c r="D22" s="43"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="43"/>
+      <c r="H22" s="43"/>
+      <c r="I22" s="44"/>
     </row>
     <row r="23" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="59" t="s">
+      <c r="C23" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="59"/>
-      <c r="E23" s="60" t="s">
+      <c r="D23" s="57"/>
+      <c r="E23" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="60"/>
-      <c r="G23" s="60"/>
-      <c r="H23" s="60"/>
-      <c r="I23" s="60"/>
+      <c r="F23" s="58"/>
+      <c r="G23" s="58"/>
+      <c r="H23" s="58"/>
+      <c r="I23" s="58"/>
     </row>
     <row r="24" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="57" t="s">
+      <c r="C24" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="D24" s="58"/>
-      <c r="E24" s="44" t="s">
+      <c r="D24" s="34"/>
+      <c r="E24" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="F24" s="61"/>
-      <c r="G24" s="61"/>
-      <c r="H24" s="61"/>
-      <c r="I24" s="62"/>
+      <c r="F24" s="59"/>
+      <c r="G24" s="59"/>
+      <c r="H24" s="59"/>
+      <c r="I24" s="60"/>
     </row>
     <row r="25" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="8">
         <v>2</v>
       </c>
-      <c r="C25" s="57" t="s">
+      <c r="C25" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="D25" s="58"/>
-      <c r="E25" s="57"/>
-      <c r="F25" s="73"/>
-      <c r="G25" s="73"/>
-      <c r="H25" s="73"/>
-      <c r="I25" s="58"/>
+      <c r="D25" s="34"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="33"/>
+      <c r="G25" s="33"/>
+      <c r="H25" s="33"/>
+      <c r="I25" s="34"/>
     </row>
     <row r="26" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="63">
+      <c r="B26" s="61">
         <v>3</v>
       </c>
-      <c r="C26" s="65" t="s">
+      <c r="C26" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="D26" s="66"/>
-      <c r="E26" s="40" t="s">
+      <c r="D26" s="22"/>
+      <c r="E26" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="F26" s="40"/>
-      <c r="G26" s="73" t="s">
+      <c r="F26" s="35"/>
+      <c r="G26" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="H26" s="73"/>
-      <c r="I26" s="58"/>
+      <c r="H26" s="33"/>
+      <c r="I26" s="34"/>
     </row>
     <row r="27" spans="2:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="64"/>
-      <c r="C27" s="67"/>
-      <c r="D27" s="68"/>
-      <c r="E27" s="35" t="s">
+      <c r="B27" s="62"/>
+      <c r="C27" s="23"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="F27" s="36"/>
-      <c r="G27" s="69" t="s">
+      <c r="F27" s="26"/>
+      <c r="G27" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="H27" s="70"/>
-      <c r="I27" s="71"/>
+      <c r="H27" s="28"/>
+      <c r="I27" s="29"/>
     </row>
     <row r="28" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="8">
         <v>4</v>
       </c>
-      <c r="C28" s="35" t="s">
+      <c r="C28" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="D28" s="36"/>
-      <c r="E28" s="30" t="s">
+      <c r="D28" s="26"/>
+      <c r="E28" s="53" t="s">
         <v>32</v>
       </c>
-      <c r="F28" s="31"/>
-      <c r="G28" s="31"/>
-      <c r="H28" s="31"/>
-      <c r="I28" s="32"/>
+      <c r="F28" s="40"/>
+      <c r="G28" s="40"/>
+      <c r="H28" s="40"/>
+      <c r="I28" s="41"/>
     </row>
     <row r="29" spans="2:9" ht="43" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="8">
         <v>5</v>
       </c>
-      <c r="C29" s="40" t="s">
+      <c r="C29" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="D29" s="40"/>
-      <c r="E29" s="33" t="s">
+      <c r="D29" s="35"/>
+      <c r="E29" s="67" t="s">
         <v>33</v>
       </c>
-      <c r="F29" s="33"/>
-      <c r="G29" s="33"/>
-      <c r="H29" s="33"/>
-      <c r="I29" s="33"/>
+      <c r="F29" s="67"/>
+      <c r="G29" s="67"/>
+      <c r="H29" s="67"/>
+      <c r="I29" s="67"/>
     </row>
     <row r="30" spans="2:9" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="8">
         <v>6</v>
       </c>
-      <c r="C30" s="35" t="s">
+      <c r="C30" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D30" s="36"/>
-      <c r="E30" s="30" t="s">
+      <c r="D30" s="26"/>
+      <c r="E30" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="F30" s="55"/>
-      <c r="G30" s="55"/>
-      <c r="H30" s="55"/>
-      <c r="I30" s="56"/>
+      <c r="F30" s="54"/>
+      <c r="G30" s="54"/>
+      <c r="H30" s="54"/>
+      <c r="I30" s="55"/>
     </row>
     <row r="31" spans="2:9" ht="53" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="8">
         <v>7</v>
       </c>
-      <c r="C31" s="40" t="s">
+      <c r="C31" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="D31" s="40"/>
-      <c r="E31" s="33" t="s">
+      <c r="D31" s="35"/>
+      <c r="E31" s="67" t="s">
         <v>35</v>
       </c>
-      <c r="F31" s="34"/>
-      <c r="G31" s="34"/>
-      <c r="H31" s="34"/>
-      <c r="I31" s="34"/>
+      <c r="F31" s="68"/>
+      <c r="G31" s="68"/>
+      <c r="H31" s="68"/>
+      <c r="I31" s="68"/>
     </row>
     <row r="32" spans="2:9" ht="53" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="8">
         <v>8</v>
       </c>
-      <c r="C32" s="35" t="s">
+      <c r="C32" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="D32" s="36"/>
-      <c r="E32" s="35"/>
-      <c r="F32" s="72"/>
-      <c r="G32" s="72"/>
-      <c r="H32" s="72"/>
-      <c r="I32" s="36"/>
+      <c r="D32" s="26"/>
+      <c r="E32" s="25"/>
+      <c r="F32" s="31"/>
+      <c r="G32" s="31"/>
+      <c r="H32" s="31"/>
+      <c r="I32" s="26"/>
     </row>
     <row r="33" spans="2:9" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="8">
         <v>9</v>
       </c>
-      <c r="C33" s="35" t="s">
+      <c r="C33" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="D33" s="36"/>
-      <c r="E33" s="37" t="s">
+      <c r="D33" s="26"/>
+      <c r="E33" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="F33" s="38"/>
-      <c r="G33" s="38"/>
-      <c r="H33" s="38"/>
-      <c r="I33" s="39"/>
+      <c r="F33" s="69"/>
+      <c r="G33" s="69"/>
+      <c r="H33" s="69"/>
+      <c r="I33" s="70"/>
     </row>
     <row r="34" spans="2:9" ht="190" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C34" s="33" t="s">
+      <c r="C34" s="67" t="s">
         <v>31</v>
       </c>
-      <c r="D34" s="33"/>
-      <c r="E34" s="33"/>
-      <c r="F34" s="33"/>
-      <c r="G34" s="33"/>
-      <c r="H34" s="33"/>
-      <c r="I34" s="33"/>
+      <c r="D34" s="67"/>
+      <c r="E34" s="67"/>
+      <c r="F34" s="67"/>
+      <c r="G34" s="67"/>
+      <c r="H34" s="67"/>
+      <c r="I34" s="67"/>
     </row>
     <row r="35" spans="2:9" ht="10" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="41"/>
-      <c r="C35" s="42"/>
-      <c r="D35" s="42"/>
-      <c r="E35" s="42"/>
-      <c r="F35" s="42"/>
-      <c r="G35" s="42"/>
-      <c r="H35" s="42"/>
-      <c r="I35" s="43"/>
+      <c r="B35" s="36"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="37"/>
+      <c r="E35" s="37"/>
+      <c r="F35" s="37"/>
+      <c r="G35" s="37"/>
+      <c r="H35" s="37"/>
+      <c r="I35" s="38"/>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B36" s="23" t="s">
+      <c r="B36" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="C36" s="23"/>
-      <c r="D36" s="23"/>
-      <c r="E36" s="23"/>
-      <c r="F36" s="23"/>
-      <c r="G36" s="23"/>
-      <c r="H36" s="23"/>
-      <c r="I36" s="23"/>
+      <c r="C36" s="56"/>
+      <c r="D36" s="56"/>
+      <c r="E36" s="56"/>
+      <c r="F36" s="56"/>
+      <c r="G36" s="56"/>
+      <c r="H36" s="56"/>
+      <c r="I36" s="56"/>
     </row>
     <row r="37" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="27" t="s">
+      <c r="B37" s="64" t="s">
         <v>48</v>
       </c>
-      <c r="C37" s="27"/>
-      <c r="D37" s="27"/>
-      <c r="E37" s="27"/>
-      <c r="F37" s="27"/>
-      <c r="G37" s="27"/>
-      <c r="H37" s="27"/>
-      <c r="I37" s="27"/>
+      <c r="C37" s="64"/>
+      <c r="D37" s="64"/>
+      <c r="E37" s="64"/>
+      <c r="F37" s="64"/>
+      <c r="G37" s="64"/>
+      <c r="H37" s="64"/>
+      <c r="I37" s="64"/>
     </row>
     <row r="38" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="27"/>
-      <c r="C38" s="27"/>
-      <c r="D38" s="27"/>
-      <c r="E38" s="27"/>
-      <c r="F38" s="27"/>
-      <c r="G38" s="27"/>
-      <c r="H38" s="27"/>
-      <c r="I38" s="27"/>
+      <c r="B38" s="64"/>
+      <c r="C38" s="64"/>
+      <c r="D38" s="64"/>
+      <c r="E38" s="64"/>
+      <c r="F38" s="64"/>
+      <c r="G38" s="64"/>
+      <c r="H38" s="64"/>
+      <c r="I38" s="64"/>
     </row>
     <row r="39" spans="2:9" ht="132" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="27"/>
-      <c r="C39" s="27"/>
-      <c r="D39" s="27"/>
-      <c r="E39" s="27"/>
-      <c r="F39" s="27"/>
-      <c r="G39" s="27"/>
-      <c r="H39" s="27"/>
-      <c r="I39" s="27"/>
+      <c r="B39" s="64"/>
+      <c r="C39" s="64"/>
+      <c r="D39" s="64"/>
+      <c r="E39" s="64"/>
+      <c r="F39" s="64"/>
+      <c r="G39" s="64"/>
+      <c r="H39" s="64"/>
+      <c r="I39" s="64"/>
     </row>
     <row r="40" spans="2:9" ht="76" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B40" s="27"/>
-      <c r="C40" s="27"/>
-      <c r="D40" s="27"/>
-      <c r="E40" s="27"/>
-      <c r="F40" s="27"/>
-      <c r="G40" s="27"/>
-      <c r="H40" s="27"/>
-      <c r="I40" s="27"/>
+      <c r="B40" s="64"/>
+      <c r="C40" s="64"/>
+      <c r="D40" s="64"/>
+      <c r="E40" s="64"/>
+      <c r="F40" s="64"/>
+      <c r="G40" s="64"/>
+      <c r="H40" s="64"/>
+      <c r="I40" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="C26:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="E32:I32"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="B36:I36"/>
+    <mergeCell ref="B10:I12"/>
+    <mergeCell ref="B9:I9"/>
+    <mergeCell ref="B37:I40"/>
+    <mergeCell ref="C15:I15"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="E28:I28"/>
+    <mergeCell ref="E29:I29"/>
+    <mergeCell ref="E31:I31"/>
+    <mergeCell ref="C34:I34"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="E33:I33"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C31:D31"/>
     <mergeCell ref="B35:I35"/>
     <mergeCell ref="B13:I13"/>
     <mergeCell ref="C21:I21"/>
@@ -3779,28 +3792,15 @@
     <mergeCell ref="E24:I24"/>
     <mergeCell ref="C25:D25"/>
     <mergeCell ref="B26:B27"/>
-    <mergeCell ref="B36:I36"/>
-    <mergeCell ref="B10:I12"/>
-    <mergeCell ref="B9:I9"/>
-    <mergeCell ref="B37:I40"/>
-    <mergeCell ref="C15:I15"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="E28:I28"/>
-    <mergeCell ref="E29:I29"/>
-    <mergeCell ref="E31:I31"/>
-    <mergeCell ref="C34:I34"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="E33:I33"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C7:I7"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="C3:I3"/>
-    <mergeCell ref="C4:I4"/>
-    <mergeCell ref="C5:I5"/>
-    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="C26:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="E32:I32"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="G26:I26"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{C9E9977D-5134-FE4B-852F-8DEBDCB543E0}"/>
@@ -3829,12 +3829,12 @@
   </cols>
   <sheetData>
     <row r="4" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B4" s="25" t="s">
+      <c r="B4" s="73" t="s">
         <v>128</v>
       </c>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
+      <c r="C4" s="73"/>
+      <c r="D4" s="73"/>
+      <c r="E4" s="73"/>
     </row>
     <row r="5" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="11" t="s">
@@ -4105,442 +4105,421 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="74" t="s">
+      <c r="C3" s="92" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="75"/>
-      <c r="E3" s="75"/>
-      <c r="F3" s="75"/>
-      <c r="G3" s="75"/>
-      <c r="H3" s="75"/>
-      <c r="I3" s="75"/>
+      <c r="D3" s="93"/>
+      <c r="E3" s="93"/>
+      <c r="F3" s="93"/>
+      <c r="G3" s="93"/>
+      <c r="H3" s="93"/>
+      <c r="I3" s="93"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="66" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
+      <c r="D4" s="66"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="66"/>
+      <c r="G4" s="66"/>
+      <c r="H4" s="66"/>
+      <c r="I4" s="66"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="22">
+      <c r="C5" s="66">
         <v>2020</v>
       </c>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
+      <c r="D5" s="66"/>
+      <c r="E5" s="66"/>
+      <c r="F5" s="66"/>
+      <c r="G5" s="66"/>
+      <c r="H5" s="66"/>
+      <c r="I5" s="66"/>
     </row>
     <row r="6" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="68" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
+      <c r="D6" s="68"/>
+      <c r="E6" s="68"/>
+      <c r="F6" s="68"/>
+      <c r="G6" s="68"/>
+      <c r="H6" s="68"/>
+      <c r="I6" s="68"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="71" t="s">
         <v>51</v>
       </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="22"/>
+      <c r="D7" s="66"/>
+      <c r="E7" s="66"/>
+      <c r="F7" s="66"/>
+      <c r="G7" s="66"/>
+      <c r="H7" s="66"/>
+      <c r="I7" s="66"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="29"/>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="29"/>
-      <c r="I8" s="29"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="56" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="23"/>
+      <c r="C9" s="56"/>
+      <c r="D9" s="56"/>
+      <c r="E9" s="56"/>
+      <c r="F9" s="56"/>
+      <c r="G9" s="56"/>
+      <c r="H9" s="56"/>
+      <c r="I9" s="56"/>
     </row>
     <row r="10" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="63" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
+      <c r="C10" s="63"/>
+      <c r="D10" s="63"/>
+      <c r="E10" s="63"/>
+      <c r="F10" s="63"/>
+      <c r="G10" s="63"/>
+      <c r="H10" s="63"/>
+      <c r="I10" s="63"/>
     </row>
     <row r="11" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="26"/>
+      <c r="B11" s="63"/>
+      <c r="C11" s="63"/>
+      <c r="D11" s="63"/>
+      <c r="E11" s="63"/>
+      <c r="F11" s="63"/>
+      <c r="G11" s="63"/>
+      <c r="H11" s="63"/>
+      <c r="I11" s="63"/>
     </row>
     <row r="12" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="26"/>
+      <c r="B12" s="63"/>
+      <c r="C12" s="63"/>
+      <c r="D12" s="63"/>
+      <c r="E12" s="63"/>
+      <c r="F12" s="63"/>
+      <c r="G12" s="63"/>
+      <c r="H12" s="63"/>
+      <c r="I12" s="63"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="29"/>
-      <c r="C13" s="29"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="29"/>
-      <c r="F13" s="29"/>
-      <c r="G13" s="29"/>
-      <c r="H13" s="29"/>
-      <c r="I13" s="29"/>
+      <c r="B13" s="30"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="30"/>
+      <c r="I13" s="30"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="23" t="s">
+      <c r="B14" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23"/>
-      <c r="H14" s="23"/>
-      <c r="I14" s="23"/>
+      <c r="C14" s="56"/>
+      <c r="D14" s="56"/>
+      <c r="E14" s="56"/>
+      <c r="F14" s="56"/>
+      <c r="G14" s="56"/>
+      <c r="H14" s="56"/>
+      <c r="I14" s="56"/>
     </row>
     <row r="15" spans="2:9" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="28" t="s">
+      <c r="C15" s="65" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="22"/>
-      <c r="I15" s="22"/>
+      <c r="D15" s="66"/>
+      <c r="E15" s="66"/>
+      <c r="F15" s="66"/>
+      <c r="G15" s="66"/>
+      <c r="H15" s="66"/>
+      <c r="I15" s="66"/>
     </row>
     <row r="16" spans="2:9" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="47" t="s">
+      <c r="B16" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="76" t="s">
+      <c r="C16" s="83" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="77"/>
-      <c r="E16" s="77"/>
-      <c r="F16" s="77"/>
-      <c r="G16" s="77"/>
-      <c r="H16" s="77"/>
-      <c r="I16" s="78"/>
+      <c r="D16" s="84"/>
+      <c r="E16" s="84"/>
+      <c r="F16" s="84"/>
+      <c r="G16" s="84"/>
+      <c r="H16" s="84"/>
+      <c r="I16" s="85"/>
     </row>
     <row r="17" spans="2:9" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="48"/>
-      <c r="C17" s="79"/>
-      <c r="D17" s="80"/>
-      <c r="E17" s="80"/>
-      <c r="F17" s="80"/>
-      <c r="G17" s="80"/>
-      <c r="H17" s="80"/>
-      <c r="I17" s="81"/>
+      <c r="B17" s="46"/>
+      <c r="C17" s="86"/>
+      <c r="D17" s="87"/>
+      <c r="E17" s="87"/>
+      <c r="F17" s="87"/>
+      <c r="G17" s="87"/>
+      <c r="H17" s="87"/>
+      <c r="I17" s="88"/>
     </row>
     <row r="18" spans="2:9" ht="135" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="65" t="s">
         <v>56</v>
       </c>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
+      <c r="D18" s="66"/>
+      <c r="E18" s="66"/>
+      <c r="F18" s="66"/>
+      <c r="G18" s="66"/>
+      <c r="H18" s="66"/>
+      <c r="I18" s="66"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="29"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="29"/>
-      <c r="G19" s="29"/>
-      <c r="H19" s="29"/>
-      <c r="I19" s="29"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="30"/>
+      <c r="I19" s="30"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="56" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="23"/>
+      <c r="C20" s="56"/>
+      <c r="D20" s="56"/>
+      <c r="E20" s="56"/>
+      <c r="F20" s="56"/>
+      <c r="G20" s="56"/>
+      <c r="H20" s="56"/>
+      <c r="I20" s="56"/>
     </row>
     <row r="21" spans="2:9" ht="160" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="82" t="s">
+      <c r="C21" s="89" t="s">
         <v>57</v>
       </c>
-      <c r="D21" s="83"/>
-      <c r="E21" s="83"/>
-      <c r="F21" s="83"/>
-      <c r="G21" s="83"/>
-      <c r="H21" s="83"/>
-      <c r="I21" s="84"/>
+      <c r="D21" s="90"/>
+      <c r="E21" s="90"/>
+      <c r="F21" s="90"/>
+      <c r="G21" s="90"/>
+      <c r="H21" s="90"/>
+      <c r="I21" s="91"/>
     </row>
     <row r="22" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="37">
+      <c r="C22" s="42">
         <v>3</v>
       </c>
-      <c r="D22" s="45"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="45"/>
-      <c r="H22" s="45"/>
-      <c r="I22" s="46"/>
+      <c r="D22" s="43"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="43"/>
+      <c r="H22" s="43"/>
+      <c r="I22" s="44"/>
     </row>
     <row r="23" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="59" t="s">
+      <c r="C23" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="59"/>
-      <c r="E23" s="60" t="s">
+      <c r="D23" s="57"/>
+      <c r="E23" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="60"/>
-      <c r="G23" s="60"/>
-      <c r="H23" s="60"/>
-      <c r="I23" s="60"/>
+      <c r="F23" s="58"/>
+      <c r="G23" s="58"/>
+      <c r="H23" s="58"/>
+      <c r="I23" s="58"/>
     </row>
     <row r="24" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="63">
+      <c r="B24" s="61">
         <v>1</v>
       </c>
-      <c r="C24" s="90" t="s">
+      <c r="C24" s="74" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="91"/>
+      <c r="D24" s="75"/>
       <c r="E24" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="F24" s="92" t="s">
+      <c r="F24" s="78" t="s">
         <v>63</v>
       </c>
-      <c r="G24" s="92"/>
-      <c r="H24" s="92"/>
-      <c r="I24" s="93"/>
+      <c r="G24" s="78"/>
+      <c r="H24" s="78"/>
+      <c r="I24" s="79"/>
     </row>
     <row r="25" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="64"/>
-      <c r="C25" s="88"/>
-      <c r="D25" s="89"/>
+      <c r="B25" s="62"/>
+      <c r="C25" s="76"/>
+      <c r="D25" s="77"/>
       <c r="E25" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="F25" s="73" t="s">
+      <c r="F25" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="G25" s="73"/>
-      <c r="H25" s="73"/>
-      <c r="I25" s="58"/>
+      <c r="G25" s="33"/>
+      <c r="H25" s="33"/>
+      <c r="I25" s="34"/>
     </row>
     <row r="26" spans="2:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="8">
         <v>2</v>
       </c>
-      <c r="C26" s="86" t="s">
+      <c r="C26" s="81" t="s">
         <v>59</v>
       </c>
-      <c r="D26" s="87"/>
-      <c r="E26" s="35"/>
-      <c r="F26" s="72"/>
-      <c r="G26" s="72"/>
-      <c r="H26" s="72"/>
-      <c r="I26" s="36"/>
+      <c r="D26" s="82"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="26"/>
     </row>
     <row r="27" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="8">
         <v>3</v>
       </c>
-      <c r="C27" s="88" t="s">
+      <c r="C27" s="76" t="s">
         <v>60</v>
       </c>
-      <c r="D27" s="89"/>
-      <c r="E27" s="35"/>
-      <c r="F27" s="72"/>
-      <c r="G27" s="72"/>
-      <c r="H27" s="72"/>
-      <c r="I27" s="36"/>
+      <c r="D27" s="77"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="31"/>
+      <c r="G27" s="31"/>
+      <c r="H27" s="31"/>
+      <c r="I27" s="26"/>
     </row>
     <row r="28" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B28" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C28" s="33" t="s">
+      <c r="C28" s="67" t="s">
         <v>65</v>
       </c>
-      <c r="D28" s="33"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="33"/>
-      <c r="H28" s="33"/>
-      <c r="I28" s="33"/>
+      <c r="D28" s="67"/>
+      <c r="E28" s="67"/>
+      <c r="F28" s="67"/>
+      <c r="G28" s="67"/>
+      <c r="H28" s="67"/>
+      <c r="I28" s="67"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B29" s="41"/>
-      <c r="C29" s="42"/>
-      <c r="D29" s="42"/>
-      <c r="E29" s="42"/>
-      <c r="F29" s="42"/>
-      <c r="G29" s="42"/>
-      <c r="H29" s="42"/>
-      <c r="I29" s="43"/>
+      <c r="B29" s="36"/>
+      <c r="C29" s="37"/>
+      <c r="D29" s="37"/>
+      <c r="E29" s="37"/>
+      <c r="F29" s="37"/>
+      <c r="G29" s="37"/>
+      <c r="H29" s="37"/>
+      <c r="I29" s="38"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B30" s="23" t="s">
+      <c r="B30" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="C30" s="23"/>
-      <c r="D30" s="23"/>
-      <c r="E30" s="23"/>
-      <c r="F30" s="23"/>
-      <c r="G30" s="23"/>
-      <c r="H30" s="23"/>
-      <c r="I30" s="23"/>
+      <c r="C30" s="56"/>
+      <c r="D30" s="56"/>
+      <c r="E30" s="56"/>
+      <c r="F30" s="56"/>
+      <c r="G30" s="56"/>
+      <c r="H30" s="56"/>
+      <c r="I30" s="56"/>
     </row>
     <row r="31" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="85" t="s">
+      <c r="B31" s="80" t="s">
         <v>66</v>
       </c>
-      <c r="C31" s="27"/>
-      <c r="D31" s="27"/>
-      <c r="E31" s="27"/>
-      <c r="F31" s="27"/>
-      <c r="G31" s="27"/>
-      <c r="H31" s="27"/>
-      <c r="I31" s="27"/>
+      <c r="C31" s="64"/>
+      <c r="D31" s="64"/>
+      <c r="E31" s="64"/>
+      <c r="F31" s="64"/>
+      <c r="G31" s="64"/>
+      <c r="H31" s="64"/>
+      <c r="I31" s="64"/>
     </row>
     <row r="32" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="27"/>
-      <c r="C32" s="27"/>
-      <c r="D32" s="27"/>
-      <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
-      <c r="G32" s="27"/>
-      <c r="H32" s="27"/>
-      <c r="I32" s="27"/>
+      <c r="B32" s="64"/>
+      <c r="C32" s="64"/>
+      <c r="D32" s="64"/>
+      <c r="E32" s="64"/>
+      <c r="F32" s="64"/>
+      <c r="G32" s="64"/>
+      <c r="H32" s="64"/>
+      <c r="I32" s="64"/>
     </row>
     <row r="33" spans="2:9" ht="124" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="27"/>
-      <c r="C33" s="27"/>
-      <c r="D33" s="27"/>
-      <c r="E33" s="27"/>
-      <c r="F33" s="27"/>
-      <c r="G33" s="27"/>
-      <c r="H33" s="27"/>
-      <c r="I33" s="27"/>
+      <c r="B33" s="64"/>
+      <c r="C33" s="64"/>
+      <c r="D33" s="64"/>
+      <c r="E33" s="64"/>
+      <c r="F33" s="64"/>
+      <c r="G33" s="64"/>
+      <c r="H33" s="64"/>
+      <c r="I33" s="64"/>
     </row>
     <row r="34" spans="2:9" ht="254" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="27"/>
-      <c r="C34" s="27"/>
-      <c r="D34" s="27"/>
-      <c r="E34" s="27"/>
-      <c r="F34" s="27"/>
-      <c r="G34" s="27"/>
-      <c r="H34" s="27"/>
-      <c r="I34" s="27"/>
+      <c r="B34" s="64"/>
+      <c r="C34" s="64"/>
+      <c r="D34" s="64"/>
+      <c r="E34" s="64"/>
+      <c r="F34" s="64"/>
+      <c r="G34" s="64"/>
+      <c r="H34" s="64"/>
+      <c r="I34" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:D25"/>
-    <mergeCell ref="F24:I24"/>
-    <mergeCell ref="F25:I25"/>
-    <mergeCell ref="C28:I28"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="B31:I34"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:I27"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="C21:I21"/>
     <mergeCell ref="C15:I15"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -4553,6 +4532,27 @@
     <mergeCell ref="B10:I12"/>
     <mergeCell ref="B13:I13"/>
     <mergeCell ref="B14:I14"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="B31:I34"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:D25"/>
+    <mergeCell ref="F24:I24"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="C28:I28"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{4DBC988E-4FF2-2C49-AA18-DD92CA6A87E8}"/>
@@ -4586,424 +4586,405 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="74" t="s">
+      <c r="C3" s="92" t="s">
         <v>67</v>
       </c>
-      <c r="D3" s="75"/>
-      <c r="E3" s="75"/>
-      <c r="F3" s="75"/>
-      <c r="G3" s="75"/>
-      <c r="H3" s="75"/>
-      <c r="I3" s="75"/>
+      <c r="D3" s="93"/>
+      <c r="E3" s="93"/>
+      <c r="F3" s="93"/>
+      <c r="G3" s="93"/>
+      <c r="H3" s="93"/>
+      <c r="I3" s="93"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="66" t="s">
         <v>68</v>
       </c>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
+      <c r="D4" s="66"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="66"/>
+      <c r="G4" s="66"/>
+      <c r="H4" s="66"/>
+      <c r="I4" s="66"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="22">
+      <c r="C5" s="66">
         <v>2022</v>
       </c>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
+      <c r="D5" s="66"/>
+      <c r="E5" s="66"/>
+      <c r="F5" s="66"/>
+      <c r="G5" s="66"/>
+      <c r="H5" s="66"/>
+      <c r="I5" s="66"/>
     </row>
     <row r="6" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="68" t="s">
         <v>69</v>
       </c>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
+      <c r="D6" s="68"/>
+      <c r="E6" s="68"/>
+      <c r="F6" s="68"/>
+      <c r="G6" s="68"/>
+      <c r="H6" s="68"/>
+      <c r="I6" s="68"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="71" t="s">
         <v>70</v>
       </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="22"/>
+      <c r="D7" s="66"/>
+      <c r="E7" s="66"/>
+      <c r="F7" s="66"/>
+      <c r="G7" s="66"/>
+      <c r="H7" s="66"/>
+      <c r="I7" s="66"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="29"/>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="29"/>
-      <c r="I8" s="29"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="56" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="23"/>
+      <c r="C9" s="56"/>
+      <c r="D9" s="56"/>
+      <c r="E9" s="56"/>
+      <c r="F9" s="56"/>
+      <c r="G9" s="56"/>
+      <c r="H9" s="56"/>
+      <c r="I9" s="56"/>
     </row>
     <row r="10" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="63" t="s">
         <v>71</v>
       </c>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
+      <c r="C10" s="63"/>
+      <c r="D10" s="63"/>
+      <c r="E10" s="63"/>
+      <c r="F10" s="63"/>
+      <c r="G10" s="63"/>
+      <c r="H10" s="63"/>
+      <c r="I10" s="63"/>
     </row>
     <row r="11" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="26"/>
+      <c r="B11" s="63"/>
+      <c r="C11" s="63"/>
+      <c r="D11" s="63"/>
+      <c r="E11" s="63"/>
+      <c r="F11" s="63"/>
+      <c r="G11" s="63"/>
+      <c r="H11" s="63"/>
+      <c r="I11" s="63"/>
     </row>
     <row r="12" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="26"/>
+      <c r="B12" s="63"/>
+      <c r="C12" s="63"/>
+      <c r="D12" s="63"/>
+      <c r="E12" s="63"/>
+      <c r="F12" s="63"/>
+      <c r="G12" s="63"/>
+      <c r="H12" s="63"/>
+      <c r="I12" s="63"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="29"/>
-      <c r="C13" s="29"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="29"/>
-      <c r="F13" s="29"/>
-      <c r="G13" s="29"/>
-      <c r="H13" s="29"/>
-      <c r="I13" s="29"/>
+      <c r="B13" s="30"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="30"/>
+      <c r="I13" s="30"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="23" t="s">
+      <c r="B14" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23"/>
-      <c r="H14" s="23"/>
-      <c r="I14" s="23"/>
+      <c r="C14" s="56"/>
+      <c r="D14" s="56"/>
+      <c r="E14" s="56"/>
+      <c r="F14" s="56"/>
+      <c r="G14" s="56"/>
+      <c r="H14" s="56"/>
+      <c r="I14" s="56"/>
     </row>
     <row r="15" spans="2:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="28" t="s">
+      <c r="C15" s="65" t="s">
         <v>73</v>
       </c>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="22"/>
-      <c r="I15" s="22"/>
+      <c r="D15" s="66"/>
+      <c r="E15" s="66"/>
+      <c r="F15" s="66"/>
+      <c r="G15" s="66"/>
+      <c r="H15" s="66"/>
+      <c r="I15" s="66"/>
     </row>
     <row r="16" spans="2:9" ht="247" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="47" t="s">
+      <c r="B16" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="76" t="s">
+      <c r="C16" s="83" t="s">
         <v>72</v>
       </c>
-      <c r="D16" s="77"/>
-      <c r="E16" s="77"/>
-      <c r="F16" s="77"/>
-      <c r="G16" s="77"/>
-      <c r="H16" s="77"/>
-      <c r="I16" s="78"/>
+      <c r="D16" s="84"/>
+      <c r="E16" s="84"/>
+      <c r="F16" s="84"/>
+      <c r="G16" s="84"/>
+      <c r="H16" s="84"/>
+      <c r="I16" s="85"/>
     </row>
     <row r="17" spans="2:9" ht="247" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="48"/>
-      <c r="C17" s="79"/>
-      <c r="D17" s="80"/>
-      <c r="E17" s="80"/>
-      <c r="F17" s="80"/>
-      <c r="G17" s="80"/>
-      <c r="H17" s="80"/>
-      <c r="I17" s="81"/>
+      <c r="B17" s="46"/>
+      <c r="C17" s="86"/>
+      <c r="D17" s="87"/>
+      <c r="E17" s="87"/>
+      <c r="F17" s="87"/>
+      <c r="G17" s="87"/>
+      <c r="H17" s="87"/>
+      <c r="I17" s="88"/>
     </row>
     <row r="18" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="94"/>
-      <c r="D18" s="95"/>
-      <c r="E18" s="95"/>
-      <c r="F18" s="95"/>
-      <c r="G18" s="95"/>
-      <c r="H18" s="95"/>
-      <c r="I18" s="95"/>
+      <c r="C18" s="100"/>
+      <c r="D18" s="101"/>
+      <c r="E18" s="101"/>
+      <c r="F18" s="101"/>
+      <c r="G18" s="101"/>
+      <c r="H18" s="101"/>
+      <c r="I18" s="101"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="29"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="29"/>
-      <c r="G19" s="29"/>
-      <c r="H19" s="29"/>
-      <c r="I19" s="29"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="30"/>
+      <c r="I19" s="30"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="56" t="s">
         <v>77</v>
       </c>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="23"/>
+      <c r="C20" s="56"/>
+      <c r="D20" s="56"/>
+      <c r="E20" s="56"/>
+      <c r="F20" s="56"/>
+      <c r="G20" s="56"/>
+      <c r="H20" s="56"/>
+      <c r="I20" s="56"/>
     </row>
     <row r="21" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="82" t="s">
+      <c r="C21" s="89" t="s">
         <v>74</v>
       </c>
-      <c r="D21" s="83"/>
-      <c r="E21" s="83"/>
-      <c r="F21" s="83"/>
-      <c r="G21" s="83"/>
-      <c r="H21" s="83"/>
-      <c r="I21" s="84"/>
+      <c r="D21" s="90"/>
+      <c r="E21" s="90"/>
+      <c r="F21" s="90"/>
+      <c r="G21" s="90"/>
+      <c r="H21" s="90"/>
+      <c r="I21" s="91"/>
     </row>
     <row r="22" spans="2:9" ht="165" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="37" t="s">
+      <c r="C22" s="42" t="s">
         <v>174</v>
       </c>
-      <c r="D22" s="45"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="45"/>
-      <c r="H22" s="45"/>
-      <c r="I22" s="46"/>
+      <c r="D22" s="43"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="43"/>
+      <c r="H22" s="43"/>
+      <c r="I22" s="44"/>
     </row>
     <row r="23" spans="2:9" ht="34" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="59" t="s">
+      <c r="C23" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="59"/>
-      <c r="E23" s="60" t="s">
+      <c r="D23" s="57"/>
+      <c r="E23" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="60"/>
-      <c r="G23" s="60"/>
-      <c r="H23" s="60"/>
-      <c r="I23" s="60"/>
+      <c r="F23" s="58"/>
+      <c r="G23" s="58"/>
+      <c r="H23" s="58"/>
+      <c r="I23" s="58"/>
     </row>
     <row r="24" spans="2:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="98" t="s">
+      <c r="C24" s="96" t="s">
         <v>75</v>
       </c>
-      <c r="D24" s="98"/>
-      <c r="E24" s="99" t="s">
+      <c r="D24" s="96"/>
+      <c r="E24" s="97" t="s">
         <v>177</v>
       </c>
-      <c r="F24" s="99"/>
-      <c r="G24" s="99"/>
-      <c r="H24" s="99"/>
-      <c r="I24" s="99"/>
+      <c r="F24" s="97"/>
+      <c r="G24" s="97"/>
+      <c r="H24" s="97"/>
+      <c r="I24" s="97"/>
     </row>
     <row r="25" spans="2:9" ht="56" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="8">
         <v>2</v>
       </c>
-      <c r="C25" s="98" t="s">
+      <c r="C25" s="96" t="s">
         <v>172</v>
       </c>
-      <c r="D25" s="98"/>
-      <c r="E25" s="74" t="s">
+      <c r="D25" s="96"/>
+      <c r="E25" s="92" t="s">
         <v>175</v>
       </c>
-      <c r="F25" s="74"/>
-      <c r="G25" s="74"/>
-      <c r="H25" s="74"/>
-      <c r="I25" s="74"/>
+      <c r="F25" s="92"/>
+      <c r="G25" s="92"/>
+      <c r="H25" s="92"/>
+      <c r="I25" s="92"/>
     </row>
     <row r="26" spans="2:9" ht="71" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="8">
         <v>3</v>
       </c>
-      <c r="C26" s="100" t="s">
+      <c r="C26" s="98" t="s">
         <v>173</v>
       </c>
-      <c r="D26" s="101"/>
-      <c r="E26" s="44" t="s">
+      <c r="D26" s="99"/>
+      <c r="E26" s="39" t="s">
         <v>176</v>
       </c>
-      <c r="F26" s="92"/>
-      <c r="G26" s="92"/>
-      <c r="H26" s="92"/>
-      <c r="I26" s="93"/>
+      <c r="F26" s="78"/>
+      <c r="G26" s="78"/>
+      <c r="H26" s="78"/>
+      <c r="I26" s="79"/>
     </row>
     <row r="27" spans="2:9" ht="68" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="33" t="s">
+      <c r="C27" s="67" t="s">
         <v>76</v>
       </c>
-      <c r="D27" s="33"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="33"/>
-      <c r="G27" s="33"/>
-      <c r="H27" s="33"/>
-      <c r="I27" s="33"/>
+      <c r="D27" s="67"/>
+      <c r="E27" s="67"/>
+      <c r="F27" s="67"/>
+      <c r="G27" s="67"/>
+      <c r="H27" s="67"/>
+      <c r="I27" s="67"/>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B28" s="41"/>
-      <c r="C28" s="42"/>
-      <c r="D28" s="42"/>
-      <c r="E28" s="42"/>
-      <c r="F28" s="42"/>
-      <c r="G28" s="42"/>
-      <c r="H28" s="42"/>
-      <c r="I28" s="43"/>
+      <c r="B28" s="36"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="37"/>
+      <c r="E28" s="37"/>
+      <c r="F28" s="37"/>
+      <c r="G28" s="37"/>
+      <c r="H28" s="37"/>
+      <c r="I28" s="38"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B29" s="23" t="s">
+      <c r="B29" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="C29" s="23"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="23"/>
-      <c r="H29" s="23"/>
-      <c r="I29" s="23"/>
+      <c r="C29" s="56"/>
+      <c r="D29" s="56"/>
+      <c r="E29" s="56"/>
+      <c r="F29" s="56"/>
+      <c r="G29" s="56"/>
+      <c r="H29" s="56"/>
+      <c r="I29" s="56"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B30" s="96"/>
-      <c r="C30" s="97"/>
-      <c r="D30" s="97"/>
-      <c r="E30" s="97"/>
-      <c r="F30" s="97"/>
-      <c r="G30" s="97"/>
-      <c r="H30" s="97"/>
-      <c r="I30" s="97"/>
+      <c r="B30" s="94"/>
+      <c r="C30" s="95"/>
+      <c r="D30" s="95"/>
+      <c r="E30" s="95"/>
+      <c r="F30" s="95"/>
+      <c r="G30" s="95"/>
+      <c r="H30" s="95"/>
+      <c r="I30" s="95"/>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B31" s="97"/>
-      <c r="C31" s="97"/>
-      <c r="D31" s="97"/>
-      <c r="E31" s="97"/>
-      <c r="F31" s="97"/>
-      <c r="G31" s="97"/>
-      <c r="H31" s="97"/>
-      <c r="I31" s="97"/>
+      <c r="B31" s="95"/>
+      <c r="C31" s="95"/>
+      <c r="D31" s="95"/>
+      <c r="E31" s="95"/>
+      <c r="F31" s="95"/>
+      <c r="G31" s="95"/>
+      <c r="H31" s="95"/>
+      <c r="I31" s="95"/>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B32" s="97"/>
-      <c r="C32" s="97"/>
-      <c r="D32" s="97"/>
-      <c r="E32" s="97"/>
-      <c r="F32" s="97"/>
-      <c r="G32" s="97"/>
-      <c r="H32" s="97"/>
-      <c r="I32" s="97"/>
+      <c r="B32" s="95"/>
+      <c r="C32" s="95"/>
+      <c r="D32" s="95"/>
+      <c r="E32" s="95"/>
+      <c r="F32" s="95"/>
+      <c r="G32" s="95"/>
+      <c r="H32" s="95"/>
+      <c r="I32" s="95"/>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B33" s="97"/>
-      <c r="C33" s="97"/>
-      <c r="D33" s="97"/>
-      <c r="E33" s="97"/>
-      <c r="F33" s="97"/>
-      <c r="G33" s="97"/>
-      <c r="H33" s="97"/>
-      <c r="I33" s="97"/>
+      <c r="B33" s="95"/>
+      <c r="C33" s="95"/>
+      <c r="D33" s="95"/>
+      <c r="E33" s="95"/>
+      <c r="F33" s="95"/>
+      <c r="G33" s="95"/>
+      <c r="H33" s="95"/>
+      <c r="I33" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:I33"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="C27:I27"/>
-    <mergeCell ref="B28:I28"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="C21:I21"/>
     <mergeCell ref="C15:I15"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -5016,6 +4997,25 @@
     <mergeCell ref="B10:I12"/>
     <mergeCell ref="B13:I13"/>
     <mergeCell ref="B14:I14"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:I33"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="C27:I27"/>
+    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:I26"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{60ABBC95-3763-1140-8147-BC4DA0DFC780}"/>
@@ -5178,499 +5178,525 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B1" s="102"/>
-      <c r="C1" s="102"/>
-      <c r="D1" s="102"/>
-      <c r="E1" s="102"/>
-      <c r="F1" s="102"/>
-      <c r="G1" s="102"/>
-      <c r="H1" s="102"/>
-      <c r="I1" s="102"/>
+      <c r="B1" s="103"/>
+      <c r="C1" s="103"/>
+      <c r="D1" s="103"/>
+      <c r="E1" s="103"/>
+      <c r="F1" s="103"/>
+      <c r="G1" s="103"/>
+      <c r="H1" s="103"/>
+      <c r="I1" s="103"/>
     </row>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
     </row>
     <row r="3" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="74" t="s">
+      <c r="C3" s="92" t="s">
         <v>78</v>
       </c>
-      <c r="D3" s="75"/>
-      <c r="E3" s="75"/>
-      <c r="F3" s="75"/>
-      <c r="G3" s="75"/>
-      <c r="H3" s="75"/>
-      <c r="I3" s="75"/>
+      <c r="D3" s="93"/>
+      <c r="E3" s="93"/>
+      <c r="F3" s="93"/>
+      <c r="G3" s="93"/>
+      <c r="H3" s="93"/>
+      <c r="I3" s="93"/>
     </row>
     <row r="4" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="66" t="s">
         <v>79</v>
       </c>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
+      <c r="D4" s="66"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="66"/>
+      <c r="G4" s="66"/>
+      <c r="H4" s="66"/>
+      <c r="I4" s="66"/>
     </row>
     <row r="5" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="22">
+      <c r="C5" s="66">
         <v>2025</v>
       </c>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
+      <c r="D5" s="66"/>
+      <c r="E5" s="66"/>
+      <c r="F5" s="66"/>
+      <c r="G5" s="66"/>
+      <c r="H5" s="66"/>
+      <c r="I5" s="66"/>
     </row>
     <row r="6" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="68" t="s">
         <v>81</v>
       </c>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
+      <c r="D6" s="68"/>
+      <c r="E6" s="68"/>
+      <c r="F6" s="68"/>
+      <c r="G6" s="68"/>
+      <c r="H6" s="68"/>
+      <c r="I6" s="68"/>
     </row>
     <row r="7" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="71" t="s">
         <v>80</v>
       </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="22"/>
+      <c r="D7" s="66"/>
+      <c r="E7" s="66"/>
+      <c r="F7" s="66"/>
+      <c r="G7" s="66"/>
+      <c r="H7" s="66"/>
+      <c r="I7" s="66"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="29"/>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="29"/>
-      <c r="I8" s="29"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="56" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="23"/>
+      <c r="C9" s="56"/>
+      <c r="D9" s="56"/>
+      <c r="E9" s="56"/>
+      <c r="F9" s="56"/>
+      <c r="G9" s="56"/>
+      <c r="H9" s="56"/>
+      <c r="I9" s="56"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="63" t="s">
         <v>82</v>
       </c>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
+      <c r="C10" s="63"/>
+      <c r="D10" s="63"/>
+      <c r="E10" s="63"/>
+      <c r="F10" s="63"/>
+      <c r="G10" s="63"/>
+      <c r="H10" s="63"/>
+      <c r="I10" s="63"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="26"/>
+      <c r="B11" s="63"/>
+      <c r="C11" s="63"/>
+      <c r="D11" s="63"/>
+      <c r="E11" s="63"/>
+      <c r="F11" s="63"/>
+      <c r="G11" s="63"/>
+      <c r="H11" s="63"/>
+      <c r="I11" s="63"/>
     </row>
     <row r="12" spans="2:9" ht="92" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="26"/>
+      <c r="B12" s="63"/>
+      <c r="C12" s="63"/>
+      <c r="D12" s="63"/>
+      <c r="E12" s="63"/>
+      <c r="F12" s="63"/>
+      <c r="G12" s="63"/>
+      <c r="H12" s="63"/>
+      <c r="I12" s="63"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="29"/>
-      <c r="C13" s="29"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="29"/>
-      <c r="F13" s="29"/>
-      <c r="G13" s="29"/>
-      <c r="H13" s="29"/>
-      <c r="I13" s="29"/>
+      <c r="B13" s="30"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="30"/>
+      <c r="I13" s="30"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="23" t="s">
+      <c r="B14" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23"/>
-      <c r="H14" s="23"/>
-      <c r="I14" s="23"/>
+      <c r="C14" s="56"/>
+      <c r="D14" s="56"/>
+      <c r="E14" s="56"/>
+      <c r="F14" s="56"/>
+      <c r="G14" s="56"/>
+      <c r="H14" s="56"/>
+      <c r="I14" s="56"/>
     </row>
     <row r="15" spans="2:9" ht="59" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="33" t="s">
+      <c r="C15" s="67" t="s">
         <v>83</v>
       </c>
-      <c r="D15" s="34"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="34"/>
-      <c r="G15" s="34"/>
-      <c r="H15" s="34"/>
-      <c r="I15" s="34"/>
+      <c r="D15" s="68"/>
+      <c r="E15" s="68"/>
+      <c r="F15" s="68"/>
+      <c r="G15" s="68"/>
+      <c r="H15" s="68"/>
+      <c r="I15" s="68"/>
     </row>
     <row r="16" spans="2:9" ht="59" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="47" t="s">
+      <c r="B16" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="76" t="s">
+      <c r="C16" s="83" t="s">
         <v>84</v>
       </c>
-      <c r="D16" s="77"/>
-      <c r="E16" s="77"/>
-      <c r="F16" s="77"/>
-      <c r="G16" s="77"/>
-      <c r="H16" s="77"/>
-      <c r="I16" s="78"/>
+      <c r="D16" s="84"/>
+      <c r="E16" s="84"/>
+      <c r="F16" s="84"/>
+      <c r="G16" s="84"/>
+      <c r="H16" s="84"/>
+      <c r="I16" s="85"/>
     </row>
     <row r="17" spans="2:9" ht="113" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="48"/>
-      <c r="C17" s="79"/>
-      <c r="D17" s="80"/>
-      <c r="E17" s="80"/>
-      <c r="F17" s="80"/>
-      <c r="G17" s="80"/>
-      <c r="H17" s="80"/>
-      <c r="I17" s="81"/>
+      <c r="B17" s="46"/>
+      <c r="C17" s="86"/>
+      <c r="D17" s="87"/>
+      <c r="E17" s="87"/>
+      <c r="F17" s="87"/>
+      <c r="G17" s="87"/>
+      <c r="H17" s="87"/>
+      <c r="I17" s="88"/>
     </row>
     <row r="18" spans="2:9" ht="358" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="26" t="s">
+      <c r="C18" s="63" t="s">
         <v>85</v>
       </c>
-      <c r="D18" s="34"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="34"/>
-      <c r="G18" s="34"/>
-      <c r="H18" s="34"/>
-      <c r="I18" s="34"/>
+      <c r="D18" s="68"/>
+      <c r="E18" s="68"/>
+      <c r="F18" s="68"/>
+      <c r="G18" s="68"/>
+      <c r="H18" s="68"/>
+      <c r="I18" s="68"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="29"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="29"/>
-      <c r="G19" s="29"/>
-      <c r="H19" s="29"/>
-      <c r="I19" s="29"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="30"/>
+      <c r="I19" s="30"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="56" t="s">
         <v>77</v>
       </c>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="23"/>
+      <c r="C20" s="56"/>
+      <c r="D20" s="56"/>
+      <c r="E20" s="56"/>
+      <c r="F20" s="56"/>
+      <c r="G20" s="56"/>
+      <c r="H20" s="56"/>
+      <c r="I20" s="56"/>
     </row>
     <row r="21" spans="2:9" ht="332" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="82" t="s">
+      <c r="C21" s="89" t="s">
         <v>86</v>
       </c>
-      <c r="D21" s="83"/>
-      <c r="E21" s="83"/>
-      <c r="F21" s="83"/>
-      <c r="G21" s="83"/>
-      <c r="H21" s="83"/>
-      <c r="I21" s="84"/>
+      <c r="D21" s="90"/>
+      <c r="E21" s="90"/>
+      <c r="F21" s="90"/>
+      <c r="G21" s="90"/>
+      <c r="H21" s="90"/>
+      <c r="I21" s="91"/>
     </row>
     <row r="22" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="37">
+      <c r="C22" s="42">
         <v>8</v>
       </c>
-      <c r="D22" s="45"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="45"/>
-      <c r="H22" s="45"/>
-      <c r="I22" s="46"/>
+      <c r="D22" s="43"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="43"/>
+      <c r="H22" s="43"/>
+      <c r="I22" s="44"/>
     </row>
     <row r="23" spans="2:9" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="59" t="s">
+      <c r="C23" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="59"/>
-      <c r="E23" s="60" t="s">
+      <c r="D23" s="57"/>
+      <c r="E23" s="58" t="s">
         <v>97</v>
       </c>
-      <c r="F23" s="60"/>
-      <c r="G23" s="60"/>
-      <c r="H23" s="60"/>
-      <c r="I23" s="60"/>
+      <c r="F23" s="58"/>
+      <c r="G23" s="58"/>
+      <c r="H23" s="58"/>
+      <c r="I23" s="58"/>
     </row>
     <row r="24" spans="2:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="103" t="s">
+      <c r="C24" s="104" t="s">
         <v>88</v>
       </c>
-      <c r="D24" s="104"/>
-      <c r="E24" s="74" t="s">
+      <c r="D24" s="105"/>
+      <c r="E24" s="92" t="s">
         <v>171</v>
       </c>
-      <c r="F24" s="74"/>
-      <c r="G24" s="74"/>
-      <c r="H24" s="74"/>
-      <c r="I24" s="74"/>
+      <c r="F24" s="92"/>
+      <c r="G24" s="92"/>
+      <c r="H24" s="92"/>
+      <c r="I24" s="92"/>
     </row>
     <row r="25" spans="2:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="8">
         <v>2</v>
       </c>
-      <c r="C25" s="100" t="s">
+      <c r="C25" s="98" t="s">
         <v>89</v>
       </c>
-      <c r="D25" s="101"/>
-      <c r="E25" s="74" t="s">
+      <c r="D25" s="99"/>
+      <c r="E25" s="92" t="s">
         <v>103</v>
       </c>
-      <c r="F25" s="74"/>
-      <c r="G25" s="74"/>
-      <c r="H25" s="74"/>
-      <c r="I25" s="74"/>
+      <c r="F25" s="92"/>
+      <c r="G25" s="92"/>
+      <c r="H25" s="92"/>
+      <c r="I25" s="92"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B26" s="8">
         <v>3</v>
       </c>
-      <c r="C26" s="100" t="s">
+      <c r="C26" s="98" t="s">
         <v>90</v>
       </c>
-      <c r="D26" s="101"/>
-      <c r="E26" s="74" t="s">
+      <c r="D26" s="99"/>
+      <c r="E26" s="92" t="s">
         <v>102</v>
       </c>
-      <c r="F26" s="74"/>
-      <c r="G26" s="74"/>
-      <c r="H26" s="74"/>
-      <c r="I26" s="74"/>
+      <c r="F26" s="92"/>
+      <c r="G26" s="92"/>
+      <c r="H26" s="92"/>
+      <c r="I26" s="92"/>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B27" s="8">
         <v>4</v>
       </c>
-      <c r="C27" s="100" t="s">
+      <c r="C27" s="98" t="s">
         <v>91</v>
       </c>
-      <c r="D27" s="101"/>
-      <c r="E27" s="74" t="s">
+      <c r="D27" s="99"/>
+      <c r="E27" s="92" t="s">
         <v>101</v>
       </c>
-      <c r="F27" s="74"/>
-      <c r="G27" s="74"/>
-      <c r="H27" s="74"/>
-      <c r="I27" s="74"/>
+      <c r="F27" s="92"/>
+      <c r="G27" s="92"/>
+      <c r="H27" s="92"/>
+      <c r="I27" s="92"/>
     </row>
     <row r="28" spans="2:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="8">
         <v>5</v>
       </c>
-      <c r="C28" s="100" t="s">
+      <c r="C28" s="98" t="s">
         <v>92</v>
       </c>
-      <c r="D28" s="101"/>
-      <c r="E28" s="74" t="s">
+      <c r="D28" s="99"/>
+      <c r="E28" s="92" t="s">
         <v>100</v>
       </c>
-      <c r="F28" s="74"/>
-      <c r="G28" s="74"/>
-      <c r="H28" s="74"/>
-      <c r="I28" s="74"/>
+      <c r="F28" s="92"/>
+      <c r="G28" s="92"/>
+      <c r="H28" s="92"/>
+      <c r="I28" s="92"/>
     </row>
     <row r="29" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="8">
         <v>6</v>
       </c>
-      <c r="C29" s="98" t="s">
+      <c r="C29" s="96" t="s">
         <v>93</v>
       </c>
-      <c r="D29" s="98"/>
-      <c r="E29" s="74" t="s">
+      <c r="D29" s="96"/>
+      <c r="E29" s="92" t="s">
         <v>99</v>
       </c>
-      <c r="F29" s="74"/>
-      <c r="G29" s="74"/>
-      <c r="H29" s="74"/>
-      <c r="I29" s="74"/>
+      <c r="F29" s="92"/>
+      <c r="G29" s="92"/>
+      <c r="H29" s="92"/>
+      <c r="I29" s="92"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B30" s="8">
         <v>7</v>
       </c>
-      <c r="C30" s="98" t="s">
+      <c r="C30" s="96" t="s">
         <v>94</v>
       </c>
-      <c r="D30" s="98"/>
-      <c r="E30" s="74" t="s">
+      <c r="D30" s="96"/>
+      <c r="E30" s="92" t="s">
         <v>98</v>
       </c>
-      <c r="F30" s="105"/>
-      <c r="G30" s="105"/>
-      <c r="H30" s="105"/>
-      <c r="I30" s="105"/>
+      <c r="F30" s="102"/>
+      <c r="G30" s="102"/>
+      <c r="H30" s="102"/>
+      <c r="I30" s="102"/>
     </row>
     <row r="31" spans="2:9" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="8">
         <v>8</v>
       </c>
-      <c r="C31" s="100" t="s">
+      <c r="C31" s="98" t="s">
         <v>95</v>
       </c>
-      <c r="D31" s="101"/>
-      <c r="E31" s="37" t="s">
+      <c r="D31" s="99"/>
+      <c r="E31" s="42" t="s">
         <v>96</v>
       </c>
-      <c r="F31" s="38"/>
-      <c r="G31" s="38"/>
-      <c r="H31" s="38"/>
-      <c r="I31" s="39"/>
+      <c r="F31" s="69"/>
+      <c r="G31" s="69"/>
+      <c r="H31" s="69"/>
+      <c r="I31" s="70"/>
     </row>
     <row r="32" spans="2:9" ht="17" x14ac:dyDescent="0.2">
       <c r="B32" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C32" s="33" t="s">
+      <c r="C32" s="67" t="s">
         <v>87</v>
       </c>
-      <c r="D32" s="33"/>
-      <c r="E32" s="33"/>
-      <c r="F32" s="33"/>
-      <c r="G32" s="33"/>
-      <c r="H32" s="33"/>
-      <c r="I32" s="33"/>
+      <c r="D32" s="67"/>
+      <c r="E32" s="67"/>
+      <c r="F32" s="67"/>
+      <c r="G32" s="67"/>
+      <c r="H32" s="67"/>
+      <c r="I32" s="67"/>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B33" s="41"/>
-      <c r="C33" s="42"/>
-      <c r="D33" s="42"/>
-      <c r="E33" s="42"/>
-      <c r="F33" s="42"/>
-      <c r="G33" s="42"/>
-      <c r="H33" s="42"/>
-      <c r="I33" s="43"/>
+      <c r="B33" s="36"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="37"/>
+      <c r="E33" s="37"/>
+      <c r="F33" s="37"/>
+      <c r="G33" s="37"/>
+      <c r="H33" s="37"/>
+      <c r="I33" s="38"/>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B34" s="23" t="s">
+      <c r="B34" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="C34" s="23"/>
-      <c r="D34" s="23"/>
-      <c r="E34" s="23"/>
-      <c r="F34" s="23"/>
-      <c r="G34" s="23"/>
-      <c r="H34" s="23"/>
-      <c r="I34" s="23"/>
+      <c r="C34" s="56"/>
+      <c r="D34" s="56"/>
+      <c r="E34" s="56"/>
+      <c r="F34" s="56"/>
+      <c r="G34" s="56"/>
+      <c r="H34" s="56"/>
+      <c r="I34" s="56"/>
     </row>
     <row r="35" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="85" t="s">
+      <c r="B35" s="80" t="s">
         <v>104</v>
       </c>
-      <c r="C35" s="27"/>
-      <c r="D35" s="27"/>
-      <c r="E35" s="27"/>
-      <c r="F35" s="27"/>
-      <c r="G35" s="27"/>
-      <c r="H35" s="27"/>
-      <c r="I35" s="27"/>
+      <c r="C35" s="64"/>
+      <c r="D35" s="64"/>
+      <c r="E35" s="64"/>
+      <c r="F35" s="64"/>
+      <c r="G35" s="64"/>
+      <c r="H35" s="64"/>
+      <c r="I35" s="64"/>
     </row>
     <row r="36" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="27"/>
-      <c r="C36" s="27"/>
-      <c r="D36" s="27"/>
-      <c r="E36" s="27"/>
-      <c r="F36" s="27"/>
-      <c r="G36" s="27"/>
-      <c r="H36" s="27"/>
-      <c r="I36" s="27"/>
+      <c r="B36" s="64"/>
+      <c r="C36" s="64"/>
+      <c r="D36" s="64"/>
+      <c r="E36" s="64"/>
+      <c r="F36" s="64"/>
+      <c r="G36" s="64"/>
+      <c r="H36" s="64"/>
+      <c r="I36" s="64"/>
     </row>
     <row r="37" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="27"/>
-      <c r="C37" s="27"/>
-      <c r="D37" s="27"/>
-      <c r="E37" s="27"/>
-      <c r="F37" s="27"/>
-      <c r="G37" s="27"/>
-      <c r="H37" s="27"/>
-      <c r="I37" s="27"/>
+      <c r="B37" s="64"/>
+      <c r="C37" s="64"/>
+      <c r="D37" s="64"/>
+      <c r="E37" s="64"/>
+      <c r="F37" s="64"/>
+      <c r="G37" s="64"/>
+      <c r="H37" s="64"/>
+      <c r="I37" s="64"/>
     </row>
     <row r="38" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="27"/>
-      <c r="C38" s="27"/>
-      <c r="D38" s="27"/>
-      <c r="E38" s="27"/>
-      <c r="F38" s="27"/>
-      <c r="G38" s="27"/>
-      <c r="H38" s="27"/>
-      <c r="I38" s="27"/>
+      <c r="B38" s="64"/>
+      <c r="C38" s="64"/>
+      <c r="D38" s="64"/>
+      <c r="E38" s="64"/>
+      <c r="F38" s="64"/>
+      <c r="G38" s="64"/>
+      <c r="H38" s="64"/>
+      <c r="I38" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="42">
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B9:I9"/>
+    <mergeCell ref="B10:I12"/>
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="C15:I15"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B19:I19"/>
     <mergeCell ref="B20:I20"/>
     <mergeCell ref="B35:I38"/>
     <mergeCell ref="C22:I22"/>
@@ -5687,32 +5713,6 @@
     <mergeCell ref="C32:I32"/>
     <mergeCell ref="B33:I33"/>
     <mergeCell ref="B34:I34"/>
-    <mergeCell ref="C6:I6"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="E27:I27"/>
-    <mergeCell ref="B1:I1"/>
-    <mergeCell ref="C7:I7"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C21:I21"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="B9:I9"/>
-    <mergeCell ref="B10:I12"/>
-    <mergeCell ref="B13:I13"/>
-    <mergeCell ref="B14:I14"/>
-    <mergeCell ref="C15:I15"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="C3:I3"/>
-    <mergeCell ref="C4:I4"/>
-    <mergeCell ref="C5:I5"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="rId1" xr:uid="{69FD07AD-7FCA-E141-8126-AFB63E0A1511}"/>

</xml_diff>